<commit_message>
Add 3 more promoters (72 total): Royal Ventures, JHOMEA, Screendomus
Also folds the Setúbal "Parque da Cidade" project into the existing
Grupo Madre entry. Regenerates the xlsx export; map artifact updated
in the same pass at the same published URL.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01SRBJwGmSsYkTHKJbGCM5ca
</commit_message>
<xml_diff>
--- a/Promotoras_Imobiliarias_Contactos.xlsx
+++ b/Promotoras_Imobiliarias_Contactos.xlsx
@@ -191,8 +191,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Promotoras" displayName="Promotoras" ref="A1:J70" headerRowCount="1">
-  <autoFilter ref="A1:J70"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Promotoras" displayName="Promotoras" ref="A1:J73" headerRowCount="1">
+  <autoFilter ref="A1:J73"/>
   <tableColumns count="10">
     <tableColumn id="1" name="Nome da Empresa"/>
     <tableColumn id="2" name="Prioritario"/>
@@ -498,7 +498,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J70"/>
+  <dimension ref="A1:J73"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1320,7 +1320,7 @@
       </c>
       <c r="I16" s="2" t="inlineStr">
         <is>
-          <t>A-Living (Areeiro) (Planeamento)</t>
+          <t>A-Living (Areeiro) (Planeamento) | Parque da Cidade (Setúbal) (Em construção)</t>
         </is>
       </c>
       <c r="J16" s="2" t="inlineStr">
@@ -2248,7 +2248,7 @@
     <row r="35" ht="30" customHeight="1">
       <c r="A35" s="2" t="inlineStr">
         <is>
-          <t>Sharp Developers</t>
+          <t>Royal Ventures</t>
         </is>
       </c>
       <c r="B35" s="3" t="inlineStr">
@@ -2258,17 +2258,17 @@
       </c>
       <c r="C35" s="4" t="inlineStr">
         <is>
-          <t>+351 933 078 094</t>
+          <t>+351 916 770 322</t>
         </is>
       </c>
       <c r="D35" s="2" t="inlineStr">
         <is>
-          <t>info@sharpdevelopers.pt</t>
+          <t>alex@royal-ventures.com</t>
         </is>
       </c>
       <c r="E35" s="2" t="inlineStr">
         <is>
-          <t>sharpdevelopers.pt</t>
+          <t>royal-ventures.com</t>
         </is>
       </c>
       <c r="F35" s="4" t="inlineStr">
@@ -2283,24 +2283,24 @@
       </c>
       <c r="H35" s="2" t="inlineStr">
         <is>
-          <t>Av. Boavista 1681, Ed. Bristol, Esc. 5.4</t>
+          <t>Edifício Oceanus, Av. da Boavista 3227, 4100-137</t>
         </is>
       </c>
       <c r="I35" s="2" t="inlineStr">
         <is>
-          <t>Residencial de luxo Porto (Em construção)</t>
+          <t>Reabilitação centro histórico do Porto (Em construção)</t>
         </is>
       </c>
       <c r="J35" s="2" t="inlineStr">
         <is>
-          <t>CEO Carla Luís</t>
+          <t>Sócios israelitas (Udi, Liad) + contacto PT Alexandre. Fonte: royal-ventures.com/contact-us</t>
         </is>
       </c>
     </row>
     <row r="36" ht="30" customHeight="1">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>SILCOGE / Grupo SIL</t>
+          <t>Sharp Developers</t>
         </is>
       </c>
       <c r="B36" s="3" t="inlineStr">
@@ -2310,49 +2310,49 @@
       </c>
       <c r="C36" s="4" t="inlineStr">
         <is>
-          <t>+351 210 124 500</t>
+          <t>+351 933 078 094</t>
         </is>
       </c>
       <c r="D36" s="2" t="inlineStr">
         <is>
-          <t>info@sil.pt</t>
+          <t>info@sharpdevelopers.pt</t>
         </is>
       </c>
       <c r="E36" s="2" t="inlineStr">
         <is>
-          <t>sil.pt</t>
+          <t>sharpdevelopers.pt</t>
         </is>
       </c>
       <c r="F36" s="4" t="inlineStr">
         <is>
-          <t>Lisboa</t>
+          <t>Porto</t>
         </is>
       </c>
       <c r="G36" s="4" t="inlineStr">
         <is>
-          <t>Lisboa</t>
+          <t>Porto</t>
         </is>
       </c>
       <c r="H36" s="2" t="inlineStr">
         <is>
-          <t>Av. Fontes Pereira de Melo 6, 5º, 1050-121</t>
+          <t>Av. Boavista 1681, Ed. Bristol, Esc. 5.4</t>
         </is>
       </c>
       <c r="I36" s="2" t="inlineStr">
         <is>
-          <t>Grande Lisboa (Em construção)</t>
+          <t>Residencial de luxo Porto (Em construção)</t>
         </is>
       </c>
       <c r="J36" s="2" t="inlineStr">
         <is>
-          <t>Promoção imobiliária desde 1949</t>
+          <t>CEO Carla Luís</t>
         </is>
       </c>
     </row>
     <row r="37" ht="30" customHeight="1">
       <c r="A37" s="2" t="inlineStr">
         <is>
-          <t>SOLYD Property Developers</t>
+          <t>SILCOGE / Grupo SIL</t>
         </is>
       </c>
       <c r="B37" s="3" t="inlineStr">
@@ -2362,22 +2362,22 @@
       </c>
       <c r="C37" s="4" t="inlineStr">
         <is>
-          <t>+351 211 214 926</t>
+          <t>+351 210 124 500</t>
         </is>
       </c>
       <c r="D37" s="2" t="inlineStr">
         <is>
-          <t>info@elou-solyd.pt</t>
+          <t>info@sil.pt</t>
         </is>
       </c>
       <c r="E37" s="2" t="inlineStr">
         <is>
-          <t>solyd.pt</t>
+          <t>sil.pt</t>
         </is>
       </c>
       <c r="F37" s="4" t="inlineStr">
         <is>
-          <t>Oeiras</t>
+          <t>Lisboa</t>
         </is>
       </c>
       <c r="G37" s="4" t="inlineStr">
@@ -2387,24 +2387,24 @@
       </c>
       <c r="H37" s="2" t="inlineStr">
         <is>
-          <t>Torre de Monsanto, Rua Afonso Praça 30, 7º, 1495-061 Algés</t>
+          <t>Av. Fontes Pereira de Melo 6, 5º, 1050-121</t>
         </is>
       </c>
       <c r="I37" s="2" t="inlineStr">
         <is>
-          <t>Luz Altear (Alta de Lisboa) (Em construção)</t>
+          <t>Grande Lisboa (Em construção)</t>
         </is>
       </c>
       <c r="J37" s="2" t="inlineStr">
         <is>
-          <t>Estoril Capital Partners + Oaktree. Tel. alternativo 210 966 905</t>
+          <t>Promoção imobiliária desde 1949</t>
         </is>
       </c>
     </row>
     <row r="38" ht="30" customHeight="1">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>Stone Capital</t>
+          <t>SOLYD Property Developers</t>
         </is>
       </c>
       <c r="B38" s="3" t="inlineStr">
@@ -2414,22 +2414,22 @@
       </c>
       <c r="C38" s="4" t="inlineStr">
         <is>
-          <t>+351 210 416 350</t>
+          <t>+351 211 214 926</t>
         </is>
       </c>
       <c r="D38" s="2" t="inlineStr">
         <is>
-          <t>info@stonecapital.pt</t>
+          <t>info@elou-solyd.pt</t>
         </is>
       </c>
       <c r="E38" s="2" t="inlineStr">
         <is>
-          <t>stonecapital.pt</t>
+          <t>solyd.pt</t>
         </is>
       </c>
       <c r="F38" s="4" t="inlineStr">
         <is>
-          <t>Lisboa</t>
+          <t>Oeiras</t>
         </is>
       </c>
       <c r="G38" s="4" t="inlineStr">
@@ -2439,24 +2439,24 @@
       </c>
       <c r="H38" s="2" t="inlineStr">
         <is>
-          <t>Av. da Liberdade 240, 1250-096</t>
+          <t>Torre de Monsanto, Rua Afonso Praça 30, 7º, 1495-061 Algés</t>
         </is>
       </c>
       <c r="I38" s="2" t="inlineStr">
         <is>
-          <t>Santa Isabel (Em construção) | Portefólio em desenvolvimento (Em construção)</t>
+          <t>Luz Altear (Alta de Lisboa) (Em construção)</t>
         </is>
       </c>
       <c r="J38" s="2" t="inlineStr">
         <is>
-          <t>Tel. móvel 965 915 993</t>
+          <t>Estoril Capital Partners + Oaktree. Tel. alternativo 210 966 905</t>
         </is>
       </c>
     </row>
     <row r="39" ht="30" customHeight="1">
       <c r="A39" s="2" t="inlineStr">
         <is>
-          <t>Teixeira Duarte Real Estate</t>
+          <t>Stone Capital</t>
         </is>
       </c>
       <c r="B39" s="3" t="inlineStr">
@@ -2466,22 +2466,22 @@
       </c>
       <c r="C39" s="4" t="inlineStr">
         <is>
-          <t>+351 217 912 300</t>
+          <t>+351 210 416 350</t>
         </is>
       </c>
       <c r="D39" s="2" t="inlineStr">
         <is>
-          <t>info@tdimobiliaria.pt</t>
+          <t>info@stonecapital.pt</t>
         </is>
       </c>
       <c r="E39" s="2" t="inlineStr">
         <is>
-          <t>tdimobiliaria.pt</t>
+          <t>stonecapital.pt</t>
         </is>
       </c>
       <c r="F39" s="4" t="inlineStr">
         <is>
-          <t>Oeiras</t>
+          <t>Lisboa</t>
         </is>
       </c>
       <c r="G39" s="4" t="inlineStr">
@@ -2491,24 +2491,24 @@
       </c>
       <c r="H39" s="2" t="inlineStr">
         <is>
-          <t>Lagoas Park, Edifício 2, 2740-265 Porto Salvo</t>
+          <t>Av. da Liberdade 240, 1250-096</t>
         </is>
       </c>
       <c r="I39" s="2" t="inlineStr">
         <is>
-          <t>Quinta de Cravel (V.N. Gaia) (Comercialização)</t>
+          <t>Santa Isabel (Em construção) | Portefólio em desenvolvimento (Em construção)</t>
         </is>
       </c>
       <c r="J39" s="2" t="inlineStr">
         <is>
-          <t>Braço imobiliário do grupo Teixeira Duarte</t>
+          <t>Tel. móvel 965 915 993</t>
         </is>
       </c>
     </row>
     <row r="40" ht="30" customHeight="1">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>Thomas &amp; Piron Portugal</t>
+          <t>Teixeira Duarte Real Estate</t>
         </is>
       </c>
       <c r="B40" s="3" t="inlineStr">
@@ -2518,49 +2518,49 @@
       </c>
       <c r="C40" s="4" t="inlineStr">
         <is>
-          <t>+351 214 422 464</t>
+          <t>+351 217 912 300</t>
         </is>
       </c>
       <c r="D40" s="2" t="inlineStr">
         <is>
-          <t>infopt@thomas-piron.eu</t>
+          <t>info@tdimobiliaria.pt</t>
         </is>
       </c>
       <c r="E40" s="2" t="inlineStr">
         <is>
-          <t>thomas-piron.pt</t>
+          <t>tdimobiliaria.pt</t>
         </is>
       </c>
       <c r="F40" s="4" t="inlineStr">
         <is>
-          <t>Matosinhos</t>
+          <t>Oeiras</t>
         </is>
       </c>
       <c r="G40" s="4" t="inlineStr">
         <is>
-          <t>Porto</t>
+          <t>Lisboa</t>
         </is>
       </c>
       <c r="H40" s="2" t="inlineStr">
         <is>
-          <t>Escritórios em Matosinhos e Sacavém</t>
+          <t>Lagoas Park, Edifício 2, 2740-265 Porto Salvo</t>
         </is>
       </c>
       <c r="I40" s="2" t="inlineStr">
         <is>
-          <t>Docks Matosinhos (Em construção) | Gaia Hills (V.N. Gaia) (Em construção) | Conde de Lima (Comercialização)</t>
+          <t>Quinta de Cravel (V.N. Gaia) (Comercialização)</t>
         </is>
       </c>
       <c r="J40" s="2" t="inlineStr">
         <is>
-          <t>Promotor belga em Portugal desde 2018. Fonte: diarioimobiliario.pt</t>
+          <t>Braço imobiliário do grupo Teixeira Duarte</t>
         </is>
       </c>
     </row>
     <row r="41" ht="30" customHeight="1">
       <c r="A41" s="2" t="inlineStr">
         <is>
-          <t>Vanguard Properties</t>
+          <t>Thomas &amp; Piron Portugal</t>
         </is>
       </c>
       <c r="B41" s="3" t="inlineStr">
@@ -2570,49 +2570,49 @@
       </c>
       <c r="C41" s="4" t="inlineStr">
         <is>
-          <t>+351 215 814 094</t>
+          <t>+351 214 422 464</t>
         </is>
       </c>
       <c r="D41" s="2" t="inlineStr">
         <is>
-          <t>info@vangproperties.com</t>
+          <t>infopt@thomas-piron.eu</t>
         </is>
       </c>
       <c r="E41" s="2" t="inlineStr">
         <is>
-          <t>vangproperties.com</t>
+          <t>thomas-piron.pt</t>
         </is>
       </c>
       <c r="F41" s="4" t="inlineStr">
         <is>
-          <t>Lisboa</t>
+          <t>Matosinhos</t>
         </is>
       </c>
       <c r="G41" s="4" t="inlineStr">
         <is>
-          <t>Lisboa</t>
+          <t>Porto</t>
         </is>
       </c>
       <c r="H41" s="2" t="inlineStr">
         <is>
-          <t>Ed. Tivoli Fórum, Av. da Liberdade 180A, 7º, 1250-146</t>
+          <t>Escritórios em Matosinhos e Sacavém</t>
         </is>
       </c>
       <c r="I41" s="2" t="inlineStr">
         <is>
-          <t>22 projetos (Lisboa, Oeiras, Algarve, Comporta) (Em construção) | Infinity (Lisboa) (Comercialização)</t>
+          <t>Docks Matosinhos (Em construção) | Gaia Hills (V.N. Gaia) (Em construção) | Conde de Lima (Comercialização)</t>
         </is>
       </c>
       <c r="J41" s="2" t="inlineStr">
         <is>
-          <t>Entidade legal Vanguardeagle Asset Management (NIF 514114215). Tel. móvel 915 292 222</t>
+          <t>Promotor belga em Portugal desde 2018. Fonte: diarioimobiliario.pt</t>
         </is>
       </c>
     </row>
     <row r="42" ht="30" customHeight="1">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>VIC Properties</t>
+          <t>Vanguard Properties</t>
         </is>
       </c>
       <c r="B42" s="3" t="inlineStr">
@@ -2622,17 +2622,17 @@
       </c>
       <c r="C42" s="4" t="inlineStr">
         <is>
-          <t>+351 219 347 112</t>
+          <t>+351 215 814 094</t>
         </is>
       </c>
       <c r="D42" s="2" t="inlineStr">
         <is>
-          <t>info@vic-properties.com</t>
+          <t>info@vangproperties.com</t>
         </is>
       </c>
       <c r="E42" s="2" t="inlineStr">
         <is>
-          <t>vic-properties.com</t>
+          <t>vangproperties.com</t>
         </is>
       </c>
       <c r="F42" s="4" t="inlineStr">
@@ -2647,120 +2647,128 @@
       </c>
       <c r="H42" s="2" t="inlineStr">
         <is>
-          <t>Av. D. João II, Ed. Mythos 42, 4.03, Parque das Nações, 1990-095</t>
+          <t>Ed. Tivoli Fórum, Av. da Liberdade 180A, 7º, 1250-146</t>
         </is>
       </c>
       <c r="I42" s="2" t="inlineStr">
         <is>
-          <t>Prata Riverside Village (Marvila) (Em construção)</t>
+          <t>22 projetos (Lisboa, Oeiras, Algarve, Comporta) (Em construção) | Infinity (Lisboa) (Comercialização)</t>
         </is>
       </c>
       <c r="J42" s="2" t="inlineStr">
         <is>
-          <t>Portefólio &gt;3B€. Fundada 2018</t>
+          <t>Entidade legal Vanguardeagle Asset Management (NIF 514114215). Tel. móvel 915 292 222</t>
         </is>
       </c>
     </row>
     <row r="43" ht="30" customHeight="1">
       <c r="A43" s="2" t="inlineStr">
         <is>
+          <t>VIC Properties</t>
+        </is>
+      </c>
+      <c r="B43" s="3" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+      <c r="C43" s="4" t="inlineStr">
+        <is>
+          <t>+351 219 347 112</t>
+        </is>
+      </c>
+      <c r="D43" s="2" t="inlineStr">
+        <is>
+          <t>info@vic-properties.com</t>
+        </is>
+      </c>
+      <c r="E43" s="2" t="inlineStr">
+        <is>
+          <t>vic-properties.com</t>
+        </is>
+      </c>
+      <c r="F43" s="4" t="inlineStr">
+        <is>
+          <t>Lisboa</t>
+        </is>
+      </c>
+      <c r="G43" s="4" t="inlineStr">
+        <is>
+          <t>Lisboa</t>
+        </is>
+      </c>
+      <c r="H43" s="2" t="inlineStr">
+        <is>
+          <t>Av. D. João II, Ed. Mythos 42, 4.03, Parque das Nações, 1990-095</t>
+        </is>
+      </c>
+      <c r="I43" s="2" t="inlineStr">
+        <is>
+          <t>Prata Riverside Village (Marvila) (Em construção)</t>
+        </is>
+      </c>
+      <c r="J43" s="2" t="inlineStr">
+        <is>
+          <t>Portefólio &gt;3B€. Fundada 2018</t>
+        </is>
+      </c>
+    </row>
+    <row r="44" ht="30" customHeight="1">
+      <c r="A44" s="2" t="inlineStr">
+        <is>
           <t>Vogue Homes</t>
         </is>
       </c>
-      <c r="B43" s="3" t="inlineStr">
-        <is>
-          <t>Sim</t>
-        </is>
-      </c>
-      <c r="C43" s="4" t="inlineStr">
+      <c r="B44" s="3" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+      <c r="C44" s="4" t="inlineStr">
         <is>
           <t>+351 213 461 246</t>
         </is>
       </c>
-      <c r="D43" s="2" t="inlineStr">
+      <c r="D44" s="2" t="inlineStr">
         <is>
           <t>comercial@vogue-homes.com</t>
         </is>
       </c>
-      <c r="E43" s="2" t="inlineStr">
+      <c r="E44" s="2" t="inlineStr">
         <is>
           <t>vogue-homes.com</t>
         </is>
       </c>
-      <c r="F43" s="4" t="inlineStr">
-        <is>
-          <t>Lisboa</t>
-        </is>
-      </c>
-      <c r="G43" s="4" t="inlineStr">
-        <is>
-          <t>Lisboa</t>
-        </is>
-      </c>
-      <c r="H43" s="2" t="inlineStr">
+      <c r="F44" s="4" t="inlineStr">
+        <is>
+          <t>Lisboa</t>
+        </is>
+      </c>
+      <c r="G44" s="4" t="inlineStr">
+        <is>
+          <t>Lisboa</t>
+        </is>
+      </c>
+      <c r="H44" s="2" t="inlineStr">
         <is>
           <t>Rua Luz Soriano 15, 1200-246</t>
         </is>
       </c>
-      <c r="I43" s="2" t="inlineStr">
+      <c r="I44" s="2" t="inlineStr">
         <is>
           <t>Dafundo 24 (Comercialização) | Bom Sucesso (Comercialização) | Westhouse (Cascais) (Comercialização)</t>
         </is>
       </c>
-      <c r="J43" s="2" t="inlineStr">
+      <c r="J44" s="2" t="inlineStr">
         <is>
           <t>NIF 510933084. Tel. móvel 913 385 846</t>
-        </is>
-      </c>
-    </row>
-    <row r="44" ht="30" customHeight="1">
-      <c r="A44" s="5" t="inlineStr">
-        <is>
-          <t>Alecrim Real Estate (Lince Capital)</t>
-        </is>
-      </c>
-      <c r="B44" s="6" t="inlineStr">
-        <is>
-          <t>Sim</t>
-        </is>
-      </c>
-      <c r="C44" s="7" t="inlineStr"/>
-      <c r="D44" s="5" t="inlineStr"/>
-      <c r="E44" s="5" t="inlineStr">
-        <is>
-          <t>lince-capital.com</t>
-        </is>
-      </c>
-      <c r="F44" s="7" t="inlineStr">
-        <is>
-          <t>Lisboa</t>
-        </is>
-      </c>
-      <c r="G44" s="7" t="inlineStr">
-        <is>
-          <t>Lisboa</t>
-        </is>
-      </c>
-      <c r="H44" s="5" t="inlineStr">
-        <is>
-          <t>Av. Eng.º Duarte Pacheco, Torre 2, piso 17, 1070-102</t>
-        </is>
-      </c>
-      <c r="I44" s="5" t="inlineStr">
-        <is>
-          <t>Metrass (Campo de Ourique) (Em construção) | 8 projetos em pipeline (Planeamento)</t>
-        </is>
-      </c>
-      <c r="J44" s="5" t="inlineStr">
-        <is>
-          <t>Nova promotora (jan/2026), CEO António Velho da Palma</t>
         </is>
       </c>
     </row>
     <row r="45" ht="30" customHeight="1">
       <c r="A45" s="5" t="inlineStr">
         <is>
-          <t>Fortera</t>
+          <t>Alecrim Real Estate (Lince Capital)</t>
         </is>
       </c>
       <c r="B45" s="6" t="inlineStr">
@@ -2770,37 +2778,41 @@
       </c>
       <c r="C45" s="7" t="inlineStr"/>
       <c r="D45" s="5" t="inlineStr"/>
-      <c r="E45" s="5" t="inlineStr"/>
+      <c r="E45" s="5" t="inlineStr">
+        <is>
+          <t>lince-capital.com</t>
+        </is>
+      </c>
       <c r="F45" s="7" t="inlineStr">
         <is>
-          <t>Vila Nova de Gaia</t>
+          <t>Lisboa</t>
         </is>
       </c>
       <c r="G45" s="7" t="inlineStr">
         <is>
-          <t>Porto</t>
+          <t>Lisboa</t>
         </is>
       </c>
       <c r="H45" s="5" t="inlineStr">
         <is>
-          <t>Porto / Gaia</t>
+          <t>Av. Eng.º Duarte Pacheco, Torre 2, piso 17, 1070-102</t>
         </is>
       </c>
       <c r="I45" s="5" t="inlineStr">
         <is>
-          <t>Skyline (V.N. Gaia) (Em construção) | 20 projetos (Porto, Gaia, Espinho, Braga) (Em construção) | Convento do Carmo (Braga) (Em construção)</t>
+          <t>Metrass (Campo de Ourique) (Em construção) | 8 projetos em pipeline (Planeamento)</t>
         </is>
       </c>
       <c r="J45" s="5" t="inlineStr">
         <is>
-          <t>Israelita (Elad Dror). Sem telefone publicado nas fontes</t>
+          <t>Nova promotora (jan/2026), CEO António Velho da Palma</t>
         </is>
       </c>
     </row>
     <row r="46" ht="30" customHeight="1">
       <c r="A46" s="5" t="inlineStr">
         <is>
-          <t>Hines Portugal</t>
+          <t>Fortera</t>
         </is>
       </c>
       <c r="B46" s="6" t="inlineStr">
@@ -2810,41 +2822,37 @@
       </c>
       <c r="C46" s="7" t="inlineStr"/>
       <c r="D46" s="5" t="inlineStr"/>
-      <c r="E46" s="5" t="inlineStr">
-        <is>
-          <t>hines.com</t>
-        </is>
-      </c>
+      <c r="E46" s="5" t="inlineStr"/>
       <c r="F46" s="7" t="inlineStr">
         <is>
-          <t>Lisboa</t>
+          <t>Vila Nova de Gaia</t>
         </is>
       </c>
       <c r="G46" s="7" t="inlineStr">
         <is>
-          <t>Lisboa</t>
+          <t>Porto</t>
         </is>
       </c>
       <c r="H46" s="5" t="inlineStr">
         <is>
-          <t>Lisboa</t>
+          <t>Porto / Gaia</t>
         </is>
       </c>
       <c r="I46" s="5" t="inlineStr">
         <is>
-          <t>Residência de estudantes Paranhos (Porto) (Em construção) | Castilho 3 (Lisboa) (Em construção)</t>
+          <t>Skyline (V.N. Gaia) (Em construção) | 20 projetos (Porto, Gaia, Espinho, Braga) (Em construção) | Convento do Carmo (Braga) (Em construção)</t>
         </is>
       </c>
       <c r="J46" s="5" t="inlineStr">
         <is>
-          <t>Gestora global · sem contacto PT publicado</t>
+          <t>Israelita (Elad Dror). Sem telefone publicado nas fontes</t>
         </is>
       </c>
     </row>
     <row r="47" ht="30" customHeight="1">
       <c r="A47" s="5" t="inlineStr">
         <is>
-          <t>Imolote</t>
+          <t>Hines Portugal</t>
         </is>
       </c>
       <c r="B47" s="6" t="inlineStr">
@@ -2856,35 +2864,39 @@
       <c r="D47" s="5" t="inlineStr"/>
       <c r="E47" s="5" t="inlineStr">
         <is>
-          <t>imolote.pt</t>
+          <t>hines.com</t>
         </is>
       </c>
       <c r="F47" s="7" t="inlineStr">
         <is>
-          <t>Porto</t>
+          <t>Lisboa</t>
         </is>
       </c>
       <c r="G47" s="7" t="inlineStr">
         <is>
-          <t>Porto</t>
-        </is>
-      </c>
-      <c r="H47" s="5" t="inlineStr"/>
+          <t>Lisboa</t>
+        </is>
+      </c>
+      <c r="H47" s="5" t="inlineStr">
+        <is>
+          <t>Lisboa</t>
+        </is>
+      </c>
       <c r="I47" s="5" t="inlineStr">
         <is>
-          <t>Monte da Virgem Flats (V.N. Gaia) (Em construção) | 21 projetos entregues (Concluído)</t>
+          <t>Residência de estudantes Paranhos (Porto) (Em construção) | Castilho 3 (Lisboa) (Em construção)</t>
         </is>
       </c>
       <c r="J47" s="5" t="inlineStr">
         <is>
-          <t>Co-promoção com investidores · CEO Paulo Vaz Ferreira</t>
+          <t>Gestora global · sem contacto PT publicado</t>
         </is>
       </c>
     </row>
     <row r="48" ht="30" customHeight="1">
       <c r="A48" s="5" t="inlineStr">
         <is>
-          <t>Overseas</t>
+          <t>Imolote</t>
         </is>
       </c>
       <c r="B48" s="6" t="inlineStr">
@@ -2894,37 +2906,37 @@
       </c>
       <c r="C48" s="7" t="inlineStr"/>
       <c r="D48" s="5" t="inlineStr"/>
-      <c r="E48" s="5" t="inlineStr"/>
+      <c r="E48" s="5" t="inlineStr">
+        <is>
+          <t>imolote.pt</t>
+        </is>
+      </c>
       <c r="F48" s="7" t="inlineStr">
         <is>
-          <t>Lisboa</t>
+          <t>Porto</t>
         </is>
       </c>
       <c r="G48" s="7" t="inlineStr">
         <is>
-          <t>Lisboa</t>
-        </is>
-      </c>
-      <c r="H48" s="5" t="inlineStr">
-        <is>
-          <t>Rua Alexandre Herculano 25, 1º, 1250-008</t>
-        </is>
-      </c>
+          <t>Porto</t>
+        </is>
+      </c>
+      <c r="H48" s="5" t="inlineStr"/>
       <c r="I48" s="5" t="inlineStr">
         <is>
-          <t>5 projetos premium (4 Lisboa + Comporta) (Em construção) | JV com Grupo André Guimarães (Lisboa) (Planeamento) | Karl Lagerfeld branded residences (Planeamento) | Telhal 72 Liberdade (Comercialização)</t>
+          <t>Monte da Virgem Flats (V.N. Gaia) (Em construção) | 21 projetos entregues (Concluído)</t>
         </is>
       </c>
       <c r="J48" s="5" t="inlineStr">
         <is>
-          <t>CEO Pedro Vicente (vice-presidente APPII). Sem telefone publicado</t>
+          <t>Co-promoção com investidores · CEO Paulo Vaz Ferreira</t>
         </is>
       </c>
     </row>
     <row r="49" ht="30" customHeight="1">
       <c r="A49" s="5" t="inlineStr">
         <is>
-          <t>Prime Portugal</t>
+          <t>Overseas</t>
         </is>
       </c>
       <c r="B49" s="6" t="inlineStr">
@@ -2947,24 +2959,24 @@
       </c>
       <c r="H49" s="5" t="inlineStr">
         <is>
-          <t>Av. Fontes Pereira de Melo 6, 1600-001</t>
+          <t>Rua Alexandre Herculano 25, 1º, 1250-008</t>
         </is>
       </c>
       <c r="I49" s="5" t="inlineStr">
         <is>
-          <t>Projetos residenciais Lisboa, Cascais e Melides (Em construção)</t>
+          <t>5 projetos premium (4 Lisboa + Comporta) (Em construção) | JV com Grupo André Guimarães (Lisboa) (Planeamento) | Karl Lagerfeld branded residences (Planeamento) | Telhal 72 Liberdade (Comercialização)</t>
         </is>
       </c>
       <c r="J49" s="5" t="inlineStr">
         <is>
-          <t>Sem telefone/site publicados (APPII)</t>
+          <t>CEO Pedro Vicente (vice-presidente APPII). Sem telefone publicado</t>
         </is>
       </c>
     </row>
     <row r="50" ht="30" customHeight="1">
       <c r="A50" s="5" t="inlineStr">
         <is>
-          <t>Round Hill Capital</t>
+          <t>Prime Portugal</t>
         </is>
       </c>
       <c r="B50" s="6" t="inlineStr">
@@ -2974,11 +2986,7 @@
       </c>
       <c r="C50" s="7" t="inlineStr"/>
       <c r="D50" s="5" t="inlineStr"/>
-      <c r="E50" s="5" t="inlineStr">
-        <is>
-          <t>roundhillcapital.com</t>
-        </is>
-      </c>
+      <c r="E50" s="5" t="inlineStr"/>
       <c r="F50" s="7" t="inlineStr">
         <is>
           <t>Lisboa</t>
@@ -2991,24 +2999,24 @@
       </c>
       <c r="H50" s="5" t="inlineStr">
         <is>
-          <t>Rua da Escola Politécnica 38, 1250-102</t>
+          <t>Av. Fontes Pereira de Melo 6, 1600-001</t>
         </is>
       </c>
       <c r="I50" s="5" t="inlineStr">
         <is>
-          <t>Student + residential Lisboa (com TPG) (Planeamento) | Tannery Amial (Porto) (Em construção)</t>
+          <t>Projetos residenciais Lisboa, Cascais e Melides (Em construção)</t>
         </is>
       </c>
       <c r="J50" s="5" t="inlineStr">
         <is>
-          <t>Sem telefone PT publicado</t>
+          <t>Sem telefone/site publicados (APPII)</t>
         </is>
       </c>
     </row>
     <row r="51" ht="30" customHeight="1">
       <c r="A51" s="5" t="inlineStr">
         <is>
-          <t>United Investments Portugal (UIP)</t>
+          <t>Round Hill Capital</t>
         </is>
       </c>
       <c r="B51" s="6" t="inlineStr">
@@ -3020,7 +3028,7 @@
       <c r="D51" s="5" t="inlineStr"/>
       <c r="E51" s="5" t="inlineStr">
         <is>
-          <t>uip.pt</t>
+          <t>roundhillcapital.com</t>
         </is>
       </c>
       <c r="F51" s="7" t="inlineStr">
@@ -3035,24 +3043,24 @@
       </c>
       <c r="H51" s="5" t="inlineStr">
         <is>
-          <t>Lisboa</t>
+          <t>Rua da Escola Politécnica 38, 1250-102</t>
         </is>
       </c>
       <c r="I51" s="5" t="inlineStr">
         <is>
-          <t>Pine Cliffs (Algarve), Sheraton Cascais, YOTEL Porto, Hyatt Regency Lisboa (Em construção)</t>
+          <t>Student + residential Lisboa (com TPG) (Planeamento) | Tannery Amial (Porto) (Em construção)</t>
         </is>
       </c>
       <c r="J51" s="5" t="inlineStr">
         <is>
-          <t>Fundada 1985 · sem telefone publicado</t>
+          <t>Sem telefone PT publicado</t>
         </is>
       </c>
     </row>
     <row r="52" ht="30" customHeight="1">
       <c r="A52" s="5" t="inlineStr">
         <is>
-          <t>VIZTA (ex-Nexity Portugal)</t>
+          <t>Screendomus (Grupo Teixeira)</t>
         </is>
       </c>
       <c r="B52" s="6" t="inlineStr">
@@ -3063,12 +3071,12 @@
       <c r="C52" s="7" t="inlineStr"/>
       <c r="D52" s="5" t="inlineStr">
         <is>
-          <t>privacidade@vizta.pt</t>
+          <t>geral@screendomus.com</t>
         </is>
       </c>
       <c r="E52" s="5" t="inlineStr">
         <is>
-          <t>vizta.pt</t>
+          <t>screendomus.com</t>
         </is>
       </c>
       <c r="F52" s="7" t="inlineStr">
@@ -3081,174 +3089,158 @@
           <t>Lisboa</t>
         </is>
       </c>
-      <c r="H52" s="5" t="inlineStr">
-        <is>
-          <t>Ed. Amoreiras Plaza, Rua Carlos Alberto da Mota Pinto 9, piso 4, Esc. 4B2, 1070-374</t>
-        </is>
-      </c>
+      <c r="H52" s="5" t="inlineStr"/>
       <c r="I52" s="5" t="inlineStr">
         <is>
-          <t>Flower Tower Aurora (Leça da Palmeira) (Em construção) | Lisboa Oriental (Olivais/Portela) (Planeamento) | Turquesa (Oeiras) (Concluído)</t>
+          <t>Altus (Alta de Lisboa) (Em construção)</t>
         </is>
       </c>
       <c r="J52" s="5" t="inlineStr">
         <is>
-          <t>Adquirida pela Orion em 2023. Formulário em vizta.pt/contactos</t>
+          <t>Integra o Grupo Teixeira. Sem telefone confirmado — contacto via screendomus.com</t>
         </is>
       </c>
     </row>
     <row r="53" ht="30" customHeight="1">
       <c r="A53" s="5" t="inlineStr">
         <is>
+          <t>United Investments Portugal (UIP)</t>
+        </is>
+      </c>
+      <c r="B53" s="6" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+      <c r="C53" s="7" t="inlineStr"/>
+      <c r="D53" s="5" t="inlineStr"/>
+      <c r="E53" s="5" t="inlineStr">
+        <is>
+          <t>uip.pt</t>
+        </is>
+      </c>
+      <c r="F53" s="7" t="inlineStr">
+        <is>
+          <t>Lisboa</t>
+        </is>
+      </c>
+      <c r="G53" s="7" t="inlineStr">
+        <is>
+          <t>Lisboa</t>
+        </is>
+      </c>
+      <c r="H53" s="5" t="inlineStr">
+        <is>
+          <t>Lisboa</t>
+        </is>
+      </c>
+      <c r="I53" s="5" t="inlineStr">
+        <is>
+          <t>Pine Cliffs (Algarve), Sheraton Cascais, YOTEL Porto, Hyatt Regency Lisboa (Em construção)</t>
+        </is>
+      </c>
+      <c r="J53" s="5" t="inlineStr">
+        <is>
+          <t>Fundada 1985 · sem telefone publicado</t>
+        </is>
+      </c>
+    </row>
+    <row r="54" ht="30" customHeight="1">
+      <c r="A54" s="5" t="inlineStr">
+        <is>
+          <t>VIZTA (ex-Nexity Portugal)</t>
+        </is>
+      </c>
+      <c r="B54" s="6" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+      <c r="C54" s="7" t="inlineStr"/>
+      <c r="D54" s="5" t="inlineStr">
+        <is>
+          <t>privacidade@vizta.pt</t>
+        </is>
+      </c>
+      <c r="E54" s="5" t="inlineStr">
+        <is>
+          <t>vizta.pt</t>
+        </is>
+      </c>
+      <c r="F54" s="7" t="inlineStr">
+        <is>
+          <t>Lisboa</t>
+        </is>
+      </c>
+      <c r="G54" s="7" t="inlineStr">
+        <is>
+          <t>Lisboa</t>
+        </is>
+      </c>
+      <c r="H54" s="5" t="inlineStr">
+        <is>
+          <t>Ed. Amoreiras Plaza, Rua Carlos Alberto da Mota Pinto 9, piso 4, Esc. 4B2, 1070-374</t>
+        </is>
+      </c>
+      <c r="I54" s="5" t="inlineStr">
+        <is>
+          <t>Flower Tower Aurora (Leça da Palmeira) (Em construção) | Lisboa Oriental (Olivais/Portela) (Planeamento) | Turquesa (Oeiras) (Concluído)</t>
+        </is>
+      </c>
+      <c r="J54" s="5" t="inlineStr">
+        <is>
+          <t>Adquirida pela Orion em 2023. Formulário em vizta.pt/contactos</t>
+        </is>
+      </c>
+    </row>
+    <row r="55" ht="30" customHeight="1">
+      <c r="A55" s="5" t="inlineStr">
+        <is>
           <t>Âncora Investments</t>
         </is>
       </c>
-      <c r="B53" s="6" t="inlineStr">
-        <is>
-          <t>Sim</t>
-        </is>
-      </c>
-      <c r="C53" s="7" t="inlineStr"/>
-      <c r="D53" s="5" t="inlineStr">
+      <c r="B55" s="6" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+      <c r="C55" s="7" t="inlineStr"/>
+      <c r="D55" s="5" t="inlineStr">
         <is>
           <t>info@ancora-inv.com</t>
         </is>
       </c>
-      <c r="E53" s="5" t="inlineStr">
+      <c r="E55" s="5" t="inlineStr">
         <is>
           <t>ancora-inv.com</t>
         </is>
       </c>
-      <c r="F53" s="7" t="inlineStr">
+      <c r="F55" s="7" t="inlineStr">
         <is>
           <t>Porto</t>
         </is>
       </c>
-      <c r="G53" s="7" t="inlineStr">
+      <c r="G55" s="7" t="inlineStr">
         <is>
           <t>Porto</t>
         </is>
       </c>
-      <c r="H53" s="5" t="inlineStr"/>
-      <c r="I53" s="5" t="inlineStr">
+      <c r="H55" s="5" t="inlineStr"/>
+      <c r="I55" s="5" t="inlineStr">
         <is>
           <t>Canelas (V.N. Gaia) + Águas Santas (Maia), com PMA (Planeamento)</t>
         </is>
       </c>
-      <c r="J53" s="5" t="inlineStr">
+      <c r="J55" s="5" t="inlineStr">
         <is>
           <t>Elad Shachar / Tamir Luria · &gt;70M€ sob gestão</t>
-        </is>
-      </c>
-    </row>
-    <row r="54" ht="30" customHeight="1">
-      <c r="A54" s="2" t="inlineStr">
-        <is>
-          <t>AEDAS Homes + LandCo (Ribamar)</t>
-        </is>
-      </c>
-      <c r="B54" s="4" t="inlineStr">
-        <is>
-          <t>Nao</t>
-        </is>
-      </c>
-      <c r="C54" s="4" t="inlineStr">
-        <is>
-          <t>900 264 096 (ES)</t>
-        </is>
-      </c>
-      <c r="D54" s="2" t="inlineStr">
-        <is>
-          <t>info@aedashomes.com</t>
-        </is>
-      </c>
-      <c r="E54" s="2" t="inlineStr">
-        <is>
-          <t>ribamarportimao.com</t>
-        </is>
-      </c>
-      <c r="F54" s="4" t="inlineStr">
-        <is>
-          <t>Portimão</t>
-        </is>
-      </c>
-      <c r="G54" s="4" t="inlineStr">
-        <is>
-          <t>Faro</t>
-        </is>
-      </c>
-      <c r="H54" s="2" t="inlineStr">
-        <is>
-          <t>Loja de vendas: Rua dos Três Castelos, Praia da Rocha</t>
-        </is>
-      </c>
-      <c r="I54" s="2" t="inlineStr">
-        <is>
-          <t>Ribamar (Praia da Rocha) (Em construção)</t>
-        </is>
-      </c>
-      <c r="J54" s="2" t="inlineStr">
-        <is>
-          <t>Número é linha gratuita espanhola · loja de vendas aberta seg-sáb</t>
-        </is>
-      </c>
-    </row>
-    <row r="55" ht="30" customHeight="1">
-      <c r="A55" s="2" t="inlineStr">
-        <is>
-          <t>Antrix</t>
-        </is>
-      </c>
-      <c r="B55" s="4" t="inlineStr">
-        <is>
-          <t>Nao</t>
-        </is>
-      </c>
-      <c r="C55" s="4" t="inlineStr">
-        <is>
-          <t>+351 917 498 714</t>
-        </is>
-      </c>
-      <c r="D55" s="2" t="inlineStr">
-        <is>
-          <t>info@antrix.pt</t>
-        </is>
-      </c>
-      <c r="E55" s="2" t="inlineStr">
-        <is>
-          <t>antrix.pt</t>
-        </is>
-      </c>
-      <c r="F55" s="4" t="inlineStr">
-        <is>
-          <t>Lagoa</t>
-        </is>
-      </c>
-      <c r="G55" s="4" t="inlineStr">
-        <is>
-          <t>Faro</t>
-        </is>
-      </c>
-      <c r="H55" s="2" t="inlineStr">
-        <is>
-          <t>Rua Jacinto Correia, Bloco A, Loja JLM, Ed. Atrium Lagoa, 8400-398</t>
-        </is>
-      </c>
-      <c r="I55" s="2" t="inlineStr">
-        <is>
-          <t>Algarve (vários projetos) (Em construção) | Lisboa, Montijo, Setúbal (Planeamento)</t>
-        </is>
-      </c>
-      <c r="J55" s="2" t="inlineStr">
-        <is>
-          <t>Mesmo CEO (Erik de Vlieger) e mesmo telefone da Carvoeiro Branco</t>
         </is>
       </c>
     </row>
     <row r="56" ht="30" customHeight="1">
       <c r="A56" s="2" t="inlineStr">
         <is>
-          <t>Carvoeiro Branco – Propriedades</t>
+          <t>AEDAS Homes + LandCo (Ribamar)</t>
         </is>
       </c>
       <c r="B56" s="4" t="inlineStr">
@@ -3258,22 +3250,22 @@
       </c>
       <c r="C56" s="4" t="inlineStr">
         <is>
-          <t>+351 917 498 714</t>
+          <t>900 264 096 (ES)</t>
         </is>
       </c>
       <c r="D56" s="2" t="inlineStr">
         <is>
-          <t>info@carvoeirobranco.com</t>
+          <t>info@aedashomes.com</t>
         </is>
       </c>
       <c r="E56" s="2" t="inlineStr">
         <is>
-          <t>carvoeirobranco.com</t>
+          <t>ribamarportimao.com</t>
         </is>
       </c>
       <c r="F56" s="4" t="inlineStr">
         <is>
-          <t>Lagoa</t>
+          <t>Portimão</t>
         </is>
       </c>
       <c r="G56" s="4" t="inlineStr">
@@ -3283,24 +3275,24 @@
       </c>
       <c r="H56" s="2" t="inlineStr">
         <is>
-          <t>Rua Jacinto Correia, Bloco A, Loja JLM, Ed. Atrium Lagoa, 8400-398</t>
+          <t>Loja de vendas: Rua dos Três Castelos, Praia da Rocha</t>
         </is>
       </c>
       <c r="I56" s="2" t="inlineStr">
         <is>
-          <t>JV com TPS (Lagoa, Portimão, Faro) (Planeamento) | Arade Premium Village / Primelife / The Court (Em construção)</t>
+          <t>Ribamar (Praia da Rocha) (Em construção)</t>
         </is>
       </c>
       <c r="J56" s="2" t="inlineStr">
         <is>
-          <t>NIF 507849183. Tel. alternativo 960 280 640</t>
+          <t>Número é linha gratuita espanhola · loja de vendas aberta seg-sáb</t>
         </is>
       </c>
     </row>
     <row r="57" ht="30" customHeight="1">
       <c r="A57" s="2" t="inlineStr">
         <is>
-          <t>Casais Imobiliária (Grupo Casais)</t>
+          <t>Antrix</t>
         </is>
       </c>
       <c r="B57" s="4" t="inlineStr">
@@ -3310,49 +3302,49 @@
       </c>
       <c r="C57" s="4" t="inlineStr">
         <is>
-          <t>+351 253 305 490</t>
+          <t>+351 917 498 714</t>
         </is>
       </c>
       <c r="D57" s="2" t="inlineStr">
         <is>
-          <t>casais@casais.pt</t>
+          <t>info@antrix.pt</t>
         </is>
       </c>
       <c r="E57" s="2" t="inlineStr">
         <is>
-          <t>casais.pt</t>
+          <t>antrix.pt</t>
         </is>
       </c>
       <c r="F57" s="4" t="inlineStr">
         <is>
-          <t>Braga</t>
+          <t>Lagoa</t>
         </is>
       </c>
       <c r="G57" s="4" t="inlineStr">
         <is>
-          <t>Braga</t>
+          <t>Faro</t>
         </is>
       </c>
       <c r="H57" s="2" t="inlineStr">
         <is>
-          <t>Rua do Anjo 27, Mire de Tibães, 4700-565</t>
+          <t>Rua Jacinto Correia, Bloco A, Loja JLM, Ed. Atrium Lagoa, 8400-398</t>
         </is>
       </c>
       <c r="I57" s="2" t="inlineStr">
         <is>
-          <t>MITH – Minho Innovation and Technology Hub (Guimarães) (Em construção)</t>
+          <t>Algarve (vários projetos) (Em construção) | Lisboa, Montijo, Setúbal (Planeamento)</t>
         </is>
       </c>
       <c r="J57" s="2" t="inlineStr">
         <is>
-          <t>Capital social 5M€, NIF 505271915. Grupo de construção top-5 nacional</t>
+          <t>Mesmo CEO (Erik de Vlieger) e mesmo telefone da Carvoeiro Branco</t>
         </is>
       </c>
     </row>
     <row r="58" ht="30" customHeight="1">
       <c r="A58" s="2" t="inlineStr">
         <is>
-          <t>Castro Group</t>
+          <t>Carvoeiro Branco – Propriedades</t>
         </is>
       </c>
       <c r="B58" s="4" t="inlineStr">
@@ -3362,49 +3354,49 @@
       </c>
       <c r="C58" s="4" t="inlineStr">
         <is>
-          <t>+351 253 461 462</t>
+          <t>+351 917 498 714</t>
         </is>
       </c>
       <c r="D58" s="2" t="inlineStr">
         <is>
-          <t>geral@castro-group.pt</t>
+          <t>info@carvoeirobranco.com</t>
         </is>
       </c>
       <c r="E58" s="2" t="inlineStr">
         <is>
-          <t>castro-group.pt</t>
+          <t>carvoeirobranco.com</t>
         </is>
       </c>
       <c r="F58" s="4" t="inlineStr">
         <is>
-          <t>Braga</t>
+          <t>Lagoa</t>
         </is>
       </c>
       <c r="G58" s="4" t="inlineStr">
         <is>
-          <t>Braga</t>
+          <t>Faro</t>
         </is>
       </c>
       <c r="H58" s="2" t="inlineStr">
         <is>
-          <t>Av. 31 de Janeiro 307, 4715-052</t>
+          <t>Rua Jacinto Correia, Bloco A, Loja JLM, Ed. Atrium Lagoa, 8400-398</t>
         </is>
       </c>
       <c r="I58" s="2" t="inlineStr">
         <is>
-          <t>Promoção + construção + gestão de ativos (Em construção)</t>
+          <t>JV com TPS (Lagoa, Portimão, Faro) (Planeamento) | Arade Premium Village / Primelife / The Court (Em construção)</t>
         </is>
       </c>
       <c r="J58" s="2" t="inlineStr">
         <is>
-          <t>50 anos de história. Fonte: APPII</t>
+          <t>NIF 507849183. Tel. alternativo 960 280 640</t>
         </is>
       </c>
     </row>
     <row r="59" ht="30" customHeight="1">
       <c r="A59" s="2" t="inlineStr">
         <is>
-          <t>Civilria</t>
+          <t>Casais Imobiliária (Grupo Casais)</t>
         </is>
       </c>
       <c r="B59" s="4" t="inlineStr">
@@ -3414,49 +3406,49 @@
       </c>
       <c r="C59" s="4" t="inlineStr">
         <is>
-          <t>+351 234 480 570</t>
+          <t>+351 253 305 490</t>
         </is>
       </c>
       <c r="D59" s="2" t="inlineStr">
         <is>
-          <t>info@civilria.pt</t>
+          <t>casais@casais.pt</t>
         </is>
       </c>
       <c r="E59" s="2" t="inlineStr">
         <is>
-          <t>civilria.pt</t>
+          <t>casais.pt</t>
         </is>
       </c>
       <c r="F59" s="4" t="inlineStr">
         <is>
-          <t>Aveiro</t>
+          <t>Braga</t>
         </is>
       </c>
       <c r="G59" s="4" t="inlineStr">
         <is>
-          <t>Aveiro</t>
+          <t>Braga</t>
         </is>
       </c>
       <c r="H59" s="2" t="inlineStr">
         <is>
-          <t>Rua Cristóvão Pinho Queimado 33, piso 3, Esc. 7, 3800-012</t>
+          <t>Rua do Anjo 27, Mire de Tibães, 4700-565</t>
         </is>
       </c>
       <c r="I59" s="2" t="inlineStr">
         <is>
-          <t>Portefólio Aveiro (Em construção)</t>
+          <t>MITH – Minho Innovation and Technology Hub (Guimarães) (Em construção)</t>
         </is>
       </c>
       <c r="J59" s="2" t="inlineStr">
         <is>
-          <t>Promotor vertical (conceção→construção→venda), 25+ anos</t>
+          <t>Capital social 5M€, NIF 505271915. Grupo de construção top-5 nacional</t>
         </is>
       </c>
     </row>
     <row r="60" ht="30" customHeight="1">
       <c r="A60" s="2" t="inlineStr">
         <is>
-          <t>Enolagest / Garvetur (Greens Vilamoura)</t>
+          <t>Castro Group</t>
         </is>
       </c>
       <c r="B60" s="4" t="inlineStr">
@@ -3466,45 +3458,49 @@
       </c>
       <c r="C60" s="4" t="inlineStr">
         <is>
-          <t>+351 289 381 550</t>
-        </is>
-      </c>
-      <c r="D60" s="2" t="inlineStr"/>
+          <t>+351 253 461 462</t>
+        </is>
+      </c>
+      <c r="D60" s="2" t="inlineStr">
+        <is>
+          <t>geral@castro-group.pt</t>
+        </is>
+      </c>
       <c r="E60" s="2" t="inlineStr">
         <is>
-          <t>enolagest.pt</t>
+          <t>castro-group.pt</t>
         </is>
       </c>
       <c r="F60" s="4" t="inlineStr">
         <is>
-          <t>Loulé</t>
+          <t>Braga</t>
         </is>
       </c>
       <c r="G60" s="4" t="inlineStr">
         <is>
-          <t>Faro</t>
+          <t>Braga</t>
         </is>
       </c>
       <c r="H60" s="2" t="inlineStr">
         <is>
-          <t>Rua Melvin Jones, Volta do Gaio, Vilamoura, 8125-406</t>
+          <t>Av. 31 de Janeiro 307, 4715-052</t>
         </is>
       </c>
       <c r="I60" s="2" t="inlineStr">
         <is>
-          <t>Greens Vilamoura (Em construção)</t>
+          <t>Promoção + construção + gestão de ativos (Em construção)</t>
         </is>
       </c>
       <c r="J60" s="2" t="inlineStr">
         <is>
-          <t>Promotor: Greens Vilamoura Investimentos Imobiliários (grupo Enolagest). Tel. alt. 289 322 488</t>
+          <t>50 anos de história. Fonte: APPII</t>
         </is>
       </c>
     </row>
     <row r="61" ht="30" customHeight="1">
       <c r="A61" s="2" t="inlineStr">
         <is>
-          <t>Garcia Garcia</t>
+          <t>Civilria</t>
         </is>
       </c>
       <c r="B61" s="4" t="inlineStr">
@@ -3514,49 +3510,49 @@
       </c>
       <c r="C61" s="4" t="inlineStr">
         <is>
-          <t>+351 253 560 230</t>
+          <t>+351 234 480 570</t>
         </is>
       </c>
       <c r="D61" s="2" t="inlineStr">
         <is>
-          <t>geral@garcia.pt</t>
+          <t>info@civilria.pt</t>
         </is>
       </c>
       <c r="E61" s="2" t="inlineStr">
         <is>
-          <t>garcia.pt</t>
+          <t>civilria.pt</t>
         </is>
       </c>
       <c r="F61" s="4" t="inlineStr">
         <is>
-          <t>Santo Tirso</t>
+          <t>Aveiro</t>
         </is>
       </c>
       <c r="G61" s="4" t="inlineStr">
         <is>
-          <t>Porto</t>
+          <t>Aveiro</t>
         </is>
       </c>
       <c r="H61" s="2" t="inlineStr">
         <is>
-          <t>Rua Comendador António Maria Lopes 15, 4780-424</t>
+          <t>Rua Cristóvão Pinho Queimado 33, piso 3, Esc. 7, 3800-012</t>
         </is>
       </c>
       <c r="I61" s="2" t="inlineStr">
         <is>
-          <t>Couros Residence (Guimarães) (Concluído) | Arco Living (Santo Tirso) (Concluído) | Residência de estudantes Hines (Porto, Paranhos) (Em construção)</t>
+          <t>Portefólio Aveiro (Em construção)</t>
         </is>
       </c>
       <c r="J61" s="2" t="inlineStr">
         <is>
-          <t>Design &amp; Build, faturação 173M€ em 2025</t>
+          <t>Promotor vertical (conceção→construção→venda), 25+ anos</t>
         </is>
       </c>
     </row>
     <row r="62" ht="30" customHeight="1">
       <c r="A62" s="2" t="inlineStr">
         <is>
-          <t>Grupo ACA / ACA Real Estate (marca Pousio)</t>
+          <t>Enolagest / Garvetur (Greens Vilamoura)</t>
         </is>
       </c>
       <c r="B62" s="4" t="inlineStr">
@@ -3566,49 +3562,45 @@
       </c>
       <c r="C62" s="4" t="inlineStr">
         <is>
-          <t>+351 252 308 250</t>
-        </is>
-      </c>
-      <c r="D62" s="2" t="inlineStr">
-        <is>
-          <t>aca@grupo-aca.com</t>
-        </is>
-      </c>
+          <t>+351 289 381 550</t>
+        </is>
+      </c>
+      <c r="D62" s="2" t="inlineStr"/>
       <c r="E62" s="2" t="inlineStr">
         <is>
-          <t>grupo-aca.com</t>
+          <t>enolagest.pt</t>
         </is>
       </c>
       <c r="F62" s="4" t="inlineStr">
         <is>
-          <t>Vila Nova de Famalicão</t>
+          <t>Loulé</t>
         </is>
       </c>
       <c r="G62" s="4" t="inlineStr">
         <is>
-          <t>Braga</t>
+          <t>Faro</t>
         </is>
       </c>
       <c r="H62" s="2" t="inlineStr">
         <is>
-          <t>Av. dos Descobrimentos, Ed. Las Vegas 3, nº63</t>
+          <t>Rua Melvin Jones, Volta do Gaio, Vilamoura, 8125-406</t>
         </is>
       </c>
       <c r="I62" s="2" t="inlineStr">
         <is>
-          <t>Pousio (Aveiro, Gaia, Lisboa) (Planeamento)</t>
+          <t>Greens Vilamoura (Em construção)</t>
         </is>
       </c>
       <c r="J62" s="2" t="inlineStr">
         <is>
-          <t>Grupo de construção com 2.000 colaboradores. Fonte: Jornal de Negócios</t>
+          <t>Promotor: Greens Vilamoura Investimentos Imobiliários (grupo Enolagest). Tel. alt. 289 322 488</t>
         </is>
       </c>
     </row>
     <row r="63" ht="30" customHeight="1">
       <c r="A63" s="2" t="inlineStr">
         <is>
-          <t>Grupo Acrescentar</t>
+          <t>Garcia Garcia</t>
         </is>
       </c>
       <c r="B63" s="4" t="inlineStr">
@@ -3618,49 +3610,49 @@
       </c>
       <c r="C63" s="4" t="inlineStr">
         <is>
-          <t>+351 253 685 109</t>
+          <t>+351 253 560 230</t>
         </is>
       </c>
       <c r="D63" s="2" t="inlineStr">
         <is>
-          <t>acrescentar@grupoacrescentar.pt</t>
+          <t>geral@garcia.pt</t>
         </is>
       </c>
       <c r="E63" s="2" t="inlineStr">
         <is>
-          <t>grupoacrescentar.pt</t>
+          <t>garcia.pt</t>
         </is>
       </c>
       <c r="F63" s="4" t="inlineStr">
         <is>
-          <t>Braga</t>
+          <t>Santo Tirso</t>
         </is>
       </c>
       <c r="G63" s="4" t="inlineStr">
         <is>
-          <t>Braga</t>
+          <t>Porto</t>
         </is>
       </c>
       <c r="H63" s="2" t="inlineStr">
         <is>
-          <t>Rua Quinta dos Lagos 24, 4700-289 Real</t>
+          <t>Rua Comendador António Maria Lopes 15, 4780-424</t>
         </is>
       </c>
       <c r="I63" s="2" t="inlineStr">
         <is>
-          <t>Green Terrace Porto (Requesende) (Em construção) | Garden Palace (Comercialização) | Strata Private Residence (Comercialização) | Vess Living (Guimarães) (Em construção)</t>
+          <t>Couros Residence (Guimarães) (Concluído) | Arco Living (Santo Tirso) (Concluído) | Residência de estudantes Hines (Porto, Paranhos) (Em construção)</t>
         </is>
       </c>
       <c r="J63" s="2" t="inlineStr">
         <is>
-          <t>Promove, constrói e vende os próprios projetos. Fonte: diarioimobiliario.pt, idealista/news</t>
+          <t>Design &amp; Build, faturação 173M€ em 2025</t>
         </is>
       </c>
     </row>
     <row r="64" ht="30" customHeight="1">
       <c r="A64" s="2" t="inlineStr">
         <is>
-          <t>Grupo Arliz</t>
+          <t>Grupo ACA / ACA Real Estate (marca Pousio)</t>
         </is>
       </c>
       <c r="B64" s="4" t="inlineStr">
@@ -3670,49 +3662,49 @@
       </c>
       <c r="C64" s="4" t="inlineStr">
         <is>
-          <t>+351 253 105 331</t>
+          <t>+351 252 308 250</t>
         </is>
       </c>
       <c r="D64" s="2" t="inlineStr">
         <is>
-          <t>geral@arliz.co</t>
+          <t>aca@grupo-aca.com</t>
         </is>
       </c>
       <c r="E64" s="2" t="inlineStr">
         <is>
-          <t>grupoarliz.pt</t>
+          <t>grupo-aca.com</t>
         </is>
       </c>
       <c r="F64" s="4" t="inlineStr">
         <is>
+          <t>Vila Nova de Famalicão</t>
+        </is>
+      </c>
+      <c r="G64" s="4" t="inlineStr">
+        <is>
           <t>Braga</t>
         </is>
       </c>
-      <c r="G64" s="4" t="inlineStr">
-        <is>
-          <t>Braga</t>
-        </is>
-      </c>
       <c r="H64" s="2" t="inlineStr">
         <is>
-          <t>Parque Industrial de Celeirós 2ª fase</t>
+          <t>Av. dos Descobrimentos, Ed. Las Vegas 3, nº63</t>
         </is>
       </c>
       <c r="I64" s="2" t="inlineStr">
         <is>
-          <t>Arc Living (Porto) (Em construção)</t>
+          <t>Pousio (Aveiro, Gaia, Lisboa) (Planeamento)</t>
         </is>
       </c>
       <c r="J64" s="2" t="inlineStr">
         <is>
-          <t>Promotor + construtor. Fonte: idealista/news, construir.pt</t>
+          <t>Grupo de construção com 2.000 colaboradores. Fonte: Jornal de Negócios</t>
         </is>
       </c>
     </row>
     <row r="65" ht="30" customHeight="1">
       <c r="A65" s="2" t="inlineStr">
         <is>
-          <t>Grupo CVM (Construções Vila Maior)</t>
+          <t>Grupo Acrescentar</t>
         </is>
       </c>
       <c r="B65" s="4" t="inlineStr">
@@ -3722,45 +3714,49 @@
       </c>
       <c r="C65" s="4" t="inlineStr">
         <is>
-          <t>273 332 784 (confirmar)</t>
-        </is>
-      </c>
-      <c r="D65" s="2" t="inlineStr"/>
+          <t>+351 253 685 109</t>
+        </is>
+      </c>
+      <c r="D65" s="2" t="inlineStr">
+        <is>
+          <t>acrescentar@grupoacrescentar.pt</t>
+        </is>
+      </c>
       <c r="E65" s="2" t="inlineStr">
         <is>
-          <t>cvmnet.com</t>
+          <t>grupoacrescentar.pt</t>
         </is>
       </c>
       <c r="F65" s="4" t="inlineStr">
         <is>
-          <t>Santa Maria da Feira</t>
+          <t>Braga</t>
         </is>
       </c>
       <c r="G65" s="4" t="inlineStr">
         <is>
-          <t>Aveiro</t>
+          <t>Braga</t>
         </is>
       </c>
       <c r="H65" s="2" t="inlineStr">
         <is>
-          <t>Parque Empresarial A32, Vila Maior</t>
+          <t>Rua Quinta dos Lagos 24, 4700-289 Real</t>
         </is>
       </c>
       <c r="I65" s="2" t="inlineStr">
         <is>
-          <t>Royal Green (V.N. Gaia, Av. Descobrimentos) (Em construção)</t>
+          <t>Green Terrace Porto (Requesende) (Em construção) | Garden Palace (Comercialização) | Strata Private Residence (Comercialização) | Vess Living (Guimarães) (Em construção)</t>
         </is>
       </c>
       <c r="J65" s="2" t="inlineStr">
         <is>
-          <t>Telefone vindo do registo — confirmar em cvmnet.com/contactos</t>
+          <t>Promove, constrói e vende os próprios projetos. Fonte: diarioimobiliario.pt, idealista/news</t>
         </is>
       </c>
     </row>
     <row r="66" ht="30" customHeight="1">
       <c r="A66" s="2" t="inlineStr">
         <is>
-          <t>Pine Hill</t>
+          <t>Grupo Arliz</t>
         </is>
       </c>
       <c r="B66" s="4" t="inlineStr">
@@ -3770,17 +3766,17 @@
       </c>
       <c r="C66" s="4" t="inlineStr">
         <is>
-          <t>+351 910 936 732</t>
+          <t>+351 253 105 331</t>
         </is>
       </c>
       <c r="D66" s="2" t="inlineStr">
         <is>
-          <t>info@pinehill.pt</t>
+          <t>geral@arliz.co</t>
         </is>
       </c>
       <c r="E66" s="2" t="inlineStr">
         <is>
-          <t>pinehill.pt</t>
+          <t>grupoarliz.pt</t>
         </is>
       </c>
       <c r="F66" s="4" t="inlineStr">
@@ -3793,22 +3789,26 @@
           <t>Braga</t>
         </is>
       </c>
-      <c r="H66" s="2" t="inlineStr"/>
+      <c r="H66" s="2" t="inlineStr">
+        <is>
+          <t>Parque Industrial de Celeirós 2ª fase</t>
+        </is>
+      </c>
       <c r="I66" s="2" t="inlineStr">
         <is>
-          <t>Braga Premium Flats (Comercialização) | 3 novos projetos em Braga (Planeamento)</t>
+          <t>Arc Living (Porto) (Em construção)</t>
         </is>
       </c>
       <c r="J66" s="2" t="inlineStr">
         <is>
-          <t>Promotora criada em 2025. Fonte: newinbraga.nit.pt, Revista Spot</t>
+          <t>Promotor + construtor. Fonte: idealista/news, construir.pt</t>
         </is>
       </c>
     </row>
     <row r="67" ht="30" customHeight="1">
       <c r="A67" s="2" t="inlineStr">
         <is>
-          <t>Quinta do Lago Resort</t>
+          <t>Grupo CVM (Construções Vila Maior)</t>
         </is>
       </c>
       <c r="B67" s="4" t="inlineStr">
@@ -3818,168 +3818,316 @@
       </c>
       <c r="C67" s="4" t="inlineStr">
         <is>
-          <t>+351 289 390 700</t>
-        </is>
-      </c>
-      <c r="D67" s="2" t="inlineStr">
-        <is>
-          <t>info@quintadolago.com</t>
-        </is>
-      </c>
+          <t>273 332 784 (confirmar)</t>
+        </is>
+      </c>
+      <c r="D67" s="2" t="inlineStr"/>
       <c r="E67" s="2" t="inlineStr">
         <is>
-          <t>quintadolago.com</t>
+          <t>cvmnet.com</t>
         </is>
       </c>
       <c r="F67" s="4" t="inlineStr">
         <is>
-          <t>Loulé</t>
+          <t>Santa Maria da Feira</t>
         </is>
       </c>
       <c r="G67" s="4" t="inlineStr">
         <is>
-          <t>Faro</t>
+          <t>Aveiro</t>
         </is>
       </c>
       <c r="H67" s="2" t="inlineStr">
         <is>
-          <t>Almancil</t>
+          <t>Parque Empresarial A32, Vila Maior</t>
         </is>
       </c>
       <c r="I67" s="2" t="inlineStr">
         <is>
-          <t>Quinta do Lago (real estate do resort) (Comercialização)</t>
+          <t>Royal Green (V.N. Gaia, Av. Descobrimentos) (Em construção)</t>
         </is>
       </c>
       <c r="J67" s="2" t="inlineStr">
         <is>
-          <t>Resort residencial/golfe</t>
+          <t>Telefone vindo do registo — confirmar em cvmnet.com/contactos</t>
         </is>
       </c>
     </row>
     <row r="68" ht="30" customHeight="1">
       <c r="A68" s="2" t="inlineStr">
         <is>
+          <t>JHOMEA Invest</t>
+        </is>
+      </c>
+      <c r="B68" s="4" t="inlineStr">
+        <is>
+          <t>Nao</t>
+        </is>
+      </c>
+      <c r="C68" s="4" t="inlineStr">
+        <is>
+          <t>+351 934 175 642</t>
+        </is>
+      </c>
+      <c r="D68" s="2" t="inlineStr">
+        <is>
+          <t>geral@jhomea.pt</t>
+        </is>
+      </c>
+      <c r="E68" s="2" t="inlineStr">
+        <is>
+          <t>jhomea.pt</t>
+        </is>
+      </c>
+      <c r="F68" s="4" t="inlineStr">
+        <is>
+          <t>Aveiro</t>
+        </is>
+      </c>
+      <c r="G68" s="4" t="inlineStr">
+        <is>
+          <t>Aveiro</t>
+        </is>
+      </c>
+      <c r="H68" s="2" t="inlineStr">
+        <is>
+          <t>Rua Cristóvão Pinho Queimado 56, 3800-012</t>
+        </is>
+      </c>
+      <c r="I68" s="2" t="inlineStr">
+        <is>
+          <t>Vacivus (Porto) (Em construção)</t>
+        </is>
+      </c>
+      <c r="J68" s="2" t="inlineStr">
+        <is>
+          <t>AMI 16355. Escritórios Aveiro (+351 914 444 764) e Lisboa (+351 912 325 143)</t>
+        </is>
+      </c>
+    </row>
+    <row r="69" ht="30" customHeight="1">
+      <c r="A69" s="2" t="inlineStr">
+        <is>
+          <t>Pine Hill</t>
+        </is>
+      </c>
+      <c r="B69" s="4" t="inlineStr">
+        <is>
+          <t>Nao</t>
+        </is>
+      </c>
+      <c r="C69" s="4" t="inlineStr">
+        <is>
+          <t>+351 910 936 732</t>
+        </is>
+      </c>
+      <c r="D69" s="2" t="inlineStr">
+        <is>
+          <t>info@pinehill.pt</t>
+        </is>
+      </c>
+      <c r="E69" s="2" t="inlineStr">
+        <is>
+          <t>pinehill.pt</t>
+        </is>
+      </c>
+      <c r="F69" s="4" t="inlineStr">
+        <is>
+          <t>Braga</t>
+        </is>
+      </c>
+      <c r="G69" s="4" t="inlineStr">
+        <is>
+          <t>Braga</t>
+        </is>
+      </c>
+      <c r="H69" s="2" t="inlineStr"/>
+      <c r="I69" s="2" t="inlineStr">
+        <is>
+          <t>Braga Premium Flats (Comercialização) | 3 novos projetos em Braga (Planeamento)</t>
+        </is>
+      </c>
+      <c r="J69" s="2" t="inlineStr">
+        <is>
+          <t>Promotora criada em 2025. Fonte: newinbraga.nit.pt, Revista Spot</t>
+        </is>
+      </c>
+    </row>
+    <row r="70" ht="30" customHeight="1">
+      <c r="A70" s="2" t="inlineStr">
+        <is>
+          <t>Quinta do Lago Resort</t>
+        </is>
+      </c>
+      <c r="B70" s="4" t="inlineStr">
+        <is>
+          <t>Nao</t>
+        </is>
+      </c>
+      <c r="C70" s="4" t="inlineStr">
+        <is>
+          <t>+351 289 390 700</t>
+        </is>
+      </c>
+      <c r="D70" s="2" t="inlineStr">
+        <is>
+          <t>info@quintadolago.com</t>
+        </is>
+      </c>
+      <c r="E70" s="2" t="inlineStr">
+        <is>
+          <t>quintadolago.com</t>
+        </is>
+      </c>
+      <c r="F70" s="4" t="inlineStr">
+        <is>
+          <t>Loulé</t>
+        </is>
+      </c>
+      <c r="G70" s="4" t="inlineStr">
+        <is>
+          <t>Faro</t>
+        </is>
+      </c>
+      <c r="H70" s="2" t="inlineStr">
+        <is>
+          <t>Almancil</t>
+        </is>
+      </c>
+      <c r="I70" s="2" t="inlineStr">
+        <is>
+          <t>Quinta do Lago (real estate do resort) (Comercialização)</t>
+        </is>
+      </c>
+      <c r="J70" s="2" t="inlineStr">
+        <is>
+          <t>Resort residencial/golfe</t>
+        </is>
+      </c>
+    </row>
+    <row r="71" ht="30" customHeight="1">
+      <c r="A71" s="2" t="inlineStr">
+        <is>
           <t>TPS – Teixeira, Pinto &amp; Soares</t>
         </is>
       </c>
-      <c r="B68" s="4" t="inlineStr">
+      <c r="B71" s="4" t="inlineStr">
         <is>
           <t>Nao</t>
         </is>
       </c>
-      <c r="C68" s="4" t="inlineStr">
+      <c r="C71" s="4" t="inlineStr">
         <is>
           <t>+351 255 433 572</t>
         </is>
       </c>
-      <c r="D68" s="2" t="inlineStr">
+      <c r="D71" s="2" t="inlineStr">
         <is>
           <t>geral@tps.com.pt</t>
         </is>
       </c>
-      <c r="E68" s="2" t="inlineStr">
+      <c r="E71" s="2" t="inlineStr">
         <is>
           <t>tps.com.pt</t>
         </is>
       </c>
-      <c r="F68" s="4" t="inlineStr">
+      <c r="F71" s="4" t="inlineStr">
         <is>
           <t>Amarante</t>
         </is>
       </c>
-      <c r="G68" s="4" t="inlineStr">
+      <c r="G71" s="4" t="inlineStr">
         <is>
           <t>Porto</t>
         </is>
       </c>
-      <c r="H68" s="2" t="inlineStr">
+      <c r="H71" s="2" t="inlineStr">
         <is>
           <t>Rua do Outeiro 677, Z.I. Telões, 4600-758</t>
         </is>
       </c>
-      <c r="I68" s="2" t="inlineStr">
+      <c r="I71" s="2" t="inlineStr">
         <is>
           <t>JV com Carvoeiro Branco (Lagoa, Portimão, Faro) (Planeamento) | One Lush (Caxias) (Em construção)</t>
         </is>
       </c>
-      <c r="J68" s="2" t="inlineStr">
+      <c r="J71" s="2" t="inlineStr">
         <is>
           <t>Uma das maiores construtoras nacionais · delegações Lisboa e Algarve</t>
         </is>
       </c>
     </row>
-    <row r="69" ht="30" customHeight="1">
-      <c r="A69" s="5" t="inlineStr">
+    <row r="72" ht="30" customHeight="1">
+      <c r="A72" s="5" t="inlineStr">
         <is>
           <t>Grupo André Guimarães (Portugal)</t>
         </is>
       </c>
-      <c r="B69" s="7" t="inlineStr">
+      <c r="B72" s="7" t="inlineStr">
         <is>
           <t>Nao</t>
         </is>
       </c>
-      <c r="C69" s="7" t="inlineStr"/>
-      <c r="D69" s="5" t="inlineStr"/>
-      <c r="E69" s="5" t="inlineStr">
+      <c r="C72" s="7" t="inlineStr"/>
+      <c r="D72" s="5" t="inlineStr"/>
+      <c r="E72" s="5" t="inlineStr">
         <is>
           <t>andreguimaraes.com.br</t>
         </is>
       </c>
-      <c r="F69" s="7" t="inlineStr"/>
-      <c r="G69" s="7" t="inlineStr"/>
-      <c r="H69" s="5" t="inlineStr"/>
-      <c r="I69" s="5" t="inlineStr">
+      <c r="F72" s="7" t="inlineStr"/>
+      <c r="G72" s="7" t="inlineStr"/>
+      <c r="H72" s="5" t="inlineStr"/>
+      <c r="I72" s="5" t="inlineStr">
         <is>
           <t>JV com Overseas (Lisboa) (Planeamento) | Porto, Algarve, Douro, Cascais, Alentejo, Amarante (Em construção)</t>
         </is>
       </c>
-      <c r="J69" s="5" t="inlineStr">
+      <c r="J72" s="5" t="inlineStr">
         <is>
           <t>Entidade PT: André Guimarães - Portugal, Lda (NIF 517865459). Sem contacto PT</t>
         </is>
       </c>
     </row>
-    <row r="70" ht="30" customHeight="1">
-      <c r="A70" s="5" t="inlineStr">
+    <row r="73" ht="30" customHeight="1">
+      <c r="A73" s="5" t="inlineStr">
         <is>
           <t>Ombria Resort (Grupo Pontos)</t>
         </is>
       </c>
-      <c r="B70" s="7" t="inlineStr">
+      <c r="B73" s="7" t="inlineStr">
         <is>
           <t>Nao</t>
         </is>
       </c>
-      <c r="C70" s="7" t="inlineStr"/>
-      <c r="D70" s="5" t="inlineStr"/>
-      <c r="E70" s="5" t="inlineStr">
+      <c r="C73" s="7" t="inlineStr"/>
+      <c r="D73" s="5" t="inlineStr"/>
+      <c r="E73" s="5" t="inlineStr">
         <is>
           <t>ombria.com</t>
         </is>
       </c>
-      <c r="F70" s="7" t="inlineStr">
+      <c r="F73" s="7" t="inlineStr">
         <is>
           <t>Loulé</t>
         </is>
       </c>
-      <c r="G70" s="7" t="inlineStr">
+      <c r="G73" s="7" t="inlineStr">
         <is>
           <t>Faro</t>
         </is>
       </c>
-      <c r="H70" s="5" t="inlineStr">
+      <c r="H73" s="5" t="inlineStr">
         <is>
           <t>Loulé</t>
         </is>
       </c>
-      <c r="I70" s="5" t="inlineStr">
+      <c r="I73" s="5" t="inlineStr">
         <is>
           <t>Ombria Algarve (Em construção)</t>
         </is>
       </c>
-      <c r="J70" s="5" t="inlineStr">
+      <c r="J73" s="5" t="inlineStr">
         <is>
           <t>Grupo finlandês Pontos · construtor Gabriel Couto</t>
         </is>
@@ -4025,7 +4173,7 @@
         </is>
       </c>
       <c r="B2" s="9" t="n">
-        <v>69</v>
+        <v>72</v>
       </c>
     </row>
     <row r="3">
@@ -4035,7 +4183,7 @@
         </is>
       </c>
       <c r="B3" s="9" t="n">
-        <v>57</v>
+        <v>59</v>
       </c>
     </row>
     <row r="4">
@@ -4045,7 +4193,7 @@
         </is>
       </c>
       <c r="B4" s="9" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
     </row>
     <row r="5">
@@ -4055,7 +4203,7 @@
         </is>
       </c>
       <c r="B5" s="9" t="n">
-        <v>52</v>
+        <v>54</v>
       </c>
     </row>
     <row r="6">

</xml_diff>

<commit_message>
Add CEO, LinkedIn and Instagram columns for all 72 promoters
Researched via targeted web search per company. LinkedIn found for most
CEOs/administrators; personal Instagram was not found with confidence
for any of them (left blank rather than guessed — company-only
Instagram accounts don't count). A few CEO names carry a confidence
note in parentheses where sources were ambiguous or homonymous.

Map artifact (same published URL) and xlsx export updated in the same
pass to surface the new fields.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01SRBJwGmSsYkTHKJbGCM5ca
</commit_message>
<xml_diff>
--- a/Promotoras_Imobiliarias_Contactos.xlsx
+++ b/Promotoras_Imobiliarias_Contactos.xlsx
@@ -191,9 +191,9 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Promotoras" displayName="Promotoras" ref="A1:J73" headerRowCount="1">
-  <autoFilter ref="A1:J73"/>
-  <tableColumns count="10">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Promotoras" displayName="Promotoras" ref="A1:M73" headerRowCount="1">
+  <autoFilter ref="A1:M73"/>
+  <tableColumns count="13">
     <tableColumn id="1" name="Nome da Empresa"/>
     <tableColumn id="2" name="Prioritario"/>
     <tableColumn id="3" name="Telefone"/>
@@ -204,6 +204,9 @@
     <tableColumn id="8" name="Morada Completa"/>
     <tableColumn id="9" name="Empreendimentos Ativos"/>
     <tableColumn id="10" name="Notas"/>
+    <tableColumn id="11" name="CEO"/>
+    <tableColumn id="12" name="LinkedIn CEO"/>
+    <tableColumn id="13" name="Instagram CEO"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showRowStripes="1"/>
 </table>
@@ -498,7 +501,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J73"/>
+  <dimension ref="A1:M73"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -511,6 +514,9 @@
     <col width="34" customWidth="1" min="8" max="8"/>
     <col width="55" customWidth="1" min="9" max="9"/>
     <col width="40" customWidth="1" min="10" max="10"/>
+    <col width="26" customWidth="1" min="11" max="11"/>
+    <col width="32" customWidth="1" min="12" max="12"/>
+    <col width="26" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
     <row r="1" ht="22" customHeight="1">
@@ -564,6 +570,21 @@
           <t>Notas</t>
         </is>
       </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>CEO</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>LinkedIn CEO</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>Instagram CEO</t>
+        </is>
+      </c>
     </row>
     <row r="2" ht="30" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
@@ -616,6 +637,9 @@
           <t>Private equity com foco imobiliário. Fonte: APPII</t>
         </is>
       </c>
+      <c r="K2" s="2" t="inlineStr"/>
+      <c r="L2" s="2" t="inlineStr"/>
+      <c r="M2" s="2" t="inlineStr"/>
     </row>
     <row r="3" ht="30" customHeight="1">
       <c r="A3" s="2" t="inlineStr">
@@ -668,6 +692,17 @@
           <t>Fundada 2022, ligada à Panhard. Tel. móvel 914 192 506</t>
         </is>
       </c>
+      <c r="K3" s="2" t="inlineStr">
+        <is>
+          <t>Carlos Morgado (Diretor Executivo)</t>
+        </is>
+      </c>
+      <c r="L3" s="2" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/cafmorgado/</t>
+        </is>
+      </c>
+      <c r="M3" s="2" t="inlineStr"/>
     </row>
     <row r="4" ht="30" customHeight="1">
       <c r="A4" s="2" t="inlineStr">
@@ -720,6 +755,17 @@
           <t>Telefone é da linha comercial Quinta do Alverde</t>
         </is>
       </c>
+      <c r="K4" s="2" t="inlineStr">
+        <is>
+          <t>Alejandro Martins (Founder &amp; CEO)</t>
+        </is>
+      </c>
+      <c r="L4" s="2" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/alejandro-martins-74b18590/</t>
+        </is>
+      </c>
+      <c r="M4" s="2" t="inlineStr"/>
     </row>
     <row r="5" ht="30" customHeight="1">
       <c r="A5" s="2" t="inlineStr">
@@ -772,6 +818,17 @@
           <t>Promotor de referência Lisboa/Porto</t>
         </is>
       </c>
+      <c r="K5" s="2" t="inlineStr">
+        <is>
+          <t>Aniceto Viegas (CEO)</t>
+        </is>
+      </c>
+      <c r="L5" s="2" t="inlineStr">
+        <is>
+          <t>https://pt.linkedin.com/in/aniceto-viegas-02586a1</t>
+        </is>
+      </c>
+      <c r="M5" s="2" t="inlineStr"/>
     </row>
     <row r="6" ht="30" customHeight="1">
       <c r="A6" s="2" t="inlineStr">
@@ -820,6 +877,13 @@
           <t>Só telefone UK publicado</t>
         </is>
       </c>
+      <c r="K6" s="2" t="inlineStr">
+        <is>
+          <t>Fredrick J. Benoit II (Director/co-fundador, 50% com Matthew Lavin)</t>
+        </is>
+      </c>
+      <c r="L6" s="2" t="inlineStr"/>
+      <c r="M6" s="2" t="inlineStr"/>
     </row>
     <row r="7" ht="30" customHeight="1">
       <c r="A7" s="2" t="inlineStr">
@@ -872,6 +936,17 @@
           <t>Promotor pan-europeu (grupo BESIX)</t>
         </is>
       </c>
+      <c r="K7" s="2" t="inlineStr">
+        <is>
+          <t>Nicolas Goffin (Country Director Portugal· CEO do grupo é Gabriel Uzgen, Bruxelas)</t>
+        </is>
+      </c>
+      <c r="L7" s="2" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/nicolas-goffin-32707487/</t>
+        </is>
+      </c>
+      <c r="M7" s="2" t="inlineStr"/>
     </row>
     <row r="8" ht="30" customHeight="1">
       <c r="A8" s="2" t="inlineStr">
@@ -924,6 +999,17 @@
           <t>Desde 2015, sócios com &gt;500M€ promovidos</t>
         </is>
       </c>
+      <c r="K8" s="2" t="inlineStr">
+        <is>
+          <t>Celma de Almeida Lavradio (Co-Founder &amp; CEO)</t>
+        </is>
+      </c>
+      <c r="L8" s="2" t="inlineStr">
+        <is>
+          <t>https://pt.linkedin.com/in/celma-de-almeida-lavradio-645baa43</t>
+        </is>
+      </c>
+      <c r="M8" s="2" t="inlineStr"/>
     </row>
     <row r="9" ht="30" customHeight="1">
       <c r="A9" s="2" t="inlineStr">
@@ -972,6 +1058,17 @@
           <t>Gestora regulada CMVM, capital internacional</t>
         </is>
       </c>
+      <c r="K9" s="2" t="inlineStr">
+        <is>
+          <t>Paulo Loureiro (fundador e CEO)</t>
+        </is>
+      </c>
+      <c r="L9" s="2" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/paulo-loureiro-8a46016/</t>
+        </is>
+      </c>
+      <c r="M9" s="2" t="inlineStr"/>
     </row>
     <row r="10" ht="30" customHeight="1">
       <c r="A10" s="2" t="inlineStr">
@@ -1024,6 +1121,13 @@
           <t>Promotor de Lisboa desde 2004</t>
         </is>
       </c>
+      <c r="K10" s="2" t="inlineStr">
+        <is>
+          <t>Sérgio Ferreira (fundador e CEO, homónimos sem confirmação total)</t>
+        </is>
+      </c>
+      <c r="L10" s="2" t="inlineStr"/>
+      <c r="M10" s="2" t="inlineStr"/>
     </row>
     <row r="11" ht="30" customHeight="1">
       <c r="A11" s="2" t="inlineStr">
@@ -1076,6 +1180,13 @@
           <t>20 anos em Príncipe Real, &gt;20 edifícios</t>
         </is>
       </c>
+      <c r="K11" s="2" t="inlineStr">
+        <is>
+          <t>Tiago Eiró (CEO)</t>
+        </is>
+      </c>
+      <c r="L11" s="2" t="inlineStr"/>
+      <c r="M11" s="2" t="inlineStr"/>
     </row>
     <row r="12" ht="30" customHeight="1">
       <c r="A12" s="2" t="inlineStr">
@@ -1128,6 +1239,17 @@
           <t>Promotora do grupo Mota-Engil</t>
         </is>
       </c>
+      <c r="K12" s="2" t="inlineStr">
+        <is>
+          <t>Vitor Paulo Pinho (CEO)</t>
+        </is>
+      </c>
+      <c r="L12" s="2" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/vitor-paulo-pinho-0a7952173/</t>
+        </is>
+      </c>
+      <c r="M12" s="2" t="inlineStr"/>
     </row>
     <row r="13" ht="30" customHeight="1">
       <c r="A13" s="2" t="inlineStr">
@@ -1176,6 +1298,13 @@
           <t>Luxo desde 1981. Fonte: reportugal.vidaimobiliaria.com</t>
         </is>
       </c>
+      <c r="K13" s="2" t="inlineStr">
+        <is>
+          <t>Mário Almeida (Administrador)</t>
+        </is>
+      </c>
+      <c r="L13" s="2" t="inlineStr"/>
+      <c r="M13" s="2" t="inlineStr"/>
     </row>
     <row r="14" ht="30" customHeight="1">
       <c r="A14" s="2" t="inlineStr">
@@ -1228,6 +1357,9 @@
           <t>Braço imobiliário da Fidelidade. Projeto: info@entrecampos.pt</t>
         </is>
       </c>
+      <c r="K14" s="2" t="inlineStr"/>
+      <c r="L14" s="2" t="inlineStr"/>
+      <c r="M14" s="2" t="inlineStr"/>
     </row>
     <row r="15" ht="30" customHeight="1">
       <c r="A15" s="2" t="inlineStr">
@@ -1276,6 +1408,9 @@
           <t>Projeto concreto não nomeado nas fontes</t>
         </is>
       </c>
+      <c r="K15" s="2" t="inlineStr"/>
+      <c r="L15" s="2" t="inlineStr"/>
+      <c r="M15" s="2" t="inlineStr"/>
     </row>
     <row r="16" ht="30" customHeight="1">
       <c r="A16" s="2" t="inlineStr">
@@ -1328,6 +1463,13 @@
           <t>Presidente António Parente. Tel. móvel 914 070 350</t>
         </is>
       </c>
+      <c r="K16" s="2" t="inlineStr">
+        <is>
+          <t>Nuno Dias (Diretor Geral da Madre Imobiliário· presidente do grupo é António Parente)</t>
+        </is>
+      </c>
+      <c r="L16" s="2" t="inlineStr"/>
+      <c r="M16" s="2" t="inlineStr"/>
     </row>
     <row r="17" ht="30" customHeight="1">
       <c r="A17" s="2" t="inlineStr">
@@ -1380,6 +1522,13 @@
           <t>Fundada 2001 · inclui Habitat Ventures/Project/Property/Broker</t>
         </is>
       </c>
+      <c r="K17" s="2" t="inlineStr">
+        <is>
+          <t>Luís Corrêa de Barros (fundador e CEO)</t>
+        </is>
+      </c>
+      <c r="L17" s="2" t="inlineStr"/>
+      <c r="M17" s="2" t="inlineStr"/>
     </row>
     <row r="18" ht="30" customHeight="1">
       <c r="A18" s="2" t="inlineStr">
@@ -1432,6 +1581,9 @@
           <t>Fundada 1960, alvará ICC 12463. Tel. móvel 961 682 789</t>
         </is>
       </c>
+      <c r="K18" s="2" t="inlineStr"/>
+      <c r="L18" s="2" t="inlineStr"/>
+      <c r="M18" s="2" t="inlineStr"/>
     </row>
     <row r="19" ht="30" customHeight="1">
       <c r="A19" s="2" t="inlineStr">
@@ -1484,6 +1636,17 @@
           <t>Promotora com construtora e imobiliária próprias</t>
         </is>
       </c>
+      <c r="K19" s="2" t="inlineStr">
+        <is>
+          <t>João Sousa (CEO)</t>
+        </is>
+      </c>
+      <c r="L19" s="2" t="inlineStr">
+        <is>
+          <t>https://pt.linkedin.com/in/joao-sousa-7802352a</t>
+        </is>
+      </c>
+      <c r="M19" s="2" t="inlineStr"/>
     </row>
     <row r="20" ht="30" customHeight="1">
       <c r="A20" s="2" t="inlineStr">
@@ -1536,6 +1699,17 @@
           <t>Belga, em Portugal desde 2014</t>
         </is>
       </c>
+      <c r="K20" s="2" t="inlineStr">
+        <is>
+          <t>Claude Kandiyoti (CEO)</t>
+        </is>
+      </c>
+      <c r="L20" s="2" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/claude-kandiyoti-287b9298/</t>
+        </is>
+      </c>
+      <c r="M20" s="2" t="inlineStr"/>
     </row>
     <row r="21" ht="30" customHeight="1">
       <c r="A21" s="2" t="inlineStr">
@@ -1584,6 +1758,17 @@
           <t>Entidade KIG Portugal (NIF 514667265)</t>
         </is>
       </c>
+      <c r="K21" s="2" t="inlineStr">
+        <is>
+          <t>Rui Meneses Ferreira (CEO)</t>
+        </is>
+      </c>
+      <c r="L21" s="2" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/rui-meneses-ferreira-97057825/</t>
+        </is>
+      </c>
+      <c r="M21" s="2" t="inlineStr"/>
     </row>
     <row r="22" ht="30" customHeight="1">
       <c r="A22" s="2" t="inlineStr">
@@ -1636,6 +1821,13 @@
           <t>Constituída em Macau 2015</t>
         </is>
       </c>
+      <c r="K22" s="2" t="inlineStr">
+        <is>
+          <t>Eduardo Kol Netto de Almeida (CEO)</t>
+        </is>
+      </c>
+      <c r="L22" s="2" t="inlineStr"/>
+      <c r="M22" s="2" t="inlineStr"/>
     </row>
     <row r="23" ht="30" customHeight="1">
       <c r="A23" s="2" t="inlineStr">
@@ -1688,6 +1880,13 @@
           <t>18 projetos no Algarve, &gt;800 unidades entregues · ISO 14001</t>
         </is>
       </c>
+      <c r="K23" s="2" t="inlineStr">
+        <is>
+          <t>António Gonçalves (Fundador)</t>
+        </is>
+      </c>
+      <c r="L23" s="2" t="inlineStr"/>
+      <c r="M23" s="2" t="inlineStr"/>
     </row>
     <row r="24" ht="30" customHeight="1">
       <c r="A24" s="2" t="inlineStr">
@@ -1740,6 +1939,17 @@
           <t>&gt;100M€ anunciados 2026. Fonte: diarioimobiliario.pt</t>
         </is>
       </c>
+      <c r="K24" s="2" t="inlineStr">
+        <is>
+          <t>Gabriel Costa (CEO, confiança baixa — só rocketreach)</t>
+        </is>
+      </c>
+      <c r="L24" s="2" t="inlineStr">
+        <is>
+          <t>https://pt.linkedin.com/in/gabriel-costa-7436b5158</t>
+        </is>
+      </c>
+      <c r="M24" s="2" t="inlineStr"/>
     </row>
     <row r="25" ht="30" customHeight="1">
       <c r="A25" s="2" t="inlineStr">
@@ -1792,6 +2002,13 @@
           <t>Capital social 5M€. Fonte: idealista/news ago/2026</t>
         </is>
       </c>
+      <c r="K25" s="2" t="inlineStr">
+        <is>
+          <t>Pedro Teixeira Paredes (CEO)</t>
+        </is>
+      </c>
+      <c r="L25" s="2" t="inlineStr"/>
+      <c r="M25" s="2" t="inlineStr"/>
     </row>
     <row r="26" ht="30" customHeight="1">
       <c r="A26" s="2" t="inlineStr">
@@ -1844,6 +2061,17 @@
           <t>Grupo suíço, 250M€ em Portugal, 71.000 m²</t>
         </is>
       </c>
+      <c r="K26" s="2" t="inlineStr">
+        <is>
+          <t>Tomas Suter (Founding Member/Partner, Suíça)</t>
+        </is>
+      </c>
+      <c r="L26" s="2" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/tomas-suter-78564b9/</t>
+        </is>
+      </c>
+      <c r="M26" s="2" t="inlineStr"/>
     </row>
     <row r="27" ht="30" customHeight="1">
       <c r="A27" s="2" t="inlineStr">
@@ -1892,6 +2120,17 @@
           <t>Gestora de investimento (2,1B€) que também promove</t>
         </is>
       </c>
+      <c r="K27" s="2" t="inlineStr">
+        <is>
+          <t>Miguel Mateus (CEO, recém-nomeado)</t>
+        </is>
+      </c>
+      <c r="L27" s="2" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/miguel-mateus-608b616/</t>
+        </is>
+      </c>
+      <c r="M27" s="2" t="inlineStr"/>
     </row>
     <row r="28" ht="30" customHeight="1">
       <c r="A28" s="2" t="inlineStr">
@@ -1944,6 +2183,17 @@
           <t>Promotor desde 1986</t>
         </is>
       </c>
+      <c r="K28" s="2" t="inlineStr">
+        <is>
+          <t>Pedro Sanches (CEO/fundador)</t>
+        </is>
+      </c>
+      <c r="L28" s="2" t="inlineStr">
+        <is>
+          <t>https://pt.linkedin.com/in/pedro-sanches-77205825</t>
+        </is>
+      </c>
+      <c r="M28" s="2" t="inlineStr"/>
     </row>
     <row r="29" ht="30" customHeight="1">
       <c r="A29" s="2" t="inlineStr">
@@ -1996,6 +2246,17 @@
           <t>1,7B€ investidos · PT e Turquia</t>
         </is>
       </c>
+      <c r="K29" s="2" t="inlineStr">
+        <is>
+          <t>William Tonnard (President &amp; COO· Chairman é Hakan Kodal)</t>
+        </is>
+      </c>
+      <c r="L29" s="2" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/william-tonnard/</t>
+        </is>
+      </c>
+      <c r="M29" s="2" t="inlineStr"/>
     </row>
     <row r="30" ht="30" customHeight="1">
       <c r="A30" s="2" t="inlineStr">
@@ -2040,6 +2301,9 @@
           <t>Telefone do registo comercial (einforma). Comercialização JLL/Predibisa</t>
         </is>
       </c>
+      <c r="K30" s="2" t="inlineStr"/>
+      <c r="L30" s="2" t="inlineStr"/>
+      <c r="M30" s="2" t="inlineStr"/>
     </row>
     <row r="31" ht="30" customHeight="1">
       <c r="A31" s="2" t="inlineStr">
@@ -2092,6 +2356,17 @@
           <t>Com Tikehau Capital. &gt;1B€ sob gestão</t>
         </is>
       </c>
+      <c r="K31" s="2" t="inlineStr">
+        <is>
+          <t>Carlos Vasconcellos (Founding Partner, CEO exato não confirmado)</t>
+        </is>
+      </c>
+      <c r="L31" s="2" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/vasconcelloscarlos/</t>
+        </is>
+      </c>
+      <c r="M31" s="2" t="inlineStr"/>
     </row>
     <row r="32" ht="30" customHeight="1">
       <c r="A32" s="2" t="inlineStr">
@@ -2144,6 +2419,17 @@
           <t>NIF 516390350, capital 800k€. Fonte: construir.pt abr/2026</t>
         </is>
       </c>
+      <c r="K32" s="2" t="inlineStr">
+        <is>
+          <t>Hugo Gonçalves Pereira (CEO)</t>
+        </is>
+      </c>
+      <c r="L32" s="2" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/hugogpereira/</t>
+        </is>
+      </c>
+      <c r="M32" s="2" t="inlineStr"/>
     </row>
     <row r="33" ht="30" customHeight="1">
       <c r="A33" s="2" t="inlineStr">
@@ -2196,6 +2482,9 @@
           <t>Grupo nascido em Monção, liderado por Nuno Afonso. Fonte: idealista/news jun/2026, Público</t>
         </is>
       </c>
+      <c r="K33" s="2" t="inlineStr"/>
+      <c r="L33" s="2" t="inlineStr"/>
+      <c r="M33" s="2" t="inlineStr"/>
     </row>
     <row r="34" ht="30" customHeight="1">
       <c r="A34" s="2" t="inlineStr">
@@ -2244,6 +2533,17 @@
           <t>ATENÇÃO: é gestor de projeto/serviços, não promotor puro</t>
         </is>
       </c>
+      <c r="K34" s="2" t="inlineStr">
+        <is>
+          <t>José Pedro Almeida Guerra (Diretor Geral)</t>
+        </is>
+      </c>
+      <c r="L34" s="2" t="inlineStr">
+        <is>
+          <t>https://pt.linkedin.com/in/josé-pedro-almeida-guerra-20723679</t>
+        </is>
+      </c>
+      <c r="M34" s="2" t="inlineStr"/>
     </row>
     <row r="35" ht="30" customHeight="1">
       <c r="A35" s="2" t="inlineStr">
@@ -2296,6 +2596,17 @@
           <t>Sócios israelitas (Udi, Liad) + contacto PT Alexandre. Fonte: royal-ventures.com/contact-us</t>
         </is>
       </c>
+      <c r="K35" s="2" t="inlineStr">
+        <is>
+          <t>Udi Yadin (fundador/General Partner)</t>
+        </is>
+      </c>
+      <c r="L35" s="2" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/udiyadin/</t>
+        </is>
+      </c>
+      <c r="M35" s="2" t="inlineStr"/>
     </row>
     <row r="36" ht="30" customHeight="1">
       <c r="A36" s="2" t="inlineStr">
@@ -2348,6 +2659,17 @@
           <t>CEO Carla Luís</t>
         </is>
       </c>
+      <c r="K36" s="2" t="inlineStr">
+        <is>
+          <t>Carla Luís (CEO/cofundadora)</t>
+        </is>
+      </c>
+      <c r="L36" s="2" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/carla-luís-b14a7616/</t>
+        </is>
+      </c>
+      <c r="M36" s="2" t="inlineStr"/>
     </row>
     <row r="37" ht="30" customHeight="1">
       <c r="A37" s="2" t="inlineStr">
@@ -2400,6 +2722,17 @@
           <t>Promoção imobiliária desde 1949</t>
         </is>
       </c>
+      <c r="K37" s="2" t="inlineStr">
+        <is>
+          <t>Pedro Silveira (acionista maioritário/ex-Chairman, destituído judicialmente mai/2025, em recurso)</t>
+        </is>
+      </c>
+      <c r="L37" s="2" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/pedro-silveira-88822a20/</t>
+        </is>
+      </c>
+      <c r="M37" s="2" t="inlineStr"/>
     </row>
     <row r="38" ht="30" customHeight="1">
       <c r="A38" s="2" t="inlineStr">
@@ -2452,6 +2785,17 @@
           <t>Estoril Capital Partners + Oaktree. Tel. alternativo 210 966 905</t>
         </is>
       </c>
+      <c r="K38" s="2" t="inlineStr">
+        <is>
+          <t>Gonçalo Cadete (CEO)</t>
+        </is>
+      </c>
+      <c r="L38" s="2" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/gon%C3%A7alo-cadete-260692/</t>
+        </is>
+      </c>
+      <c r="M38" s="2" t="inlineStr"/>
     </row>
     <row r="39" ht="30" customHeight="1">
       <c r="A39" s="2" t="inlineStr">
@@ -2504,6 +2848,13 @@
           <t>Tel. móvel 965 915 993</t>
         </is>
       </c>
+      <c r="K39" s="2" t="inlineStr">
+        <is>
+          <t>Geoffroy Moreno (Co-Founder)</t>
+        </is>
+      </c>
+      <c r="L39" s="2" t="inlineStr"/>
+      <c r="M39" s="2" t="inlineStr"/>
     </row>
     <row r="40" ht="30" customHeight="1">
       <c r="A40" s="2" t="inlineStr">
@@ -2556,6 +2907,9 @@
           <t>Braço imobiliário do grupo Teixeira Duarte</t>
         </is>
       </c>
+      <c r="K40" s="2" t="inlineStr"/>
+      <c r="L40" s="2" t="inlineStr"/>
+      <c r="M40" s="2" t="inlineStr"/>
     </row>
     <row r="41" ht="30" customHeight="1">
       <c r="A41" s="2" t="inlineStr">
@@ -2608,6 +2962,17 @@
           <t>Promotor belga em Portugal desde 2018. Fonte: diarioimobiliario.pt</t>
         </is>
       </c>
+      <c r="K41" s="2" t="inlineStr">
+        <is>
+          <t>David Carreira (Diretor Geral/Country Manager)</t>
+        </is>
+      </c>
+      <c r="L41" s="2" t="inlineStr">
+        <is>
+          <t>https://lu.linkedin.com/in/david-carreira-a4082050</t>
+        </is>
+      </c>
+      <c r="M41" s="2" t="inlineStr"/>
     </row>
     <row r="42" ht="30" customHeight="1">
       <c r="A42" s="2" t="inlineStr">
@@ -2660,6 +3025,17 @@
           <t>Entidade legal Vanguardeagle Asset Management (NIF 514114215). Tel. móvel 915 292 222</t>
         </is>
       </c>
+      <c r="K42" s="2" t="inlineStr">
+        <is>
+          <t>Henrique Rodrigues da Silva (CEO desde fev/2026)</t>
+        </is>
+      </c>
+      <c r="L42" s="2" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/henrique-rodrigues-da-silva-b396643/</t>
+        </is>
+      </c>
+      <c r="M42" s="2" t="inlineStr"/>
     </row>
     <row r="43" ht="30" customHeight="1">
       <c r="A43" s="2" t="inlineStr">
@@ -2712,6 +3088,17 @@
           <t>Portefólio &gt;3B€. Fundada 2018</t>
         </is>
       </c>
+      <c r="K43" s="2" t="inlineStr">
+        <is>
+          <t>João Cabaça (Co-fundador e CEO)</t>
+        </is>
+      </c>
+      <c r="L43" s="2" t="inlineStr">
+        <is>
+          <t>https://pt.linkedin.com/in/jo%C3%A3o-caba%C3%A7a-6b293614b</t>
+        </is>
+      </c>
+      <c r="M43" s="2" t="inlineStr"/>
     </row>
     <row r="44" ht="30" customHeight="1">
       <c r="A44" s="2" t="inlineStr">
@@ -2764,6 +3151,17 @@
           <t>NIF 510933084. Tel. móvel 913 385 846</t>
         </is>
       </c>
+      <c r="K44" s="2" t="inlineStr">
+        <is>
+          <t>Joaquim Lico (CEO)</t>
+        </is>
+      </c>
+      <c r="L44" s="2" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/joaquim-lico-4383239/</t>
+        </is>
+      </c>
+      <c r="M44" s="2" t="inlineStr"/>
     </row>
     <row r="45" ht="30" customHeight="1">
       <c r="A45" s="5" t="inlineStr">
@@ -2808,6 +3206,17 @@
           <t>Nova promotora (jan/2026), CEO António Velho da Palma</t>
         </is>
       </c>
+      <c r="K45" s="5" t="inlineStr">
+        <is>
+          <t>António Velho da Palma (CEO Alecrim RE)· CEO da holding Lince Capital é Vasco Pereira Coutinho</t>
+        </is>
+      </c>
+      <c r="L45" s="5" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/ant%C3%B3nio-velho-da-palma-82112282/</t>
+        </is>
+      </c>
+      <c r="M45" s="5" t="inlineStr"/>
     </row>
     <row r="46" ht="30" customHeight="1">
       <c r="A46" s="5" t="inlineStr">
@@ -2848,6 +3257,13 @@
           <t>Israelita (Elad Dror). Sem telefone publicado nas fontes</t>
         </is>
       </c>
+      <c r="K46" s="5" t="inlineStr">
+        <is>
+          <t>Pedro Ferreira (CEO desde jun/2023· fundador anterior Elad Dror saiu em 2023)</t>
+        </is>
+      </c>
+      <c r="L46" s="5" t="inlineStr"/>
+      <c r="M46" s="5" t="inlineStr"/>
     </row>
     <row r="47" ht="30" customHeight="1">
       <c r="A47" s="5" t="inlineStr">
@@ -2892,6 +3308,13 @@
           <t>Gestora global · sem contacto PT publicado</t>
         </is>
       </c>
+      <c r="K47" s="5" t="inlineStr">
+        <is>
+          <t>Vanessa Gelado (Senior Managing Director, Head of Southern Europe)</t>
+        </is>
+      </c>
+      <c r="L47" s="5" t="inlineStr"/>
+      <c r="M47" s="5" t="inlineStr"/>
     </row>
     <row r="48" ht="30" customHeight="1">
       <c r="A48" s="5" t="inlineStr">
@@ -2932,6 +3355,13 @@
           <t>Co-promoção com investidores · CEO Paulo Vaz Ferreira</t>
         </is>
       </c>
+      <c r="K48" s="5" t="inlineStr">
+        <is>
+          <t>Paulo Vaz Ferreira (sócio e CEO desde 2019, confiança moderada)</t>
+        </is>
+      </c>
+      <c r="L48" s="5" t="inlineStr"/>
+      <c r="M48" s="5" t="inlineStr"/>
     </row>
     <row r="49" ht="30" customHeight="1">
       <c r="A49" s="5" t="inlineStr">
@@ -2972,6 +3402,17 @@
           <t>CEO Pedro Vicente (vice-presidente APPII). Sem telefone publicado</t>
         </is>
       </c>
+      <c r="K49" s="5" t="inlineStr">
+        <is>
+          <t>Pedro Vicente (CEO)</t>
+        </is>
+      </c>
+      <c r="L49" s="5" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/pedro-vicente-9aa0b424/</t>
+        </is>
+      </c>
+      <c r="M49" s="5" t="inlineStr"/>
     </row>
     <row r="50" ht="30" customHeight="1">
       <c r="A50" s="5" t="inlineStr">
@@ -3012,6 +3453,13 @@
           <t>Sem telefone/site publicados (APPII)</t>
         </is>
       </c>
+      <c r="K50" s="5" t="inlineStr">
+        <is>
+          <t>Federico Rosales (cofundador e CEO)</t>
+        </is>
+      </c>
+      <c r="L50" s="5" t="inlineStr"/>
+      <c r="M50" s="5" t="inlineStr"/>
     </row>
     <row r="51" ht="30" customHeight="1">
       <c r="A51" s="5" t="inlineStr">
@@ -3056,6 +3504,13 @@
           <t>Sem telefone PT publicado</t>
         </is>
       </c>
+      <c r="K51" s="5" t="inlineStr">
+        <is>
+          <t>Michael Bickford (Founder &amp; CEO global· sem responsável PT confirmado)</t>
+        </is>
+      </c>
+      <c r="L51" s="5" t="inlineStr"/>
+      <c r="M51" s="5" t="inlineStr"/>
     </row>
     <row r="52" ht="30" customHeight="1">
       <c r="A52" s="5" t="inlineStr">
@@ -3100,6 +3555,13 @@
           <t>Integra o Grupo Teixeira. Sem telefone confirmado — contacto via screendomus.com</t>
         </is>
       </c>
+      <c r="K52" s="5" t="inlineStr">
+        <is>
+          <t>Nuno Teixeira (Administrador, perfil LinkedIn não confirmado)</t>
+        </is>
+      </c>
+      <c r="L52" s="5" t="inlineStr"/>
+      <c r="M52" s="5" t="inlineStr"/>
     </row>
     <row r="53" ht="30" customHeight="1">
       <c r="A53" s="5" t="inlineStr">
@@ -3144,6 +3606,17 @@
           <t>Fundada 1985 · sem telefone publicado</t>
         </is>
       </c>
+      <c r="K53" s="5" t="inlineStr">
+        <is>
+          <t>Carlos Leal (CEO)</t>
+        </is>
+      </c>
+      <c r="L53" s="5" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/carlos-leal-62797227/</t>
+        </is>
+      </c>
+      <c r="M53" s="5" t="inlineStr"/>
     </row>
     <row r="54" ht="30" customHeight="1">
       <c r="A54" s="5" t="inlineStr">
@@ -3192,6 +3665,17 @@
           <t>Adquirida pela Orion em 2023. Formulário em vizta.pt/contactos</t>
         </is>
       </c>
+      <c r="K54" s="5" t="inlineStr">
+        <is>
+          <t>Fernando Vasco Costa (CEO)</t>
+        </is>
+      </c>
+      <c r="L54" s="5" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/fernando-vasco-costa/</t>
+        </is>
+      </c>
+      <c r="M54" s="5" t="inlineStr"/>
     </row>
     <row r="55" ht="30" customHeight="1">
       <c r="A55" s="5" t="inlineStr">
@@ -3236,6 +3720,17 @@
           <t>Elad Shachar / Tamir Luria · &gt;70M€ sob gestão</t>
         </is>
       </c>
+      <c r="K55" s="5" t="inlineStr">
+        <is>
+          <t>Elad Shachar e Tamir Luria (co-líderes/investidores)</t>
+        </is>
+      </c>
+      <c r="L55" s="5" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/tamir-luria/</t>
+        </is>
+      </c>
+      <c r="M55" s="5" t="inlineStr"/>
     </row>
     <row r="56" ht="30" customHeight="1">
       <c r="A56" s="2" t="inlineStr">
@@ -3288,6 +3783,17 @@
           <t>Número é linha gratuita espanhola · loja de vendas aberta seg-sáb</t>
         </is>
       </c>
+      <c r="K56" s="2" t="inlineStr">
+        <is>
+          <t>José Ignacio Fernández (AEDAS Homes PT) / Javier M. Prieto Ruiz (Diretor Promoção, LandCo)</t>
+        </is>
+      </c>
+      <c r="L56" s="2" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/javier-m-prieto-ruiz-583b9227/</t>
+        </is>
+      </c>
+      <c r="M56" s="2" t="inlineStr"/>
     </row>
     <row r="57" ht="30" customHeight="1">
       <c r="A57" s="2" t="inlineStr">
@@ -3340,6 +3846,17 @@
           <t>Mesmo CEO (Erik de Vlieger) e mesmo telefone da Carvoeiro Branco</t>
         </is>
       </c>
+      <c r="K57" s="2" t="inlineStr">
+        <is>
+          <t>Erik de Vlieger (President, mesmo grupo da Carvoeiro Branco)</t>
+        </is>
+      </c>
+      <c r="L57" s="2" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/erik-de-vlieger-12a06a181/</t>
+        </is>
+      </c>
+      <c r="M57" s="2" t="inlineStr"/>
     </row>
     <row r="58" ht="30" customHeight="1">
       <c r="A58" s="2" t="inlineStr">
@@ -3392,6 +3909,17 @@
           <t>NIF 507849183. Tel. alternativo 960 280 640</t>
         </is>
       </c>
+      <c r="K58" s="2" t="inlineStr">
+        <is>
+          <t>Erik de Vlieger (CEO)</t>
+        </is>
+      </c>
+      <c r="L58" s="2" t="inlineStr">
+        <is>
+          <t>https://pt.linkedin.com/in/erik-de-vlieger-12a06a181</t>
+        </is>
+      </c>
+      <c r="M58" s="2" t="inlineStr"/>
     </row>
     <row r="59" ht="30" customHeight="1">
       <c r="A59" s="2" t="inlineStr">
@@ -3444,6 +3972,13 @@
           <t>Capital social 5M€, NIF 505271915. Grupo de construção top-5 nacional</t>
         </is>
       </c>
+      <c r="K59" s="2" t="inlineStr">
+        <is>
+          <t>António Carlos Rodrigues (CEO do Grupo Casais, não específico da divisão imobiliária)</t>
+        </is>
+      </c>
+      <c r="L59" s="2" t="inlineStr"/>
+      <c r="M59" s="2" t="inlineStr"/>
     </row>
     <row r="60" ht="30" customHeight="1">
       <c r="A60" s="2" t="inlineStr">
@@ -3496,6 +4031,17 @@
           <t>50 anos de história. Fonte: APPII</t>
         </is>
       </c>
+      <c r="K60" s="2" t="inlineStr">
+        <is>
+          <t>Paulo Castro (CEO)</t>
+        </is>
+      </c>
+      <c r="L60" s="2" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/paulo-castro-75946a37/</t>
+        </is>
+      </c>
+      <c r="M60" s="2" t="inlineStr"/>
     </row>
     <row r="61" ht="30" customHeight="1">
       <c r="A61" s="2" t="inlineStr">
@@ -3548,6 +4094,17 @@
           <t>Promotor vertical (conceção→construção→venda), 25+ anos</t>
         </is>
       </c>
+      <c r="K61" s="2" t="inlineStr">
+        <is>
+          <t>Artur Varum (CEO)</t>
+        </is>
+      </c>
+      <c r="L61" s="2" t="inlineStr">
+        <is>
+          <t>https://pt.linkedin.com/in/artur-varum-63599125</t>
+        </is>
+      </c>
+      <c r="M61" s="2" t="inlineStr"/>
     </row>
     <row r="62" ht="30" customHeight="1">
       <c r="A62" s="2" t="inlineStr">
@@ -3596,6 +4153,17 @@
           <t>Promotor: Greens Vilamoura Investimentos Imobiliários (grupo Enolagest). Tel. alt. 289 322 488</t>
         </is>
       </c>
+      <c r="K62" s="2" t="inlineStr">
+        <is>
+          <t>Reinaldo Teixeira (Administrador)</t>
+        </is>
+      </c>
+      <c r="L62" s="2" t="inlineStr">
+        <is>
+          <t>https://pt.linkedin.com/in/reinaldo-teixeira-821a3419</t>
+        </is>
+      </c>
+      <c r="M62" s="2" t="inlineStr"/>
     </row>
     <row r="63" ht="30" customHeight="1">
       <c r="A63" s="2" t="inlineStr">
@@ -3648,6 +4216,13 @@
           <t>Design &amp; Build, faturação 173M€ em 2025</t>
         </is>
       </c>
+      <c r="K63" s="2" t="inlineStr">
+        <is>
+          <t>Miguel Garcia (administrador, confiança moderada)</t>
+        </is>
+      </c>
+      <c r="L63" s="2" t="inlineStr"/>
+      <c r="M63" s="2" t="inlineStr"/>
     </row>
     <row r="64" ht="30" customHeight="1">
       <c r="A64" s="2" t="inlineStr">
@@ -3700,6 +4275,17 @@
           <t>Grupo de construção com 2.000 colaboradores. Fonte: Jornal de Negócios</t>
         </is>
       </c>
+      <c r="K64" s="2" t="inlineStr">
+        <is>
+          <t>Alberto Couto Alves (Presidente/CEO)</t>
+        </is>
+      </c>
+      <c r="L64" s="2" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/alberto-couto-alves-000343125/</t>
+        </is>
+      </c>
+      <c r="M64" s="2" t="inlineStr"/>
     </row>
     <row r="65" ht="30" customHeight="1">
       <c r="A65" s="2" t="inlineStr">
@@ -3752,6 +4338,13 @@
           <t>Promove, constrói e vende os próprios projetos. Fonte: diarioimobiliario.pt, idealista/news</t>
         </is>
       </c>
+      <c r="K65" s="2" t="inlineStr">
+        <is>
+          <t>Pedro Ferreira (administrador, confiança moderada)</t>
+        </is>
+      </c>
+      <c r="L65" s="2" t="inlineStr"/>
+      <c r="M65" s="2" t="inlineStr"/>
     </row>
     <row r="66" ht="30" customHeight="1">
       <c r="A66" s="2" t="inlineStr">
@@ -3804,6 +4397,17 @@
           <t>Promotor + construtor. Fonte: idealista/news, construir.pt</t>
         </is>
       </c>
+      <c r="K66" s="2" t="inlineStr">
+        <is>
+          <t>Domingos Correia (CEO)</t>
+        </is>
+      </c>
+      <c r="L66" s="2" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/domingos-correia-4453ab32/</t>
+        </is>
+      </c>
+      <c r="M66" s="2" t="inlineStr"/>
     </row>
     <row r="67" ht="30" customHeight="1">
       <c r="A67" s="2" t="inlineStr">
@@ -3852,6 +4456,13 @@
           <t>Telefone vindo do registo — confirmar em cvmnet.com/contactos</t>
         </is>
       </c>
+      <c r="K67" s="2" t="inlineStr">
+        <is>
+          <t>Severino Ponte (Administração, com Ângelo Marques)</t>
+        </is>
+      </c>
+      <c r="L67" s="2" t="inlineStr"/>
+      <c r="M67" s="2" t="inlineStr"/>
     </row>
     <row r="68" ht="30" customHeight="1">
       <c r="A68" s="2" t="inlineStr">
@@ -3904,6 +4515,13 @@
           <t>AMI 16355. Escritórios Aveiro (+351 914 444 764) e Lisboa (+351 912 325 143)</t>
         </is>
       </c>
+      <c r="K68" s="2" t="inlineStr">
+        <is>
+          <t>José Miguel Afonso (CEO/fundador)</t>
+        </is>
+      </c>
+      <c r="L68" s="2" t="inlineStr"/>
+      <c r="M68" s="2" t="inlineStr"/>
     </row>
     <row r="69" ht="30" customHeight="1">
       <c r="A69" s="2" t="inlineStr">
@@ -3952,6 +4570,17 @@
           <t>Promotora criada em 2025. Fonte: newinbraga.nit.pt, Revista Spot</t>
         </is>
       </c>
+      <c r="K69" s="2" t="inlineStr">
+        <is>
+          <t>Nuno Pinheiro (fundador)</t>
+        </is>
+      </c>
+      <c r="L69" s="2" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/nuno-pinheiro-39968aa4/</t>
+        </is>
+      </c>
+      <c r="M69" s="2" t="inlineStr"/>
     </row>
     <row r="70" ht="30" customHeight="1">
       <c r="A70" s="2" t="inlineStr">
@@ -4004,6 +4633,17 @@
           <t>Resort residencial/golfe</t>
         </is>
       </c>
+      <c r="K70" s="2" t="inlineStr">
+        <is>
+          <t>Sean Moriarty (CEO)</t>
+        </is>
+      </c>
+      <c r="L70" s="2" t="inlineStr">
+        <is>
+          <t>https://pt.linkedin.com/in/sean-moriarty-6a749133</t>
+        </is>
+      </c>
+      <c r="M70" s="2" t="inlineStr"/>
     </row>
     <row r="71" ht="30" customHeight="1">
       <c r="A71" s="2" t="inlineStr">
@@ -4056,6 +4696,13 @@
           <t>Uma das maiores construtoras nacionais · delegações Lisboa e Algarve</t>
         </is>
       </c>
+      <c r="K71" s="2" t="inlineStr">
+        <is>
+          <t>Bruno Fernando Macedo Soares (CEO/Presidente do CA)</t>
+        </is>
+      </c>
+      <c r="L71" s="2" t="inlineStr"/>
+      <c r="M71" s="2" t="inlineStr"/>
     </row>
     <row r="72" ht="30" customHeight="1">
       <c r="A72" s="5" t="inlineStr">
@@ -4088,6 +4735,13 @@
           <t>Entidade PT: André Guimarães - Portugal, Lda (NIF 517865459). Sem contacto PT</t>
         </is>
       </c>
+      <c r="K72" s="5" t="inlineStr">
+        <is>
+          <t>Fundador falecido· hoje liderado pelos filhos (Brasil), sem responsável PT confirmado</t>
+        </is>
+      </c>
+      <c r="L72" s="5" t="inlineStr"/>
+      <c r="M72" s="5" t="inlineStr"/>
     </row>
     <row r="73" ht="30" customHeight="1">
       <c r="A73" s="5" t="inlineStr">
@@ -4132,6 +4786,17 @@
           <t>Grupo finlandês Pontos · construtor Gabriel Couto</t>
         </is>
       </c>
+      <c r="K73" s="5" t="inlineStr">
+        <is>
+          <t>Patrick Freeman (CEO Ombria desde 2023)· CEO do Grupo Pontos é Timo Kokkila</t>
+        </is>
+      </c>
+      <c r="L73" s="5" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/patricksfreeman/</t>
+        </is>
+      </c>
+      <c r="M73" s="5" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -4147,7 +4812,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B7"/>
+  <dimension ref="A1:B10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="42" customWidth="1" min="1" max="1"/>
@@ -4207,18 +4872,50 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="9" t="n"/>
-      <c r="B6" s="9" t="n"/>
+      <c r="A6" s="9" t="inlineStr">
+        <is>
+          <t>Com nome de CEO/administrador identificado</t>
+        </is>
+      </c>
+      <c r="B6" s="9" t="n">
+        <v>65</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="9" t="inlineStr">
         <is>
+          <t>Com LinkedIn pessoal do CEO confirmado</t>
+        </is>
+      </c>
+      <c r="B7" s="9" t="n">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="9" t="n"/>
+      <c r="B8" s="9" t="n"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="9" t="inlineStr">
+        <is>
           <t>Nota</t>
         </is>
       </c>
-      <c r="B7" s="9" t="inlineStr">
+      <c r="B9" s="9" t="inlineStr">
         <is>
           <t>Linhas com fundo laranja claro na folha 'Promotoras' não têm telefone confirmado — use o email, o site ou o LinkedIn indicado nas Notas.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="9" t="inlineStr">
+        <is>
+          <t>Nota CEO/LinkedIn/Instagram</t>
+        </is>
+      </c>
+      <c r="B10" s="9" t="inlineStr">
+        <is>
+          <t>Nenhum handle de Instagram pessoal foi encontrado com confiança para nenhum CEO — por isso a coluna vem vazia em todas as linhas (não foi inventado nenhum perfil). Alguns nomes de CEO/LinkedIn têm confiança moderada — ver texto entre parênteses na coluna CEO.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Fill in CEO/LinkedIn for the 75 newly added promoters
Researched via targeted web search (spawned subagents hit an account
spend-limit mid-run, so this pass ran through direct searches instead).
44 of 75 now have a confirmed CEO/administrator name; 20 of those also
have a personal LinkedIn profile. The remaining 31 are left blank —
searched but not found with confidence, never guessed. No personal
Instagram was found for any CEO in this batch either, consistent with
the original 72.

Map artifact (same published URL) and xlsx export updated in the same
pass.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01SRBJwGmSsYkTHKJbGCM5ca
</commit_message>
<xml_diff>
--- a/Promotoras_Imobiliarias_Contactos.xlsx
+++ b/Promotoras_Imobiliarias_Contactos.xlsx
@@ -3245,7 +3245,11 @@
           <t>Fonte: diarioimobiliario.pt</t>
         </is>
       </c>
-      <c r="K46" s="5" t="inlineStr"/>
+      <c r="K46" s="5" t="inlineStr">
+        <is>
+          <t>Victor de Sousa (Diretor-Geral AFA Real Estate)</t>
+        </is>
+      </c>
       <c r="L46" s="5" t="inlineStr"/>
       <c r="M46" s="5" t="inlineStr"/>
     </row>
@@ -3421,7 +3425,11 @@
           <t>Fonte: viva-porto.pt</t>
         </is>
       </c>
-      <c r="K50" s="5" t="inlineStr"/>
+      <c r="K50" s="5" t="inlineStr">
+        <is>
+          <t>Bruno Soares (CEO, família Soares/Latitude Capital)</t>
+        </is>
+      </c>
       <c r="L50" s="5" t="inlineStr"/>
       <c r="M50" s="5" t="inlineStr"/>
     </row>
@@ -3605,7 +3613,11 @@
           <t>Fonte: construir.pt</t>
         </is>
       </c>
-      <c r="K54" s="5" t="inlineStr"/>
+      <c r="K54" s="5" t="inlineStr">
+        <is>
+          <t>João Magalhães e Alexandre Magalhães (promotores individuais)</t>
+        </is>
+      </c>
       <c r="L54" s="5" t="inlineStr"/>
       <c r="M54" s="5" t="inlineStr"/>
     </row>
@@ -3644,7 +3656,11 @@
           <t>Fonte: vidaimobiliaria.com</t>
         </is>
       </c>
-      <c r="K55" s="5" t="inlineStr"/>
+      <c r="K55" s="5" t="inlineStr">
+        <is>
+          <t>Vera Kendall (administradora, dados de 2018 · confiança baixa)</t>
+        </is>
+      </c>
       <c r="L55" s="5" t="inlineStr"/>
       <c r="M55" s="5" t="inlineStr"/>
     </row>
@@ -3734,7 +3750,11 @@
           <t>Fonte: construir.pt</t>
         </is>
       </c>
-      <c r="K57" s="5" t="inlineStr"/>
+      <c r="K57" s="5" t="inlineStr">
+        <is>
+          <t>Nuno Cunha (Managing Director)</t>
+        </is>
+      </c>
       <c r="L57" s="5" t="inlineStr"/>
       <c r="M57" s="5" t="inlineStr"/>
     </row>
@@ -3820,7 +3840,11 @@
           <t>Fonte: dinheirovivo.pt, construir.pt</t>
         </is>
       </c>
-      <c r="K59" s="5" t="inlineStr"/>
+      <c r="K59" s="5" t="inlineStr">
+        <is>
+          <t>Paula Fernandes (CEO)</t>
+        </is>
+      </c>
       <c r="L59" s="5" t="inlineStr"/>
       <c r="M59" s="5" t="inlineStr"/>
     </row>
@@ -4098,8 +4122,16 @@
           <t>Fonte: idealista.pt</t>
         </is>
       </c>
-      <c r="K65" s="5" t="inlineStr"/>
-      <c r="L65" s="5" t="inlineStr"/>
+      <c r="K65" s="5" t="inlineStr">
+        <is>
+          <t>Paula Santos (Diretora Geral Visabeirahouse)</t>
+        </is>
+      </c>
+      <c r="L65" s="5" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/paula-santos-71083337/</t>
+        </is>
+      </c>
       <c r="M65" s="5" t="inlineStr"/>
     </row>
     <row r="66" ht="30" customHeight="1">
@@ -4385,8 +4417,16 @@
           <t>Fonte: diarioimobiliario.pt</t>
         </is>
       </c>
-      <c r="K70" s="2" t="inlineStr"/>
-      <c r="L70" s="2" t="inlineStr"/>
+      <c r="K70" s="2" t="inlineStr">
+        <is>
+          <t>Rosalía Torres Ruiz-Olivares (Co-founder)</t>
+        </is>
+      </c>
+      <c r="L70" s="2" t="inlineStr">
+        <is>
+          <t>https://ae.linkedin.com/in/rosal%C3%ADa-torres-ruiz-olivares-51702725</t>
+        </is>
+      </c>
       <c r="M70" s="2" t="inlineStr"/>
     </row>
     <row r="71" ht="30" customHeight="1">
@@ -4680,7 +4720,11 @@
           <t>Fonte: idealista.pt</t>
         </is>
       </c>
-      <c r="K75" s="2" t="inlineStr"/>
+      <c r="K75" s="2" t="inlineStr">
+        <is>
+          <t>Diogo Baptista Antunes (CEO)</t>
+        </is>
+      </c>
       <c r="L75" s="2" t="inlineStr"/>
       <c r="M75" s="2" t="inlineStr"/>
     </row>
@@ -5085,8 +5129,16 @@
           <t>Fonte: sapo.pt</t>
         </is>
       </c>
-      <c r="K82" s="2" t="inlineStr"/>
-      <c r="L82" s="2" t="inlineStr"/>
+      <c r="K82" s="2" t="inlineStr">
+        <is>
+          <t>Miguel Tilli (fundador e CEO)</t>
+        </is>
+      </c>
+      <c r="L82" s="2" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/miguel-tilli-a7a41587/</t>
+        </is>
+      </c>
       <c r="M82" s="2" t="inlineStr"/>
     </row>
     <row r="83" ht="30" customHeight="1">
@@ -5313,7 +5365,11 @@
           <t>Fonte: vidaimobiliaria.com</t>
         </is>
       </c>
-      <c r="K86" s="2" t="inlineStr"/>
+      <c r="K86" s="2" t="inlineStr">
+        <is>
+          <t>João Luís Ferreira (Chairman &amp; Partner)</t>
+        </is>
+      </c>
       <c r="L86" s="2" t="inlineStr"/>
       <c r="M86" s="2" t="inlineStr"/>
     </row>
@@ -5360,8 +5416,16 @@
           <t>Fonte: vidaimobiliaria.com</t>
         </is>
       </c>
-      <c r="K87" s="2" t="inlineStr"/>
-      <c r="L87" s="2" t="inlineStr"/>
+      <c r="K87" s="2" t="inlineStr">
+        <is>
+          <t>Diogo Sá Viana Rebelo (Co-Founder)</t>
+        </is>
+      </c>
+      <c r="L87" s="2" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/diogo-s%C3%A1-viana-rebelo-910104143/</t>
+        </is>
+      </c>
       <c r="M87" s="2" t="inlineStr"/>
     </row>
     <row r="88" ht="30" customHeight="1">
@@ -5466,7 +5530,11 @@
           <t>Fonte: omirante.pt</t>
         </is>
       </c>
-      <c r="K89" s="2" t="inlineStr"/>
+      <c r="K89" s="2" t="inlineStr">
+        <is>
+          <t>Sérgio Santos (CEO/fundador, com Delphine Gerardo)</t>
+        </is>
+      </c>
       <c r="L89" s="2" t="inlineStr"/>
       <c r="M89" s="2" t="inlineStr"/>
     </row>
@@ -5544,7 +5612,11 @@
           <t>Fonte: idealista.pt, vidaimobiliaria.com</t>
         </is>
       </c>
-      <c r="K91" s="5" t="inlineStr"/>
+      <c r="K91" s="5" t="inlineStr">
+        <is>
+          <t>Miguel Guedes de Sousa (Founder &amp; CEO)</t>
+        </is>
+      </c>
       <c r="L91" s="5" t="inlineStr"/>
       <c r="M91" s="5" t="inlineStr"/>
     </row>
@@ -5622,7 +5694,11 @@
           <t>Fonte: idealista.pt, jornaleconomico.sapo.pt</t>
         </is>
       </c>
-      <c r="K93" s="5" t="inlineStr"/>
+      <c r="K93" s="5" t="inlineStr">
+        <is>
+          <t>João Bugalho (CEO)</t>
+        </is>
+      </c>
       <c r="L93" s="5" t="inlineStr"/>
       <c r="M93" s="5" t="inlineStr"/>
     </row>
@@ -5665,7 +5741,11 @@
           <t>Fonte: ominho.pt</t>
         </is>
       </c>
-      <c r="K94" s="5" t="inlineStr"/>
+      <c r="K94" s="5" t="inlineStr">
+        <is>
+          <t>Paulo Balinha e Bruno Torres (fundadores, 2008)</t>
+        </is>
+      </c>
       <c r="L94" s="5" t="inlineStr"/>
       <c r="M94" s="5" t="inlineStr"/>
     </row>
@@ -5946,8 +6026,16 @@
           <t>Fonte: idealista.pt</t>
         </is>
       </c>
-      <c r="K101" s="5" t="inlineStr"/>
-      <c r="L101" s="5" t="inlineStr"/>
+      <c r="K101" s="5" t="inlineStr">
+        <is>
+          <t>David Faria (CEO e sócio único)</t>
+        </is>
+      </c>
+      <c r="L101" s="5" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/david-faria-a301a466/</t>
+        </is>
+      </c>
       <c r="M101" s="5" t="inlineStr"/>
     </row>
     <row r="102" ht="30" customHeight="1">
@@ -5985,7 +6073,11 @@
           <t>Fonte: noticiasdeaveiro.pt, terranova.pt</t>
         </is>
       </c>
-      <c r="K102" s="5" t="inlineStr"/>
+      <c r="K102" s="5" t="inlineStr">
+        <is>
+          <t>Aristides Alferes (administrador)</t>
+        </is>
+      </c>
       <c r="L102" s="5" t="inlineStr"/>
       <c r="M102" s="5" t="inlineStr"/>
     </row>
@@ -6024,7 +6116,11 @@
           <t>Fonte: vidaimobiliaria.com</t>
         </is>
       </c>
-      <c r="K103" s="5" t="inlineStr"/>
+      <c r="K103" s="5" t="inlineStr">
+        <is>
+          <t>Hugo Mendes Pinto (Managing Partner)</t>
+        </is>
+      </c>
       <c r="L103" s="5" t="inlineStr"/>
       <c r="M103" s="5" t="inlineStr"/>
     </row>
@@ -6067,7 +6163,11 @@
           <t>Fonte: jornaldenegocios.pt</t>
         </is>
       </c>
-      <c r="K104" s="5" t="inlineStr"/>
+      <c r="K104" s="5" t="inlineStr">
+        <is>
+          <t>Elizabeth Rothfield (CEO, Founding Partner)</t>
+        </is>
+      </c>
       <c r="L104" s="5" t="inlineStr"/>
       <c r="M104" s="5" t="inlineStr"/>
     </row>
@@ -6106,7 +6206,11 @@
           <t>Fonte: jornaldenegocios.pt, idealista.pt</t>
         </is>
       </c>
-      <c r="K105" s="5" t="inlineStr"/>
+      <c r="K105" s="5" t="inlineStr">
+        <is>
+          <t>Paul Henri Schelfhout (Presidente do CA) / Armando Lacerda Queiroz (administrador)</t>
+        </is>
+      </c>
       <c r="L105" s="5" t="inlineStr"/>
       <c r="M105" s="5" t="inlineStr"/>
     </row>
@@ -6309,7 +6413,11 @@
           <t>Fonte: eco.sapo.pt, jornaldenegocios.pt</t>
         </is>
       </c>
-      <c r="K110" s="5" t="inlineStr"/>
+      <c r="K110" s="5" t="inlineStr">
+        <is>
+          <t>Joaquim Silva (CEO Ferreira Build Power)</t>
+        </is>
+      </c>
       <c r="L110" s="5" t="inlineStr"/>
       <c r="M110" s="5" t="inlineStr"/>
     </row>
@@ -6473,7 +6581,11 @@
           <t>Fonte: idealista.pt</t>
         </is>
       </c>
-      <c r="K114" s="5" t="inlineStr"/>
+      <c r="K114" s="5" t="inlineStr">
+        <is>
+          <t>Gilberto Jordan (CEO desde 2009 · sucede a André Jordan, falecido 2024)</t>
+        </is>
+      </c>
       <c r="L114" s="5" t="inlineStr"/>
       <c r="M114" s="5" t="inlineStr"/>
     </row>
@@ -6512,7 +6624,11 @@
           <t>Fonte: linkedin.com/company/grupo-aoc</t>
         </is>
       </c>
-      <c r="K115" s="5" t="inlineStr"/>
+      <c r="K115" s="5" t="inlineStr">
+        <is>
+          <t>Aníbal Cristina (fundador, 1990)</t>
+        </is>
+      </c>
       <c r="L115" s="5" t="inlineStr"/>
       <c r="M115" s="5" t="inlineStr"/>
     </row>
@@ -6551,8 +6667,16 @@
           <t>Fonte: idealista.pt</t>
         </is>
       </c>
-      <c r="K116" s="5" t="inlineStr"/>
-      <c r="L116" s="5" t="inlineStr"/>
+      <c r="K116" s="5" t="inlineStr">
+        <is>
+          <t>Carlos Silva Neves (administrador)</t>
+        </is>
+      </c>
+      <c r="L116" s="5" t="inlineStr">
+        <is>
+          <t>https://pt.linkedin.com/in/carlos-silva-neves-3b0711142</t>
+        </is>
+      </c>
       <c r="M116" s="5" t="inlineStr"/>
     </row>
     <row r="117" ht="30" customHeight="1">
@@ -6637,7 +6761,11 @@
           <t>Fonte: gruponb.pt</t>
         </is>
       </c>
-      <c r="K118" s="5" t="inlineStr"/>
+      <c r="K118" s="5" t="inlineStr">
+        <is>
+          <t>Ioav Blanche (presidente)</t>
+        </is>
+      </c>
       <c r="L118" s="5" t="inlineStr"/>
       <c r="M118" s="5" t="inlineStr"/>
     </row>
@@ -6680,7 +6808,11 @@
           <t>Fonte: publico.pt, construir.pt</t>
         </is>
       </c>
-      <c r="K119" s="5" t="inlineStr"/>
+      <c r="K119" s="5" t="inlineStr">
+        <is>
+          <t>Dionísio Pestana (Chairman/dono)</t>
+        </is>
+      </c>
       <c r="L119" s="5" t="inlineStr"/>
       <c r="M119" s="5" t="inlineStr"/>
     </row>
@@ -6848,8 +6980,16 @@
           <t>Fonte: jpaiva.pt</t>
         </is>
       </c>
-      <c r="K123" s="5" t="inlineStr"/>
-      <c r="L123" s="5" t="inlineStr"/>
+      <c r="K123" s="5" t="inlineStr">
+        <is>
+          <t>Igor Castro (CEO)</t>
+        </is>
+      </c>
+      <c r="L123" s="5" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/igor-castro-a0026b22b/</t>
+        </is>
+      </c>
       <c r="M123" s="5" t="inlineStr"/>
     </row>
     <row r="124" ht="30" customHeight="1">
@@ -6891,7 +7031,11 @@
           <t>Fonte: luxpremium.net</t>
         </is>
       </c>
-      <c r="K124" s="5" t="inlineStr"/>
+      <c r="K124" s="5" t="inlineStr">
+        <is>
+          <t>Claude Berda (fundador)</t>
+        </is>
+      </c>
       <c r="L124" s="5" t="inlineStr"/>
       <c r="M124" s="5" t="inlineStr"/>
     </row>
@@ -6930,7 +7074,11 @@
           <t>Fonte: oconnormurphy.ie</t>
         </is>
       </c>
-      <c r="K125" s="5" t="inlineStr"/>
+      <c r="K125" s="5" t="inlineStr">
+        <is>
+          <t>Manuel António e Jorge Almeida (fundadores, 1972)</t>
+        </is>
+      </c>
       <c r="L125" s="5" t="inlineStr"/>
       <c r="M125" s="5" t="inlineStr"/>
     </row>
@@ -7012,7 +7160,11 @@
           <t>Fonte: maveninvest.pt</t>
         </is>
       </c>
-      <c r="K127" s="5" t="inlineStr"/>
+      <c r="K127" s="5" t="inlineStr">
+        <is>
+          <t>Yehonatan Gourvitch (CEO)</t>
+        </is>
+      </c>
       <c r="L127" s="5" t="inlineStr"/>
       <c r="M127" s="5" t="inlineStr"/>
     </row>
@@ -7055,8 +7207,16 @@
           <t>Fonte: vidaimobiliaria.com</t>
         </is>
       </c>
-      <c r="K128" s="5" t="inlineStr"/>
-      <c r="L128" s="5" t="inlineStr"/>
+      <c r="K128" s="5" t="inlineStr">
+        <is>
+          <t>António Ribeiro da Cunha (CEO)</t>
+        </is>
+      </c>
+      <c r="L128" s="5" t="inlineStr">
+        <is>
+          <t>https://pt.linkedin.com/in/ant%C3%B3nio-ribeiro-da-cunha-77b974112</t>
+        </is>
+      </c>
       <c r="M128" s="5" t="inlineStr"/>
     </row>
     <row r="129" ht="30" customHeight="1">
@@ -7133,7 +7293,11 @@
           <t>Fonte: jornaleconomico.sapo.pt</t>
         </is>
       </c>
-      <c r="K130" s="5" t="inlineStr"/>
+      <c r="K130" s="5" t="inlineStr">
+        <is>
+          <t>Matan Amitai (co-fundador)</t>
+        </is>
+      </c>
       <c r="L130" s="5" t="inlineStr"/>
       <c r="M130" s="5" t="inlineStr"/>
     </row>
@@ -7309,7 +7473,11 @@
           <t>Fonte: racius.com, cnnportugal.iol.pt</t>
         </is>
       </c>
-      <c r="K134" s="5" t="inlineStr"/>
+      <c r="K134" s="5" t="inlineStr">
+        <is>
+          <t>Joaquim Da Cunha Mendes Duarte (Presidente) / Sergio Manuel Mendes Gomes (Administrador)</t>
+        </is>
+      </c>
       <c r="L134" s="5" t="inlineStr"/>
       <c r="M134" s="5" t="inlineStr"/>
     </row>
@@ -7426,7 +7594,11 @@
           <t>Fonte: jornaldenegocios.pt</t>
         </is>
       </c>
-      <c r="K137" s="5" t="inlineStr"/>
+      <c r="K137" s="5" t="inlineStr">
+        <is>
+          <t>João Ribeiro (CEO e fundador, com Jorge Duarte e Fernando Santos)</t>
+        </is>
+      </c>
       <c r="L137" s="5" t="inlineStr"/>
       <c r="M137" s="5" t="inlineStr"/>
     </row>
@@ -7469,7 +7641,11 @@
           <t>Fonte: sava.pt, thepreplan.com</t>
         </is>
       </c>
-      <c r="K138" s="5" t="inlineStr"/>
+      <c r="K138" s="5" t="inlineStr">
+        <is>
+          <t>Celestino Vermelho Rodrigues (contacto)</t>
+        </is>
+      </c>
       <c r="L138" s="5" t="inlineStr"/>
       <c r="M138" s="5" t="inlineStr"/>
     </row>
@@ -7512,8 +7688,16 @@
           <t>Fonte: eco.sapo.pt</t>
         </is>
       </c>
-      <c r="K139" s="5" t="inlineStr"/>
-      <c r="L139" s="5" t="inlineStr"/>
+      <c r="K139" s="5" t="inlineStr">
+        <is>
+          <t>António Vaz (fundador e CEO)</t>
+        </is>
+      </c>
+      <c r="L139" s="5" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/antonio-vaz-9444998a/</t>
+        </is>
+      </c>
       <c r="M139" s="5" t="inlineStr"/>
     </row>
     <row r="140" ht="30" customHeight="1">
@@ -7555,8 +7739,16 @@
           <t>Fonte: reportugal.vidaimobiliaria.com</t>
         </is>
       </c>
-      <c r="K140" s="5" t="inlineStr"/>
-      <c r="L140" s="5" t="inlineStr"/>
+      <c r="K140" s="5" t="inlineStr">
+        <is>
+          <t>Alain Gross (Co-Founder e CEO)</t>
+        </is>
+      </c>
+      <c r="L140" s="5" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/alain-gross-3351411/</t>
+        </is>
+      </c>
       <c r="M140" s="5" t="inlineStr"/>
     </row>
     <row r="141" ht="30" customHeight="1">
@@ -7637,7 +7829,11 @@
           <t>Fonte: rtp.pt, idealista.pt</t>
         </is>
       </c>
-      <c r="K142" s="5" t="inlineStr"/>
+      <c r="K142" s="5" t="inlineStr">
+        <is>
+          <t>Fernando Guedes de Oliveira (CEO)</t>
+        </is>
+      </c>
       <c r="L142" s="5" t="inlineStr"/>
       <c r="M142" s="5" t="inlineStr"/>
     </row>
@@ -7723,7 +7919,11 @@
           <t>Fonte: squareview.pt</t>
         </is>
       </c>
-      <c r="K144" s="5" t="inlineStr"/>
+      <c r="K144" s="5" t="inlineStr">
+        <is>
+          <t>Luis Horta e Costa (CEO/Fundador)</t>
+        </is>
+      </c>
       <c r="L144" s="5" t="inlineStr"/>
       <c r="M144" s="5" t="inlineStr"/>
     </row>
@@ -7844,7 +8044,11 @@
           <t>Fonte: theshipyard.pt, barlavento.pt</t>
         </is>
       </c>
-      <c r="K147" s="5" t="inlineStr"/>
+      <c r="K147" s="5" t="inlineStr">
+        <is>
+          <t>Thomas Coughlan (fundador)</t>
+        </is>
+      </c>
       <c r="L147" s="5" t="inlineStr"/>
       <c r="M147" s="5" t="inlineStr"/>
     </row>
@@ -7971,7 +8175,7 @@
         </is>
       </c>
       <c r="B6" s="9" t="n">
-        <v>65</v>
+        <v>106</v>
       </c>
     </row>
     <row r="7">
@@ -7981,7 +8185,7 @@
         </is>
       </c>
       <c r="B7" s="9" t="n">
-        <v>42</v>
+        <v>52</v>
       </c>
     </row>
     <row r="8">

</xml_diff>

<commit_message>
Add 3 more promoters (160 total): DST Real Estate, Le Parc, The Epic Group
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01SRBJwGmSsYkTHKJbGCM5ca
</commit_message>
<xml_diff>
--- a/Promotoras_Imobiliarias_Contactos.xlsx
+++ b/Promotoras_Imobiliarias_Contactos.xlsx
@@ -191,8 +191,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Promotoras" displayName="Promotoras" ref="A1:M158" headerRowCount="1">
-  <autoFilter ref="A1:M158"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Promotoras" displayName="Promotoras" ref="A1:M161" headerRowCount="1">
+  <autoFilter ref="A1:M161"/>
   <tableColumns count="13">
     <tableColumn id="1" name="Nome da Empresa"/>
     <tableColumn id="2" name="Prioritario"/>
@@ -501,7 +501,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M158"/>
+  <dimension ref="A1:M161"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -5013,7 +5013,7 @@
     <row r="82" ht="30" customHeight="1">
       <c r="A82" s="2" t="inlineStr">
         <is>
-          <t>Enolagest / Garvetur (Greens Vilamoura)</t>
+          <t>DST Real Estate (Grupo dst)</t>
         </is>
       </c>
       <c r="B82" s="4" t="inlineStr">
@@ -5023,56 +5023,52 @@
       </c>
       <c r="C82" s="4" t="inlineStr">
         <is>
-          <t>+351 289 381 550</t>
-        </is>
-      </c>
-      <c r="D82" s="2" t="inlineStr"/>
+          <t>+351 253 307 200</t>
+        </is>
+      </c>
+      <c r="D82" s="2" t="inlineStr">
+        <is>
+          <t>geral@dstsgps.com</t>
+        </is>
+      </c>
       <c r="E82" s="2" t="inlineStr">
         <is>
-          <t>enolagest.pt</t>
+          <t>dstsgps.com</t>
         </is>
       </c>
       <c r="F82" s="4" t="inlineStr">
         <is>
-          <t>Loulé</t>
+          <t>Braga</t>
         </is>
       </c>
       <c r="G82" s="4" t="inlineStr">
         <is>
-          <t>Faro</t>
+          <t>Braga</t>
         </is>
       </c>
       <c r="H82" s="2" t="inlineStr">
         <is>
-          <t>Rua Melvin Jones, Volta do Gaio, Vilamoura, 8125-406</t>
+          <t>Rua de Pitancinhos - Palmeira, 4700-727</t>
         </is>
       </c>
       <c r="I82" s="2" t="inlineStr">
         <is>
-          <t>Greens Vilamoura (Em construção)</t>
+          <t>Museu no centro histórico de Braga (Em construção)</t>
         </is>
       </c>
       <c r="J82" s="2" t="inlineStr">
         <is>
-          <t>Promotor: Greens Vilamoura Investimentos Imobiliários (grupo Enolagest). Tel. alt. 289 322 488</t>
-        </is>
-      </c>
-      <c r="K82" s="2" t="inlineStr">
-        <is>
-          <t>Reinaldo Teixeira (Administrador)</t>
-        </is>
-      </c>
-      <c r="L82" s="2" t="inlineStr">
-        <is>
-          <t>https://pt.linkedin.com/in/reinaldo-teixeira-821a3419</t>
-        </is>
-      </c>
+          <t>Braço imobiliário do Grupo dst (Domingos da Silva Teixeira)</t>
+        </is>
+      </c>
+      <c r="K82" s="2" t="inlineStr"/>
+      <c r="L82" s="2" t="inlineStr"/>
       <c r="M82" s="2" t="inlineStr"/>
     </row>
     <row r="83" ht="30" customHeight="1">
       <c r="A83" s="2" t="inlineStr">
         <is>
-          <t>Garcia Garcia</t>
+          <t>Enolagest / Garvetur (Greens Vilamoura)</t>
         </is>
       </c>
       <c r="B83" s="4" t="inlineStr">
@@ -5082,56 +5078,56 @@
       </c>
       <c r="C83" s="4" t="inlineStr">
         <is>
-          <t>+351 253 560 230</t>
-        </is>
-      </c>
-      <c r="D83" s="2" t="inlineStr">
-        <is>
-          <t>geral@garcia.pt</t>
-        </is>
-      </c>
+          <t>+351 289 381 550</t>
+        </is>
+      </c>
+      <c r="D83" s="2" t="inlineStr"/>
       <c r="E83" s="2" t="inlineStr">
         <is>
-          <t>garcia.pt</t>
+          <t>enolagest.pt</t>
         </is>
       </c>
       <c r="F83" s="4" t="inlineStr">
         <is>
-          <t>Santo Tirso</t>
+          <t>Loulé</t>
         </is>
       </c>
       <c r="G83" s="4" t="inlineStr">
         <is>
-          <t>Porto</t>
+          <t>Faro</t>
         </is>
       </c>
       <c r="H83" s="2" t="inlineStr">
         <is>
-          <t>Rua Comendador António Maria Lopes 15, 4780-424</t>
+          <t>Rua Melvin Jones, Volta do Gaio, Vilamoura, 8125-406</t>
         </is>
       </c>
       <c r="I83" s="2" t="inlineStr">
         <is>
-          <t>Couros Residence (Guimarães) (Concluído) | Arco Living (Santo Tirso) (Concluído) | Residência de estudantes Hines (Porto, Paranhos) (Em construção)</t>
+          <t>Greens Vilamoura (Em construção)</t>
         </is>
       </c>
       <c r="J83" s="2" t="inlineStr">
         <is>
-          <t>Design &amp; Build, faturação 173M€ em 2025</t>
+          <t>Promotor: Greens Vilamoura Investimentos Imobiliários (grupo Enolagest). Tel. alt. 289 322 488</t>
         </is>
       </c>
       <c r="K83" s="2" t="inlineStr">
         <is>
-          <t>Miguel Garcia (administrador, confiança moderada)</t>
-        </is>
-      </c>
-      <c r="L83" s="2" t="inlineStr"/>
+          <t>Reinaldo Teixeira (Administrador)</t>
+        </is>
+      </c>
+      <c r="L83" s="2" t="inlineStr">
+        <is>
+          <t>https://pt.linkedin.com/in/reinaldo-teixeira-821a3419</t>
+        </is>
+      </c>
       <c r="M83" s="2" t="inlineStr"/>
     </row>
     <row r="84" ht="30" customHeight="1">
       <c r="A84" s="2" t="inlineStr">
         <is>
-          <t>Grupo ACA / ACA Real Estate (marca Pousio)</t>
+          <t>Garcia Garcia</t>
         </is>
       </c>
       <c r="B84" s="4" t="inlineStr">
@@ -5141,60 +5137,56 @@
       </c>
       <c r="C84" s="4" t="inlineStr">
         <is>
-          <t>+351 252 308 250</t>
+          <t>+351 253 560 230</t>
         </is>
       </c>
       <c r="D84" s="2" t="inlineStr">
         <is>
-          <t>aca@grupo-aca.com</t>
+          <t>geral@garcia.pt</t>
         </is>
       </c>
       <c r="E84" s="2" t="inlineStr">
         <is>
-          <t>grupo-aca.com</t>
+          <t>garcia.pt</t>
         </is>
       </c>
       <c r="F84" s="4" t="inlineStr">
         <is>
-          <t>Vila Nova de Famalicão</t>
+          <t>Santo Tirso</t>
         </is>
       </c>
       <c r="G84" s="4" t="inlineStr">
         <is>
-          <t>Braga</t>
+          <t>Porto</t>
         </is>
       </c>
       <c r="H84" s="2" t="inlineStr">
         <is>
-          <t>Av. dos Descobrimentos, Ed. Las Vegas 3, nº63</t>
+          <t>Rua Comendador António Maria Lopes 15, 4780-424</t>
         </is>
       </c>
       <c r="I84" s="2" t="inlineStr">
         <is>
-          <t>Pousio (Aveiro, Gaia, Lisboa) (Planeamento)</t>
+          <t>Couros Residence (Guimarães) (Concluído) | Arco Living (Santo Tirso) (Concluído) | Residência de estudantes Hines (Porto, Paranhos) (Em construção)</t>
         </is>
       </c>
       <c r="J84" s="2" t="inlineStr">
         <is>
-          <t>Grupo de construção com 2.000 colaboradores. Fonte: Jornal de Negócios</t>
+          <t>Design &amp; Build, faturação 173M€ em 2025</t>
         </is>
       </c>
       <c r="K84" s="2" t="inlineStr">
         <is>
-          <t>Alberto Couto Alves (Presidente/CEO)</t>
-        </is>
-      </c>
-      <c r="L84" s="2" t="inlineStr">
-        <is>
-          <t>https://www.linkedin.com/in/alberto-couto-alves-000343125/</t>
-        </is>
-      </c>
+          <t>Miguel Garcia (administrador, confiança moderada)</t>
+        </is>
+      </c>
+      <c r="L84" s="2" t="inlineStr"/>
       <c r="M84" s="2" t="inlineStr"/>
     </row>
     <row r="85" ht="30" customHeight="1">
       <c r="A85" s="2" t="inlineStr">
         <is>
-          <t>Grupo Acrescentar</t>
+          <t>Grupo ACA / ACA Real Estate (marca Pousio)</t>
         </is>
       </c>
       <c r="B85" s="4" t="inlineStr">
@@ -5204,56 +5196,60 @@
       </c>
       <c r="C85" s="4" t="inlineStr">
         <is>
-          <t>+351 253 685 109</t>
+          <t>+351 252 308 250</t>
         </is>
       </c>
       <c r="D85" s="2" t="inlineStr">
         <is>
-          <t>acrescentar@grupoacrescentar.pt</t>
+          <t>aca@grupo-aca.com</t>
         </is>
       </c>
       <c r="E85" s="2" t="inlineStr">
         <is>
-          <t>grupoacrescentar.pt</t>
+          <t>grupo-aca.com</t>
         </is>
       </c>
       <c r="F85" s="4" t="inlineStr">
         <is>
+          <t>Vila Nova de Famalicão</t>
+        </is>
+      </c>
+      <c r="G85" s="4" t="inlineStr">
+        <is>
           <t>Braga</t>
         </is>
       </c>
-      <c r="G85" s="4" t="inlineStr">
-        <is>
-          <t>Braga</t>
-        </is>
-      </c>
       <c r="H85" s="2" t="inlineStr">
         <is>
-          <t>Rua Quinta dos Lagos 24, 4700-289 Real</t>
+          <t>Av. dos Descobrimentos, Ed. Las Vegas 3, nº63</t>
         </is>
       </c>
       <c r="I85" s="2" t="inlineStr">
         <is>
-          <t>Green Terrace Porto (Requesende) (Em construção) | Garden Palace (Comercialização) | Strata Private Residence (Comercialização) | Vess Living (Guimarães) (Em construção)</t>
+          <t>Pousio (Aveiro, Gaia, Lisboa) (Planeamento)</t>
         </is>
       </c>
       <c r="J85" s="2" t="inlineStr">
         <is>
-          <t>Promove, constrói e vende os próprios projetos. Fonte: diarioimobiliario.pt, idealista/news</t>
+          <t>Grupo de construção com 2.000 colaboradores. Fonte: Jornal de Negócios</t>
         </is>
       </c>
       <c r="K85" s="2" t="inlineStr">
         <is>
-          <t>Pedro Ferreira (administrador, confiança moderada)</t>
-        </is>
-      </c>
-      <c r="L85" s="2" t="inlineStr"/>
+          <t>Alberto Couto Alves (Presidente/CEO)</t>
+        </is>
+      </c>
+      <c r="L85" s="2" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/alberto-couto-alves-000343125/</t>
+        </is>
+      </c>
       <c r="M85" s="2" t="inlineStr"/>
     </row>
     <row r="86" ht="30" customHeight="1">
       <c r="A86" s="2" t="inlineStr">
         <is>
-          <t>Grupo Arliz</t>
+          <t>Grupo Acrescentar</t>
         </is>
       </c>
       <c r="B86" s="4" t="inlineStr">
@@ -5263,17 +5259,17 @@
       </c>
       <c r="C86" s="4" t="inlineStr">
         <is>
-          <t>+351 253 105 331</t>
+          <t>+351 253 685 109</t>
         </is>
       </c>
       <c r="D86" s="2" t="inlineStr">
         <is>
-          <t>geral@arliz.co</t>
+          <t>acrescentar@grupoacrescentar.pt</t>
         </is>
       </c>
       <c r="E86" s="2" t="inlineStr">
         <is>
-          <t>grupoarliz.pt</t>
+          <t>grupoacrescentar.pt</t>
         </is>
       </c>
       <c r="F86" s="4" t="inlineStr">
@@ -5288,35 +5284,31 @@
       </c>
       <c r="H86" s="2" t="inlineStr">
         <is>
-          <t>Parque Industrial de Celeirós 2ª fase</t>
+          <t>Rua Quinta dos Lagos 24, 4700-289 Real</t>
         </is>
       </c>
       <c r="I86" s="2" t="inlineStr">
         <is>
-          <t>Arc Living (Porto) (Em construção)</t>
+          <t>Green Terrace Porto (Requesende) (Em construção) | Garden Palace (Comercialização) | Strata Private Residence (Comercialização) | Vess Living (Guimarães) (Em construção)</t>
         </is>
       </c>
       <c r="J86" s="2" t="inlineStr">
         <is>
-          <t>Promotor + construtor. Fonte: idealista/news, construir.pt</t>
+          <t>Promove, constrói e vende os próprios projetos. Fonte: diarioimobiliario.pt, idealista/news</t>
         </is>
       </c>
       <c r="K86" s="2" t="inlineStr">
         <is>
-          <t>Domingos Correia (CEO)</t>
-        </is>
-      </c>
-      <c r="L86" s="2" t="inlineStr">
-        <is>
-          <t>https://www.linkedin.com/in/domingos-correia-4453ab32/</t>
-        </is>
-      </c>
+          <t>Pedro Ferreira (administrador, confiança moderada)</t>
+        </is>
+      </c>
+      <c r="L86" s="2" t="inlineStr"/>
       <c r="M86" s="2" t="inlineStr"/>
     </row>
     <row r="87" ht="30" customHeight="1">
       <c r="A87" s="2" t="inlineStr">
         <is>
-          <t>Grupo CVM (Construções Vila Maior)</t>
+          <t>Grupo Arliz</t>
         </is>
       </c>
       <c r="B87" s="4" t="inlineStr">
@@ -5326,52 +5318,60 @@
       </c>
       <c r="C87" s="4" t="inlineStr">
         <is>
-          <t>273 332 784 (confirmar)</t>
-        </is>
-      </c>
-      <c r="D87" s="2" t="inlineStr"/>
+          <t>+351 253 105 331</t>
+        </is>
+      </c>
+      <c r="D87" s="2" t="inlineStr">
+        <is>
+          <t>geral@arliz.co</t>
+        </is>
+      </c>
       <c r="E87" s="2" t="inlineStr">
         <is>
-          <t>cvmnet.com</t>
+          <t>grupoarliz.pt</t>
         </is>
       </c>
       <c r="F87" s="4" t="inlineStr">
         <is>
-          <t>Santa Maria da Feira</t>
+          <t>Braga</t>
         </is>
       </c>
       <c r="G87" s="4" t="inlineStr">
         <is>
-          <t>Aveiro</t>
+          <t>Braga</t>
         </is>
       </c>
       <c r="H87" s="2" t="inlineStr">
         <is>
-          <t>Parque Empresarial A32, Vila Maior</t>
+          <t>Parque Industrial de Celeirós 2ª fase</t>
         </is>
       </c>
       <c r="I87" s="2" t="inlineStr">
         <is>
-          <t>Royal Green (V.N. Gaia, Av. Descobrimentos) (Em construção)</t>
+          <t>Arc Living (Porto) (Em construção)</t>
         </is>
       </c>
       <c r="J87" s="2" t="inlineStr">
         <is>
-          <t>Telefone vindo do registo — confirmar em cvmnet.com/contactos</t>
+          <t>Promotor + construtor. Fonte: idealista/news, construir.pt</t>
         </is>
       </c>
       <c r="K87" s="2" t="inlineStr">
         <is>
-          <t>Severino Ponte (Administração, com Ângelo Marques)</t>
-        </is>
-      </c>
-      <c r="L87" s="2" t="inlineStr"/>
+          <t>Domingos Correia (CEO)</t>
+        </is>
+      </c>
+      <c r="L87" s="2" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/domingos-correia-4453ab32/</t>
+        </is>
+      </c>
       <c r="M87" s="2" t="inlineStr"/>
     </row>
     <row r="88" ht="30" customHeight="1">
       <c r="A88" s="2" t="inlineStr">
         <is>
-          <t>HomeLovers Investment</t>
+          <t>Grupo CVM (Construções Vila Maior)</t>
         </is>
       </c>
       <c r="B88" s="4" t="inlineStr">
@@ -5381,52 +5381,52 @@
       </c>
       <c r="C88" s="4" t="inlineStr">
         <is>
-          <t>+351 913 470 147</t>
+          <t>273 332 784 (confirmar)</t>
         </is>
       </c>
       <c r="D88" s="2" t="inlineStr"/>
       <c r="E88" s="2" t="inlineStr">
         <is>
-          <t>homelovers.pt</t>
+          <t>cvmnet.com</t>
         </is>
       </c>
       <c r="F88" s="4" t="inlineStr">
         <is>
-          <t>Setúbal</t>
+          <t>Santa Maria da Feira</t>
         </is>
       </c>
       <c r="G88" s="4" t="inlineStr">
         <is>
-          <t>Setúbal</t>
-        </is>
-      </c>
-      <c r="H88" s="2" t="inlineStr"/>
+          <t>Aveiro</t>
+        </is>
+      </c>
+      <c r="H88" s="2" t="inlineStr">
+        <is>
+          <t>Parque Empresarial A32, Vila Maior</t>
+        </is>
+      </c>
       <c r="I88" s="2" t="inlineStr">
         <is>
-          <t>Parque da Cidade – Riverside Living Setúbal (Em construção)</t>
+          <t>Royal Green (V.N. Gaia, Av. Descobrimentos) (Em construção)</t>
         </is>
       </c>
       <c r="J88" s="2" t="inlineStr">
         <is>
-          <t>Fonte: sapo.pt</t>
+          <t>Telefone vindo do registo — confirmar em cvmnet.com/contactos</t>
         </is>
       </c>
       <c r="K88" s="2" t="inlineStr">
         <is>
-          <t>Miguel Tilli (fundador e CEO)</t>
-        </is>
-      </c>
-      <c r="L88" s="2" t="inlineStr">
-        <is>
-          <t>https://www.linkedin.com/in/miguel-tilli-a7a41587/</t>
-        </is>
-      </c>
+          <t>Severino Ponte (Administração, com Ângelo Marques)</t>
+        </is>
+      </c>
+      <c r="L88" s="2" t="inlineStr"/>
       <c r="M88" s="2" t="inlineStr"/>
     </row>
     <row r="89" ht="30" customHeight="1">
       <c r="A89" s="2" t="inlineStr">
         <is>
-          <t>JHOMEA Invest</t>
+          <t>HomeLovers Investment</t>
         </is>
       </c>
       <c r="B89" s="4" t="inlineStr">
@@ -5436,56 +5436,52 @@
       </c>
       <c r="C89" s="4" t="inlineStr">
         <is>
-          <t>+351 934 175 642</t>
-        </is>
-      </c>
-      <c r="D89" s="2" t="inlineStr">
-        <is>
-          <t>geral@jhomea.pt</t>
-        </is>
-      </c>
+          <t>+351 913 470 147</t>
+        </is>
+      </c>
+      <c r="D89" s="2" t="inlineStr"/>
       <c r="E89" s="2" t="inlineStr">
         <is>
-          <t>jhomea.pt</t>
+          <t>homelovers.pt</t>
         </is>
       </c>
       <c r="F89" s="4" t="inlineStr">
         <is>
-          <t>Aveiro</t>
+          <t>Setúbal</t>
         </is>
       </c>
       <c r="G89" s="4" t="inlineStr">
         <is>
-          <t>Aveiro</t>
-        </is>
-      </c>
-      <c r="H89" s="2" t="inlineStr">
-        <is>
-          <t>Rua Cristóvão Pinho Queimado 56, 3800-012</t>
-        </is>
-      </c>
+          <t>Setúbal</t>
+        </is>
+      </c>
+      <c r="H89" s="2" t="inlineStr"/>
       <c r="I89" s="2" t="inlineStr">
         <is>
-          <t>Vacivus (Porto) (Em construção)</t>
+          <t>Parque da Cidade – Riverside Living Setúbal (Em construção)</t>
         </is>
       </c>
       <c r="J89" s="2" t="inlineStr">
         <is>
-          <t>AMI 16355. Escritórios Aveiro (+351 914 444 764) e Lisboa (+351 912 325 143)</t>
+          <t>Fonte: sapo.pt</t>
         </is>
       </c>
       <c r="K89" s="2" t="inlineStr">
         <is>
-          <t>José Miguel Afonso (CEO/fundador)</t>
-        </is>
-      </c>
-      <c r="L89" s="2" t="inlineStr"/>
+          <t>Miguel Tilli (fundador e CEO)</t>
+        </is>
+      </c>
+      <c r="L89" s="2" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/miguel-tilli-a7a41587/</t>
+        </is>
+      </c>
       <c r="M89" s="2" t="inlineStr"/>
     </row>
     <row r="90" ht="30" customHeight="1">
       <c r="A90" s="2" t="inlineStr">
         <is>
-          <t>Metathesis</t>
+          <t>JHOMEA Invest</t>
         </is>
       </c>
       <c r="B90" s="4" t="inlineStr">
@@ -5495,43 +5491,47 @@
       </c>
       <c r="C90" s="4" t="inlineStr">
         <is>
-          <t>+351 211 650 420</t>
-        </is>
-      </c>
-      <c r="D90" s="2" t="inlineStr"/>
+          <t>+351 934 175 642</t>
+        </is>
+      </c>
+      <c r="D90" s="2" t="inlineStr">
+        <is>
+          <t>geral@jhomea.pt</t>
+        </is>
+      </c>
       <c r="E90" s="2" t="inlineStr">
         <is>
-          <t>metathesis.pt</t>
+          <t>jhomea.pt</t>
         </is>
       </c>
       <c r="F90" s="4" t="inlineStr">
         <is>
-          <t>Almada</t>
+          <t>Aveiro</t>
         </is>
       </c>
       <c r="G90" s="4" t="inlineStr">
         <is>
-          <t>Setúbal</t>
+          <t>Aveiro</t>
         </is>
       </c>
       <c r="H90" s="2" t="inlineStr">
         <is>
-          <t>R. Marcos de Assunção nº4A, 2805-290</t>
+          <t>Rua Cristóvão Pinho Queimado 56, 3800-012</t>
         </is>
       </c>
       <c r="I90" s="2" t="inlineStr">
         <is>
-          <t>Reabilitação de imóveis residenciais (Almada) (Em construção)</t>
+          <t>Vacivus (Porto) (Em construção)</t>
         </is>
       </c>
       <c r="J90" s="2" t="inlineStr">
         <is>
-          <t>Gerente: Maria Elisabete da Fonseca Dionísio Dias. Tel. alt. 967 364 611</t>
+          <t>AMI 16355. Escritórios Aveiro (+351 914 444 764) e Lisboa (+351 912 325 143)</t>
         </is>
       </c>
       <c r="K90" s="2" t="inlineStr">
         <is>
-          <t>Maria Elisabete da Fonseca Dionísio Dias (gerente)</t>
+          <t>José Miguel Afonso (CEO/fundador)</t>
         </is>
       </c>
       <c r="L90" s="2" t="inlineStr"/>
@@ -5540,7 +5540,7 @@
     <row r="91" ht="30" customHeight="1">
       <c r="A91" s="2" t="inlineStr">
         <is>
-          <t>Pine Hill</t>
+          <t>Metathesis</t>
         </is>
       </c>
       <c r="B91" s="4" t="inlineStr">
@@ -5550,56 +5550,52 @@
       </c>
       <c r="C91" s="4" t="inlineStr">
         <is>
-          <t>+351 910 936 732</t>
-        </is>
-      </c>
-      <c r="D91" s="2" t="inlineStr">
-        <is>
-          <t>info@pinehill.pt</t>
-        </is>
-      </c>
+          <t>+351 211 650 420</t>
+        </is>
+      </c>
+      <c r="D91" s="2" t="inlineStr"/>
       <c r="E91" s="2" t="inlineStr">
         <is>
-          <t>pinehill.pt</t>
+          <t>metathesis.pt</t>
         </is>
       </c>
       <c r="F91" s="4" t="inlineStr">
         <is>
-          <t>Braga</t>
+          <t>Almada</t>
         </is>
       </c>
       <c r="G91" s="4" t="inlineStr">
         <is>
-          <t>Braga</t>
-        </is>
-      </c>
-      <c r="H91" s="2" t="inlineStr"/>
+          <t>Setúbal</t>
+        </is>
+      </c>
+      <c r="H91" s="2" t="inlineStr">
+        <is>
+          <t>R. Marcos de Assunção nº4A, 2805-290</t>
+        </is>
+      </c>
       <c r="I91" s="2" t="inlineStr">
         <is>
-          <t>Braga Premium Flats (Comercialização) | 3 novos projetos em Braga (Planeamento)</t>
+          <t>Reabilitação de imóveis residenciais (Almada) (Em construção)</t>
         </is>
       </c>
       <c r="J91" s="2" t="inlineStr">
         <is>
-          <t>Promotora criada em 2025. Fonte: newinbraga.nit.pt, Revista Spot</t>
+          <t>Gerente: Maria Elisabete da Fonseca Dionísio Dias. Tel. alt. 967 364 611</t>
         </is>
       </c>
       <c r="K91" s="2" t="inlineStr">
         <is>
-          <t>Nuno Pinheiro (fundador)</t>
-        </is>
-      </c>
-      <c r="L91" s="2" t="inlineStr">
-        <is>
-          <t>https://www.linkedin.com/in/nuno-pinheiro-39968aa4/</t>
-        </is>
-      </c>
+          <t>Maria Elisabete da Fonseca Dionísio Dias (gerente)</t>
+        </is>
+      </c>
+      <c r="L91" s="2" t="inlineStr"/>
       <c r="M91" s="2" t="inlineStr"/>
     </row>
     <row r="92" ht="30" customHeight="1">
       <c r="A92" s="2" t="inlineStr">
         <is>
-          <t>Quinta do Lago Resort</t>
+          <t>Pine Hill</t>
         </is>
       </c>
       <c r="B92" s="4" t="inlineStr">
@@ -5609,52 +5605,48 @@
       </c>
       <c r="C92" s="4" t="inlineStr">
         <is>
-          <t>+351 289 390 700</t>
+          <t>+351 910 936 732</t>
         </is>
       </c>
       <c r="D92" s="2" t="inlineStr">
         <is>
-          <t>info@quintadolago.com</t>
+          <t>info@pinehill.pt</t>
         </is>
       </c>
       <c r="E92" s="2" t="inlineStr">
         <is>
-          <t>quintadolago.com</t>
+          <t>pinehill.pt</t>
         </is>
       </c>
       <c r="F92" s="4" t="inlineStr">
         <is>
-          <t>Loulé</t>
+          <t>Braga</t>
         </is>
       </c>
       <c r="G92" s="4" t="inlineStr">
         <is>
-          <t>Faro</t>
-        </is>
-      </c>
-      <c r="H92" s="2" t="inlineStr">
-        <is>
-          <t>Almancil</t>
-        </is>
-      </c>
+          <t>Braga</t>
+        </is>
+      </c>
+      <c r="H92" s="2" t="inlineStr"/>
       <c r="I92" s="2" t="inlineStr">
         <is>
-          <t>Quinta do Lago (real estate do resort) (Comercialização)</t>
+          <t>Braga Premium Flats (Comercialização) | 3 novos projetos em Braga (Planeamento)</t>
         </is>
       </c>
       <c r="J92" s="2" t="inlineStr">
         <is>
-          <t>Resort residencial/golfe</t>
+          <t>Promotora criada em 2025. Fonte: newinbraga.nit.pt, Revista Spot</t>
         </is>
       </c>
       <c r="K92" s="2" t="inlineStr">
         <is>
-          <t>Sean Moriarty (CEO)</t>
+          <t>Nuno Pinheiro (fundador)</t>
         </is>
       </c>
       <c r="L92" s="2" t="inlineStr">
         <is>
-          <t>https://pt.linkedin.com/in/sean-moriarty-6a749133</t>
+          <t>https://www.linkedin.com/in/nuno-pinheiro-39968aa4/</t>
         </is>
       </c>
       <c r="M92" s="2" t="inlineStr"/>
@@ -5662,7 +5654,7 @@
     <row r="93" ht="30" customHeight="1">
       <c r="A93" s="2" t="inlineStr">
         <is>
-          <t>Royal Prime</t>
+          <t>Quinta do Lago Resort</t>
         </is>
       </c>
       <c r="B93" s="4" t="inlineStr">
@@ -5672,52 +5664,60 @@
       </c>
       <c r="C93" s="4" t="inlineStr">
         <is>
-          <t>+351 910 181 312</t>
+          <t>+351 289 390 700</t>
         </is>
       </c>
       <c r="D93" s="2" t="inlineStr">
         <is>
-          <t>rgodinho@royalprime.pt</t>
+          <t>info@quintadolago.com</t>
         </is>
       </c>
       <c r="E93" s="2" t="inlineStr">
         <is>
-          <t>royalprime.pt</t>
+          <t>quintadolago.com</t>
         </is>
       </c>
       <c r="F93" s="4" t="inlineStr">
         <is>
-          <t>Covilhã</t>
+          <t>Loulé</t>
         </is>
       </c>
       <c r="G93" s="4" t="inlineStr">
         <is>
-          <t>Castelo Branco</t>
+          <t>Faro</t>
         </is>
       </c>
       <c r="H93" s="2" t="inlineStr">
         <is>
-          <t>R. Doutor Mário Soares, lote 3, 6200-026</t>
+          <t>Almancil</t>
         </is>
       </c>
       <c r="I93" s="2" t="inlineStr">
         <is>
-          <t>Tower Residences (Covilhã) (Concluído)</t>
+          <t>Quinta do Lago (real estate do resort) (Comercialização)</t>
         </is>
       </c>
       <c r="J93" s="2" t="inlineStr">
         <is>
-          <t>Contacto comercial Rita Godinho</t>
-        </is>
-      </c>
-      <c r="K93" s="2" t="inlineStr"/>
-      <c r="L93" s="2" t="inlineStr"/>
+          <t>Resort residencial/golfe</t>
+        </is>
+      </c>
+      <c r="K93" s="2" t="inlineStr">
+        <is>
+          <t>Sean Moriarty (CEO)</t>
+        </is>
+      </c>
+      <c r="L93" s="2" t="inlineStr">
+        <is>
+          <t>https://pt.linkedin.com/in/sean-moriarty-6a749133</t>
+        </is>
+      </c>
       <c r="M93" s="2" t="inlineStr"/>
     </row>
     <row r="94" ht="30" customHeight="1">
       <c r="A94" s="2" t="inlineStr">
         <is>
-          <t>Salk Properties Portugal</t>
+          <t>Royal Prime</t>
         </is>
       </c>
       <c r="B94" s="4" t="inlineStr">
@@ -5727,48 +5727,52 @@
       </c>
       <c r="C94" s="4" t="inlineStr">
         <is>
-          <t>+351 939 443 765</t>
-        </is>
-      </c>
-      <c r="D94" s="2" t="inlineStr"/>
+          <t>+351 910 181 312</t>
+        </is>
+      </c>
+      <c r="D94" s="2" t="inlineStr">
+        <is>
+          <t>rgodinho@royalprime.pt</t>
+        </is>
+      </c>
       <c r="E94" s="2" t="inlineStr">
         <is>
-          <t>salkproperties.com</t>
+          <t>royalprime.pt</t>
         </is>
       </c>
       <c r="F94" s="4" t="inlineStr">
         <is>
-          <t>Alcácer do Sal</t>
+          <t>Covilhã</t>
         </is>
       </c>
       <c r="G94" s="4" t="inlineStr">
         <is>
-          <t>Setúbal</t>
-        </is>
-      </c>
-      <c r="H94" s="2" t="inlineStr"/>
+          <t>Castelo Branco</t>
+        </is>
+      </c>
+      <c r="H94" s="2" t="inlineStr">
+        <is>
+          <t>R. Doutor Mário Soares, lote 3, 6200-026</t>
+        </is>
+      </c>
       <c r="I94" s="2" t="inlineStr">
         <is>
-          <t>Alcácer Vintage (Planeamento (consulta pública))</t>
+          <t>Tower Residences (Covilhã) (Concluído)</t>
         </is>
       </c>
       <c r="J94" s="2" t="inlineStr">
         <is>
-          <t>Fonte: vidaimobiliaria.com</t>
-        </is>
-      </c>
-      <c r="K94" s="2" t="inlineStr">
-        <is>
-          <t>João Luís Ferreira (Chairman &amp; Partner)</t>
-        </is>
-      </c>
+          <t>Contacto comercial Rita Godinho</t>
+        </is>
+      </c>
+      <c r="K94" s="2" t="inlineStr"/>
       <c r="L94" s="2" t="inlineStr"/>
       <c r="M94" s="2" t="inlineStr"/>
     </row>
     <row r="95" ht="30" customHeight="1">
       <c r="A95" s="2" t="inlineStr">
         <is>
-          <t>Scale Property Development</t>
+          <t>Salk Properties Portugal</t>
         </is>
       </c>
       <c r="B95" s="4" t="inlineStr">
@@ -5778,18 +5782,18 @@
       </c>
       <c r="C95" s="4" t="inlineStr">
         <is>
-          <t>+351 219 362 960</t>
+          <t>+351 939 443 765</t>
         </is>
       </c>
       <c r="D95" s="2" t="inlineStr"/>
       <c r="E95" s="2" t="inlineStr">
         <is>
-          <t>scalepropertydevelopment.com</t>
+          <t>salkproperties.com</t>
         </is>
       </c>
       <c r="F95" s="4" t="inlineStr">
         <is>
-          <t>Setúbal</t>
+          <t>Alcácer do Sal</t>
         </is>
       </c>
       <c r="G95" s="4" t="inlineStr">
@@ -5800,7 +5804,7 @@
       <c r="H95" s="2" t="inlineStr"/>
       <c r="I95" s="2" t="inlineStr">
         <is>
-          <t>Parque da Cidade – Riverside Living Setúbal (Em construção)</t>
+          <t>Alcácer Vintage (Planeamento (consulta pública))</t>
         </is>
       </c>
       <c r="J95" s="2" t="inlineStr">
@@ -5810,20 +5814,16 @@
       </c>
       <c r="K95" s="2" t="inlineStr">
         <is>
-          <t>Diogo Sá Viana Rebelo (Co-Founder)</t>
-        </is>
-      </c>
-      <c r="L95" s="2" t="inlineStr">
-        <is>
-          <t>https://www.linkedin.com/in/diogo-s%C3%A1-viana-rebelo-910104143/</t>
-        </is>
-      </c>
+          <t>João Luís Ferreira (Chairman &amp; Partner)</t>
+        </is>
+      </c>
+      <c r="L95" s="2" t="inlineStr"/>
       <c r="M95" s="2" t="inlineStr"/>
     </row>
     <row r="96" ht="30" customHeight="1">
       <c r="A96" s="2" t="inlineStr">
         <is>
-          <t>TPS – Teixeira, Pinto &amp; Soares</t>
+          <t>Scale Property Development</t>
         </is>
       </c>
       <c r="B96" s="4" t="inlineStr">
@@ -5833,56 +5833,52 @@
       </c>
       <c r="C96" s="4" t="inlineStr">
         <is>
-          <t>+351 255 433 572</t>
-        </is>
-      </c>
-      <c r="D96" s="2" t="inlineStr">
-        <is>
-          <t>geral@tps.com.pt</t>
-        </is>
-      </c>
+          <t>+351 219 362 960</t>
+        </is>
+      </c>
+      <c r="D96" s="2" t="inlineStr"/>
       <c r="E96" s="2" t="inlineStr">
         <is>
-          <t>tps.com.pt</t>
+          <t>scalepropertydevelopment.com</t>
         </is>
       </c>
       <c r="F96" s="4" t="inlineStr">
         <is>
-          <t>Amarante</t>
+          <t>Setúbal</t>
         </is>
       </c>
       <c r="G96" s="4" t="inlineStr">
         <is>
-          <t>Porto</t>
-        </is>
-      </c>
-      <c r="H96" s="2" t="inlineStr">
-        <is>
-          <t>Rua do Outeiro 677, Z.I. Telões, 4600-758</t>
-        </is>
-      </c>
+          <t>Setúbal</t>
+        </is>
+      </c>
+      <c r="H96" s="2" t="inlineStr"/>
       <c r="I96" s="2" t="inlineStr">
         <is>
-          <t>JV com Carvoeiro Branco (Lagoa, Portimão, Faro) (Planeamento) | One Lush (Caxias) (Em construção)</t>
+          <t>Parque da Cidade – Riverside Living Setúbal (Em construção)</t>
         </is>
       </c>
       <c r="J96" s="2" t="inlineStr">
         <is>
-          <t>Uma das maiores construtoras nacionais · delegações Lisboa e Algarve</t>
+          <t>Fonte: vidaimobiliaria.com</t>
         </is>
       </c>
       <c r="K96" s="2" t="inlineStr">
         <is>
-          <t>Bruno Fernando Macedo Soares (CEO/Presidente do CA)</t>
-        </is>
-      </c>
-      <c r="L96" s="2" t="inlineStr"/>
+          <t>Diogo Sá Viana Rebelo (Co-Founder)</t>
+        </is>
+      </c>
+      <c r="L96" s="2" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/diogo-s%C3%A1-viana-rebelo-910104143/</t>
+        </is>
+      </c>
       <c r="M96" s="2" t="inlineStr"/>
     </row>
     <row r="97" ht="30" customHeight="1">
       <c r="A97" s="2" t="inlineStr">
         <is>
-          <t>Vomera Group</t>
+          <t>TPS – Teixeira, Pinto &amp; Soares</t>
         </is>
       </c>
       <c r="B97" s="4" t="inlineStr">
@@ -5892,87 +5888,107 @@
       </c>
       <c r="C97" s="4" t="inlineStr">
         <is>
-          <t>351 243 078 442</t>
-        </is>
-      </c>
-      <c r="D97" s="2" t="inlineStr"/>
+          <t>+351 255 433 572</t>
+        </is>
+      </c>
+      <c r="D97" s="2" t="inlineStr">
+        <is>
+          <t>geral@tps.com.pt</t>
+        </is>
+      </c>
       <c r="E97" s="2" t="inlineStr">
         <is>
-          <t>vomera.pt</t>
+          <t>tps.com.pt</t>
         </is>
       </c>
       <c r="F97" s="4" t="inlineStr">
         <is>
-          <t>Santarém</t>
+          <t>Amarante</t>
         </is>
       </c>
       <c r="G97" s="4" t="inlineStr">
         <is>
-          <t>Santarém</t>
-        </is>
-      </c>
-      <c r="H97" s="2" t="inlineStr"/>
+          <t>Porto</t>
+        </is>
+      </c>
+      <c r="H97" s="2" t="inlineStr">
+        <is>
+          <t>Rua do Outeiro 677, Z.I. Telões, 4600-758</t>
+        </is>
+      </c>
       <c r="I97" s="2" t="inlineStr">
         <is>
-          <t>Empreendimento residencial de luxo (nome não divulgado) (Comercialização/Lançamento)</t>
+          <t>JV com Carvoeiro Branco (Lagoa, Portimão, Faro) (Planeamento) | One Lush (Caxias) (Em construção)</t>
         </is>
       </c>
       <c r="J97" s="2" t="inlineStr">
         <is>
-          <t>Fonte: omirante.pt</t>
+          <t>Uma das maiores construtoras nacionais · delegações Lisboa e Algarve</t>
         </is>
       </c>
       <c r="K97" s="2" t="inlineStr">
         <is>
-          <t>Sérgio Santos (CEO/fundador, com Delphine Gerardo)</t>
+          <t>Bruno Fernando Macedo Soares (CEO/Presidente do CA)</t>
         </is>
       </c>
       <c r="L97" s="2" t="inlineStr"/>
       <c r="M97" s="2" t="inlineStr"/>
     </row>
     <row r="98" ht="30" customHeight="1">
-      <c r="A98" s="5" t="inlineStr">
-        <is>
-          <t>Algarve Property Shops</t>
-        </is>
-      </c>
-      <c r="B98" s="7" t="inlineStr">
+      <c r="A98" s="2" t="inlineStr">
+        <is>
+          <t>Vomera Group</t>
+        </is>
+      </c>
+      <c r="B98" s="4" t="inlineStr">
         <is>
           <t>Nao</t>
         </is>
       </c>
-      <c r="C98" s="7" t="inlineStr"/>
-      <c r="D98" s="5" t="inlineStr"/>
-      <c r="E98" s="5" t="inlineStr"/>
-      <c r="F98" s="7" t="inlineStr">
-        <is>
-          <t>Tavira</t>
-        </is>
-      </c>
-      <c r="G98" s="7" t="inlineStr">
-        <is>
-          <t>Faro</t>
-        </is>
-      </c>
-      <c r="H98" s="5" t="inlineStr"/>
-      <c r="I98" s="5" t="inlineStr">
-        <is>
-          <t>Varandas de Cabanas (Em construção/Comercialização)</t>
-        </is>
-      </c>
-      <c r="J98" s="5" t="inlineStr">
-        <is>
-          <t>Fonte: idealista.pt</t>
-        </is>
-      </c>
-      <c r="K98" s="5" t="inlineStr"/>
-      <c r="L98" s="5" t="inlineStr"/>
-      <c r="M98" s="5" t="inlineStr"/>
+      <c r="C98" s="4" t="inlineStr">
+        <is>
+          <t>351 243 078 442</t>
+        </is>
+      </c>
+      <c r="D98" s="2" t="inlineStr"/>
+      <c r="E98" s="2" t="inlineStr">
+        <is>
+          <t>vomera.pt</t>
+        </is>
+      </c>
+      <c r="F98" s="4" t="inlineStr">
+        <is>
+          <t>Santarém</t>
+        </is>
+      </c>
+      <c r="G98" s="4" t="inlineStr">
+        <is>
+          <t>Santarém</t>
+        </is>
+      </c>
+      <c r="H98" s="2" t="inlineStr"/>
+      <c r="I98" s="2" t="inlineStr">
+        <is>
+          <t>Empreendimento residencial de luxo (nome não divulgado) (Comercialização/Lançamento)</t>
+        </is>
+      </c>
+      <c r="J98" s="2" t="inlineStr">
+        <is>
+          <t>Fonte: omirante.pt</t>
+        </is>
+      </c>
+      <c r="K98" s="2" t="inlineStr">
+        <is>
+          <t>Sérgio Santos (CEO/fundador, com Delphine Gerardo)</t>
+        </is>
+      </c>
+      <c r="L98" s="2" t="inlineStr"/>
+      <c r="M98" s="2" t="inlineStr"/>
     </row>
     <row r="99" ht="30" customHeight="1">
       <c r="A99" s="5" t="inlineStr">
         <is>
-          <t>Amorim Luxury</t>
+          <t>Algarve Property Shops</t>
         </is>
       </c>
       <c r="B99" s="7" t="inlineStr">
@@ -5985,37 +6001,33 @@
       <c r="E99" s="5" t="inlineStr"/>
       <c r="F99" s="7" t="inlineStr">
         <is>
-          <t>Lisboa/Grândola/Lagoa</t>
+          <t>Tavira</t>
         </is>
       </c>
       <c r="G99" s="7" t="inlineStr">
         <is>
-          <t>Lisboa</t>
+          <t>Faro</t>
         </is>
       </c>
       <c r="H99" s="5" t="inlineStr"/>
       <c r="I99" s="5" t="inlineStr">
         <is>
-          <t>JNcQUOI House (Av. Liberdade) (Em construção)</t>
+          <t>Varandas de Cabanas (Em construção/Comercialização)</t>
         </is>
       </c>
       <c r="J99" s="5" t="inlineStr">
         <is>
-          <t>Fonte: idealista.pt, vidaimobiliaria.com</t>
-        </is>
-      </c>
-      <c r="K99" s="5" t="inlineStr">
-        <is>
-          <t>Miguel Guedes de Sousa (Founder &amp; CEO)</t>
-        </is>
-      </c>
+          <t>Fonte: idealista.pt</t>
+        </is>
+      </c>
+      <c r="K99" s="5" t="inlineStr"/>
       <c r="L99" s="5" t="inlineStr"/>
       <c r="M99" s="5" t="inlineStr"/>
     </row>
     <row r="100" ht="30" customHeight="1">
       <c r="A100" s="5" t="inlineStr">
         <is>
-          <t>Aresta Vitalicia</t>
+          <t>Amorim Luxury</t>
         </is>
       </c>
       <c r="B100" s="7" t="inlineStr">
@@ -6028,33 +6040,37 @@
       <c r="E100" s="5" t="inlineStr"/>
       <c r="F100" s="7" t="inlineStr">
         <is>
-          <t>Setúbal</t>
+          <t>Lisboa/Grândola/Lagoa</t>
         </is>
       </c>
       <c r="G100" s="7" t="inlineStr">
         <is>
-          <t>Setúbal</t>
+          <t>Lisboa</t>
         </is>
       </c>
       <c r="H100" s="5" t="inlineStr"/>
       <c r="I100" s="5" t="inlineStr">
         <is>
-          <t>WeBuild Castelo (Comercialização)</t>
+          <t>JNcQUOI House (Av. Liberdade) (Em construção)</t>
         </is>
       </c>
       <c r="J100" s="5" t="inlineStr">
         <is>
-          <t>Fonte: construir.pt</t>
-        </is>
-      </c>
-      <c r="K100" s="5" t="inlineStr"/>
+          <t>Fonte: idealista.pt, vidaimobiliaria.com</t>
+        </is>
+      </c>
+      <c r="K100" s="5" t="inlineStr">
+        <is>
+          <t>Miguel Guedes de Sousa (Founder &amp; CEO)</t>
+        </is>
+      </c>
       <c r="L100" s="5" t="inlineStr"/>
       <c r="M100" s="5" t="inlineStr"/>
     </row>
     <row r="101" ht="30" customHeight="1">
       <c r="A101" s="5" t="inlineStr">
         <is>
-          <t>Arrow Global Portugal</t>
+          <t>Aresta Vitalicia</t>
         </is>
       </c>
       <c r="B101" s="7" t="inlineStr">
@@ -6067,37 +6083,33 @@
       <c r="E101" s="5" t="inlineStr"/>
       <c r="F101" s="7" t="inlineStr">
         <is>
-          <t>Loulé (Almancil/Quinta do Lago)</t>
+          <t>Setúbal</t>
         </is>
       </c>
       <c r="G101" s="7" t="inlineStr">
         <is>
-          <t>Faro</t>
+          <t>Setúbal</t>
         </is>
       </c>
       <c r="H101" s="5" t="inlineStr"/>
       <c r="I101" s="5" t="inlineStr">
         <is>
-          <t>The Shore Residences (Comercialização)</t>
+          <t>WeBuild Castelo (Comercialização)</t>
         </is>
       </c>
       <c r="J101" s="5" t="inlineStr">
         <is>
-          <t>Fonte: idealista.pt, jornaleconomico.sapo.pt</t>
-        </is>
-      </c>
-      <c r="K101" s="5" t="inlineStr">
-        <is>
-          <t>João Bugalho (CEO)</t>
-        </is>
-      </c>
+          <t>Fonte: construir.pt</t>
+        </is>
+      </c>
+      <c r="K101" s="5" t="inlineStr"/>
       <c r="L101" s="5" t="inlineStr"/>
       <c r="M101" s="5" t="inlineStr"/>
     </row>
     <row r="102" ht="30" customHeight="1">
       <c r="A102" s="5" t="inlineStr">
         <is>
-          <t>Baltor – Engenharia e Construção</t>
+          <t>Arrow Global Portugal</t>
         </is>
       </c>
       <c r="B102" s="7" t="inlineStr">
@@ -6107,35 +6119,31 @@
       </c>
       <c r="C102" s="7" t="inlineStr"/>
       <c r="D102" s="5" t="inlineStr"/>
-      <c r="E102" s="5" t="inlineStr">
-        <is>
-          <t>baltor.pt</t>
-        </is>
-      </c>
+      <c r="E102" s="5" t="inlineStr"/>
       <c r="F102" s="7" t="inlineStr">
         <is>
-          <t>Setúbal (sede Viana do Castelo)</t>
+          <t>Loulé (Almancil/Quinta do Lago)</t>
         </is>
       </c>
       <c r="G102" s="7" t="inlineStr">
         <is>
-          <t>Setúbal</t>
+          <t>Faro</t>
         </is>
       </c>
       <c r="H102" s="5" t="inlineStr"/>
       <c r="I102" s="5" t="inlineStr">
         <is>
-          <t>Parque da Cidade – Riverside III (Em construção)</t>
+          <t>The Shore Residences (Comercialização)</t>
         </is>
       </c>
       <c r="J102" s="5" t="inlineStr">
         <is>
-          <t>Fonte: ominho.pt</t>
+          <t>Fonte: idealista.pt, jornaleconomico.sapo.pt</t>
         </is>
       </c>
       <c r="K102" s="5" t="inlineStr">
         <is>
-          <t>Paulo Balinha e Bruno Torres (fundadores, 2008)</t>
+          <t>João Bugalho (CEO)</t>
         </is>
       </c>
       <c r="L102" s="5" t="inlineStr"/>
@@ -6144,7 +6152,7 @@
     <row r="103" ht="30" customHeight="1">
       <c r="A103" s="5" t="inlineStr">
         <is>
-          <t>Bond Group</t>
+          <t>Baltor – Engenharia e Construção</t>
         </is>
       </c>
       <c r="B103" s="7" t="inlineStr">
@@ -6154,36 +6162,44 @@
       </c>
       <c r="C103" s="7" t="inlineStr"/>
       <c r="D103" s="5" t="inlineStr"/>
-      <c r="E103" s="5" t="inlineStr"/>
+      <c r="E103" s="5" t="inlineStr">
+        <is>
+          <t>baltor.pt</t>
+        </is>
+      </c>
       <c r="F103" s="7" t="inlineStr">
         <is>
-          <t>Amares</t>
+          <t>Setúbal (sede Viana do Castelo)</t>
         </is>
       </c>
       <c r="G103" s="7" t="inlineStr">
         <is>
-          <t>Braga</t>
+          <t>Setúbal</t>
         </is>
       </c>
       <c r="H103" s="5" t="inlineStr"/>
       <c r="I103" s="5" t="inlineStr">
         <is>
-          <t>José Azevedo Prime Living (Ferreiros, Amares) (Em construção)</t>
+          <t>Parque da Cidade – Riverside III (Em construção)</t>
         </is>
       </c>
       <c r="J103" s="5" t="inlineStr">
         <is>
-          <t>Grupo imobiliário do Minho. Sem contacto direto confirmado nas fontes</t>
-        </is>
-      </c>
-      <c r="K103" s="5" t="inlineStr"/>
+          <t>Fonte: ominho.pt</t>
+        </is>
+      </c>
+      <c r="K103" s="5" t="inlineStr">
+        <is>
+          <t>Paulo Balinha e Bruno Torres (fundadores, 2008)</t>
+        </is>
+      </c>
       <c r="L103" s="5" t="inlineStr"/>
       <c r="M103" s="5" t="inlineStr"/>
     </row>
     <row r="104" ht="30" customHeight="1">
       <c r="A104" s="5" t="inlineStr">
         <is>
-          <t>Branco Real Estate</t>
+          <t>Bond Group</t>
         </is>
       </c>
       <c r="B104" s="7" t="inlineStr">
@@ -6196,23 +6212,23 @@
       <c r="E104" s="5" t="inlineStr"/>
       <c r="F104" s="7" t="inlineStr">
         <is>
-          <t>Lagos</t>
+          <t>Amares</t>
         </is>
       </c>
       <c r="G104" s="7" t="inlineStr">
         <is>
-          <t>Faro</t>
+          <t>Braga</t>
         </is>
       </c>
       <c r="H104" s="5" t="inlineStr"/>
       <c r="I104" s="5" t="inlineStr">
         <is>
-          <t>Domus (Em construção)</t>
+          <t>José Azevedo Prime Living (Ferreiros, Amares) (Em construção)</t>
         </is>
       </c>
       <c r="J104" s="5" t="inlineStr">
         <is>
-          <t>Fonte: idealista.pt/empreendimento/35004962</t>
+          <t>Grupo imobiliário do Minho. Sem contacto direto confirmado nas fontes</t>
         </is>
       </c>
       <c r="K104" s="5" t="inlineStr"/>
@@ -6222,7 +6238,7 @@
     <row r="105" ht="30" customHeight="1">
       <c r="A105" s="5" t="inlineStr">
         <is>
-          <t>Casas do Sotavento</t>
+          <t>Branco Real Estate</t>
         </is>
       </c>
       <c r="B105" s="7" t="inlineStr">
@@ -6232,14 +6248,10 @@
       </c>
       <c r="C105" s="7" t="inlineStr"/>
       <c r="D105" s="5" t="inlineStr"/>
-      <c r="E105" s="5" t="inlineStr">
-        <is>
-          <t>casasdosotavento.pt</t>
-        </is>
-      </c>
+      <c r="E105" s="5" t="inlineStr"/>
       <c r="F105" s="7" t="inlineStr">
         <is>
-          <t>Tavira</t>
+          <t>Lagos</t>
         </is>
       </c>
       <c r="G105" s="7" t="inlineStr">
@@ -6250,12 +6262,12 @@
       <c r="H105" s="5" t="inlineStr"/>
       <c r="I105" s="5" t="inlineStr">
         <is>
-          <t>Boavista Ocean Tavira (Comercialização)</t>
+          <t>Domus (Em construção)</t>
         </is>
       </c>
       <c r="J105" s="5" t="inlineStr">
         <is>
-          <t>Fonte: boavistaoceantavira.com</t>
+          <t>Fonte: idealista.pt/empreendimento/35004962</t>
         </is>
       </c>
       <c r="K105" s="5" t="inlineStr"/>
@@ -6265,7 +6277,7 @@
     <row r="106" ht="30" customHeight="1">
       <c r="A106" s="5" t="inlineStr">
         <is>
-          <t>Confidential Sphere – Investimento Imobiliário</t>
+          <t>Casas do Sotavento</t>
         </is>
       </c>
       <c r="B106" s="7" t="inlineStr">
@@ -6275,10 +6287,14 @@
       </c>
       <c r="C106" s="7" t="inlineStr"/>
       <c r="D106" s="5" t="inlineStr"/>
-      <c r="E106" s="5" t="inlineStr"/>
+      <c r="E106" s="5" t="inlineStr">
+        <is>
+          <t>casasdosotavento.pt</t>
+        </is>
+      </c>
       <c r="F106" s="7" t="inlineStr">
         <is>
-          <t>Silves</t>
+          <t>Tavira</t>
         </is>
       </c>
       <c r="G106" s="7" t="inlineStr">
@@ -6289,12 +6305,12 @@
       <c r="H106" s="5" t="inlineStr"/>
       <c r="I106" s="5" t="inlineStr">
         <is>
-          <t>Quinta do Pateiro / Silves Hills (Planeamento)</t>
+          <t>Boavista Ocean Tavira (Comercialização)</t>
         </is>
       </c>
       <c r="J106" s="5" t="inlineStr">
         <is>
-          <t>Fonte: terraruiva.pt, barlavento.pt</t>
+          <t>Fonte: boavistaoceantavira.com</t>
         </is>
       </c>
       <c r="K106" s="5" t="inlineStr"/>
@@ -6304,7 +6320,7 @@
     <row r="107" ht="30" customHeight="1">
       <c r="A107" s="5" t="inlineStr">
         <is>
-          <t>CS Ribeiro</t>
+          <t>Confidential Sphere – Investimento Imobiliário</t>
         </is>
       </c>
       <c r="B107" s="7" t="inlineStr">
@@ -6317,23 +6333,23 @@
       <c r="E107" s="5" t="inlineStr"/>
       <c r="F107" s="7" t="inlineStr">
         <is>
-          <t>Guarda (atua Viseu/Coimbra)</t>
+          <t>Silves</t>
         </is>
       </c>
       <c r="G107" s="7" t="inlineStr">
         <is>
-          <t>Guarda</t>
+          <t>Faro</t>
         </is>
       </c>
       <c r="H107" s="5" t="inlineStr"/>
       <c r="I107" s="5" t="inlineStr">
         <is>
-          <t>The Town Signature (Solum, Coimbra) (Em construção)</t>
+          <t>Quinta do Pateiro / Silves Hills (Planeamento)</t>
         </is>
       </c>
       <c r="J107" s="5" t="inlineStr">
         <is>
-          <t>Fonte: diariocoimbra.pt</t>
+          <t>Fonte: terraruiva.pt, barlavento.pt</t>
         </is>
       </c>
       <c r="K107" s="5" t="inlineStr"/>
@@ -6343,7 +6359,7 @@
     <row r="108" ht="30" customHeight="1">
       <c r="A108" s="5" t="inlineStr">
         <is>
-          <t>Discovery Land Company</t>
+          <t>CS Ribeiro</t>
         </is>
       </c>
       <c r="B108" s="7" t="inlineStr">
@@ -6353,30 +6369,26 @@
       </c>
       <c r="C108" s="7" t="inlineStr"/>
       <c r="D108" s="5" t="inlineStr"/>
-      <c r="E108" s="5" t="inlineStr">
-        <is>
-          <t>discoverylandco.com</t>
-        </is>
-      </c>
+      <c r="E108" s="5" t="inlineStr"/>
       <c r="F108" s="7" t="inlineStr">
         <is>
-          <t>Grândola (Melides)</t>
+          <t>Guarda (atua Viseu/Coimbra)</t>
         </is>
       </c>
       <c r="G108" s="7" t="inlineStr">
         <is>
-          <t>Setúbal</t>
+          <t>Guarda</t>
         </is>
       </c>
       <c r="H108" s="5" t="inlineStr"/>
       <c r="I108" s="5" t="inlineStr">
         <is>
-          <t>CostaTerra Golf &amp; Ocean Club (Em construção/Comercialização)</t>
+          <t>The Town Signature (Solum, Coimbra) (Em construção)</t>
         </is>
       </c>
       <c r="J108" s="5" t="inlineStr">
         <is>
-          <t>Fonte: brainsre.news</t>
+          <t>Fonte: diariocoimbra.pt</t>
         </is>
       </c>
       <c r="K108" s="5" t="inlineStr"/>
@@ -6386,7 +6398,7 @@
     <row r="109" ht="30" customHeight="1">
       <c r="A109" s="5" t="inlineStr">
         <is>
-          <t>DUJA – Sociedade de Construções, Lda</t>
+          <t>Discovery Land Company</t>
         </is>
       </c>
       <c r="B109" s="7" t="inlineStr">
@@ -6396,26 +6408,30 @@
       </c>
       <c r="C109" s="7" t="inlineStr"/>
       <c r="D109" s="5" t="inlineStr"/>
-      <c r="E109" s="5" t="inlineStr"/>
+      <c r="E109" s="5" t="inlineStr">
+        <is>
+          <t>discoverylandco.com</t>
+        </is>
+      </c>
       <c r="F109" s="7" t="inlineStr">
         <is>
-          <t>Tavira</t>
+          <t>Grândola (Melides)</t>
         </is>
       </c>
       <c r="G109" s="7" t="inlineStr">
         <is>
-          <t>Faro</t>
+          <t>Setúbal</t>
         </is>
       </c>
       <c r="H109" s="5" t="inlineStr"/>
       <c r="I109" s="5" t="inlineStr">
         <is>
-          <t>Royal Cabanas Beach I e II (Comercialização)</t>
+          <t>CostaTerra Golf &amp; Ocean Club (Em construção/Comercialização)</t>
         </is>
       </c>
       <c r="J109" s="5" t="inlineStr">
         <is>
-          <t>Fonte: remax.pt, tavitel.pt</t>
+          <t>Fonte: brainsre.news</t>
         </is>
       </c>
       <c r="K109" s="5" t="inlineStr"/>
@@ -6425,7 +6441,7 @@
     <row r="110" ht="30" customHeight="1">
       <c r="A110" s="5" t="inlineStr">
         <is>
-          <t>Emblezart</t>
+          <t>DUJA – Sociedade de Construções, Lda</t>
         </is>
       </c>
       <c r="B110" s="7" t="inlineStr">
@@ -6438,41 +6454,33 @@
       <c r="E110" s="5" t="inlineStr"/>
       <c r="F110" s="7" t="inlineStr">
         <is>
-          <t>Guimarães</t>
+          <t>Tavira</t>
         </is>
       </c>
       <c r="G110" s="7" t="inlineStr">
         <is>
-          <t>Braga</t>
+          <t>Faro</t>
         </is>
       </c>
       <c r="H110" s="5" t="inlineStr"/>
       <c r="I110" s="5" t="inlineStr">
         <is>
-          <t>Botânico Avenida (Em construção (fase inicial))</t>
+          <t>Royal Cabanas Beach I e II (Comercialização)</t>
         </is>
       </c>
       <c r="J110" s="5" t="inlineStr">
         <is>
-          <t>Fonte: idealista.pt</t>
-        </is>
-      </c>
-      <c r="K110" s="5" t="inlineStr">
-        <is>
-          <t>David Faria (CEO e sócio único)</t>
-        </is>
-      </c>
-      <c r="L110" s="5" t="inlineStr">
-        <is>
-          <t>https://www.linkedin.com/in/david-faria-a301a466/</t>
-        </is>
-      </c>
+          <t>Fonte: remax.pt, tavitel.pt</t>
+        </is>
+      </c>
+      <c r="K110" s="5" t="inlineStr"/>
+      <c r="L110" s="5" t="inlineStr"/>
       <c r="M110" s="5" t="inlineStr"/>
     </row>
     <row r="111" ht="30" customHeight="1">
       <c r="A111" s="5" t="inlineStr">
         <is>
-          <t>Encobarra</t>
+          <t>Emblezart</t>
         </is>
       </c>
       <c r="B111" s="7" t="inlineStr">
@@ -6485,37 +6493,41 @@
       <c r="E111" s="5" t="inlineStr"/>
       <c r="F111" s="7" t="inlineStr">
         <is>
-          <t>Aveiro (Aradas)</t>
+          <t>Guimarães</t>
         </is>
       </c>
       <c r="G111" s="7" t="inlineStr">
         <is>
-          <t>Aveiro</t>
+          <t>Braga</t>
         </is>
       </c>
       <c r="H111" s="5" t="inlineStr"/>
       <c r="I111" s="5" t="inlineStr">
         <is>
-          <t>Quinta da Pinheira (Em construção)</t>
+          <t>Botânico Avenida (Em construção (fase inicial))</t>
         </is>
       </c>
       <c r="J111" s="5" t="inlineStr">
         <is>
-          <t>Fonte: noticiasdeaveiro.pt, terranova.pt</t>
+          <t>Fonte: idealista.pt</t>
         </is>
       </c>
       <c r="K111" s="5" t="inlineStr">
         <is>
-          <t>Aristides Alferes (administrador)</t>
-        </is>
-      </c>
-      <c r="L111" s="5" t="inlineStr"/>
+          <t>David Faria (CEO e sócio único)</t>
+        </is>
+      </c>
+      <c r="L111" s="5" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/david-faria-a301a466/</t>
+        </is>
+      </c>
       <c r="M111" s="5" t="inlineStr"/>
     </row>
     <row r="112" ht="30" customHeight="1">
       <c r="A112" s="5" t="inlineStr">
         <is>
-          <t>Estrutural Group</t>
+          <t>Encobarra</t>
         </is>
       </c>
       <c r="B112" s="7" t="inlineStr">
@@ -6528,28 +6540,28 @@
       <c r="E112" s="5" t="inlineStr"/>
       <c r="F112" s="7" t="inlineStr">
         <is>
-          <t>Vila Franca de Xira</t>
+          <t>Aveiro (Aradas)</t>
         </is>
       </c>
       <c r="G112" s="7" t="inlineStr">
         <is>
-          <t>Lisboa</t>
+          <t>Aveiro</t>
         </is>
       </c>
       <c r="H112" s="5" t="inlineStr"/>
       <c r="I112" s="5" t="inlineStr">
         <is>
-          <t>Vila Viva (Em construção)</t>
+          <t>Quinta da Pinheira (Em construção)</t>
         </is>
       </c>
       <c r="J112" s="5" t="inlineStr">
         <is>
-          <t>Fonte: vidaimobiliaria.com</t>
+          <t>Fonte: noticiasdeaveiro.pt, terranova.pt</t>
         </is>
       </c>
       <c r="K112" s="5" t="inlineStr">
         <is>
-          <t>Hugo Mendes Pinto (Managing Partner)</t>
+          <t>Aristides Alferes (administrador)</t>
         </is>
       </c>
       <c r="L112" s="5" t="inlineStr"/>
@@ -6558,7 +6570,7 @@
     <row r="113" ht="30" customHeight="1">
       <c r="A113" s="5" t="inlineStr">
         <is>
-          <t>Explorer Investments (Explorer Real Estate)</t>
+          <t>Estrutural Group</t>
         </is>
       </c>
       <c r="B113" s="7" t="inlineStr">
@@ -6568,14 +6580,10 @@
       </c>
       <c r="C113" s="7" t="inlineStr"/>
       <c r="D113" s="5" t="inlineStr"/>
-      <c r="E113" s="5" t="inlineStr">
-        <is>
-          <t>explorerinvestments.com</t>
-        </is>
-      </c>
+      <c r="E113" s="5" t="inlineStr"/>
       <c r="F113" s="7" t="inlineStr">
         <is>
-          <t>Sintra</t>
+          <t>Vila Franca de Xira</t>
         </is>
       </c>
       <c r="G113" s="7" t="inlineStr">
@@ -6586,17 +6594,17 @@
       <c r="H113" s="5" t="inlineStr"/>
       <c r="I113" s="5" t="inlineStr">
         <is>
-          <t>CPHP / Penha Longa (Operação/Asset management (desde 2018))</t>
+          <t>Vila Viva (Em construção)</t>
         </is>
       </c>
       <c r="J113" s="5" t="inlineStr">
         <is>
-          <t>Fonte: jornaldenegocios.pt</t>
+          <t>Fonte: vidaimobiliaria.com</t>
         </is>
       </c>
       <c r="K113" s="5" t="inlineStr">
         <is>
-          <t>Elizabeth Rothfield (CEO, Founding Partner)</t>
+          <t>Hugo Mendes Pinto (Managing Partner)</t>
         </is>
       </c>
       <c r="L113" s="5" t="inlineStr"/>
@@ -6605,7 +6613,7 @@
     <row r="114" ht="30" customHeight="1">
       <c r="A114" s="5" t="inlineStr">
         <is>
-          <t>Finangeste, S.A.</t>
+          <t>Explorer Investments (Explorer Real Estate)</t>
         </is>
       </c>
       <c r="B114" s="7" t="inlineStr">
@@ -6615,31 +6623,35 @@
       </c>
       <c r="C114" s="7" t="inlineStr"/>
       <c r="D114" s="5" t="inlineStr"/>
-      <c r="E114" s="5" t="inlineStr"/>
+      <c r="E114" s="5" t="inlineStr">
+        <is>
+          <t>explorerinvestments.com</t>
+        </is>
+      </c>
       <c r="F114" s="7" t="inlineStr">
         <is>
-          <t>Faro</t>
+          <t>Sintra</t>
         </is>
       </c>
       <c r="G114" s="7" t="inlineStr">
         <is>
-          <t>Faro</t>
+          <t>Lisboa</t>
         </is>
       </c>
       <c r="H114" s="5" t="inlineStr"/>
       <c r="I114" s="5" t="inlineStr">
         <is>
-          <t>PUVA (Planeamento/Em construção)</t>
+          <t>CPHP / Penha Longa (Operação/Asset management (desde 2018))</t>
         </is>
       </c>
       <c r="J114" s="5" t="inlineStr">
         <is>
-          <t>Fonte: jornaldenegocios.pt, idealista.pt</t>
+          <t>Fonte: jornaldenegocios.pt</t>
         </is>
       </c>
       <c r="K114" s="5" t="inlineStr">
         <is>
-          <t>Paul Henri Schelfhout (Presidente do CA) / Armando Lacerda Queiroz (administrador)</t>
+          <t>Elizabeth Rothfield (CEO, Founding Partner)</t>
         </is>
       </c>
       <c r="L114" s="5" t="inlineStr"/>
@@ -6648,7 +6660,7 @@
     <row r="115" ht="30" customHeight="1">
       <c r="A115" s="5" t="inlineStr">
         <is>
-          <t>FourPromo, Lda (Grupo M2O)</t>
+          <t>Finangeste, S.A.</t>
         </is>
       </c>
       <c r="B115" s="7" t="inlineStr">
@@ -6661,7 +6673,7 @@
       <c r="E115" s="5" t="inlineStr"/>
       <c r="F115" s="7" t="inlineStr">
         <is>
-          <t>Loulé (Vilamoura)</t>
+          <t>Faro</t>
         </is>
       </c>
       <c r="G115" s="7" t="inlineStr">
@@ -6672,22 +6684,26 @@
       <c r="H115" s="5" t="inlineStr"/>
       <c r="I115" s="5" t="inlineStr">
         <is>
-          <t>Rivus (Em construção/Comercialização)</t>
+          <t>PUVA (Planeamento/Em construção)</t>
         </is>
       </c>
       <c r="J115" s="5" t="inlineStr">
         <is>
-          <t>Fonte: construir.pt, idealista.pt</t>
-        </is>
-      </c>
-      <c r="K115" s="5" t="inlineStr"/>
+          <t>Fonte: jornaldenegocios.pt, idealista.pt</t>
+        </is>
+      </c>
+      <c r="K115" s="5" t="inlineStr">
+        <is>
+          <t>Paul Henri Schelfhout (Presidente do CA) / Armando Lacerda Queiroz (administrador)</t>
+        </is>
+      </c>
       <c r="L115" s="5" t="inlineStr"/>
       <c r="M115" s="5" t="inlineStr"/>
     </row>
     <row r="116" ht="30" customHeight="1">
       <c r="A116" s="5" t="inlineStr">
         <is>
-          <t>Foz Gala Investments</t>
+          <t>FourPromo, Lda (Grupo M2O)</t>
         </is>
       </c>
       <c r="B116" s="7" t="inlineStr">
@@ -6700,23 +6716,23 @@
       <c r="E116" s="5" t="inlineStr"/>
       <c r="F116" s="7" t="inlineStr">
         <is>
-          <t>Figueira da Foz</t>
+          <t>Loulé (Vilamoura)</t>
         </is>
       </c>
       <c r="G116" s="7" t="inlineStr">
         <is>
-          <t>Coimbra</t>
+          <t>Faro</t>
         </is>
       </c>
       <c r="H116" s="5" t="inlineStr"/>
       <c r="I116" s="5" t="inlineStr">
         <is>
-          <t>Urbanização antiga fábrica Alberto Gaspar (Planeamento (estudo prévio))</t>
+          <t>Rivus (Em construção/Comercialização)</t>
         </is>
       </c>
       <c r="J116" s="5" t="inlineStr">
         <is>
-          <t>Fonte: idealista.pt, asbeiras.pt</t>
+          <t>Fonte: construir.pt, idealista.pt</t>
         </is>
       </c>
       <c r="K116" s="5" t="inlineStr"/>
@@ -6726,7 +6742,7 @@
     <row r="117" ht="30" customHeight="1">
       <c r="A117" s="5" t="inlineStr">
         <is>
-          <t>Galvana Investimentos Imobiliários e Turísticos, Lda</t>
+          <t>Foz Gala Investments</t>
         </is>
       </c>
       <c r="B117" s="7" t="inlineStr">
@@ -6739,23 +6755,23 @@
       <c r="E117" s="5" t="inlineStr"/>
       <c r="F117" s="7" t="inlineStr">
         <is>
-          <t>Albufeira</t>
+          <t>Figueira da Foz</t>
         </is>
       </c>
       <c r="G117" s="7" t="inlineStr">
         <is>
-          <t>Faro</t>
+          <t>Coimbra</t>
         </is>
       </c>
       <c r="H117" s="5" t="inlineStr"/>
       <c r="I117" s="5" t="inlineStr">
         <is>
-          <t>Quinta Dourada (Em construção)</t>
+          <t>Urbanização antiga fábrica Alberto Gaspar (Planeamento (estudo prévio))</t>
         </is>
       </c>
       <c r="J117" s="5" t="inlineStr">
         <is>
-          <t>Fonte: oconnormurphy.ie, postal.pt</t>
+          <t>Fonte: idealista.pt, asbeiras.pt</t>
         </is>
       </c>
       <c r="K117" s="5" t="inlineStr"/>
@@ -6765,7 +6781,7 @@
     <row r="118" ht="30" customHeight="1">
       <c r="A118" s="5" t="inlineStr">
         <is>
-          <t>Genuino Investments</t>
+          <t>Galvana Investimentos Imobiliários e Turísticos, Lda</t>
         </is>
       </c>
       <c r="B118" s="7" t="inlineStr">
@@ -6775,14 +6791,10 @@
       </c>
       <c r="C118" s="7" t="inlineStr"/>
       <c r="D118" s="5" t="inlineStr"/>
-      <c r="E118" s="5" t="inlineStr">
-        <is>
-          <t>genuinoinvestments.com</t>
-        </is>
-      </c>
+      <c r="E118" s="5" t="inlineStr"/>
       <c r="F118" s="7" t="inlineStr">
         <is>
-          <t>Portimão</t>
+          <t>Albufeira</t>
         </is>
       </c>
       <c r="G118" s="7" t="inlineStr">
@@ -6793,12 +6805,12 @@
       <c r="H118" s="5" t="inlineStr"/>
       <c r="I118" s="5" t="inlineStr">
         <is>
-          <t>Genuíno Resort / Praia da Rocha (Comercialização)</t>
+          <t>Quinta Dourada (Em construção)</t>
         </is>
       </c>
       <c r="J118" s="5" t="inlineStr">
         <is>
-          <t>Fonte: genuinoinvestments.com</t>
+          <t>Fonte: oconnormurphy.ie, postal.pt</t>
         </is>
       </c>
       <c r="K118" s="5" t="inlineStr"/>
@@ -6808,7 +6820,7 @@
     <row r="119" ht="30" customHeight="1">
       <c r="A119" s="5" t="inlineStr">
         <is>
-          <t>GFH (Grupo Ferreira Holding) / Ferreira Build Power (marca BeLiving)</t>
+          <t>Genuino Investments</t>
         </is>
       </c>
       <c r="B119" s="7" t="inlineStr">
@@ -6820,12 +6832,12 @@
       <c r="D119" s="5" t="inlineStr"/>
       <c r="E119" s="5" t="inlineStr">
         <is>
-          <t>ferreirabuildpower.com</t>
+          <t>genuinoinvestments.com</t>
         </is>
       </c>
       <c r="F119" s="7" t="inlineStr">
         <is>
-          <t>Faro/Loulé</t>
+          <t>Portimão</t>
         </is>
       </c>
       <c r="G119" s="7" t="inlineStr">
@@ -6836,26 +6848,22 @@
       <c r="H119" s="5" t="inlineStr"/>
       <c r="I119" s="5" t="inlineStr">
         <is>
-          <t>BeLiving Faro / BeLiving HCC Loulé (Em construção)</t>
+          <t>Genuíno Resort / Praia da Rocha (Comercialização)</t>
         </is>
       </c>
       <c r="J119" s="5" t="inlineStr">
         <is>
-          <t>Fonte: eco.sapo.pt, jornaldenegocios.pt</t>
-        </is>
-      </c>
-      <c r="K119" s="5" t="inlineStr">
-        <is>
-          <t>Joaquim Silva (CEO Ferreira Build Power)</t>
-        </is>
-      </c>
+          <t>Fonte: genuinoinvestments.com</t>
+        </is>
+      </c>
+      <c r="K119" s="5" t="inlineStr"/>
       <c r="L119" s="5" t="inlineStr"/>
       <c r="M119" s="5" t="inlineStr"/>
     </row>
     <row r="120" ht="30" customHeight="1">
       <c r="A120" s="5" t="inlineStr">
         <is>
-          <t>Glowing</t>
+          <t>GFH (Grupo Ferreira Holding) / Ferreira Build Power (marca BeLiving)</t>
         </is>
       </c>
       <c r="B120" s="7" t="inlineStr">
@@ -6867,38 +6875,42 @@
       <c r="D120" s="5" t="inlineStr"/>
       <c r="E120" s="5" t="inlineStr">
         <is>
-          <t>glowing.pt</t>
+          <t>ferreirabuildpower.com</t>
         </is>
       </c>
       <c r="F120" s="7" t="inlineStr">
         <is>
-          <t>Alcácer do Sal</t>
+          <t>Faro/Loulé</t>
         </is>
       </c>
       <c r="G120" s="7" t="inlineStr">
         <is>
-          <t>Setúbal</t>
+          <t>Faro</t>
         </is>
       </c>
       <c r="H120" s="5" t="inlineStr"/>
       <c r="I120" s="5" t="inlineStr">
         <is>
-          <t>FiniSal (Em construção/Comercialização)</t>
+          <t>BeLiving Faro / BeLiving HCC Loulé (Em construção)</t>
         </is>
       </c>
       <c r="J120" s="5" t="inlineStr">
         <is>
-          <t>Fonte: idealista.pt</t>
-        </is>
-      </c>
-      <c r="K120" s="5" t="inlineStr"/>
+          <t>Fonte: eco.sapo.pt, jornaldenegocios.pt</t>
+        </is>
+      </c>
+      <c r="K120" s="5" t="inlineStr">
+        <is>
+          <t>Joaquim Silva (CEO Ferreira Build Power)</t>
+        </is>
+      </c>
       <c r="L120" s="5" t="inlineStr"/>
       <c r="M120" s="5" t="inlineStr"/>
     </row>
     <row r="121" ht="30" customHeight="1">
       <c r="A121" s="5" t="inlineStr">
         <is>
-          <t>Grupo A. Silva &amp; Silva</t>
+          <t>Glowing</t>
         </is>
       </c>
       <c r="B121" s="7" t="inlineStr">
@@ -6908,10 +6920,14 @@
       </c>
       <c r="C121" s="7" t="inlineStr"/>
       <c r="D121" s="5" t="inlineStr"/>
-      <c r="E121" s="5" t="inlineStr"/>
+      <c r="E121" s="5" t="inlineStr">
+        <is>
+          <t>glowing.pt</t>
+        </is>
+      </c>
       <c r="F121" s="7" t="inlineStr">
         <is>
-          <t>Seixal</t>
+          <t>Alcácer do Sal</t>
         </is>
       </c>
       <c r="G121" s="7" t="inlineStr">
@@ -6922,12 +6938,12 @@
       <c r="H121" s="5" t="inlineStr"/>
       <c r="I121" s="5" t="inlineStr">
         <is>
-          <t>Seixal Baía (Planeamento)</t>
+          <t>FiniSal (Em construção/Comercialização)</t>
         </is>
       </c>
       <c r="J121" s="5" t="inlineStr">
         <is>
-          <t>Fonte: novoperfil.pt</t>
+          <t>Fonte: idealista.pt</t>
         </is>
       </c>
       <c r="K121" s="5" t="inlineStr"/>
@@ -6937,7 +6953,7 @@
     <row r="122" ht="30" customHeight="1">
       <c r="A122" s="5" t="inlineStr">
         <is>
-          <t>Grupo André Guimarães (Portugal)</t>
+          <t>Grupo A. Silva &amp; Silva</t>
         </is>
       </c>
       <c r="B122" s="7" t="inlineStr">
@@ -6947,36 +6963,36 @@
       </c>
       <c r="C122" s="7" t="inlineStr"/>
       <c r="D122" s="5" t="inlineStr"/>
-      <c r="E122" s="5" t="inlineStr">
-        <is>
-          <t>andreguimaraes.com.br</t>
-        </is>
-      </c>
-      <c r="F122" s="7" t="inlineStr"/>
-      <c r="G122" s="7" t="inlineStr"/>
+      <c r="E122" s="5" t="inlineStr"/>
+      <c r="F122" s="7" t="inlineStr">
+        <is>
+          <t>Seixal</t>
+        </is>
+      </c>
+      <c r="G122" s="7" t="inlineStr">
+        <is>
+          <t>Setúbal</t>
+        </is>
+      </c>
       <c r="H122" s="5" t="inlineStr"/>
       <c r="I122" s="5" t="inlineStr">
         <is>
-          <t>JV com Overseas (Lisboa) (Planeamento) | Porto, Algarve, Douro, Cascais, Alentejo, Amarante (Em construção)</t>
+          <t>Seixal Baía (Planeamento)</t>
         </is>
       </c>
       <c r="J122" s="5" t="inlineStr">
         <is>
-          <t>Entidade PT: André Guimarães - Portugal, Lda (NIF 517865459). Sem contacto PT</t>
-        </is>
-      </c>
-      <c r="K122" s="5" t="inlineStr">
-        <is>
-          <t>Fundador falecido· hoje liderado pelos filhos (Brasil), sem responsável PT confirmado</t>
-        </is>
-      </c>
+          <t>Fonte: novoperfil.pt</t>
+        </is>
+      </c>
+      <c r="K122" s="5" t="inlineStr"/>
       <c r="L122" s="5" t="inlineStr"/>
       <c r="M122" s="5" t="inlineStr"/>
     </row>
     <row r="123" ht="30" customHeight="1">
       <c r="A123" s="5" t="inlineStr">
         <is>
-          <t>Grupo André Jordan</t>
+          <t>Grupo André Guimarães (Portugal)</t>
         </is>
       </c>
       <c r="B123" s="7" t="inlineStr">
@@ -6988,33 +7004,25 @@
       <c r="D123" s="5" t="inlineStr"/>
       <c r="E123" s="5" t="inlineStr">
         <is>
-          <t>andrejordangroup.pt</t>
-        </is>
-      </c>
-      <c r="F123" s="7" t="inlineStr">
-        <is>
-          <t>Sintra</t>
-        </is>
-      </c>
-      <c r="G123" s="7" t="inlineStr">
-        <is>
-          <t>Lisboa</t>
-        </is>
-      </c>
+          <t>andreguimaraes.com.br</t>
+        </is>
+      </c>
+      <c r="F123" s="7" t="inlineStr"/>
+      <c r="G123" s="7" t="inlineStr"/>
       <c r="H123" s="5" t="inlineStr"/>
       <c r="I123" s="5" t="inlineStr">
         <is>
-          <t>Lisbon Green Valley (Belas Clube de Campo) (Em construção)</t>
+          <t>JV com Overseas (Lisboa) (Planeamento) | Porto, Algarve, Douro, Cascais, Alentejo, Amarante (Em construção)</t>
         </is>
       </c>
       <c r="J123" s="5" t="inlineStr">
         <is>
-          <t>Fonte: idealista.pt</t>
+          <t>Entidade PT: André Guimarães - Portugal, Lda (NIF 517865459). Sem contacto PT</t>
         </is>
       </c>
       <c r="K123" s="5" t="inlineStr">
         <is>
-          <t>Gilberto Jordan (CEO desde 2009 · sucede a André Jordan, falecido 2024)</t>
+          <t>Fundador falecido· hoje liderado pelos filhos (Brasil), sem responsável PT confirmado</t>
         </is>
       </c>
       <c r="L123" s="5" t="inlineStr"/>
@@ -7023,7 +7031,7 @@
     <row r="124" ht="30" customHeight="1">
       <c r="A124" s="5" t="inlineStr">
         <is>
-          <t>Grupo AOC (Aníbal de Oliveira Cristina)</t>
+          <t>Grupo André Jordan</t>
         </is>
       </c>
       <c r="B124" s="7" t="inlineStr">
@@ -7033,31 +7041,35 @@
       </c>
       <c r="C124" s="7" t="inlineStr"/>
       <c r="D124" s="5" t="inlineStr"/>
-      <c r="E124" s="5" t="inlineStr"/>
+      <c r="E124" s="5" t="inlineStr">
+        <is>
+          <t>andrejordangroup.pt</t>
+        </is>
+      </c>
       <c r="F124" s="7" t="inlineStr">
         <is>
-          <t>Setúbal</t>
+          <t>Sintra</t>
         </is>
       </c>
       <c r="G124" s="7" t="inlineStr">
         <is>
-          <t>Setúbal</t>
+          <t>Lisboa</t>
         </is>
       </c>
       <c r="H124" s="5" t="inlineStr"/>
       <c r="I124" s="5" t="inlineStr">
         <is>
-          <t>Parque da Cidade – Riverside IV (Em construção)</t>
+          <t>Lisbon Green Valley (Belas Clube de Campo) (Em construção)</t>
         </is>
       </c>
       <c r="J124" s="5" t="inlineStr">
         <is>
-          <t>Fonte: linkedin.com/company/grupo-aoc</t>
+          <t>Fonte: idealista.pt</t>
         </is>
       </c>
       <c r="K124" s="5" t="inlineStr">
         <is>
-          <t>Aníbal Cristina (fundador, 1990)</t>
+          <t>Gilberto Jordan (CEO desde 2009 · sucede a André Jordan, falecido 2024)</t>
         </is>
       </c>
       <c r="L124" s="5" t="inlineStr"/>
@@ -7066,7 +7078,7 @@
     <row r="125" ht="30" customHeight="1">
       <c r="A125" s="5" t="inlineStr">
         <is>
-          <t>Grupo Azinor</t>
+          <t>Grupo AOC (Aníbal de Oliveira Cristina)</t>
         </is>
       </c>
       <c r="B125" s="7" t="inlineStr">
@@ -7079,41 +7091,37 @@
       <c r="E125" s="5" t="inlineStr"/>
       <c r="F125" s="7" t="inlineStr">
         <is>
-          <t>Oeiras</t>
+          <t>Setúbal</t>
         </is>
       </c>
       <c r="G125" s="7" t="inlineStr">
         <is>
-          <t>Lisboa</t>
+          <t>Setúbal</t>
         </is>
       </c>
       <c r="H125" s="5" t="inlineStr"/>
       <c r="I125" s="5" t="inlineStr">
         <is>
-          <t>Porto Cruz (Planeamento (consulta pública))</t>
+          <t>Parque da Cidade – Riverside IV (Em construção)</t>
         </is>
       </c>
       <c r="J125" s="5" t="inlineStr">
         <is>
-          <t>Fonte: idealista.pt</t>
+          <t>Fonte: linkedin.com/company/grupo-aoc</t>
         </is>
       </c>
       <c r="K125" s="5" t="inlineStr">
         <is>
-          <t>Carlos Silva Neves (administrador)</t>
-        </is>
-      </c>
-      <c r="L125" s="5" t="inlineStr">
-        <is>
-          <t>https://pt.linkedin.com/in/carlos-silva-neves-3b0711142</t>
-        </is>
-      </c>
+          <t>Aníbal Cristina (fundador, 1990)</t>
+        </is>
+      </c>
+      <c r="L125" s="5" t="inlineStr"/>
       <c r="M125" s="5" t="inlineStr"/>
     </row>
     <row r="126" ht="30" customHeight="1">
       <c r="A126" s="5" t="inlineStr">
         <is>
-          <t>Grupo Mais Empresas / Construções Mais</t>
+          <t>Grupo Azinor</t>
         </is>
       </c>
       <c r="B126" s="7" t="inlineStr">
@@ -7123,25 +7131,21 @@
       </c>
       <c r="C126" s="7" t="inlineStr"/>
       <c r="D126" s="5" t="inlineStr"/>
-      <c r="E126" s="5" t="inlineStr">
-        <is>
-          <t>grupomaisempresas.pt</t>
-        </is>
-      </c>
+      <c r="E126" s="5" t="inlineStr"/>
       <c r="F126" s="7" t="inlineStr">
         <is>
-          <t>Leiria</t>
+          <t>Oeiras</t>
         </is>
       </c>
       <c r="G126" s="7" t="inlineStr">
         <is>
-          <t>Leiria</t>
+          <t>Lisboa</t>
         </is>
       </c>
       <c r="H126" s="5" t="inlineStr"/>
       <c r="I126" s="5" t="inlineStr">
         <is>
-          <t>Golden Wolf (Em construção)</t>
+          <t>Porto Cruz (Planeamento (consulta pública))</t>
         </is>
       </c>
       <c r="J126" s="5" t="inlineStr">
@@ -7149,14 +7153,22 @@
           <t>Fonte: idealista.pt</t>
         </is>
       </c>
-      <c r="K126" s="5" t="inlineStr"/>
-      <c r="L126" s="5" t="inlineStr"/>
+      <c r="K126" s="5" t="inlineStr">
+        <is>
+          <t>Carlos Silva Neves (administrador)</t>
+        </is>
+      </c>
+      <c r="L126" s="5" t="inlineStr">
+        <is>
+          <t>https://pt.linkedin.com/in/carlos-silva-neves-3b0711142</t>
+        </is>
+      </c>
       <c r="M126" s="5" t="inlineStr"/>
     </row>
     <row r="127" ht="30" customHeight="1">
       <c r="A127" s="5" t="inlineStr">
         <is>
-          <t>Grupo NB Portugal</t>
+          <t>Grupo Mais Empresas / Construções Mais</t>
         </is>
       </c>
       <c r="B127" s="7" t="inlineStr">
@@ -7168,42 +7180,38 @@
       <c r="D127" s="5" t="inlineStr"/>
       <c r="E127" s="5" t="inlineStr">
         <is>
-          <t>gruponbportugal.pt</t>
+          <t>grupomaisempresas.pt</t>
         </is>
       </c>
       <c r="F127" s="7" t="inlineStr">
         <is>
-          <t>Aveiro</t>
+          <t>Leiria</t>
         </is>
       </c>
       <c r="G127" s="7" t="inlineStr">
         <is>
-          <t>Aveiro</t>
+          <t>Leiria</t>
         </is>
       </c>
       <c r="H127" s="5" t="inlineStr"/>
       <c r="I127" s="5" t="inlineStr">
         <is>
-          <t>NB 2040 / NB Garden (estado não confirmado)</t>
+          <t>Golden Wolf (Em construção)</t>
         </is>
       </c>
       <c r="J127" s="5" t="inlineStr">
         <is>
-          <t>Fonte: gruponb.pt</t>
-        </is>
-      </c>
-      <c r="K127" s="5" t="inlineStr">
-        <is>
-          <t>Ioav Blanche (presidente)</t>
-        </is>
-      </c>
+          <t>Fonte: idealista.pt</t>
+        </is>
+      </c>
+      <c r="K127" s="5" t="inlineStr"/>
       <c r="L127" s="5" t="inlineStr"/>
       <c r="M127" s="5" t="inlineStr"/>
     </row>
     <row r="128" ht="30" customHeight="1">
       <c r="A128" s="5" t="inlineStr">
         <is>
-          <t>Grupo Pestana (Pestana Residences)</t>
+          <t>Grupo NB Portugal</t>
         </is>
       </c>
       <c r="B128" s="7" t="inlineStr">
@@ -7215,33 +7223,33 @@
       <c r="D128" s="5" t="inlineStr"/>
       <c r="E128" s="5" t="inlineStr">
         <is>
-          <t>pestana.com</t>
+          <t>gruponbportugal.pt</t>
         </is>
       </c>
       <c r="F128" s="7" t="inlineStr">
         <is>
-          <t>Sines/Lagoa</t>
+          <t>Aveiro</t>
         </is>
       </c>
       <c r="G128" s="7" t="inlineStr">
         <is>
-          <t>Setúbal</t>
+          <t>Aveiro</t>
         </is>
       </c>
       <c r="H128" s="5" t="inlineStr"/>
       <c r="I128" s="5" t="inlineStr">
         <is>
-          <t>Pestana Porto Covo Beach Residences (Licenciamento)</t>
+          <t>NB 2040 / NB Garden (estado não confirmado)</t>
         </is>
       </c>
       <c r="J128" s="5" t="inlineStr">
         <is>
-          <t>Fonte: publico.pt, construir.pt</t>
+          <t>Fonte: gruponb.pt</t>
         </is>
       </c>
       <c r="K128" s="5" t="inlineStr">
         <is>
-          <t>Dionísio Pestana (Chairman/dono)</t>
+          <t>Ioav Blanche (presidente)</t>
         </is>
       </c>
       <c r="L128" s="5" t="inlineStr"/>
@@ -7250,7 +7258,7 @@
     <row r="129" ht="30" customHeight="1">
       <c r="A129" s="5" t="inlineStr">
         <is>
-          <t>Hillside House Coimbra, Lda</t>
+          <t>Grupo Pestana (Pestana Residences)</t>
         </is>
       </c>
       <c r="B129" s="7" t="inlineStr">
@@ -7262,38 +7270,42 @@
       <c r="D129" s="5" t="inlineStr"/>
       <c r="E129" s="5" t="inlineStr">
         <is>
-          <t>hillside.pt</t>
+          <t>pestana.com</t>
         </is>
       </c>
       <c r="F129" s="7" t="inlineStr">
         <is>
-          <t>Mealhada (projeto em Coimbra)</t>
+          <t>Sines/Lagoa</t>
         </is>
       </c>
       <c r="G129" s="7" t="inlineStr">
         <is>
-          <t>Aveiro</t>
+          <t>Setúbal</t>
         </is>
       </c>
       <c r="H129" s="5" t="inlineStr"/>
       <c r="I129" s="5" t="inlineStr">
         <is>
-          <t>Hillside – Areeiro (2ª fase) (Em construção)</t>
+          <t>Pestana Porto Covo Beach Residences (Licenciamento)</t>
         </is>
       </c>
       <c r="J129" s="5" t="inlineStr">
         <is>
-          <t>Fonte: remax.pt, hillside.pt</t>
-        </is>
-      </c>
-      <c r="K129" s="5" t="inlineStr"/>
+          <t>Fonte: publico.pt, construir.pt</t>
+        </is>
+      </c>
+      <c r="K129" s="5" t="inlineStr">
+        <is>
+          <t>Dionísio Pestana (Chairman/dono)</t>
+        </is>
+      </c>
       <c r="L129" s="5" t="inlineStr"/>
       <c r="M129" s="5" t="inlineStr"/>
     </row>
     <row r="130" ht="30" customHeight="1">
       <c r="A130" s="5" t="inlineStr">
         <is>
-          <t>Iconic Jeunesse, Unipessoal, Lda</t>
+          <t>Hillside House Coimbra, Lda</t>
         </is>
       </c>
       <c r="B130" s="7" t="inlineStr">
@@ -7305,28 +7317,28 @@
       <c r="D130" s="5" t="inlineStr"/>
       <c r="E130" s="5" t="inlineStr">
         <is>
-          <t>zenithresidences.pt</t>
+          <t>hillside.pt</t>
         </is>
       </c>
       <c r="F130" s="7" t="inlineStr">
         <is>
-          <t>Portimão</t>
+          <t>Mealhada (projeto em Coimbra)</t>
         </is>
       </c>
       <c r="G130" s="7" t="inlineStr">
         <is>
-          <t>Faro</t>
+          <t>Aveiro</t>
         </is>
       </c>
       <c r="H130" s="5" t="inlineStr"/>
       <c r="I130" s="5" t="inlineStr">
         <is>
-          <t>Zenith Residences (Em construção/Planeamento)</t>
+          <t>Hillside – Areeiro (2ª fase) (Em construção)</t>
         </is>
       </c>
       <c r="J130" s="5" t="inlineStr">
         <is>
-          <t>Fonte: zenithresidences.pt, jamesedition.com</t>
+          <t>Fonte: remax.pt, hillside.pt</t>
         </is>
       </c>
       <c r="K130" s="5" t="inlineStr"/>
@@ -7336,7 +7348,7 @@
     <row r="131" ht="30" customHeight="1">
       <c r="A131" s="5" t="inlineStr">
         <is>
-          <t>Invesquart – Real Estate Promotor</t>
+          <t>Iconic Jeunesse, Unipessoal, Lda</t>
         </is>
       </c>
       <c r="B131" s="7" t="inlineStr">
@@ -7346,10 +7358,14 @@
       </c>
       <c r="C131" s="7" t="inlineStr"/>
       <c r="D131" s="5" t="inlineStr"/>
-      <c r="E131" s="5" t="inlineStr"/>
+      <c r="E131" s="5" t="inlineStr">
+        <is>
+          <t>zenithresidences.pt</t>
+        </is>
+      </c>
       <c r="F131" s="7" t="inlineStr">
         <is>
-          <t>Loulé (Quarteira)</t>
+          <t>Portimão</t>
         </is>
       </c>
       <c r="G131" s="7" t="inlineStr">
@@ -7360,12 +7376,12 @@
       <c r="H131" s="5" t="inlineStr"/>
       <c r="I131" s="5" t="inlineStr">
         <is>
-          <t>Terraços de Quarteira (Comercialização)</t>
+          <t>Zenith Residences (Em construção/Planeamento)</t>
         </is>
       </c>
       <c r="J131" s="5" t="inlineStr">
         <is>
-          <t>Fonte: facebook.com/TerracosQuarteira</t>
+          <t>Fonte: zenithresidences.pt, jamesedition.com</t>
         </is>
       </c>
       <c r="K131" s="5" t="inlineStr"/>
@@ -7375,7 +7391,7 @@
     <row r="132" ht="30" customHeight="1">
       <c r="A132" s="5" t="inlineStr">
         <is>
-          <t>JPAIVA Investimentos / JPAIVA Engenharia e Construção</t>
+          <t>Invesquart – Real Estate Promotor</t>
         </is>
       </c>
       <c r="B132" s="7" t="inlineStr">
@@ -7385,48 +7401,36 @@
       </c>
       <c r="C132" s="7" t="inlineStr"/>
       <c r="D132" s="5" t="inlineStr"/>
-      <c r="E132" s="5" t="inlineStr">
-        <is>
-          <t>jpaiva.pt</t>
-        </is>
-      </c>
+      <c r="E132" s="5" t="inlineStr"/>
       <c r="F132" s="7" t="inlineStr">
         <is>
-          <t>Coimbra</t>
+          <t>Loulé (Quarteira)</t>
         </is>
       </c>
       <c r="G132" s="7" t="inlineStr">
         <is>
-          <t>Coimbra</t>
+          <t>Faro</t>
         </is>
       </c>
       <c r="H132" s="5" t="inlineStr"/>
       <c r="I132" s="5" t="inlineStr">
         <is>
-          <t>Garden Residence 2 (Antanhol) (Em construção/comercialização)</t>
+          <t>Terraços de Quarteira (Comercialização)</t>
         </is>
       </c>
       <c r="J132" s="5" t="inlineStr">
         <is>
-          <t>Fonte: jpaiva.pt</t>
-        </is>
-      </c>
-      <c r="K132" s="5" t="inlineStr">
-        <is>
-          <t>Igor Castro (CEO)</t>
-        </is>
-      </c>
-      <c r="L132" s="5" t="inlineStr">
-        <is>
-          <t>https://www.linkedin.com/in/igor-castro-a0026b22b/</t>
-        </is>
-      </c>
+          <t>Fonte: facebook.com/TerracosQuarteira</t>
+        </is>
+      </c>
+      <c r="K132" s="5" t="inlineStr"/>
+      <c r="L132" s="5" t="inlineStr"/>
       <c r="M132" s="5" t="inlineStr"/>
     </row>
     <row r="133" ht="30" customHeight="1">
       <c r="A133" s="5" t="inlineStr">
         <is>
-          <t>Lux Premium</t>
+          <t>JPAIVA Investimentos / JPAIVA Engenharia e Construção</t>
         </is>
       </c>
       <c r="B133" s="7" t="inlineStr">
@@ -7438,7 +7442,7 @@
       <c r="D133" s="5" t="inlineStr"/>
       <c r="E133" s="5" t="inlineStr">
         <is>
-          <t>luxpremium.net</t>
+          <t>jpaiva.pt</t>
         </is>
       </c>
       <c r="F133" s="7" t="inlineStr">
@@ -7454,26 +7458,30 @@
       <c r="H133" s="5" t="inlineStr"/>
       <c r="I133" s="5" t="inlineStr">
         <is>
-          <t>Coimbra Premium (Planeamento)</t>
+          <t>Garden Residence 2 (Antanhol) (Em construção/comercialização)</t>
         </is>
       </c>
       <c r="J133" s="5" t="inlineStr">
         <is>
-          <t>Fonte: luxpremium.net</t>
+          <t>Fonte: jpaiva.pt</t>
         </is>
       </c>
       <c r="K133" s="5" t="inlineStr">
         <is>
-          <t>Claude Berda (fundador)</t>
-        </is>
-      </c>
-      <c r="L133" s="5" t="inlineStr"/>
+          <t>Igor Castro (CEO)</t>
+        </is>
+      </c>
+      <c r="L133" s="5" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/igor-castro-a0026b22b/</t>
+        </is>
+      </c>
       <c r="M133" s="5" t="inlineStr"/>
     </row>
     <row r="134" ht="30" customHeight="1">
       <c r="A134" s="5" t="inlineStr">
         <is>
-          <t>MAJA Construções, S.A.</t>
+          <t>Le Parc</t>
         </is>
       </c>
       <c r="B134" s="7" t="inlineStr">
@@ -7483,10 +7491,14 @@
       </c>
       <c r="C134" s="7" t="inlineStr"/>
       <c r="D134" s="5" t="inlineStr"/>
-      <c r="E134" s="5" t="inlineStr"/>
+      <c r="E134" s="5" t="inlineStr">
+        <is>
+          <t>leparc.pt</t>
+        </is>
+      </c>
       <c r="F134" s="7" t="inlineStr">
         <is>
-          <t>Albufeira</t>
+          <t>Faro</t>
         </is>
       </c>
       <c r="G134" s="7" t="inlineStr">
@@ -7497,26 +7509,22 @@
       <c r="H134" s="5" t="inlineStr"/>
       <c r="I134" s="5" t="inlineStr">
         <is>
-          <t>Quinta Dourada (Em construção)</t>
+          <t>Le Parc Faro (Comercialização) | Le Parc Canidelo (V.N. Gaia) (Comercialização)</t>
         </is>
       </c>
       <c r="J134" s="5" t="inlineStr">
         <is>
-          <t>Fonte: oconnormurphy.ie</t>
-        </is>
-      </c>
-      <c r="K134" s="5" t="inlineStr">
-        <is>
-          <t>Manuel António e Jorge Almeida (fundadores, 1972)</t>
-        </is>
-      </c>
+          <t>Sem telefone próprio confirmado — número encontrado é da comercializadora JLL</t>
+        </is>
+      </c>
+      <c r="K134" s="5" t="inlineStr"/>
       <c r="L134" s="5" t="inlineStr"/>
       <c r="M134" s="5" t="inlineStr"/>
     </row>
     <row r="135" ht="30" customHeight="1">
       <c r="A135" s="5" t="inlineStr">
         <is>
-          <t>Mariano Investe – Empreendimentos Imobiliários</t>
+          <t>Lux Premium</t>
         </is>
       </c>
       <c r="B135" s="7" t="inlineStr">
@@ -7526,36 +7534,44 @@
       </c>
       <c r="C135" s="7" t="inlineStr"/>
       <c r="D135" s="5" t="inlineStr"/>
-      <c r="E135" s="5" t="inlineStr"/>
+      <c r="E135" s="5" t="inlineStr">
+        <is>
+          <t>luxpremium.net</t>
+        </is>
+      </c>
       <c r="F135" s="7" t="inlineStr">
         <is>
-          <t>Santarém</t>
+          <t>Coimbra</t>
         </is>
       </c>
       <c r="G135" s="7" t="inlineStr">
         <is>
-          <t>Santarém</t>
+          <t>Coimbra</t>
         </is>
       </c>
       <c r="H135" s="5" t="inlineStr"/>
       <c r="I135" s="5" t="inlineStr">
         <is>
-          <t>Quinta de São Pedro Valley (Em construção)</t>
+          <t>Coimbra Premium (Planeamento)</t>
         </is>
       </c>
       <c r="J135" s="5" t="inlineStr">
         <is>
-          <t>Fonte: idealista.pt</t>
-        </is>
-      </c>
-      <c r="K135" s="5" t="inlineStr"/>
+          <t>Fonte: luxpremium.net</t>
+        </is>
+      </c>
+      <c r="K135" s="5" t="inlineStr">
+        <is>
+          <t>Claude Berda (fundador)</t>
+        </is>
+      </c>
       <c r="L135" s="5" t="inlineStr"/>
       <c r="M135" s="5" t="inlineStr"/>
     </row>
     <row r="136" ht="30" customHeight="1">
       <c r="A136" s="5" t="inlineStr">
         <is>
-          <t>Maven (Maven Invest)</t>
+          <t>MAJA Construções, S.A.</t>
         </is>
       </c>
       <c r="B136" s="7" t="inlineStr">
@@ -7565,35 +7581,31 @@
       </c>
       <c r="C136" s="7" t="inlineStr"/>
       <c r="D136" s="5" t="inlineStr"/>
-      <c r="E136" s="5" t="inlineStr">
-        <is>
-          <t>maveninvest.pt</t>
-        </is>
-      </c>
+      <c r="E136" s="5" t="inlineStr"/>
       <c r="F136" s="7" t="inlineStr">
         <is>
-          <t>Setúbal</t>
+          <t>Albufeira</t>
         </is>
       </c>
       <c r="G136" s="7" t="inlineStr">
         <is>
-          <t>Setúbal</t>
+          <t>Faro</t>
         </is>
       </c>
       <c r="H136" s="5" t="inlineStr"/>
       <c r="I136" s="5" t="inlineStr">
         <is>
-          <t>WeBuild Castelo (Comercialização)</t>
+          <t>Quinta Dourada (Em construção)</t>
         </is>
       </c>
       <c r="J136" s="5" t="inlineStr">
         <is>
-          <t>Fonte: maveninvest.pt</t>
+          <t>Fonte: oconnormurphy.ie</t>
         </is>
       </c>
       <c r="K136" s="5" t="inlineStr">
         <is>
-          <t>Yehonatan Gourvitch (CEO)</t>
+          <t>Manuel António e Jorge Almeida (fundadores, 1972)</t>
         </is>
       </c>
       <c r="L136" s="5" t="inlineStr"/>
@@ -7602,7 +7614,7 @@
     <row r="137" ht="30" customHeight="1">
       <c r="A137" s="5" t="inlineStr">
         <is>
-          <t>Mello RDC</t>
+          <t>Mariano Investe – Empreendimentos Imobiliários</t>
         </is>
       </c>
       <c r="B137" s="7" t="inlineStr">
@@ -7612,48 +7624,36 @@
       </c>
       <c r="C137" s="7" t="inlineStr"/>
       <c r="D137" s="5" t="inlineStr"/>
-      <c r="E137" s="5" t="inlineStr">
-        <is>
-          <t>mellordc.pt</t>
-        </is>
-      </c>
+      <c r="E137" s="5" t="inlineStr"/>
       <c r="F137" s="7" t="inlineStr">
         <is>
-          <t>Grândola (Melides)</t>
+          <t>Santarém</t>
         </is>
       </c>
       <c r="G137" s="7" t="inlineStr">
         <is>
-          <t>Setúbal</t>
+          <t>Santarém</t>
         </is>
       </c>
       <c r="H137" s="5" t="inlineStr"/>
       <c r="I137" s="5" t="inlineStr">
         <is>
-          <t>Projeto hoteleiro em Melides (não divulgado) (Planeamento)</t>
+          <t>Quinta de São Pedro Valley (Em construção)</t>
         </is>
       </c>
       <c r="J137" s="5" t="inlineStr">
         <is>
-          <t>Fonte: vidaimobiliaria.com</t>
-        </is>
-      </c>
-      <c r="K137" s="5" t="inlineStr">
-        <is>
-          <t>António Ribeiro da Cunha (CEO)</t>
-        </is>
-      </c>
-      <c r="L137" s="5" t="inlineStr">
-        <is>
-          <t>https://pt.linkedin.com/in/ant%C3%B3nio-ribeiro-da-cunha-77b974112</t>
-        </is>
-      </c>
+          <t>Fonte: idealista.pt</t>
+        </is>
+      </c>
+      <c r="K137" s="5" t="inlineStr"/>
+      <c r="L137" s="5" t="inlineStr"/>
       <c r="M137" s="5" t="inlineStr"/>
     </row>
     <row r="138" ht="30" customHeight="1">
       <c r="A138" s="5" t="inlineStr">
         <is>
-          <t>Máscarazul – Mediação Imobiliária, Lda</t>
+          <t>Maven (Maven Invest)</t>
         </is>
       </c>
       <c r="B138" s="7" t="inlineStr">
@@ -7663,36 +7663,44 @@
       </c>
       <c r="C138" s="7" t="inlineStr"/>
       <c r="D138" s="5" t="inlineStr"/>
-      <c r="E138" s="5" t="inlineStr"/>
+      <c r="E138" s="5" t="inlineStr">
+        <is>
+          <t>maveninvest.pt</t>
+        </is>
+      </c>
       <c r="F138" s="7" t="inlineStr">
         <is>
-          <t>Albufeira</t>
+          <t>Setúbal</t>
         </is>
       </c>
       <c r="G138" s="7" t="inlineStr">
         <is>
-          <t>Faro</t>
+          <t>Setúbal</t>
         </is>
       </c>
       <c r="H138" s="5" t="inlineStr"/>
       <c r="I138" s="5" t="inlineStr">
         <is>
-          <t>Quinta Dourada (Em construção)</t>
+          <t>WeBuild Castelo (Comercialização)</t>
         </is>
       </c>
       <c r="J138" s="5" t="inlineStr">
         <is>
-          <t>Fonte: ireland-portugal.com</t>
-        </is>
-      </c>
-      <c r="K138" s="5" t="inlineStr"/>
+          <t>Fonte: maveninvest.pt</t>
+        </is>
+      </c>
+      <c r="K138" s="5" t="inlineStr">
+        <is>
+          <t>Yehonatan Gourvitch (CEO)</t>
+        </is>
+      </c>
       <c r="L138" s="5" t="inlineStr"/>
       <c r="M138" s="5" t="inlineStr"/>
     </row>
     <row r="139" ht="30" customHeight="1">
       <c r="A139" s="5" t="inlineStr">
         <is>
-          <t>Nova Atlantic</t>
+          <t>Mello RDC</t>
         </is>
       </c>
       <c r="B139" s="7" t="inlineStr">
@@ -7702,40 +7710,48 @@
       </c>
       <c r="C139" s="7" t="inlineStr"/>
       <c r="D139" s="5" t="inlineStr"/>
-      <c r="E139" s="5" t="inlineStr"/>
+      <c r="E139" s="5" t="inlineStr">
+        <is>
+          <t>mellordc.pt</t>
+        </is>
+      </c>
       <c r="F139" s="7" t="inlineStr">
         <is>
-          <t>Viana do Castelo</t>
+          <t>Grândola (Melides)</t>
         </is>
       </c>
       <c r="G139" s="7" t="inlineStr">
         <is>
-          <t>Viana do Castelo</t>
+          <t>Setúbal</t>
         </is>
       </c>
       <c r="H139" s="5" t="inlineStr"/>
       <c r="I139" s="5" t="inlineStr">
         <is>
-          <t>GREEN HILLS Viana Residences (Comercialização (arrancou set/2026))</t>
+          <t>Projeto hoteleiro em Melides (não divulgado) (Planeamento)</t>
         </is>
       </c>
       <c r="J139" s="5" t="inlineStr">
         <is>
-          <t>Fonte: jornaleconomico.sapo.pt</t>
+          <t>Fonte: vidaimobiliaria.com</t>
         </is>
       </c>
       <c r="K139" s="5" t="inlineStr">
         <is>
-          <t>Matan Amitai (co-fundador)</t>
-        </is>
-      </c>
-      <c r="L139" s="5" t="inlineStr"/>
+          <t>António Ribeiro da Cunha (CEO)</t>
+        </is>
+      </c>
+      <c r="L139" s="5" t="inlineStr">
+        <is>
+          <t>https://pt.linkedin.com/in/ant%C3%B3nio-ribeiro-da-cunha-77b974112</t>
+        </is>
+      </c>
       <c r="M139" s="5" t="inlineStr"/>
     </row>
     <row r="140" ht="30" customHeight="1">
       <c r="A140" s="5" t="inlineStr">
         <is>
-          <t>OCM Portugal (O'Connor Murphy)</t>
+          <t>Máscarazul – Mediação Imobiliária, Lda</t>
         </is>
       </c>
       <c r="B140" s="7" t="inlineStr">
@@ -7745,14 +7761,10 @@
       </c>
       <c r="C140" s="7" t="inlineStr"/>
       <c r="D140" s="5" t="inlineStr"/>
-      <c r="E140" s="5" t="inlineStr">
-        <is>
-          <t>oconnormurphy.ie</t>
-        </is>
-      </c>
+      <c r="E140" s="5" t="inlineStr"/>
       <c r="F140" s="7" t="inlineStr">
         <is>
-          <t>Olhão</t>
+          <t>Albufeira</t>
         </is>
       </c>
       <c r="G140" s="7" t="inlineStr">
@@ -7763,12 +7775,12 @@
       <c r="H140" s="5" t="inlineStr"/>
       <c r="I140" s="5" t="inlineStr">
         <is>
-          <t>Del Mar Waterfront Living (Comercialização)</t>
+          <t>Quinta Dourada (Em construção)</t>
         </is>
       </c>
       <c r="J140" s="5" t="inlineStr">
         <is>
-          <t>Fonte: jll.pt, delmarliving.pt</t>
+          <t>Fonte: ireland-portugal.com</t>
         </is>
       </c>
       <c r="K140" s="5" t="inlineStr"/>
@@ -7778,7 +7790,7 @@
     <row r="141" ht="30" customHeight="1">
       <c r="A141" s="5" t="inlineStr">
         <is>
-          <t>Ombria Resort (Grupo Pontos)</t>
+          <t>Nova Atlantic</t>
         </is>
       </c>
       <c r="B141" s="7" t="inlineStr">
@@ -7788,52 +7800,40 @@
       </c>
       <c r="C141" s="7" t="inlineStr"/>
       <c r="D141" s="5" t="inlineStr"/>
-      <c r="E141" s="5" t="inlineStr">
-        <is>
-          <t>ombria.com</t>
-        </is>
-      </c>
+      <c r="E141" s="5" t="inlineStr"/>
       <c r="F141" s="7" t="inlineStr">
         <is>
-          <t>Loulé</t>
+          <t>Viana do Castelo</t>
         </is>
       </c>
       <c r="G141" s="7" t="inlineStr">
         <is>
-          <t>Faro</t>
-        </is>
-      </c>
-      <c r="H141" s="5" t="inlineStr">
-        <is>
-          <t>Loulé</t>
-        </is>
-      </c>
+          <t>Viana do Castelo</t>
+        </is>
+      </c>
+      <c r="H141" s="5" t="inlineStr"/>
       <c r="I141" s="5" t="inlineStr">
         <is>
-          <t>Ombria Algarve (Em construção)</t>
+          <t>GREEN HILLS Viana Residences (Comercialização (arrancou set/2026))</t>
         </is>
       </c>
       <c r="J141" s="5" t="inlineStr">
         <is>
-          <t>Grupo finlandês Pontos · construtor Gabriel Couto</t>
+          <t>Fonte: jornaleconomico.sapo.pt</t>
         </is>
       </c>
       <c r="K141" s="5" t="inlineStr">
         <is>
-          <t>Patrick Freeman (CEO Ombria desde 2023)· CEO do Grupo Pontos é Timo Kokkila</t>
-        </is>
-      </c>
-      <c r="L141" s="5" t="inlineStr">
-        <is>
-          <t>https://www.linkedin.com/in/patricksfreeman/</t>
-        </is>
-      </c>
+          <t>Matan Amitai (co-fundador)</t>
+        </is>
+      </c>
+      <c r="L141" s="5" t="inlineStr"/>
       <c r="M141" s="5" t="inlineStr"/>
     </row>
     <row r="142" ht="30" customHeight="1">
       <c r="A142" s="5" t="inlineStr">
         <is>
-          <t>PATRIMOINIMMO PORTUGAL</t>
+          <t>OCM Portugal (O'Connor Murphy)</t>
         </is>
       </c>
       <c r="B142" s="7" t="inlineStr">
@@ -7843,10 +7843,14 @@
       </c>
       <c r="C142" s="7" t="inlineStr"/>
       <c r="D142" s="5" t="inlineStr"/>
-      <c r="E142" s="5" t="inlineStr"/>
+      <c r="E142" s="5" t="inlineStr">
+        <is>
+          <t>oconnormurphy.ie</t>
+        </is>
+      </c>
       <c r="F142" s="7" t="inlineStr">
         <is>
-          <t>Lagoa</t>
+          <t>Olhão</t>
         </is>
       </c>
       <c r="G142" s="7" t="inlineStr">
@@ -7857,12 +7861,12 @@
       <c r="H142" s="5" t="inlineStr"/>
       <c r="I142" s="5" t="inlineStr">
         <is>
-          <t>Ferragudo Hills Residência (Comercialização)</t>
+          <t>Del Mar Waterfront Living (Comercialização)</t>
         </is>
       </c>
       <c r="J142" s="5" t="inlineStr">
         <is>
-          <t>Fonte: ferreirabuildpower.com</t>
+          <t>Fonte: jll.pt, delmarliving.pt</t>
         </is>
       </c>
       <c r="K142" s="5" t="inlineStr"/>
@@ -7872,7 +7876,7 @@
     <row r="143" ht="30" customHeight="1">
       <c r="A143" s="5" t="inlineStr">
         <is>
-          <t>Pelicano – Investimento Imobiliário, S.A.</t>
+          <t>Ombria Resort (Grupo Pontos)</t>
         </is>
       </c>
       <c r="B143" s="7" t="inlineStr">
@@ -7882,40 +7886,52 @@
       </c>
       <c r="C143" s="7" t="inlineStr"/>
       <c r="D143" s="5" t="inlineStr"/>
-      <c r="E143" s="5" t="inlineStr"/>
+      <c r="E143" s="5" t="inlineStr">
+        <is>
+          <t>ombria.com</t>
+        </is>
+      </c>
       <c r="F143" s="7" t="inlineStr">
         <is>
-          <t>Palmela</t>
+          <t>Loulé</t>
         </is>
       </c>
       <c r="G143" s="7" t="inlineStr">
         <is>
-          <t>Setúbal</t>
-        </is>
-      </c>
-      <c r="H143" s="5" t="inlineStr"/>
+          <t>Faro</t>
+        </is>
+      </c>
+      <c r="H143" s="5" t="inlineStr">
+        <is>
+          <t>Loulé</t>
+        </is>
+      </c>
       <c r="I143" s="5" t="inlineStr">
         <is>
-          <t>Palmela Village (Comercialização)</t>
+          <t>Ombria Algarve (Em construção)</t>
         </is>
       </c>
       <c r="J143" s="5" t="inlineStr">
         <is>
-          <t>Fonte: racius.com, cnnportugal.iol.pt</t>
+          <t>Grupo finlandês Pontos · construtor Gabriel Couto</t>
         </is>
       </c>
       <c r="K143" s="5" t="inlineStr">
         <is>
-          <t>Joaquim Da Cunha Mendes Duarte (Presidente) / Sergio Manuel Mendes Gomes (Administrador)</t>
-        </is>
-      </c>
-      <c r="L143" s="5" t="inlineStr"/>
+          <t>Patrick Freeman (CEO Ombria desde 2023)· CEO do Grupo Pontos é Timo Kokkila</t>
+        </is>
+      </c>
+      <c r="L143" s="5" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/patricksfreeman/</t>
+        </is>
+      </c>
       <c r="M143" s="5" t="inlineStr"/>
     </row>
     <row r="144" ht="30" customHeight="1">
       <c r="A144" s="5" t="inlineStr">
         <is>
-          <t>Pensaplano</t>
+          <t>PATRIMOINIMMO PORTUGAL</t>
         </is>
       </c>
       <c r="B144" s="7" t="inlineStr">
@@ -7928,23 +7944,23 @@
       <c r="E144" s="5" t="inlineStr"/>
       <c r="F144" s="7" t="inlineStr">
         <is>
-          <t>Coimbra</t>
+          <t>Lagoa</t>
         </is>
       </c>
       <c r="G144" s="7" t="inlineStr">
         <is>
-          <t>Coimbra</t>
+          <t>Faro</t>
         </is>
       </c>
       <c r="H144" s="5" t="inlineStr"/>
       <c r="I144" s="5" t="inlineStr">
         <is>
-          <t>Eleven (Em construção)</t>
+          <t>Ferragudo Hills Residência (Comercialização)</t>
         </is>
       </c>
       <c r="J144" s="5" t="inlineStr">
         <is>
-          <t>Fonte: idealista.pt, construir.pt</t>
+          <t>Fonte: ferreirabuildpower.com</t>
         </is>
       </c>
       <c r="K144" s="5" t="inlineStr"/>
@@ -7954,7 +7970,7 @@
     <row r="145" ht="30" customHeight="1">
       <c r="A145" s="5" t="inlineStr">
         <is>
-          <t>Portugal Slow Living</t>
+          <t>Pelicano – Investimento Imobiliário, S.A.</t>
         </is>
       </c>
       <c r="B145" s="7" t="inlineStr">
@@ -7967,7 +7983,7 @@
       <c r="E145" s="5" t="inlineStr"/>
       <c r="F145" s="7" t="inlineStr">
         <is>
-          <t>Montijo</t>
+          <t>Palmela</t>
         </is>
       </c>
       <c r="G145" s="7" t="inlineStr">
@@ -7978,22 +7994,26 @@
       <c r="H145" s="5" t="inlineStr"/>
       <c r="I145" s="5" t="inlineStr">
         <is>
-          <t>Monville (Comercialização)</t>
+          <t>Palmela Village (Comercialização)</t>
         </is>
       </c>
       <c r="J145" s="5" t="inlineStr">
         <is>
-          <t>Fonte: idealista.pt</t>
-        </is>
-      </c>
-      <c r="K145" s="5" t="inlineStr"/>
+          <t>Fonte: racius.com, cnnportugal.iol.pt</t>
+        </is>
+      </c>
+      <c r="K145" s="5" t="inlineStr">
+        <is>
+          <t>Joaquim Da Cunha Mendes Duarte (Presidente) / Sergio Manuel Mendes Gomes (Administrador)</t>
+        </is>
+      </c>
       <c r="L145" s="5" t="inlineStr"/>
       <c r="M145" s="5" t="inlineStr"/>
     </row>
     <row r="146" ht="30" customHeight="1">
       <c r="A146" s="5" t="inlineStr">
         <is>
-          <t>Rivage Properties</t>
+          <t>Pensaplano</t>
         </is>
       </c>
       <c r="B146" s="7" t="inlineStr">
@@ -8006,37 +8026,33 @@
       <c r="E146" s="5" t="inlineStr"/>
       <c r="F146" s="7" t="inlineStr">
         <is>
-          <t>Gondomar</t>
+          <t>Coimbra</t>
         </is>
       </c>
       <c r="G146" s="7" t="inlineStr">
         <is>
-          <t>Porto</t>
+          <t>Coimbra</t>
         </is>
       </c>
       <c r="H146" s="5" t="inlineStr"/>
       <c r="I146" s="5" t="inlineStr">
         <is>
-          <t>The View II (Em construção (conclusão 2026))</t>
+          <t>Eleven (Em construção)</t>
         </is>
       </c>
       <c r="J146" s="5" t="inlineStr">
         <is>
-          <t>Fonte: jornaldenegocios.pt</t>
-        </is>
-      </c>
-      <c r="K146" s="5" t="inlineStr">
-        <is>
-          <t>João Ribeiro (CEO e fundador, com Jorge Duarte e Fernando Santos)</t>
-        </is>
-      </c>
+          <t>Fonte: idealista.pt, construir.pt</t>
+        </is>
+      </c>
+      <c r="K146" s="5" t="inlineStr"/>
       <c r="L146" s="5" t="inlineStr"/>
       <c r="M146" s="5" t="inlineStr"/>
     </row>
     <row r="147" ht="30" customHeight="1">
       <c r="A147" s="5" t="inlineStr">
         <is>
-          <t>Rodrigues &amp; Vermelho – Construções, S.A.</t>
+          <t>Portugal Slow Living</t>
         </is>
       </c>
       <c r="B147" s="7" t="inlineStr">
@@ -8046,44 +8062,36 @@
       </c>
       <c r="C147" s="7" t="inlineStr"/>
       <c r="D147" s="5" t="inlineStr"/>
-      <c r="E147" s="5" t="inlineStr">
-        <is>
-          <t>rodriguesevermelho.com</t>
-        </is>
-      </c>
+      <c r="E147" s="5" t="inlineStr"/>
       <c r="F147" s="7" t="inlineStr">
         <is>
-          <t>Lagos</t>
+          <t>Montijo</t>
         </is>
       </c>
       <c r="G147" s="7" t="inlineStr">
         <is>
-          <t>Faro</t>
+          <t>Setúbal</t>
         </is>
       </c>
       <c r="H147" s="5" t="inlineStr"/>
       <c r="I147" s="5" t="inlineStr">
         <is>
-          <t>Domus (Domus 22 e 23) (Em construção)</t>
+          <t>Monville (Comercialização)</t>
         </is>
       </c>
       <c r="J147" s="5" t="inlineStr">
         <is>
-          <t>Fonte: sava.pt, thepreplan.com</t>
-        </is>
-      </c>
-      <c r="K147" s="5" t="inlineStr">
-        <is>
-          <t>Celestino Vermelho Rodrigues (contacto)</t>
-        </is>
-      </c>
+          <t>Fonte: idealista.pt</t>
+        </is>
+      </c>
+      <c r="K147" s="5" t="inlineStr"/>
       <c r="L147" s="5" t="inlineStr"/>
       <c r="M147" s="5" t="inlineStr"/>
     </row>
     <row r="148" ht="30" customHeight="1">
       <c r="A148" s="5" t="inlineStr">
         <is>
-          <t>Soccal &amp; Vaz Invest</t>
+          <t>Rivage Properties</t>
         </is>
       </c>
       <c r="B148" s="7" t="inlineStr">
@@ -8093,48 +8101,40 @@
       </c>
       <c r="C148" s="7" t="inlineStr"/>
       <c r="D148" s="5" t="inlineStr"/>
-      <c r="E148" s="5" t="inlineStr">
-        <is>
-          <t>soccal-vaz.com</t>
-        </is>
-      </c>
+      <c r="E148" s="5" t="inlineStr"/>
       <c r="F148" s="7" t="inlineStr">
         <is>
-          <t>Sines</t>
+          <t>Gondomar</t>
         </is>
       </c>
       <c r="G148" s="7" t="inlineStr">
         <is>
-          <t>Setúbal</t>
+          <t>Porto</t>
         </is>
       </c>
       <c r="H148" s="5" t="inlineStr"/>
       <c r="I148" s="5" t="inlineStr">
         <is>
-          <t>Brisa Mar (Em construção)</t>
+          <t>The View II (Em construção (conclusão 2026))</t>
         </is>
       </c>
       <c r="J148" s="5" t="inlineStr">
         <is>
-          <t>Fonte: eco.sapo.pt</t>
+          <t>Fonte: jornaldenegocios.pt</t>
         </is>
       </c>
       <c r="K148" s="5" t="inlineStr">
         <is>
-          <t>António Vaz (fundador e CEO)</t>
-        </is>
-      </c>
-      <c r="L148" s="5" t="inlineStr">
-        <is>
-          <t>https://www.linkedin.com/in/antonio-vaz-9444998a/</t>
-        </is>
-      </c>
+          <t>João Ribeiro (CEO e fundador, com Jorge Duarte e Fernando Santos)</t>
+        </is>
+      </c>
+      <c r="L148" s="5" t="inlineStr"/>
       <c r="M148" s="5" t="inlineStr"/>
     </row>
     <row r="149" ht="30" customHeight="1">
       <c r="A149" s="5" t="inlineStr">
         <is>
-          <t>Solid Sentinel</t>
+          <t>Rodrigues &amp; Vermelho – Construções, S.A.</t>
         </is>
       </c>
       <c r="B149" s="7" t="inlineStr">
@@ -8146,46 +8146,42 @@
       <c r="D149" s="5" t="inlineStr"/>
       <c r="E149" s="5" t="inlineStr">
         <is>
-          <t>solidsentinel.pt</t>
+          <t>rodriguesevermelho.com</t>
         </is>
       </c>
       <c r="F149" s="7" t="inlineStr">
         <is>
-          <t>Barreiro</t>
+          <t>Lagos</t>
         </is>
       </c>
       <c r="G149" s="7" t="inlineStr">
         <is>
-          <t>Setúbal</t>
+          <t>Faro</t>
         </is>
       </c>
       <c r="H149" s="5" t="inlineStr"/>
       <c r="I149" s="5" t="inlineStr">
         <is>
-          <t>NOOBA (Em construção/comercialização)</t>
+          <t>Domus (Domus 22 e 23) (Em construção)</t>
         </is>
       </c>
       <c r="J149" s="5" t="inlineStr">
         <is>
-          <t>Fonte: reportugal.vidaimobiliaria.com</t>
+          <t>Fonte: sava.pt, thepreplan.com</t>
         </is>
       </c>
       <c r="K149" s="5" t="inlineStr">
         <is>
-          <t>Alain Gross (Co-Founder e CEO)</t>
-        </is>
-      </c>
-      <c r="L149" s="5" t="inlineStr">
-        <is>
-          <t>https://www.linkedin.com/in/alain-gross-3351411/</t>
-        </is>
-      </c>
+          <t>Celestino Vermelho Rodrigues (contacto)</t>
+        </is>
+      </c>
+      <c r="L149" s="5" t="inlineStr"/>
       <c r="M149" s="5" t="inlineStr"/>
     </row>
     <row r="150" ht="30" customHeight="1">
       <c r="A150" s="5" t="inlineStr">
         <is>
-          <t>SOLUM PROGRESS</t>
+          <t>Soccal &amp; Vaz Invest</t>
         </is>
       </c>
       <c r="B150" s="7" t="inlineStr">
@@ -8195,36 +8191,48 @@
       </c>
       <c r="C150" s="7" t="inlineStr"/>
       <c r="D150" s="5" t="inlineStr"/>
-      <c r="E150" s="5" t="inlineStr"/>
+      <c r="E150" s="5" t="inlineStr">
+        <is>
+          <t>soccal-vaz.com</t>
+        </is>
+      </c>
       <c r="F150" s="7" t="inlineStr">
         <is>
-          <t>Coimbra</t>
+          <t>Sines</t>
         </is>
       </c>
       <c r="G150" s="7" t="inlineStr">
         <is>
-          <t>Coimbra</t>
+          <t>Setúbal</t>
         </is>
       </c>
       <c r="H150" s="5" t="inlineStr"/>
       <c r="I150" s="5" t="inlineStr">
         <is>
-          <t>Namora Residence (Solum, Sto. António dos Olivais) (Em construção/comercialização)</t>
+          <t>Brisa Mar (Em construção)</t>
         </is>
       </c>
       <c r="J150" s="5" t="inlineStr">
         <is>
-          <t>Fonte: jpaiva.pt, zome.pt</t>
-        </is>
-      </c>
-      <c r="K150" s="5" t="inlineStr"/>
-      <c r="L150" s="5" t="inlineStr"/>
+          <t>Fonte: eco.sapo.pt</t>
+        </is>
+      </c>
+      <c r="K150" s="5" t="inlineStr">
+        <is>
+          <t>António Vaz (fundador e CEO)</t>
+        </is>
+      </c>
+      <c r="L150" s="5" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/antonio-vaz-9444998a/</t>
+        </is>
+      </c>
       <c r="M150" s="5" t="inlineStr"/>
     </row>
     <row r="151" ht="30" customHeight="1">
       <c r="A151" s="5" t="inlineStr">
         <is>
-          <t>Sonae Sierra</t>
+          <t>Solid Sentinel</t>
         </is>
       </c>
       <c r="B151" s="7" t="inlineStr">
@@ -8236,42 +8244,46 @@
       <c r="D151" s="5" t="inlineStr"/>
       <c r="E151" s="5" t="inlineStr">
         <is>
-          <t>sonaesierra.com</t>
+          <t>solidsentinel.pt</t>
         </is>
       </c>
       <c r="F151" s="7" t="inlineStr">
         <is>
-          <t>Lisboa/Porto</t>
+          <t>Barreiro</t>
         </is>
       </c>
       <c r="G151" s="7" t="inlineStr">
         <is>
-          <t>nacional</t>
+          <t>Setúbal</t>
         </is>
       </c>
       <c r="H151" s="5" t="inlineStr"/>
       <c r="I151" s="5" t="inlineStr">
         <is>
-          <t>Pulse Lisboa (Em construção)</t>
+          <t>NOOBA (Em construção/comercialização)</t>
         </is>
       </c>
       <c r="J151" s="5" t="inlineStr">
         <is>
-          <t>Fonte: rtp.pt, idealista.pt</t>
+          <t>Fonte: reportugal.vidaimobiliaria.com</t>
         </is>
       </c>
       <c r="K151" s="5" t="inlineStr">
         <is>
-          <t>Fernando Guedes de Oliveira (CEO)</t>
-        </is>
-      </c>
-      <c r="L151" s="5" t="inlineStr"/>
+          <t>Alain Gross (Co-Founder e CEO)</t>
+        </is>
+      </c>
+      <c r="L151" s="5" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/alain-gross-3351411/</t>
+        </is>
+      </c>
       <c r="M151" s="5" t="inlineStr"/>
     </row>
     <row r="152" ht="30" customHeight="1">
       <c r="A152" s="5" t="inlineStr">
         <is>
-          <t>Southshore Investments</t>
+          <t>SOLUM PROGRESS</t>
         </is>
       </c>
       <c r="B152" s="7" t="inlineStr">
@@ -8281,30 +8293,26 @@
       </c>
       <c r="C152" s="7" t="inlineStr"/>
       <c r="D152" s="5" t="inlineStr"/>
-      <c r="E152" s="5" t="inlineStr">
-        <is>
-          <t>southshoreinvest.com</t>
-        </is>
-      </c>
+      <c r="E152" s="5" t="inlineStr"/>
       <c r="F152" s="7" t="inlineStr">
         <is>
-          <t>Almada</t>
+          <t>Coimbra</t>
         </is>
       </c>
       <c r="G152" s="7" t="inlineStr">
         <is>
-          <t>Setúbal</t>
+          <t>Coimbra</t>
         </is>
       </c>
       <c r="H152" s="5" t="inlineStr"/>
       <c r="I152" s="5" t="inlineStr">
         <is>
-          <t>Tejo City District (Planeamento)</t>
+          <t>Namora Residence (Solum, Sto. António dos Olivais) (Em construção/comercialização)</t>
         </is>
       </c>
       <c r="J152" s="5" t="inlineStr">
         <is>
-          <t>Fonte: southshoreinvest.com</t>
+          <t>Fonte: jpaiva.pt, zome.pt</t>
         </is>
       </c>
       <c r="K152" s="5" t="inlineStr"/>
@@ -8314,7 +8322,7 @@
     <row r="153" ht="30" customHeight="1">
       <c r="A153" s="5" t="inlineStr">
         <is>
-          <t>Square View</t>
+          <t>Sonae Sierra</t>
         </is>
       </c>
       <c r="B153" s="7" t="inlineStr">
@@ -8326,33 +8334,33 @@
       <c r="D153" s="5" t="inlineStr"/>
       <c r="E153" s="5" t="inlineStr">
         <is>
-          <t>squareview.pt</t>
+          <t>sonaesierra.com</t>
         </is>
       </c>
       <c r="F153" s="7" t="inlineStr">
         <is>
-          <t>Lisboa/Ericeira/Melides</t>
+          <t>Lisboa/Porto</t>
         </is>
       </c>
       <c r="G153" s="7" t="inlineStr">
         <is>
-          <t>Lisboa</t>
+          <t>nacional</t>
         </is>
       </c>
       <c r="H153" s="5" t="inlineStr"/>
       <c r="I153" s="5" t="inlineStr">
         <is>
-          <t>4 projetos residenciais multifamiliares (nomes não encontrados) (Em desenvolvimento)</t>
+          <t>Pulse Lisboa (Em construção)</t>
         </is>
       </c>
       <c r="J153" s="5" t="inlineStr">
         <is>
-          <t>Fonte: squareview.pt</t>
+          <t>Fonte: rtp.pt, idealista.pt</t>
         </is>
       </c>
       <c r="K153" s="5" t="inlineStr">
         <is>
-          <t>Luis Horta e Costa (CEO/Fundador)</t>
+          <t>Fernando Guedes de Oliveira (CEO)</t>
         </is>
       </c>
       <c r="L153" s="5" t="inlineStr"/>
@@ -8361,7 +8369,7 @@
     <row r="154" ht="30" customHeight="1">
       <c r="A154" s="5" t="inlineStr">
         <is>
-          <t>Terrace Benefit, Lda</t>
+          <t>Southshore Investments</t>
         </is>
       </c>
       <c r="B154" s="7" t="inlineStr">
@@ -8371,26 +8379,30 @@
       </c>
       <c r="C154" s="7" t="inlineStr"/>
       <c r="D154" s="5" t="inlineStr"/>
-      <c r="E154" s="5" t="inlineStr"/>
+      <c r="E154" s="5" t="inlineStr">
+        <is>
+          <t>southshoreinvest.com</t>
+        </is>
+      </c>
       <c r="F154" s="7" t="inlineStr">
         <is>
-          <t>Loulé (Quarteira)</t>
+          <t>Almada</t>
         </is>
       </c>
       <c r="G154" s="7" t="inlineStr">
         <is>
-          <t>Faro</t>
+          <t>Setúbal</t>
         </is>
       </c>
       <c r="H154" s="5" t="inlineStr"/>
       <c r="I154" s="5" t="inlineStr">
         <is>
-          <t>Forte Novo (Em construção)</t>
+          <t>Tejo City District (Planeamento)</t>
         </is>
       </c>
       <c r="J154" s="5" t="inlineStr">
         <is>
-          <t>Fonte: racius.com, idealista.pt</t>
+          <t>Fonte: southshoreinvest.com</t>
         </is>
       </c>
       <c r="K154" s="5" t="inlineStr"/>
@@ -8400,7 +8412,7 @@
     <row r="155" ht="30" customHeight="1">
       <c r="A155" s="5" t="inlineStr">
         <is>
-          <t>Udra – Grupo San José</t>
+          <t>Square View</t>
         </is>
       </c>
       <c r="B155" s="7" t="inlineStr">
@@ -8410,36 +8422,44 @@
       </c>
       <c r="C155" s="7" t="inlineStr"/>
       <c r="D155" s="5" t="inlineStr"/>
-      <c r="E155" s="5" t="inlineStr"/>
+      <c r="E155" s="5" t="inlineStr">
+        <is>
+          <t>squareview.pt</t>
+        </is>
+      </c>
       <c r="F155" s="7" t="inlineStr">
         <is>
-          <t>Setúbal</t>
+          <t>Lisboa/Ericeira/Melides</t>
         </is>
       </c>
       <c r="G155" s="7" t="inlineStr">
         <is>
-          <t>Setúbal</t>
+          <t>Lisboa</t>
         </is>
       </c>
       <c r="H155" s="5" t="inlineStr"/>
       <c r="I155" s="5" t="inlineStr">
         <is>
-          <t>Parque da Cidade – Riverside II (Em construção)</t>
+          <t>4 projetos residenciais multifamiliares (nomes não encontrados) (Em desenvolvimento)</t>
         </is>
       </c>
       <c r="J155" s="5" t="inlineStr">
         <is>
-          <t>Fonte: idealista.pt</t>
-        </is>
-      </c>
-      <c r="K155" s="5" t="inlineStr"/>
+          <t>Fonte: squareview.pt</t>
+        </is>
+      </c>
+      <c r="K155" s="5" t="inlineStr">
+        <is>
+          <t>Luis Horta e Costa (CEO/Fundador)</t>
+        </is>
+      </c>
       <c r="L155" s="5" t="inlineStr"/>
       <c r="M155" s="5" t="inlineStr"/>
     </row>
     <row r="156" ht="30" customHeight="1">
       <c r="A156" s="5" t="inlineStr">
         <is>
-          <t>Urban Green Private (UGP)</t>
+          <t>Terrace Benefit, Lda</t>
         </is>
       </c>
       <c r="B156" s="7" t="inlineStr">
@@ -8449,14 +8469,10 @@
       </c>
       <c r="C156" s="7" t="inlineStr"/>
       <c r="D156" s="5" t="inlineStr"/>
-      <c r="E156" s="5" t="inlineStr">
-        <is>
-          <t>ugp.ie</t>
-        </is>
-      </c>
+      <c r="E156" s="5" t="inlineStr"/>
       <c r="F156" s="7" t="inlineStr">
         <is>
-          <t>Faro</t>
+          <t>Loulé (Quarteira)</t>
         </is>
       </c>
       <c r="G156" s="7" t="inlineStr">
@@ -8467,26 +8483,22 @@
       <c r="H156" s="5" t="inlineStr"/>
       <c r="I156" s="5" t="inlineStr">
         <is>
-          <t>The Shipyard (Comercialização)</t>
+          <t>Forte Novo (Em construção)</t>
         </is>
       </c>
       <c r="J156" s="5" t="inlineStr">
         <is>
-          <t>Fonte: theshipyard.pt, barlavento.pt</t>
-        </is>
-      </c>
-      <c r="K156" s="5" t="inlineStr">
-        <is>
-          <t>Thomas Coughlan (fundador)</t>
-        </is>
-      </c>
+          <t>Fonte: racius.com, idealista.pt</t>
+        </is>
+      </c>
+      <c r="K156" s="5" t="inlineStr"/>
       <c r="L156" s="5" t="inlineStr"/>
       <c r="M156" s="5" t="inlineStr"/>
     </row>
     <row r="157" ht="30" customHeight="1">
       <c r="A157" s="5" t="inlineStr">
         <is>
-          <t>Vale do Lobo Resort</t>
+          <t>The Epic Group</t>
         </is>
       </c>
       <c r="B157" s="7" t="inlineStr">
@@ -8498,32 +8510,28 @@
       <c r="D157" s="5" t="inlineStr"/>
       <c r="E157" s="5" t="inlineStr">
         <is>
-          <t>valedolobo.com</t>
+          <t>valentavillas.com</t>
         </is>
       </c>
       <c r="F157" s="7" t="inlineStr">
         <is>
-          <t>Loulé</t>
+          <t>Ílhavo</t>
         </is>
       </c>
       <c r="G157" s="7" t="inlineStr">
         <is>
-          <t>Faro</t>
-        </is>
-      </c>
-      <c r="H157" s="5" t="inlineStr">
-        <is>
-          <t>Parque do Golfe</t>
-        </is>
-      </c>
+          <t>Aveiro</t>
+        </is>
+      </c>
+      <c r="H157" s="5" t="inlineStr"/>
       <c r="I157" s="5" t="inlineStr">
         <is>
-          <t>Vale Real (lotes/moradias em planta) (Planeamento) | Oceano Clube (Comercialização) | The Residences (Comercialização)</t>
+          <t>Valenta Villas (Ermida, Ílhavo) (Comercialização)</t>
         </is>
       </c>
       <c r="J157" s="5" t="inlineStr">
         <is>
-          <t>Adquirido 2022 por fundo assessorado pela Davidson Kempner Capital Management. Promotor/gestor operacional: Kronos Real Estate Group</t>
+          <t>Sem telefone/CEO confirmados nas fontes</t>
         </is>
       </c>
       <c r="K157" s="5" t="inlineStr"/>
@@ -8533,7 +8541,7 @@
     <row r="158" ht="30" customHeight="1">
       <c r="A158" s="5" t="inlineStr">
         <is>
-          <t>Vila Galé</t>
+          <t>Udra – Grupo San José</t>
         </is>
       </c>
       <c r="B158" s="7" t="inlineStr">
@@ -8543,25 +8551,21 @@
       </c>
       <c r="C158" s="7" t="inlineStr"/>
       <c r="D158" s="5" t="inlineStr"/>
-      <c r="E158" s="5" t="inlineStr">
-        <is>
-          <t>vilagale.com</t>
-        </is>
-      </c>
+      <c r="E158" s="5" t="inlineStr"/>
       <c r="F158" s="7" t="inlineStr">
         <is>
-          <t>Golegã</t>
+          <t>Setúbal</t>
         </is>
       </c>
       <c r="G158" s="7" t="inlineStr">
         <is>
-          <t>Santarém</t>
+          <t>Setúbal</t>
         </is>
       </c>
       <c r="H158" s="5" t="inlineStr"/>
       <c r="I158" s="5" t="inlineStr">
         <is>
-          <t>Vila Galé Collection Tejo (Quinta da Cardiga) (Em construção)</t>
+          <t>Parque da Cidade – Riverside II (Em construção)</t>
         </is>
       </c>
       <c r="J158" s="5" t="inlineStr">
@@ -8572,6 +8576,143 @@
       <c r="K158" s="5" t="inlineStr"/>
       <c r="L158" s="5" t="inlineStr"/>
       <c r="M158" s="5" t="inlineStr"/>
+    </row>
+    <row r="159" ht="30" customHeight="1">
+      <c r="A159" s="5" t="inlineStr">
+        <is>
+          <t>Urban Green Private (UGP)</t>
+        </is>
+      </c>
+      <c r="B159" s="7" t="inlineStr">
+        <is>
+          <t>Nao</t>
+        </is>
+      </c>
+      <c r="C159" s="7" t="inlineStr"/>
+      <c r="D159" s="5" t="inlineStr"/>
+      <c r="E159" s="5" t="inlineStr">
+        <is>
+          <t>ugp.ie</t>
+        </is>
+      </c>
+      <c r="F159" s="7" t="inlineStr">
+        <is>
+          <t>Faro</t>
+        </is>
+      </c>
+      <c r="G159" s="7" t="inlineStr">
+        <is>
+          <t>Faro</t>
+        </is>
+      </c>
+      <c r="H159" s="5" t="inlineStr"/>
+      <c r="I159" s="5" t="inlineStr">
+        <is>
+          <t>The Shipyard (Comercialização)</t>
+        </is>
+      </c>
+      <c r="J159" s="5" t="inlineStr">
+        <is>
+          <t>Fonte: theshipyard.pt, barlavento.pt</t>
+        </is>
+      </c>
+      <c r="K159" s="5" t="inlineStr">
+        <is>
+          <t>Thomas Coughlan (fundador)</t>
+        </is>
+      </c>
+      <c r="L159" s="5" t="inlineStr"/>
+      <c r="M159" s="5" t="inlineStr"/>
+    </row>
+    <row r="160" ht="30" customHeight="1">
+      <c r="A160" s="5" t="inlineStr">
+        <is>
+          <t>Vale do Lobo Resort</t>
+        </is>
+      </c>
+      <c r="B160" s="7" t="inlineStr">
+        <is>
+          <t>Nao</t>
+        </is>
+      </c>
+      <c r="C160" s="7" t="inlineStr"/>
+      <c r="D160" s="5" t="inlineStr"/>
+      <c r="E160" s="5" t="inlineStr">
+        <is>
+          <t>valedolobo.com</t>
+        </is>
+      </c>
+      <c r="F160" s="7" t="inlineStr">
+        <is>
+          <t>Loulé</t>
+        </is>
+      </c>
+      <c r="G160" s="7" t="inlineStr">
+        <is>
+          <t>Faro</t>
+        </is>
+      </c>
+      <c r="H160" s="5" t="inlineStr">
+        <is>
+          <t>Parque do Golfe</t>
+        </is>
+      </c>
+      <c r="I160" s="5" t="inlineStr">
+        <is>
+          <t>Vale Real (lotes/moradias em planta) (Planeamento) | Oceano Clube (Comercialização) | The Residences (Comercialização)</t>
+        </is>
+      </c>
+      <c r="J160" s="5" t="inlineStr">
+        <is>
+          <t>Adquirido 2022 por fundo assessorado pela Davidson Kempner Capital Management. Promotor/gestor operacional: Kronos Real Estate Group</t>
+        </is>
+      </c>
+      <c r="K160" s="5" t="inlineStr"/>
+      <c r="L160" s="5" t="inlineStr"/>
+      <c r="M160" s="5" t="inlineStr"/>
+    </row>
+    <row r="161" ht="30" customHeight="1">
+      <c r="A161" s="5" t="inlineStr">
+        <is>
+          <t>Vila Galé</t>
+        </is>
+      </c>
+      <c r="B161" s="7" t="inlineStr">
+        <is>
+          <t>Nao</t>
+        </is>
+      </c>
+      <c r="C161" s="7" t="inlineStr"/>
+      <c r="D161" s="5" t="inlineStr"/>
+      <c r="E161" s="5" t="inlineStr">
+        <is>
+          <t>vilagale.com</t>
+        </is>
+      </c>
+      <c r="F161" s="7" t="inlineStr">
+        <is>
+          <t>Golegã</t>
+        </is>
+      </c>
+      <c r="G161" s="7" t="inlineStr">
+        <is>
+          <t>Santarém</t>
+        </is>
+      </c>
+      <c r="H161" s="5" t="inlineStr"/>
+      <c r="I161" s="5" t="inlineStr">
+        <is>
+          <t>Vila Galé Collection Tejo (Quinta da Cardiga) (Em construção)</t>
+        </is>
+      </c>
+      <c r="J161" s="5" t="inlineStr">
+        <is>
+          <t>Fonte: idealista.pt</t>
+        </is>
+      </c>
+      <c r="K161" s="5" t="inlineStr"/>
+      <c r="L161" s="5" t="inlineStr"/>
+      <c r="M161" s="5" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -8613,7 +8754,7 @@
         </is>
       </c>
       <c r="B2" s="9" t="n">
-        <v>157</v>
+        <v>160</v>
       </c>
     </row>
     <row r="3">
@@ -8623,7 +8764,7 @@
         </is>
       </c>
       <c r="B3" s="9" t="n">
-        <v>70</v>
+        <v>71</v>
       </c>
     </row>
     <row r="4">
@@ -8633,7 +8774,7 @@
         </is>
       </c>
       <c r="B4" s="9" t="n">
-        <v>87</v>
+        <v>89</v>
       </c>
     </row>
     <row r="5">

</xml_diff>

<commit_message>
Find phone numbers for 11 priority companies without one
Fortera, Overseas, RAR Imobiliária, Visabeirahouse, Nhood Portugal,
Arts Investments, Round Hill Capital, Screendomus, AFA, Prime Portugal
(flagged as possibly the same entity as "Prime Lisbon", same address —
worth confirming), United Investments Portugal. Also upgrades RAR
Imobiliária's CEO entry with her full name and LinkedIn.

161 companies total; phones with a confirmed PT number go from 69 to 80.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01SRBJwGmSsYkTHKJbGCM5ca
</commit_message>
<xml_diff>
--- a/Promotoras_Imobiliarias_Contactos.xlsx
+++ b/Promotoras_Imobiliarias_Contactos.xlsx
@@ -644,7 +644,7 @@
     <row r="3" ht="30" customHeight="1">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>ALMA Development</t>
+          <t>AFA (Grupo AFA)</t>
         </is>
       </c>
       <c r="B3" s="3" t="inlineStr">
@@ -654,17 +654,17 @@
       </c>
       <c r="C3" s="4" t="inlineStr">
         <is>
-          <t>+351 218 019 249</t>
+          <t>+351 218 981 190</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>geral@almadevelopment.pt</t>
+          <t>anaborges@afa.pt</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>almadevelopment.pt</t>
+          <t>afa-realestate.com</t>
         </is>
       </c>
       <c r="F3" s="4" t="inlineStr">
@@ -679,35 +679,31 @@
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t>Torre Duarte Pacheco, 1070-101</t>
+          <t>Av. D. João II, nº25, 2º, 1990-079</t>
         </is>
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>Caxias Heights (Oeiras) (Comercialização) | 3 projetos Grande Porto/Lisboa (Em construção)</t>
+          <t>Savoy Residence D'Ávila (Em construção)</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>Fundada 2022, ligada à Panhard. Tel. móvel 914 192 506</t>
+          <t>Fonte: diarioimobiliario.pt</t>
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr">
         <is>
-          <t>Carlos Morgado (Diretor Executivo)</t>
-        </is>
-      </c>
-      <c r="L3" s="2" t="inlineStr">
-        <is>
-          <t>https://www.linkedin.com/in/cafmorgado/</t>
-        </is>
-      </c>
+          <t>Victor de Sousa (Diretor-Geral AFA Real Estate)</t>
+        </is>
+      </c>
+      <c r="L3" s="2" t="inlineStr"/>
       <c r="M3" s="2" t="inlineStr"/>
     </row>
     <row r="4" ht="30" customHeight="1">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>AM48</t>
+          <t>ALMA Development</t>
         </is>
       </c>
       <c r="B4" s="3" t="inlineStr">
@@ -717,17 +713,17 @@
       </c>
       <c r="C4" s="4" t="inlineStr">
         <is>
-          <t>+351 910 713 848</t>
+          <t>+351 218 019 249</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>quintadoalverde@am48.pt</t>
+          <t>geral@almadevelopment.pt</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>am48.pt</t>
+          <t>almadevelopment.pt</t>
         </is>
       </c>
       <c r="F4" s="4" t="inlineStr">
@@ -742,27 +738,27 @@
       </c>
       <c r="H4" s="2" t="inlineStr">
         <is>
-          <t>Lisboa (sede) · Aveiro</t>
+          <t>Torre Duarte Pacheco, 1070-101</t>
         </is>
       </c>
       <c r="I4" s="2" t="inlineStr">
         <is>
-          <t>Quinta do Alverde (Oeiras) (Comercialização) | Foz de Prata + Ceramium (Aveiro) (Em construção) | Ópera LX / Focus LX / Promenade (Lisboa) (Concluído)</t>
+          <t>Caxias Heights (Oeiras) (Comercialização) | 3 projetos Grande Porto/Lisboa (Em construção)</t>
         </is>
       </c>
       <c r="J4" s="2" t="inlineStr">
         <is>
-          <t>Telefone é da linha comercial Quinta do Alverde</t>
+          <t>Fundada 2022, ligada à Panhard. Tel. móvel 914 192 506</t>
         </is>
       </c>
       <c r="K4" s="2" t="inlineStr">
         <is>
-          <t>Alejandro Martins (Founder &amp; CEO)</t>
+          <t>Carlos Morgado (Diretor Executivo)</t>
         </is>
       </c>
       <c r="L4" s="2" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/in/alejandro-martins-74b18590/</t>
+          <t>https://www.linkedin.com/in/cafmorgado/</t>
         </is>
       </c>
       <c r="M4" s="2" t="inlineStr"/>
@@ -770,7 +766,7 @@
     <row r="5" ht="30" customHeight="1">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>AVENUE</t>
+          <t>AM48</t>
         </is>
       </c>
       <c r="B5" s="3" t="inlineStr">
@@ -780,17 +776,17 @@
       </c>
       <c r="C5" s="4" t="inlineStr">
         <is>
-          <t>+351 215 989 523</t>
+          <t>+351 910 713 848</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>geral@avenue.pt</t>
+          <t>quintadoalverde@am48.pt</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>avenue.pt</t>
+          <t>am48.pt</t>
         </is>
       </c>
       <c r="F5" s="4" t="inlineStr">
@@ -805,27 +801,27 @@
       </c>
       <c r="H5" s="2" t="inlineStr">
         <is>
-          <t>Rua Serpa Pinto 14A, 3º, 1200-445 (Porto: Av. Boavista 772, +351 220 990 530)</t>
+          <t>Lisboa (sede) · Aveiro</t>
         </is>
       </c>
       <c r="I5" s="2" t="inlineStr">
         <is>
-          <t>Nolipa (Campo Grande) (Em construção) | Bonjardim (Porto) (Concluído)</t>
+          <t>Quinta do Alverde (Oeiras) (Comercialização) | Foz de Prata + Ceramium (Aveiro) (Em construção) | Ópera LX / Focus LX / Promenade (Lisboa) (Concluído)</t>
         </is>
       </c>
       <c r="J5" s="2" t="inlineStr">
         <is>
-          <t>Promotor de referência Lisboa/Porto</t>
+          <t>Telefone é da linha comercial Quinta do Alverde</t>
         </is>
       </c>
       <c r="K5" s="2" t="inlineStr">
         <is>
-          <t>Aniceto Viegas (CEO)</t>
+          <t>Alejandro Martins (Founder &amp; CEO)</t>
         </is>
       </c>
       <c r="L5" s="2" t="inlineStr">
         <is>
-          <t>https://pt.linkedin.com/in/aniceto-viegas-02586a1</t>
+          <t>https://www.linkedin.com/in/alejandro-martins-74b18590/</t>
         </is>
       </c>
       <c r="M5" s="2" t="inlineStr"/>
@@ -833,7 +829,7 @@
     <row r="6" ht="30" customHeight="1">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>Benoit Properties International</t>
+          <t>Arts Investments, SA</t>
         </is>
       </c>
       <c r="B6" s="3" t="inlineStr">
@@ -843,13 +839,13 @@
       </c>
       <c r="C6" s="4" t="inlineStr">
         <is>
-          <t>+44 161 250 5300 (UK)</t>
+          <t>+351 291 281 182</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr"/>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>benoitproperties.com</t>
+          <t>artsinvestments.com</t>
         </is>
       </c>
       <c r="F6" s="4" t="inlineStr">
@@ -864,31 +860,27 @@
       </c>
       <c r="H6" s="2" t="inlineStr">
         <is>
-          <t>Rua Tierno Galvan, Amoreiras Torre 3, piso 6, sala 612, 1070-274</t>
+          <t>Av. Eng. Duarte Pacheco, Amoreiras Torre 2, 10º, sala 10, 1070-101</t>
         </is>
       </c>
       <c r="I6" s="2" t="inlineStr">
         <is>
-          <t>114 Avenida Central (Braga) (Comercialização) | Alexandre Braga 10 (Lisboa) (Em construção)</t>
+          <t>3 projetos em curso (nomes não encontrados) (Em construção/desenvolvimento)</t>
         </is>
       </c>
       <c r="J6" s="2" t="inlineStr">
         <is>
-          <t>Só telefone UK publicado</t>
-        </is>
-      </c>
-      <c r="K6" s="2" t="inlineStr">
-        <is>
-          <t>Fredrick J. Benoit II (Director/co-fundador, 50% com Matthew Lavin)</t>
-        </is>
-      </c>
+          <t>Fonte: vidaimobiliaria.com. Nota: nº de telefone tem indicativo da Madeira (291) — confirmar antes de ligar</t>
+        </is>
+      </c>
+      <c r="K6" s="2" t="inlineStr"/>
       <c r="L6" s="2" t="inlineStr"/>
       <c r="M6" s="2" t="inlineStr"/>
     </row>
     <row r="7" ht="30" customHeight="1">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>BESIX RED Portugal</t>
+          <t>AVENUE</t>
         </is>
       </c>
       <c r="B7" s="3" t="inlineStr">
@@ -898,17 +890,17 @@
       </c>
       <c r="C7" s="4" t="inlineStr">
         <is>
-          <t>+351 216 037 894</t>
+          <t>+351 215 989 523</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>info@besixred.com</t>
+          <t>geral@avenue.pt</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>besixred.com</t>
+          <t>avenue.pt</t>
         </is>
       </c>
       <c r="F7" s="4" t="inlineStr">
@@ -923,27 +915,27 @@
       </c>
       <c r="H7" s="2" t="inlineStr">
         <is>
-          <t>Av. Duque de Loulé 106, 9º, 1050-093</t>
+          <t>Rua Serpa Pinto 14A, 3º, 1200-445 (Porto: Av. Boavista 772, +351 220 990 530)</t>
         </is>
       </c>
       <c r="I7" s="2" t="inlineStr">
         <is>
-          <t>DUUO (Praça de Espanha) (Em construção) | Parque Oriente (Parque das Nações) (Em construção) | WellBe (Em construção)</t>
+          <t>Nolipa (Campo Grande) (Em construção) | Bonjardim (Porto) (Concluído)</t>
         </is>
       </c>
       <c r="J7" s="2" t="inlineStr">
         <is>
-          <t>Promotor pan-europeu (grupo BESIX)</t>
+          <t>Promotor de referência Lisboa/Porto</t>
         </is>
       </c>
       <c r="K7" s="2" t="inlineStr">
         <is>
-          <t>Nicolas Goffin (Country Director Portugal· CEO do grupo é Gabriel Uzgen, Bruxelas)</t>
+          <t>Aniceto Viegas (CEO)</t>
         </is>
       </c>
       <c r="L7" s="2" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/in/nicolas-goffin-32707487/</t>
+          <t>https://pt.linkedin.com/in/aniceto-viegas-02586a1</t>
         </is>
       </c>
       <c r="M7" s="2" t="inlineStr"/>
@@ -951,7 +943,7 @@
     <row r="8" ht="30" customHeight="1">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>Blue Buffalo Capital</t>
+          <t>Benoit Properties International</t>
         </is>
       </c>
       <c r="B8" s="3" t="inlineStr">
@@ -961,22 +953,18 @@
       </c>
       <c r="C8" s="4" t="inlineStr">
         <is>
-          <t>+351 934 643 306</t>
-        </is>
-      </c>
-      <c r="D8" s="2" t="inlineStr">
-        <is>
-          <t>geral@bluebuffalocapital.com</t>
-        </is>
-      </c>
+          <t>+44 161 250 5300 (UK)</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr"/>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>bluebuffalocapital.com</t>
+          <t>benoitproperties.com</t>
         </is>
       </c>
       <c r="F8" s="4" t="inlineStr">
         <is>
-          <t>Cascais</t>
+          <t>Lisboa</t>
         </is>
       </c>
       <c r="G8" s="4" t="inlineStr">
@@ -986,35 +974,31 @@
       </c>
       <c r="H8" s="2" t="inlineStr">
         <is>
-          <t>Rua de São Tomé e Príncipe 23 B, 2765-282 Estoril</t>
+          <t>Rua Tierno Galvan, Amoreiras Torre 3, piso 6, sala 612, 1070-274</t>
         </is>
       </c>
       <c r="I8" s="2" t="inlineStr">
         <is>
-          <t>Residencial de luxo Grande Lisboa (Em construção)</t>
+          <t>114 Avenida Central (Braga) (Comercialização) | Alexandre Braga 10 (Lisboa) (Em construção)</t>
         </is>
       </c>
       <c r="J8" s="2" t="inlineStr">
         <is>
-          <t>Desde 2015, sócios com &gt;500M€ promovidos</t>
+          <t>Só telefone UK publicado</t>
         </is>
       </c>
       <c r="K8" s="2" t="inlineStr">
         <is>
-          <t>Celma de Almeida Lavradio (Co-Founder &amp; CEO)</t>
-        </is>
-      </c>
-      <c r="L8" s="2" t="inlineStr">
-        <is>
-          <t>https://pt.linkedin.com/in/celma-de-almeida-lavradio-645baa43</t>
-        </is>
-      </c>
+          <t>Fredrick J. Benoit II (Director/co-fundador, 50% com Matthew Lavin)</t>
+        </is>
+      </c>
+      <c r="L8" s="2" t="inlineStr"/>
       <c r="M8" s="2" t="inlineStr"/>
     </row>
     <row r="9" ht="30" customHeight="1">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>Bondstone</t>
+          <t>BESIX RED Portugal</t>
         </is>
       </c>
       <c r="B9" s="3" t="inlineStr">
@@ -1024,13 +1008,17 @@
       </c>
       <c r="C9" s="4" t="inlineStr">
         <is>
-          <t>+351 211 349 157</t>
-        </is>
-      </c>
-      <c r="D9" s="2" t="inlineStr"/>
+          <t>+351 216 037 894</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>info@besixred.com</t>
+        </is>
+      </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>bondstone.com</t>
+          <t>besixred.com</t>
         </is>
       </c>
       <c r="F9" s="4" t="inlineStr">
@@ -1045,27 +1033,27 @@
       </c>
       <c r="H9" s="2" t="inlineStr">
         <is>
-          <t>Rua Castilho 39, 10º C, 1250-068</t>
+          <t>Av. Duque de Loulé 106, 9º, 1050-093</t>
         </is>
       </c>
       <c r="I9" s="2" t="inlineStr">
         <is>
-          <t>The Coral (Cascais) (Em construção)</t>
+          <t>DUUO (Praça de Espanha) (Em construção) | Parque Oriente (Parque das Nações) (Em construção) | WellBe (Em construção)</t>
         </is>
       </c>
       <c r="J9" s="2" t="inlineStr">
         <is>
-          <t>Gestora regulada CMVM, capital internacional</t>
+          <t>Promotor pan-europeu (grupo BESIX)</t>
         </is>
       </c>
       <c r="K9" s="2" t="inlineStr">
         <is>
-          <t>Paulo Loureiro (fundador e CEO)</t>
+          <t>Nicolas Goffin (Country Director Portugal· CEO do grupo é Gabriel Uzgen, Bruxelas)</t>
         </is>
       </c>
       <c r="L9" s="2" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/in/paulo-loureiro-8a46016/</t>
+          <t>https://www.linkedin.com/in/nicolas-goffin-32707487/</t>
         </is>
       </c>
       <c r="M9" s="2" t="inlineStr"/>
@@ -1073,7 +1061,7 @@
     <row r="10" ht="30" customHeight="1">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>Coporgest</t>
+          <t>Blue Buffalo Capital</t>
         </is>
       </c>
       <c r="B10" s="3" t="inlineStr">
@@ -1083,22 +1071,22 @@
       </c>
       <c r="C10" s="4" t="inlineStr">
         <is>
-          <t>+351 213 108 900</t>
+          <t>+351 934 643 306</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>geral@coporgest.com</t>
+          <t>geral@bluebuffalocapital.com</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>coporgest.com</t>
+          <t>bluebuffalocapital.com</t>
         </is>
       </c>
       <c r="F10" s="4" t="inlineStr">
         <is>
-          <t>Lisboa</t>
+          <t>Cascais</t>
         </is>
       </c>
       <c r="G10" s="4" t="inlineStr">
@@ -1108,31 +1096,35 @@
       </c>
       <c r="H10" s="2" t="inlineStr">
         <is>
-          <t>Av. da Liberdade 245, 9º C, 1250-143</t>
+          <t>Rua de São Tomé e Príncipe 23 B, 2765-282 Estoril</t>
         </is>
       </c>
       <c r="I10" s="2" t="inlineStr">
         <is>
-          <t>Comporta Beach Resort (Em construção)</t>
+          <t>Residencial de luxo Grande Lisboa (Em construção)</t>
         </is>
       </c>
       <c r="J10" s="2" t="inlineStr">
         <is>
-          <t>Promotor de Lisboa desde 2004</t>
+          <t>Desde 2015, sócios com &gt;500M€ promovidos</t>
         </is>
       </c>
       <c r="K10" s="2" t="inlineStr">
         <is>
-          <t>Sérgio Ferreira (fundador e CEO, homónimos sem confirmação total)</t>
-        </is>
-      </c>
-      <c r="L10" s="2" t="inlineStr"/>
+          <t>Celma de Almeida Lavradio (Co-Founder &amp; CEO)</t>
+        </is>
+      </c>
+      <c r="L10" s="2" t="inlineStr">
+        <is>
+          <t>https://pt.linkedin.com/in/celma-de-almeida-lavradio-645baa43</t>
+        </is>
+      </c>
       <c r="M10" s="2" t="inlineStr"/>
     </row>
     <row r="11" ht="30" customHeight="1">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>EastBanc Portugal</t>
+          <t>Bondstone</t>
         </is>
       </c>
       <c r="B11" s="3" t="inlineStr">
@@ -1142,17 +1134,13 @@
       </c>
       <c r="C11" s="4" t="inlineStr">
         <is>
-          <t>+351 213 404 150</t>
-        </is>
-      </c>
-      <c r="D11" s="2" t="inlineStr">
-        <is>
-          <t>geral@eastbanc.com</t>
-        </is>
-      </c>
+          <t>+351 211 349 157</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr"/>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>eastbanc.pt</t>
+          <t>bondstone.com</t>
         </is>
       </c>
       <c r="F11" s="4" t="inlineStr">
@@ -1167,31 +1155,35 @@
       </c>
       <c r="H11" s="2" t="inlineStr">
         <is>
-          <t>Rua da Escola Politécnica 38, 2º, 1250-102</t>
+          <t>Rua Castilho 39, 10º C, 1250-068</t>
         </is>
       </c>
       <c r="I11" s="2" t="inlineStr">
         <is>
-          <t>8 projetos Príncipe Real (Em construção) | DPV Block (Comercialização) | EmbaiXada (Concluído)</t>
+          <t>The Coral (Cascais) (Em construção)</t>
         </is>
       </c>
       <c r="J11" s="2" t="inlineStr">
         <is>
-          <t>20 anos em Príncipe Real, &gt;20 edifícios</t>
+          <t>Gestora regulada CMVM, capital internacional</t>
         </is>
       </c>
       <c r="K11" s="2" t="inlineStr">
         <is>
-          <t>Tiago Eiró (CEO)</t>
-        </is>
-      </c>
-      <c r="L11" s="2" t="inlineStr"/>
+          <t>Paulo Loureiro (fundador e CEO)</t>
+        </is>
+      </c>
+      <c r="L11" s="2" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/paulo-loureiro-8a46016/</t>
+        </is>
+      </c>
       <c r="M11" s="2" t="inlineStr"/>
     </row>
     <row r="12" ht="30" customHeight="1">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>Easyliving</t>
+          <t>Ceetrus / Nhood Portugal</t>
         </is>
       </c>
       <c r="B12" s="3" t="inlineStr">
@@ -1201,38 +1193,42 @@
       </c>
       <c r="C12" s="4" t="inlineStr">
         <is>
-          <t>+351 961 866 297</t>
+          <t>+351 210 537 815</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>info@easyliving.pt</t>
+          <t>news@nhood.pt</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>easyliving.pt</t>
+          <t>nhood.pt</t>
         </is>
       </c>
       <c r="F12" s="4" t="inlineStr">
         <is>
-          <t>Porto</t>
+          <t>Lisboa</t>
         </is>
       </c>
       <c r="G12" s="4" t="inlineStr">
         <is>
-          <t>Porto</t>
-        </is>
-      </c>
-      <c r="H12" s="2" t="inlineStr"/>
+          <t>nacional</t>
+        </is>
+      </c>
+      <c r="H12" s="2" t="inlineStr">
+        <is>
+          <t>Rua Artilharia 1, nº51, Páteo Bagatela, Ed. 3, 1250-038</t>
+        </is>
+      </c>
       <c r="I12" s="2" t="inlineStr">
         <is>
-          <t>Boavista Garden (Av. da Boavista) (Em construção) | Aspreladas Easy (Comercialização)</t>
+          <t>Pipeline nacional 15 cidades (nomes não encontrados) (Planeamento)</t>
         </is>
       </c>
       <c r="J12" s="2" t="inlineStr">
         <is>
-          <t>Compra, reabilitação e construção. Comercialização via RE/MAX Collection</t>
+          <t>Fonte: idealista.pt</t>
         </is>
       </c>
       <c r="K12" s="2" t="inlineStr"/>
@@ -1242,7 +1238,7 @@
     <row r="13" ht="30" customHeight="1">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>EMERGE – Mota-Engil Real Estate</t>
+          <t>Coporgest</t>
         </is>
       </c>
       <c r="B13" s="3" t="inlineStr">
@@ -1252,60 +1248,56 @@
       </c>
       <c r="C13" s="4" t="inlineStr">
         <is>
-          <t>+351 225 190 362</t>
+          <t>+351 213 108 900</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>emerge@mota-engil.pt</t>
+          <t>geral@coporgest.com</t>
         </is>
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>emerge-realestate.pt</t>
+          <t>coporgest.com</t>
         </is>
       </c>
       <c r="F13" s="4" t="inlineStr">
         <is>
-          <t>Porto</t>
+          <t>Lisboa</t>
         </is>
       </c>
       <c r="G13" s="4" t="inlineStr">
         <is>
-          <t>Porto</t>
+          <t>Lisboa</t>
         </is>
       </c>
       <c r="H13" s="2" t="inlineStr">
         <is>
-          <t>Calçada do Rêgo Lameiro 38, 4300-454</t>
+          <t>Av. da Liberdade 245, 9º C, 1250-143</t>
         </is>
       </c>
       <c r="I13" s="2" t="inlineStr">
         <is>
-          <t>OPO-City (Porto/Matosinhos) (Comercialização) | AURIOS (Comercialização)</t>
+          <t>Comporta Beach Resort (Em construção)</t>
         </is>
       </c>
       <c r="J13" s="2" t="inlineStr">
         <is>
-          <t>Promotora do grupo Mota-Engil</t>
+          <t>Promotor de Lisboa desde 2004</t>
         </is>
       </c>
       <c r="K13" s="2" t="inlineStr">
         <is>
-          <t>Vitor Paulo Pinho (CEO)</t>
-        </is>
-      </c>
-      <c r="L13" s="2" t="inlineStr">
-        <is>
-          <t>https://www.linkedin.com/in/vitor-paulo-pinho-0a7952173/</t>
-        </is>
-      </c>
+          <t>Sérgio Ferreira (fundador e CEO, homónimos sem confirmação total)</t>
+        </is>
+      </c>
+      <c r="L13" s="2" t="inlineStr"/>
       <c r="M13" s="2" t="inlineStr"/>
     </row>
     <row r="14" ht="30" customHeight="1">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>Fercopor</t>
+          <t>EastBanc Portugal</t>
         </is>
       </c>
       <c r="B14" s="3" t="inlineStr">
@@ -1315,43 +1307,47 @@
       </c>
       <c r="C14" s="4" t="inlineStr">
         <is>
-          <t>+351 226 091 113</t>
-        </is>
-      </c>
-      <c r="D14" s="2" t="inlineStr"/>
+          <t>+351 213 404 150</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>geral@eastbanc.com</t>
+        </is>
+      </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>fercopor.pt</t>
+          <t>eastbanc.pt</t>
         </is>
       </c>
       <c r="F14" s="4" t="inlineStr">
         <is>
-          <t>Porto</t>
+          <t>Lisboa</t>
         </is>
       </c>
       <c r="G14" s="4" t="inlineStr">
         <is>
-          <t>Porto</t>
+          <t>Lisboa</t>
         </is>
       </c>
       <c r="H14" s="2" t="inlineStr">
         <is>
-          <t>Av. da França 20, Sala 509, 4050-275</t>
+          <t>Rua da Escola Politécnica 38, 2º, 1250-102</t>
         </is>
       </c>
       <c r="I14" s="2" t="inlineStr">
         <is>
-          <t>Boavista (2 projetos) (Planeamento) | Vila do Conde (Planeamento)</t>
+          <t>8 projetos Príncipe Real (Em construção) | DPV Block (Comercialização) | EmbaiXada (Concluído)</t>
         </is>
       </c>
       <c r="J14" s="2" t="inlineStr">
         <is>
-          <t>Luxo desde 1981. Fonte: reportugal.vidaimobiliaria.com</t>
+          <t>20 anos em Príncipe Real, &gt;20 edifícios</t>
         </is>
       </c>
       <c r="K14" s="2" t="inlineStr">
         <is>
-          <t>Mário Almeida (Administrador)</t>
+          <t>Tiago Eiró (CEO)</t>
         </is>
       </c>
       <c r="L14" s="2" t="inlineStr"/>
@@ -1360,7 +1356,7 @@
     <row r="15" ht="30" customHeight="1">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>Fidelidade Property</t>
+          <t>Easyliving</t>
         </is>
       </c>
       <c r="B15" s="3" t="inlineStr">
@@ -1370,42 +1366,38 @@
       </c>
       <c r="C15" s="4" t="inlineStr">
         <is>
-          <t>+351 217 807 772</t>
+          <t>+351 961 866 297</t>
         </is>
       </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
-          <t>geral@fidelidadeproperty.pt</t>
+          <t>info@easyliving.pt</t>
         </is>
       </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
-          <t>fidelidadeproperty.pt</t>
+          <t>easyliving.pt</t>
         </is>
       </c>
       <c r="F15" s="4" t="inlineStr">
         <is>
-          <t>Lisboa</t>
+          <t>Porto</t>
         </is>
       </c>
       <c r="G15" s="4" t="inlineStr">
         <is>
-          <t>Lisboa</t>
-        </is>
-      </c>
-      <c r="H15" s="2" t="inlineStr">
-        <is>
-          <t>Largo do Calhariz 30, 1249-001</t>
-        </is>
-      </c>
+          <t>Porto</t>
+        </is>
+      </c>
+      <c r="H15" s="2" t="inlineStr"/>
       <c r="I15" s="2" t="inlineStr">
         <is>
-          <t>EntreCampos (antiga Feira Popular) (Em construção)</t>
+          <t>Boavista Garden (Av. da Boavista) (Em construção) | Aspreladas Easy (Comercialização)</t>
         </is>
       </c>
       <c r="J15" s="2" t="inlineStr">
         <is>
-          <t>Braço imobiliário da Fidelidade. Projeto: info@entrecampos.pt</t>
+          <t>Compra, reabilitação e construção. Comercialização via RE/MAX Collection</t>
         </is>
       </c>
       <c r="K15" s="2" t="inlineStr"/>
@@ -1415,7 +1407,7 @@
     <row r="16" ht="30" customHeight="1">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>FIDES – Investimentos e Gestão Imobiliária</t>
+          <t>EMERGE – Mota-Engil Real Estate</t>
         </is>
       </c>
       <c r="B16" s="3" t="inlineStr">
@@ -1425,48 +1417,60 @@
       </c>
       <c r="C16" s="4" t="inlineStr">
         <is>
-          <t>+351 213 877 749</t>
+          <t>+351 225 190 362</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>diogopintogoncalves@imofides.com</t>
-        </is>
-      </c>
-      <c r="E16" s="2" t="inlineStr"/>
+          <t>emerge@mota-engil.pt</t>
+        </is>
+      </c>
+      <c r="E16" s="2" t="inlineStr">
+        <is>
+          <t>emerge-realestate.pt</t>
+        </is>
+      </c>
       <c r="F16" s="4" t="inlineStr">
         <is>
-          <t>Lisboa</t>
+          <t>Porto</t>
         </is>
       </c>
       <c r="G16" s="4" t="inlineStr">
         <is>
-          <t>Lisboa</t>
+          <t>Porto</t>
         </is>
       </c>
       <c r="H16" s="2" t="inlineStr">
         <is>
-          <t>Rua Tierno Galvan, Amoreiras Torre 3, 6º, sala 607, 1070-274</t>
+          <t>Calçada do Rêgo Lameiro 38, 4300-454</t>
         </is>
       </c>
       <c r="I16" s="2" t="inlineStr">
         <is>
-          <t>Promoção residencial (Em construção)</t>
+          <t>OPO-City (Porto/Matosinhos) (Comercialização) | AURIOS (Comercialização)</t>
         </is>
       </c>
       <c r="J16" s="2" t="inlineStr">
         <is>
-          <t>Projeto concreto não nomeado nas fontes</t>
-        </is>
-      </c>
-      <c r="K16" s="2" t="inlineStr"/>
-      <c r="L16" s="2" t="inlineStr"/>
+          <t>Promotora do grupo Mota-Engil</t>
+        </is>
+      </c>
+      <c r="K16" s="2" t="inlineStr">
+        <is>
+          <t>Vitor Paulo Pinho (CEO)</t>
+        </is>
+      </c>
+      <c r="L16" s="2" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/vitor-paulo-pinho-0a7952173/</t>
+        </is>
+      </c>
       <c r="M16" s="2" t="inlineStr"/>
     </row>
     <row r="17" ht="30" customHeight="1">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>Grupo Madre / Madre Imobiliário</t>
+          <t>Fercopor</t>
         </is>
       </c>
       <c r="B17" s="3" t="inlineStr">
@@ -1476,47 +1480,43 @@
       </c>
       <c r="C17" s="4" t="inlineStr">
         <is>
-          <t>+351 213 243 220</t>
-        </is>
-      </c>
-      <c r="D17" s="2" t="inlineStr">
-        <is>
-          <t>geral@madreimobiliario.com</t>
-        </is>
-      </c>
+          <t>+351 226 091 113</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="inlineStr"/>
       <c r="E17" s="2" t="inlineStr">
         <is>
-          <t>madreimobiliario.com</t>
+          <t>fercopor.pt</t>
         </is>
       </c>
       <c r="F17" s="4" t="inlineStr">
         <is>
-          <t>Lisboa</t>
+          <t>Porto</t>
         </is>
       </c>
       <c r="G17" s="4" t="inlineStr">
         <is>
-          <t>Lisboa</t>
+          <t>Porto</t>
         </is>
       </c>
       <c r="H17" s="2" t="inlineStr">
         <is>
-          <t>Campo Grande 28, 11º, 1700-093</t>
+          <t>Av. da França 20, Sala 509, 4050-275</t>
         </is>
       </c>
       <c r="I17" s="2" t="inlineStr">
         <is>
-          <t>A-Living (Areeiro) (Planeamento) | Parque da Cidade (Setúbal) (Em construção)</t>
+          <t>Boavista (2 projetos) (Planeamento) | Vila do Conde (Planeamento)</t>
         </is>
       </c>
       <c r="J17" s="2" t="inlineStr">
         <is>
-          <t>Presidente António Parente. Tel. móvel 914 070 350</t>
+          <t>Luxo desde 1981. Fonte: reportugal.vidaimobiliaria.com</t>
         </is>
       </c>
       <c r="K17" s="2" t="inlineStr">
         <is>
-          <t>Nuno Dias (Diretor Geral da Madre Imobiliário· presidente do grupo é António Parente)</t>
+          <t>Mário Almeida (Administrador)</t>
         </is>
       </c>
       <c r="L17" s="2" t="inlineStr"/>
@@ -1525,7 +1525,7 @@
     <row r="18" ht="30" customHeight="1">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>Habitat Invest</t>
+          <t>Fidelidade Property</t>
         </is>
       </c>
       <c r="B18" s="3" t="inlineStr">
@@ -1535,17 +1535,17 @@
       </c>
       <c r="C18" s="4" t="inlineStr">
         <is>
-          <t>+351 213 461 024</t>
+          <t>+351 217 807 772</t>
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
-          <t>info@habitatinvest.pt</t>
+          <t>geral@fidelidadeproperty.pt</t>
         </is>
       </c>
       <c r="E18" s="2" t="inlineStr">
         <is>
-          <t>habitatinvest.pt</t>
+          <t>fidelidadeproperty.pt</t>
         </is>
       </c>
       <c r="F18" s="4" t="inlineStr">
@@ -1560,31 +1560,27 @@
       </c>
       <c r="H18" s="2" t="inlineStr">
         <is>
-          <t>Rua da Moeda 4, 1200-275</t>
+          <t>Largo do Calhariz 30, 1249-001</t>
         </is>
       </c>
       <c r="I18" s="2" t="inlineStr">
         <is>
-          <t>15 projetos em desenvolvimento (Em construção) | ALMAR SOUTH LIVING (Almada) (Em construção/comercialização) | AURYA (Santo António dos Cavaleiros, Loures) (Em construção)</t>
+          <t>EntreCampos (antiga Feira Popular) (Em construção)</t>
         </is>
       </c>
       <c r="J18" s="2" t="inlineStr">
         <is>
-          <t>Fundada 2001 · inclui Habitat Ventures/Project/Property/Broker</t>
-        </is>
-      </c>
-      <c r="K18" s="2" t="inlineStr">
-        <is>
-          <t>Luís Corrêa de Barros (fundador e CEO)</t>
-        </is>
-      </c>
+          <t>Braço imobiliário da Fidelidade. Projeto: info@entrecampos.pt</t>
+        </is>
+      </c>
+      <c r="K18" s="2" t="inlineStr"/>
       <c r="L18" s="2" t="inlineStr"/>
       <c r="M18" s="2" t="inlineStr"/>
     </row>
     <row r="19" ht="30" customHeight="1">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>J. Dias &amp; Dias</t>
+          <t>FIDES – Investimentos e Gestão Imobiliária</t>
         </is>
       </c>
       <c r="B19" s="3" t="inlineStr">
@@ -1594,22 +1590,18 @@
       </c>
       <c r="C19" s="4" t="inlineStr">
         <is>
-          <t>+351 214 422 593</t>
+          <t>+351 213 877 749</t>
         </is>
       </c>
       <c r="D19" s="2" t="inlineStr">
         <is>
-          <t>geral@jdiasdias.pt</t>
-        </is>
-      </c>
-      <c r="E19" s="2" t="inlineStr">
-        <is>
-          <t>jdiasdias.pt</t>
-        </is>
-      </c>
+          <t>diogopintogoncalves@imofides.com</t>
+        </is>
+      </c>
+      <c r="E19" s="2" t="inlineStr"/>
       <c r="F19" s="4" t="inlineStr">
         <is>
-          <t>Cascais</t>
+          <t>Lisboa</t>
         </is>
       </c>
       <c r="G19" s="4" t="inlineStr">
@@ -1619,17 +1611,17 @@
       </c>
       <c r="H19" s="2" t="inlineStr">
         <is>
-          <t>Av. Venceslau Balseiro da Grande Guerra, Quinta das Marianas, Parede</t>
+          <t>Rua Tierno Galvan, Amoreiras Torre 3, 6º, sala 607, 1070-274</t>
         </is>
       </c>
       <c r="I19" s="2" t="inlineStr">
         <is>
-          <t>Urban Living (Carcavelos/Parede) (Comercialização)</t>
+          <t>Promoção residencial (Em construção)</t>
         </is>
       </c>
       <c r="J19" s="2" t="inlineStr">
         <is>
-          <t>Fundada 1960, alvará ICC 12463. Tel. móvel 961 682 789</t>
+          <t>Projeto concreto não nomeado nas fontes</t>
         </is>
       </c>
       <c r="K19" s="2" t="inlineStr"/>
@@ -1639,7 +1631,7 @@
     <row r="20" ht="30" customHeight="1">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>JPS Group</t>
+          <t>Fortera</t>
         </is>
       </c>
       <c r="B20" s="3" t="inlineStr">
@@ -1649,60 +1641,56 @@
       </c>
       <c r="C20" s="4" t="inlineStr">
         <is>
-          <t>+351 218 371 025</t>
+          <t>+351 220 110 929</t>
         </is>
       </c>
       <c r="D20" s="2" t="inlineStr">
         <is>
-          <t>secretariado@jpsgroup.pt</t>
+          <t>info@fortera.pt</t>
         </is>
       </c>
       <c r="E20" s="2" t="inlineStr">
         <is>
-          <t>jpsgroup.pt</t>
+          <t>fortera.pt</t>
         </is>
       </c>
       <c r="F20" s="4" t="inlineStr">
         <is>
-          <t>Lisboa</t>
+          <t>Vila Nova de Gaia</t>
         </is>
       </c>
       <c r="G20" s="4" t="inlineStr">
         <is>
-          <t>Lisboa</t>
+          <t>Porto</t>
         </is>
       </c>
       <c r="H20" s="2" t="inlineStr">
         <is>
-          <t>Av. Almirante Gago Coutinho 126</t>
+          <t>Rua de Rei Ramiro 870, 5º A, 4400-281</t>
         </is>
       </c>
       <c r="I20" s="2" t="inlineStr">
         <is>
-          <t>SkyCity (Carnaxide) (Em construção) | Herdade Real de Santiago (Comercialização) | Terraços de São Francisco (Comercialização)</t>
+          <t>Skyline (V.N. Gaia) (Em construção) | 20 projetos (Porto, Gaia, Espinho, Braga) (Em construção) | Convento do Carmo (Braga) (Em construção)</t>
         </is>
       </c>
       <c r="J20" s="2" t="inlineStr">
         <is>
-          <t>Promotora com construtora e imobiliária próprias</t>
+          <t>Fundadores Elad Dror e Nir Shalom. Nota: Elad Dror foi detido na Operação Babel (2023, corrupção) — confirmar situação atual antes de contacto</t>
         </is>
       </c>
       <c r="K20" s="2" t="inlineStr">
         <is>
-          <t>João Sousa (CEO)</t>
-        </is>
-      </c>
-      <c r="L20" s="2" t="inlineStr">
-        <is>
-          <t>https://pt.linkedin.com/in/joao-sousa-7802352a</t>
-        </is>
-      </c>
+          <t>Pedro Ferreira (CEO desde jun/2023· fundador anterior Elad Dror saiu em 2023)</t>
+        </is>
+      </c>
+      <c r="L20" s="2" t="inlineStr"/>
       <c r="M20" s="2" t="inlineStr"/>
     </row>
     <row r="21" ht="30" customHeight="1">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>Krest Investments</t>
+          <t>Grupo Madre / Madre Imobiliário</t>
         </is>
       </c>
       <c r="B21" s="3" t="inlineStr">
@@ -1712,17 +1700,17 @@
       </c>
       <c r="C21" s="4" t="inlineStr">
         <is>
-          <t>+351 215 873 920</t>
+          <t>+351 213 243 220</t>
         </is>
       </c>
       <c r="D21" s="2" t="inlineStr">
         <is>
-          <t>info@krestinvestments.com</t>
+          <t>geral@madreimobiliario.com</t>
         </is>
       </c>
       <c r="E21" s="2" t="inlineStr">
         <is>
-          <t>krestinvestments.com</t>
+          <t>madreimobiliario.com</t>
         </is>
       </c>
       <c r="F21" s="4" t="inlineStr">
@@ -1737,35 +1725,31 @@
       </c>
       <c r="H21" s="2" t="inlineStr">
         <is>
-          <t>Av. Eng.º Duarte Pacheco, Amoreiras Torre 1, piso 14, sala 2, 1070-101</t>
+          <t>Campo Grande 28, 11º, 1700-093</t>
         </is>
       </c>
       <c r="I21" s="2" t="inlineStr">
         <is>
-          <t>Lisboa / Porto / Algarve (Comercialização)</t>
+          <t>A-Living (Areeiro) (Planeamento) | Parque da Cidade (Setúbal) (Em construção)</t>
         </is>
       </c>
       <c r="J21" s="2" t="inlineStr">
         <is>
-          <t>Belga, em Portugal desde 2014</t>
+          <t>Presidente António Parente. Tel. móvel 914 070 350</t>
         </is>
       </c>
       <c r="K21" s="2" t="inlineStr">
         <is>
-          <t>Claude Kandiyoti (CEO)</t>
-        </is>
-      </c>
-      <c r="L21" s="2" t="inlineStr">
-        <is>
-          <t>https://www.linkedin.com/in/claude-kandiyoti-287b9298/</t>
-        </is>
-      </c>
+          <t>Nuno Dias (Diretor Geral da Madre Imobiliário· presidente do grupo é António Parente)</t>
+        </is>
+      </c>
+      <c r="L21" s="2" t="inlineStr"/>
       <c r="M21" s="2" t="inlineStr"/>
     </row>
     <row r="22" ht="30" customHeight="1">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>Kronos Homes Portugal</t>
+          <t>Habitat Invest</t>
         </is>
       </c>
       <c r="B22" s="3" t="inlineStr">
@@ -1775,13 +1759,17 @@
       </c>
       <c r="C22" s="4" t="inlineStr">
         <is>
-          <t>+351 211 227 710</t>
-        </is>
-      </c>
-      <c r="D22" s="2" t="inlineStr"/>
+          <t>+351 213 461 024</t>
+        </is>
+      </c>
+      <c r="D22" s="2" t="inlineStr">
+        <is>
+          <t>info@habitatinvest.pt</t>
+        </is>
+      </c>
       <c r="E22" s="2" t="inlineStr">
         <is>
-          <t>kronoshomes.com</t>
+          <t>habitatinvest.pt</t>
         </is>
       </c>
       <c r="F22" s="4" t="inlineStr">
@@ -1796,35 +1784,31 @@
       </c>
       <c r="H22" s="2" t="inlineStr">
         <is>
-          <t>Av. da Liberdade 245, 1250-143</t>
+          <t>Rua da Moeda 4, 1200-275</t>
         </is>
       </c>
       <c r="I22" s="2" t="inlineStr">
         <is>
-          <t>The One (Lisboa) (Comercialização) | Lagos e Alcantarilha (Comercialização) | Flamingos Salgados (Comercialização) | Monte Santo (Carvoeiro) (Comercialização)</t>
+          <t>15 projetos em desenvolvimento (Em construção) | ALMAR SOUTH LIVING (Almada) (Em construção/comercialização) | AURYA (Santo António dos Cavaleiros, Loures) (Em construção)</t>
         </is>
       </c>
       <c r="J22" s="2" t="inlineStr">
         <is>
-          <t>Entidade KIG Portugal (NIF 514667265)</t>
+          <t>Fundada 2001 · inclui Habitat Ventures/Project/Property/Broker</t>
         </is>
       </c>
       <c r="K22" s="2" t="inlineStr">
         <is>
-          <t>Rui Meneses Ferreira (CEO)</t>
-        </is>
-      </c>
-      <c r="L22" s="2" t="inlineStr">
-        <is>
-          <t>https://www.linkedin.com/in/rui-meneses-ferreira-97057825/</t>
-        </is>
-      </c>
+          <t>Luís Corrêa de Barros (fundador e CEO)</t>
+        </is>
+      </c>
+      <c r="L22" s="2" t="inlineStr"/>
       <c r="M22" s="2" t="inlineStr"/>
     </row>
     <row r="23" ht="30" customHeight="1">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>Lantia</t>
+          <t>J. Dias &amp; Dias</t>
         </is>
       </c>
       <c r="B23" s="3" t="inlineStr">
@@ -1834,22 +1818,22 @@
       </c>
       <c r="C23" s="4" t="inlineStr">
         <is>
-          <t>+351 211 165 360</t>
+          <t>+351 214 422 593</t>
         </is>
       </c>
       <c r="D23" s="2" t="inlineStr">
         <is>
-          <t>geral@lantia.pt</t>
+          <t>geral@jdiasdias.pt</t>
         </is>
       </c>
       <c r="E23" s="2" t="inlineStr">
         <is>
-          <t>lantia.pt</t>
+          <t>jdiasdias.pt</t>
         </is>
       </c>
       <c r="F23" s="4" t="inlineStr">
         <is>
-          <t>Lisboa</t>
+          <t>Cascais</t>
         </is>
       </c>
       <c r="G23" s="4" t="inlineStr">
@@ -1859,31 +1843,27 @@
       </c>
       <c r="H23" s="2" t="inlineStr">
         <is>
-          <t>Praça Duque de Saldanha 1, 4F, 1050-054</t>
+          <t>Av. Venceslau Balseiro da Grande Guerra, Quinta das Marianas, Parede</t>
         </is>
       </c>
       <c r="I23" s="2" t="inlineStr">
         <is>
-          <t>Residencial e turístico Grande Lisboa (Em construção)</t>
+          <t>Urban Living (Carcavelos/Parede) (Comercialização)</t>
         </is>
       </c>
       <c r="J23" s="2" t="inlineStr">
         <is>
-          <t>Constituída em Macau 2015</t>
-        </is>
-      </c>
-      <c r="K23" s="2" t="inlineStr">
-        <is>
-          <t>Eduardo Kol Netto de Almeida (CEO)</t>
-        </is>
-      </c>
+          <t>Fundada 1960, alvará ICC 12463. Tel. móvel 961 682 789</t>
+        </is>
+      </c>
+      <c r="K23" s="2" t="inlineStr"/>
       <c r="L23" s="2" t="inlineStr"/>
       <c r="M23" s="2" t="inlineStr"/>
     </row>
     <row r="24" ht="30" customHeight="1">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>Libertas – Investimentos Imobiliários</t>
+          <t>JPS Group</t>
         </is>
       </c>
       <c r="B24" s="3" t="inlineStr">
@@ -1893,17 +1873,17 @@
       </c>
       <c r="C24" s="4" t="inlineStr">
         <is>
-          <t>+351 213 243 050</t>
+          <t>+351 218 371 025</t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr">
         <is>
-          <t>libertas@libertas.pt</t>
+          <t>secretariado@jpsgroup.pt</t>
         </is>
       </c>
       <c r="E24" s="2" t="inlineStr">
         <is>
-          <t>libertas.pt</t>
+          <t>jpsgroup.pt</t>
         </is>
       </c>
       <c r="F24" s="4" t="inlineStr">
@@ -1918,31 +1898,35 @@
       </c>
       <c r="H24" s="2" t="inlineStr">
         <is>
-          <t>Av. da Liberdade 129, 8º A, 1250-140</t>
+          <t>Av. Almirante Gago Coutinho 126</t>
         </is>
       </c>
       <c r="I24" s="2" t="inlineStr">
         <is>
-          <t>Lux Garden EVO (Faro) (Em construção) | Novos projetos Algarve (Planeamento)</t>
+          <t>SkyCity (Carnaxide) (Em construção) | Herdade Real de Santiago (Comercialização) | Terraços de São Francisco (Comercialização)</t>
         </is>
       </c>
       <c r="J24" s="2" t="inlineStr">
         <is>
-          <t>18 projetos no Algarve, &gt;800 unidades entregues · ISO 14001</t>
+          <t>Promotora com construtora e imobiliária próprias</t>
         </is>
       </c>
       <c r="K24" s="2" t="inlineStr">
         <is>
-          <t>António Gonçalves (Fundador)</t>
-        </is>
-      </c>
-      <c r="L24" s="2" t="inlineStr"/>
+          <t>João Sousa (CEO)</t>
+        </is>
+      </c>
+      <c r="L24" s="2" t="inlineStr">
+        <is>
+          <t>https://pt.linkedin.com/in/joao-sousa-7802352a</t>
+        </is>
+      </c>
       <c r="M24" s="2" t="inlineStr"/>
     </row>
     <row r="25" ht="30" customHeight="1">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>Major Development</t>
+          <t>Krest Investments</t>
         </is>
       </c>
       <c r="B25" s="3" t="inlineStr">
@@ -1952,17 +1936,17 @@
       </c>
       <c r="C25" s="4" t="inlineStr">
         <is>
-          <t>+351 210 912 130</t>
+          <t>+351 215 873 920</t>
         </is>
       </c>
       <c r="D25" s="2" t="inlineStr">
         <is>
-          <t>contacto@majordevelop.com</t>
+          <t>info@krestinvestments.com</t>
         </is>
       </c>
       <c r="E25" s="2" t="inlineStr">
         <is>
-          <t>majordevelop.com</t>
+          <t>krestinvestments.com</t>
         </is>
       </c>
       <c r="F25" s="4" t="inlineStr">
@@ -1977,27 +1961,27 @@
       </c>
       <c r="H25" s="2" t="inlineStr">
         <is>
-          <t>Cais do Gás, Armazém H, 1200-109</t>
+          <t>Av. Eng.º Duarte Pacheco, Amoreiras Torre 1, piso 14, sala 2, 1070-101</t>
         </is>
       </c>
       <c r="I25" s="2" t="inlineStr">
         <is>
-          <t>Garden Cascais (Planeamento) | Solo Oeiras (Planeamento) | Vistabella (Oeiras) (Planeamento) | Santa Apolónia (Planeamento) | Nouveau Lisboa (Av. Berna) (Concluído)</t>
+          <t>Lisboa / Porto / Algarve (Comercialização)</t>
         </is>
       </c>
       <c r="J25" s="2" t="inlineStr">
         <is>
-          <t>&gt;100M€ anunciados 2026. Fonte: diarioimobiliario.pt</t>
+          <t>Belga, em Portugal desde 2014</t>
         </is>
       </c>
       <c r="K25" s="2" t="inlineStr">
         <is>
-          <t>Gabriel Costa (CEO, confiança baixa — só rocketreach)</t>
+          <t>Claude Kandiyoti (CEO)</t>
         </is>
       </c>
       <c r="L25" s="2" t="inlineStr">
         <is>
-          <t>https://pt.linkedin.com/in/gabriel-costa-7436b5158</t>
+          <t>https://www.linkedin.com/in/claude-kandiyoti-287b9298/</t>
         </is>
       </c>
       <c r="M25" s="2" t="inlineStr"/>
@@ -2005,7 +1989,7 @@
     <row r="26" ht="30" customHeight="1">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>Mesmo Valor (Mesmovalor, S.A.)</t>
+          <t>Kronos Homes Portugal</t>
         </is>
       </c>
       <c r="B26" s="3" t="inlineStr">
@@ -2015,56 +1999,56 @@
       </c>
       <c r="C26" s="4" t="inlineStr">
         <is>
-          <t>+351 223 274 626</t>
-        </is>
-      </c>
-      <c r="D26" s="2" t="inlineStr">
-        <is>
-          <t>geral@mesmovalor.pt</t>
-        </is>
-      </c>
+          <t>+351 211 227 710</t>
+        </is>
+      </c>
+      <c r="D26" s="2" t="inlineStr"/>
       <c r="E26" s="2" t="inlineStr">
         <is>
-          <t>mesmovalor.pt</t>
+          <t>kronoshomes.com</t>
         </is>
       </c>
       <c r="F26" s="4" t="inlineStr">
         <is>
-          <t>Porto</t>
+          <t>Lisboa</t>
         </is>
       </c>
       <c r="G26" s="4" t="inlineStr">
         <is>
-          <t>Porto</t>
+          <t>Lisboa</t>
         </is>
       </c>
       <c r="H26" s="2" t="inlineStr">
         <is>
-          <t>Rua do Pinheiro Manso 147, 4100-412</t>
+          <t>Av. da Liberdade 245, 1250-143</t>
         </is>
       </c>
       <c r="I26" s="2" t="inlineStr">
         <is>
-          <t>Boavista Tower (Comercialização)</t>
+          <t>The One (Lisboa) (Comercialização) | Lagos e Alcantarilha (Comercialização) | Flamingos Salgados (Comercialização) | Monte Santo (Carvoeiro) (Comercialização)</t>
         </is>
       </c>
       <c r="J26" s="2" t="inlineStr">
         <is>
-          <t>Capital social 5M€. Fonte: idealista/news ago/2026</t>
+          <t>Entidade KIG Portugal (NIF 514667265)</t>
         </is>
       </c>
       <c r="K26" s="2" t="inlineStr">
         <is>
-          <t>Pedro Teixeira Paredes (CEO)</t>
-        </is>
-      </c>
-      <c r="L26" s="2" t="inlineStr"/>
+          <t>Rui Meneses Ferreira (CEO)</t>
+        </is>
+      </c>
+      <c r="L26" s="2" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/rui-meneses-ferreira-97057825/</t>
+        </is>
+      </c>
       <c r="M26" s="2" t="inlineStr"/>
     </row>
     <row r="27" ht="30" customHeight="1">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>MEXTO Property Investment</t>
+          <t>Lantia</t>
         </is>
       </c>
       <c r="B27" s="3" t="inlineStr">
@@ -2074,17 +2058,17 @@
       </c>
       <c r="C27" s="4" t="inlineStr">
         <is>
-          <t>+351 213 461 050</t>
+          <t>+351 211 165 360</t>
         </is>
       </c>
       <c r="D27" s="2" t="inlineStr">
         <is>
-          <t>info@mexto.pt</t>
+          <t>geral@lantia.pt</t>
         </is>
       </c>
       <c r="E27" s="2" t="inlineStr">
         <is>
-          <t>mexto.pt</t>
+          <t>lantia.pt</t>
         </is>
       </c>
       <c r="F27" s="4" t="inlineStr">
@@ -2099,35 +2083,31 @@
       </c>
       <c r="H27" s="2" t="inlineStr">
         <is>
-          <t>Rua Nova do Almada 81, 4º Dto</t>
+          <t>Praça Duque de Saldanha 1, 4F, 1050-054</t>
         </is>
       </c>
       <c r="I27" s="2" t="inlineStr">
         <is>
-          <t>Castilho 3 (Em construção) | São Gens (Graça) (Em construção)</t>
+          <t>Residencial e turístico Grande Lisboa (Em construção)</t>
         </is>
       </c>
       <c r="J27" s="2" t="inlineStr">
         <is>
-          <t>Grupo suíço, 250M€ em Portugal, 71.000 m²</t>
+          <t>Constituída em Macau 2015</t>
         </is>
       </c>
       <c r="K27" s="2" t="inlineStr">
         <is>
-          <t>Tomas Suter (Founding Member/Partner, Suíça)</t>
-        </is>
-      </c>
-      <c r="L27" s="2" t="inlineStr">
-        <is>
-          <t>https://www.linkedin.com/in/tomas-suter-78564b9/</t>
-        </is>
-      </c>
+          <t>Eduardo Kol Netto de Almeida (CEO)</t>
+        </is>
+      </c>
+      <c r="L27" s="2" t="inlineStr"/>
       <c r="M27" s="2" t="inlineStr"/>
     </row>
     <row r="28" ht="30" customHeight="1">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>Norfin</t>
+          <t>Libertas – Investimentos Imobiliários</t>
         </is>
       </c>
       <c r="B28" s="3" t="inlineStr">
@@ -2137,13 +2117,17 @@
       </c>
       <c r="C28" s="4" t="inlineStr">
         <is>
-          <t>+351 213 182 520</t>
-        </is>
-      </c>
-      <c r="D28" s="2" t="inlineStr"/>
+          <t>+351 213 243 050</t>
+        </is>
+      </c>
+      <c r="D28" s="2" t="inlineStr">
+        <is>
+          <t>libertas@libertas.pt</t>
+        </is>
+      </c>
       <c r="E28" s="2" t="inlineStr">
         <is>
-          <t>norfin.pt</t>
+          <t>libertas.pt</t>
         </is>
       </c>
       <c r="F28" s="4" t="inlineStr">
@@ -2158,35 +2142,31 @@
       </c>
       <c r="H28" s="2" t="inlineStr">
         <is>
-          <t>Av. Almirante Gago Coutinho 30, piso 0, 1000-017</t>
+          <t>Av. da Liberdade 129, 8º A, 1250-140</t>
         </is>
       </c>
       <c r="I28" s="2" t="inlineStr">
         <is>
-          <t>Lisbon Heights (Alta de Lisboa) (Comercialização) | Lote Alta de Lisboa (Planeamento) | Oriente Green Campus / Campo Novo (Em construção)</t>
+          <t>Lux Garden EVO (Faro) (Em construção) | Novos projetos Algarve (Planeamento)</t>
         </is>
       </c>
       <c r="J28" s="2" t="inlineStr">
         <is>
-          <t>Gestora de investimento (2,1B€) que também promove</t>
+          <t>18 projetos no Algarve, &gt;800 unidades entregues · ISO 14001</t>
         </is>
       </c>
       <c r="K28" s="2" t="inlineStr">
         <is>
-          <t>Miguel Mateus (CEO, recém-nomeado)</t>
-        </is>
-      </c>
-      <c r="L28" s="2" t="inlineStr">
-        <is>
-          <t>https://www.linkedin.com/in/miguel-mateus-608b616/</t>
-        </is>
-      </c>
+          <t>António Gonçalves (Fundador)</t>
+        </is>
+      </c>
+      <c r="L28" s="2" t="inlineStr"/>
       <c r="M28" s="2" t="inlineStr"/>
     </row>
     <row r="29" ht="30" customHeight="1">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>Noronha Sanches</t>
+          <t>Major Development</t>
         </is>
       </c>
       <c r="B29" s="3" t="inlineStr">
@@ -2196,17 +2176,17 @@
       </c>
       <c r="C29" s="4" t="inlineStr">
         <is>
-          <t>+351 217 220 620</t>
+          <t>+351 210 912 130</t>
         </is>
       </c>
       <c r="D29" s="2" t="inlineStr">
         <is>
-          <t>sales@noronhasanches.com</t>
+          <t>contacto@majordevelop.com</t>
         </is>
       </c>
       <c r="E29" s="2" t="inlineStr">
         <is>
-          <t>noronhasanches.com</t>
+          <t>majordevelop.com</t>
         </is>
       </c>
       <c r="F29" s="4" t="inlineStr">
@@ -2221,27 +2201,27 @@
       </c>
       <c r="H29" s="2" t="inlineStr">
         <is>
-          <t>Campo Grande 28, 3º G, 1700-093</t>
+          <t>Cais do Gás, Armazém H, 1200-109</t>
         </is>
       </c>
       <c r="I29" s="2" t="inlineStr">
         <is>
-          <t>One Lush (Caxias) (Em construção) | Vila Praia (Comercialização) | Marinha Prime (Comercialização)</t>
+          <t>Garden Cascais (Planeamento) | Solo Oeiras (Planeamento) | Vistabella (Oeiras) (Planeamento) | Santa Apolónia (Planeamento) | Nouveau Lisboa (Av. Berna) (Concluído)</t>
         </is>
       </c>
       <c r="J29" s="2" t="inlineStr">
         <is>
-          <t>Promotor desde 1986</t>
+          <t>&gt;100M€ anunciados 2026. Fonte: diarioimobiliario.pt</t>
         </is>
       </c>
       <c r="K29" s="2" t="inlineStr">
         <is>
-          <t>Pedro Sanches (CEO/fundador)</t>
+          <t>Gabriel Costa (CEO, confiança baixa — só rocketreach)</t>
         </is>
       </c>
       <c r="L29" s="2" t="inlineStr">
         <is>
-          <t>https://pt.linkedin.com/in/pedro-sanches-77205825</t>
+          <t>https://pt.linkedin.com/in/gabriel-costa-7436b5158</t>
         </is>
       </c>
       <c r="M29" s="2" t="inlineStr"/>
@@ -2249,7 +2229,7 @@
     <row r="30" ht="30" customHeight="1">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>Névoa, S.A.</t>
+          <t>Mesmo Valor (Mesmovalor, S.A.)</t>
         </is>
       </c>
       <c r="B30" s="3" t="inlineStr">
@@ -2259,44 +2239,56 @@
       </c>
       <c r="C30" s="4" t="inlineStr">
         <is>
-          <t>+351 253 240 010</t>
-        </is>
-      </c>
-      <c r="D30" s="2" t="inlineStr"/>
+          <t>+351 223 274 626</t>
+        </is>
+      </c>
+      <c r="D30" s="2" t="inlineStr">
+        <is>
+          <t>geral@mesmovalor.pt</t>
+        </is>
+      </c>
       <c r="E30" s="2" t="inlineStr">
         <is>
-          <t>nevoa.pt</t>
+          <t>mesmovalor.pt</t>
         </is>
       </c>
       <c r="F30" s="4" t="inlineStr">
         <is>
-          <t>Lisboa</t>
+          <t>Porto</t>
         </is>
       </c>
       <c r="G30" s="4" t="inlineStr">
         <is>
-          <t>Lisboa</t>
-        </is>
-      </c>
-      <c r="H30" s="2" t="inlineStr"/>
+          <t>Porto</t>
+        </is>
+      </c>
+      <c r="H30" s="2" t="inlineStr">
+        <is>
+          <t>Rua do Pinheiro Manso 147, 4100-412</t>
+        </is>
+      </c>
       <c r="I30" s="2" t="inlineStr">
         <is>
-          <t>Portfólio nacional de empreendimentos (Comercialização)</t>
+          <t>Boavista Tower (Comercialização)</t>
         </is>
       </c>
       <c r="J30" s="2" t="inlineStr">
         <is>
-          <t>Fonte: vidaimobiliaria.com, racius.com</t>
-        </is>
-      </c>
-      <c r="K30" s="2" t="inlineStr"/>
+          <t>Capital social 5M€. Fonte: idealista/news ago/2026</t>
+        </is>
+      </c>
+      <c r="K30" s="2" t="inlineStr">
+        <is>
+          <t>Pedro Teixeira Paredes (CEO)</t>
+        </is>
+      </c>
       <c r="L30" s="2" t="inlineStr"/>
       <c r="M30" s="2" t="inlineStr"/>
     </row>
     <row r="31" ht="30" customHeight="1">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>Optylon Krea</t>
+          <t>MEXTO Property Investment</t>
         </is>
       </c>
       <c r="B31" s="3" t="inlineStr">
@@ -2306,17 +2298,17 @@
       </c>
       <c r="C31" s="4" t="inlineStr">
         <is>
-          <t>+351 212 400 124</t>
+          <t>+351 213 461 050</t>
         </is>
       </c>
       <c r="D31" s="2" t="inlineStr">
         <is>
-          <t>sales@optylonkrea.com</t>
+          <t>info@mexto.pt</t>
         </is>
       </c>
       <c r="E31" s="2" t="inlineStr">
         <is>
-          <t>optylonkrea.com</t>
+          <t>mexto.pt</t>
         </is>
       </c>
       <c r="F31" s="4" t="inlineStr">
@@ -2331,27 +2323,27 @@
       </c>
       <c r="H31" s="2" t="inlineStr">
         <is>
-          <t>Rua Alexandre Herculano 50, 10º/11º, 1250-096</t>
+          <t>Rua Nova do Almada 81, 4º Dto</t>
         </is>
       </c>
       <c r="I31" s="2" t="inlineStr">
         <is>
-          <t>Ando Living – Alfama Club e Liberdade Club (Em construção) | Augusta Townhouse + Santos Townhouse (Comercialização)</t>
+          <t>Castilho 3 (Em construção) | São Gens (Graça) (Em construção)</t>
         </is>
       </c>
       <c r="J31" s="2" t="inlineStr">
         <is>
-          <t>1,7B€ investidos · PT e Turquia</t>
+          <t>Grupo suíço, 250M€ em Portugal, 71.000 m²</t>
         </is>
       </c>
       <c r="K31" s="2" t="inlineStr">
         <is>
-          <t>William Tonnard (President &amp; COO· Chairman é Hakan Kodal)</t>
+          <t>Tomas Suter (Founding Member/Partner, Suíça)</t>
         </is>
       </c>
       <c r="L31" s="2" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/in/william-tonnard/</t>
+          <t>https://www.linkedin.com/in/tomas-suter-78564b9/</t>
         </is>
       </c>
       <c r="M31" s="2" t="inlineStr"/>
@@ -2359,7 +2351,7 @@
     <row r="32" ht="30" customHeight="1">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>Qualive</t>
+          <t>Norfin</t>
         </is>
       </c>
       <c r="B32" s="3" t="inlineStr">
@@ -2369,44 +2361,56 @@
       </c>
       <c r="C32" s="4" t="inlineStr">
         <is>
-          <t>+351 226 090 545</t>
+          <t>+351 213 182 520</t>
         </is>
       </c>
       <c r="D32" s="2" t="inlineStr"/>
-      <c r="E32" s="2" t="inlineStr"/>
+      <c r="E32" s="2" t="inlineStr">
+        <is>
+          <t>norfin.pt</t>
+        </is>
+      </c>
       <c r="F32" s="4" t="inlineStr">
         <is>
-          <t>Porto</t>
+          <t>Lisboa</t>
         </is>
       </c>
       <c r="G32" s="4" t="inlineStr">
         <is>
-          <t>Porto</t>
+          <t>Lisboa</t>
         </is>
       </c>
       <c r="H32" s="2" t="inlineStr">
         <is>
-          <t>Rua D. Pedro V 410, 2º, 4150-601</t>
+          <t>Av. Almirante Gago Coutinho 30, piso 0, 1000-017</t>
         </is>
       </c>
       <c r="I32" s="2" t="inlineStr">
         <is>
-          <t>Fábrica do Prado (Matosinhos) (Em construção)</t>
+          <t>Lisbon Heights (Alta de Lisboa) (Comercialização) | Lote Alta de Lisboa (Planeamento) | Oriente Green Campus / Campo Novo (Em construção)</t>
         </is>
       </c>
       <c r="J32" s="2" t="inlineStr">
         <is>
-          <t>Telefone do registo comercial (einforma). Comercialização JLL/Predibisa</t>
-        </is>
-      </c>
-      <c r="K32" s="2" t="inlineStr"/>
-      <c r="L32" s="2" t="inlineStr"/>
+          <t>Gestora de investimento (2,1B€) que também promove</t>
+        </is>
+      </c>
+      <c r="K32" s="2" t="inlineStr">
+        <is>
+          <t>Miguel Mateus (CEO, recém-nomeado)</t>
+        </is>
+      </c>
+      <c r="L32" s="2" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/miguel-mateus-608b616/</t>
+        </is>
+      </c>
       <c r="M32" s="2" t="inlineStr"/>
     </row>
     <row r="33" ht="30" customHeight="1">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t>Quest Capital</t>
+          <t>Noronha Sanches</t>
         </is>
       </c>
       <c r="B33" s="3" t="inlineStr">
@@ -2416,17 +2420,17 @@
       </c>
       <c r="C33" s="4" t="inlineStr">
         <is>
-          <t>+351 213 472 435</t>
+          <t>+351 217 220 620</t>
         </is>
       </c>
       <c r="D33" s="2" t="inlineStr">
         <is>
-          <t>info@questcapital.eu</t>
+          <t>sales@noronhasanches.com</t>
         </is>
       </c>
       <c r="E33" s="2" t="inlineStr">
         <is>
-          <t>questcapital.eu</t>
+          <t>noronhasanches.com</t>
         </is>
       </c>
       <c r="F33" s="4" t="inlineStr">
@@ -2441,27 +2445,27 @@
       </c>
       <c r="H33" s="2" t="inlineStr">
         <is>
-          <t>Rua António Maria Cardoso 2, 1200-027 (escritório Porto: Rua Fernandes Tomás 546)</t>
+          <t>Campo Grande 28, 3º G, 1700-093</t>
         </is>
       </c>
       <c r="I33" s="2" t="inlineStr">
         <is>
-          <t>Antas Atrium (Porto, antigo estádio) (Em construção)</t>
+          <t>One Lush (Caxias) (Em construção) | Vila Praia (Comercialização) | Marinha Prime (Comercialização)</t>
         </is>
       </c>
       <c r="J33" s="2" t="inlineStr">
         <is>
-          <t>Com Tikehau Capital. &gt;1B€ sob gestão</t>
+          <t>Promotor desde 1986</t>
         </is>
       </c>
       <c r="K33" s="2" t="inlineStr">
         <is>
-          <t>Carlos Vasconcellos (Founding Partner, CEO exato não confirmado)</t>
+          <t>Pedro Sanches (CEO/fundador)</t>
         </is>
       </c>
       <c r="L33" s="2" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/in/vasconcelloscarlos/</t>
+          <t>https://pt.linkedin.com/in/pedro-sanches-77205825</t>
         </is>
       </c>
       <c r="M33" s="2" t="inlineStr"/>
@@ -2469,7 +2473,7 @@
     <row r="34" ht="30" customHeight="1">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>ReVentures – Property Developers</t>
+          <t>Névoa, S.A.</t>
         </is>
       </c>
       <c r="B34" s="3" t="inlineStr">
@@ -2479,17 +2483,13 @@
       </c>
       <c r="C34" s="4" t="inlineStr">
         <is>
-          <t>+351 212 402 489</t>
-        </is>
-      </c>
-      <c r="D34" s="2" t="inlineStr">
-        <is>
-          <t>info@reventures.pt</t>
-        </is>
-      </c>
+          <t>+351 253 240 010</t>
+        </is>
+      </c>
+      <c r="D34" s="2" t="inlineStr"/>
       <c r="E34" s="2" t="inlineStr">
         <is>
-          <t>reventures.pt</t>
+          <t>nevoa.pt</t>
         </is>
       </c>
       <c r="F34" s="4" t="inlineStr">
@@ -2502,37 +2502,25 @@
           <t>Lisboa</t>
         </is>
       </c>
-      <c r="H34" s="2" t="inlineStr">
-        <is>
-          <t>Campo Grande 28, 3º A, 1700-093</t>
-        </is>
-      </c>
+      <c r="H34" s="2" t="inlineStr"/>
       <c r="I34" s="2" t="inlineStr">
         <is>
-          <t>7 residências de estudantes (rede nacional) (Em construção) | Senior Living (Planeamento)</t>
+          <t>Portfólio nacional de empreendimentos (Comercialização)</t>
         </is>
       </c>
       <c r="J34" s="2" t="inlineStr">
         <is>
-          <t>NIF 516390350, capital 800k€. Fonte: construir.pt abr/2026</t>
-        </is>
-      </c>
-      <c r="K34" s="2" t="inlineStr">
-        <is>
-          <t>Hugo Gonçalves Pereira (CEO)</t>
-        </is>
-      </c>
-      <c r="L34" s="2" t="inlineStr">
-        <is>
-          <t>https://www.linkedin.com/in/hugogpereira/</t>
-        </is>
-      </c>
+          <t>Fonte: vidaimobiliaria.com, racius.com</t>
+        </is>
+      </c>
+      <c r="K34" s="2" t="inlineStr"/>
+      <c r="L34" s="2" t="inlineStr"/>
       <c r="M34" s="2" t="inlineStr"/>
     </row>
     <row r="35" ht="30" customHeight="1">
       <c r="A35" s="2" t="inlineStr">
         <is>
-          <t>Rio Capital / Grupo Rio</t>
+          <t>Optylon Krea</t>
         </is>
       </c>
       <c r="B35" s="3" t="inlineStr">
@@ -2542,17 +2530,17 @@
       </c>
       <c r="C35" s="4" t="inlineStr">
         <is>
-          <t>+351 213 861 065</t>
+          <t>+351 212 400 124</t>
         </is>
       </c>
       <c r="D35" s="2" t="inlineStr">
         <is>
-          <t>geral@riocapital.pt</t>
+          <t>sales@optylonkrea.com</t>
         </is>
       </c>
       <c r="E35" s="2" t="inlineStr">
         <is>
-          <t>riocapital.pt</t>
+          <t>optylonkrea.com</t>
         </is>
       </c>
       <c r="F35" s="4" t="inlineStr">
@@ -2567,27 +2555,35 @@
       </c>
       <c r="H35" s="2" t="inlineStr">
         <is>
-          <t>Av. Duarte Pacheco, Amoreiras Torre 2, 14º D</t>
+          <t>Rua Alexandre Herculano 50, 10º/11º, 1250-096</t>
         </is>
       </c>
       <c r="I35" s="2" t="inlineStr">
         <is>
-          <t>21 projetos residenciais Grande Porto (Em construção) | Velaris (Porto) (Planeamento) | São Vicente (Maia) (Planeamento) | Metropólis Estúdio Residence (Matosinhos) (Planeamento)</t>
+          <t>Ando Living – Alfama Club e Liberdade Club (Em construção) | Augusta Townhouse + Santos Townhouse (Comercialização)</t>
         </is>
       </c>
       <c r="J35" s="2" t="inlineStr">
         <is>
-          <t>Grupo nascido em Monção, liderado por Nuno Afonso. Fonte: idealista/news jun/2026, Público</t>
-        </is>
-      </c>
-      <c r="K35" s="2" t="inlineStr"/>
-      <c r="L35" s="2" t="inlineStr"/>
+          <t>1,7B€ investidos · PT e Turquia</t>
+        </is>
+      </c>
+      <c r="K35" s="2" t="inlineStr">
+        <is>
+          <t>William Tonnard (President &amp; COO· Chairman é Hakan Kodal)</t>
+        </is>
+      </c>
+      <c r="L35" s="2" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/william-tonnard/</t>
+        </is>
+      </c>
       <c r="M35" s="2" t="inlineStr"/>
     </row>
     <row r="36" ht="30" customHeight="1">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>Rockbuilding – Soluções Imobiliárias</t>
+          <t>Overseas</t>
         </is>
       </c>
       <c r="B36" s="3" t="inlineStr">
@@ -2597,13 +2593,17 @@
       </c>
       <c r="C36" s="4" t="inlineStr">
         <is>
-          <t>+351 217 996 700</t>
-        </is>
-      </c>
-      <c r="D36" s="2" t="inlineStr"/>
+          <t>+351 911 741 900</t>
+        </is>
+      </c>
+      <c r="D36" s="2" t="inlineStr">
+        <is>
+          <t>info@overseasglobal.com</t>
+        </is>
+      </c>
       <c r="E36" s="2" t="inlineStr">
         <is>
-          <t>rockbuilding.com</t>
+          <t>overseasglobal.com</t>
         </is>
       </c>
       <c r="F36" s="4" t="inlineStr">
@@ -2618,27 +2618,27 @@
       </c>
       <c r="H36" s="2" t="inlineStr">
         <is>
-          <t>Ed. Amoreiras Plaza, Rua Carlos Alberto da Mota Pinto 9, 7º A, 1070-374</t>
+          <t>Rua Alexandre Herculano 25, 1º, 1250-008</t>
         </is>
       </c>
       <c r="I36" s="2" t="inlineStr">
         <is>
-          <t>Serviços de desenvolvimento para promotores (Em construção)</t>
+          <t>5 projetos premium (4 Lisboa + Comporta) (Em construção) | JV com Grupo André Guimarães (Lisboa) (Planeamento) | Karl Lagerfeld branded residences (Planeamento) | Telhal 72 Liberdade (Comercialização)</t>
         </is>
       </c>
       <c r="J36" s="2" t="inlineStr">
         <is>
-          <t>ATENÇÃO: é gestor de projeto/serviços, não promotor puro</t>
+          <t>CEO Pedro Vicente (vice-presidente APPII). Sem telefone publicado</t>
         </is>
       </c>
       <c r="K36" s="2" t="inlineStr">
         <is>
-          <t>José Pedro Almeida Guerra (Diretor Geral)</t>
+          <t>Pedro Vicente (CEO)</t>
         </is>
       </c>
       <c r="L36" s="2" t="inlineStr">
         <is>
-          <t>https://pt.linkedin.com/in/josé-pedro-almeida-guerra-20723679</t>
+          <t>https://www.linkedin.com/in/pedro-vicente-9aa0b424/</t>
         </is>
       </c>
       <c r="M36" s="2" t="inlineStr"/>
@@ -2646,7 +2646,7 @@
     <row r="37" ht="30" customHeight="1">
       <c r="A37" s="2" t="inlineStr">
         <is>
-          <t>Royal Ventures</t>
+          <t>Prime Portugal</t>
         </is>
       </c>
       <c r="B37" s="3" t="inlineStr">
@@ -2656,60 +2656,56 @@
       </c>
       <c r="C37" s="4" t="inlineStr">
         <is>
-          <t>+351 916 770 322</t>
+          <t>+351 915 896 265</t>
         </is>
       </c>
       <c r="D37" s="2" t="inlineStr">
         <is>
-          <t>alex@royal-ventures.com</t>
+          <t>info@primelisbon.com</t>
         </is>
       </c>
       <c r="E37" s="2" t="inlineStr">
         <is>
-          <t>royal-ventures.com</t>
+          <t>primelisbon.com</t>
         </is>
       </c>
       <c r="F37" s="4" t="inlineStr">
         <is>
-          <t>Porto</t>
+          <t>Lisboa</t>
         </is>
       </c>
       <c r="G37" s="4" t="inlineStr">
         <is>
-          <t>Porto</t>
+          <t>Lisboa</t>
         </is>
       </c>
       <c r="H37" s="2" t="inlineStr">
         <is>
-          <t>Edifício Oceanus, Av. da Boavista 3227, 4100-137</t>
+          <t>Av. Fontes Pereira de Melo 6, 1600-001</t>
         </is>
       </c>
       <c r="I37" s="2" t="inlineStr">
         <is>
-          <t>Reabilitação centro histórico do Porto (Em construção)</t>
+          <t>Projetos residenciais Lisboa, Cascais e Melides (Em construção)</t>
         </is>
       </c>
       <c r="J37" s="2" t="inlineStr">
         <is>
-          <t>Sócios israelitas (Udi, Liad) + contacto PT Alexandre. Fonte: royal-ventures.com/contact-us</t>
+          <t>Telefone/site é da 'Prime Lisbon', mesma morada — confirmar que é a mesma entidade antes de contactar</t>
         </is>
       </c>
       <c r="K37" s="2" t="inlineStr">
         <is>
-          <t>Udi Yadin (fundador/General Partner)</t>
-        </is>
-      </c>
-      <c r="L37" s="2" t="inlineStr">
-        <is>
-          <t>https://www.linkedin.com/in/udiyadin/</t>
-        </is>
-      </c>
+          <t>Federico Rosales (cofundador e CEO)</t>
+        </is>
+      </c>
+      <c r="L37" s="2" t="inlineStr"/>
       <c r="M37" s="2" t="inlineStr"/>
     </row>
     <row r="38" ht="30" customHeight="1">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>Sharp Developers</t>
+          <t>Qualive</t>
         </is>
       </c>
       <c r="B38" s="3" t="inlineStr">
@@ -2719,19 +2715,11 @@
       </c>
       <c r="C38" s="4" t="inlineStr">
         <is>
-          <t>+351 933 078 094</t>
-        </is>
-      </c>
-      <c r="D38" s="2" t="inlineStr">
-        <is>
-          <t>info@sharpdevelopers.pt</t>
-        </is>
-      </c>
-      <c r="E38" s="2" t="inlineStr">
-        <is>
-          <t>sharpdevelopers.pt</t>
-        </is>
-      </c>
+          <t>+351 226 090 545</t>
+        </is>
+      </c>
+      <c r="D38" s="2" t="inlineStr"/>
+      <c r="E38" s="2" t="inlineStr"/>
       <c r="F38" s="4" t="inlineStr">
         <is>
           <t>Porto</t>
@@ -2744,35 +2732,27 @@
       </c>
       <c r="H38" s="2" t="inlineStr">
         <is>
-          <t>Av. Boavista 1681, Ed. Bristol, Esc. 5.4</t>
+          <t>Rua D. Pedro V 410, 2º, 4150-601</t>
         </is>
       </c>
       <c r="I38" s="2" t="inlineStr">
         <is>
-          <t>Residencial de luxo Porto (Em construção)</t>
+          <t>Fábrica do Prado (Matosinhos) (Em construção)</t>
         </is>
       </c>
       <c r="J38" s="2" t="inlineStr">
         <is>
-          <t>CEO Carla Luís</t>
-        </is>
-      </c>
-      <c r="K38" s="2" t="inlineStr">
-        <is>
-          <t>Carla Luís (CEO/cofundadora)</t>
-        </is>
-      </c>
-      <c r="L38" s="2" t="inlineStr">
-        <is>
-          <t>https://www.linkedin.com/in/carla-luís-b14a7616/</t>
-        </is>
-      </c>
+          <t>Telefone do registo comercial (einforma). Comercialização JLL/Predibisa</t>
+        </is>
+      </c>
+      <c r="K38" s="2" t="inlineStr"/>
+      <c r="L38" s="2" t="inlineStr"/>
       <c r="M38" s="2" t="inlineStr"/>
     </row>
     <row r="39" ht="30" customHeight="1">
       <c r="A39" s="2" t="inlineStr">
         <is>
-          <t>SILCOGE / Grupo SIL</t>
+          <t>Quest Capital</t>
         </is>
       </c>
       <c r="B39" s="3" t="inlineStr">
@@ -2782,17 +2762,17 @@
       </c>
       <c r="C39" s="4" t="inlineStr">
         <is>
-          <t>+351 210 124 500</t>
+          <t>+351 213 472 435</t>
         </is>
       </c>
       <c r="D39" s="2" t="inlineStr">
         <is>
-          <t>info@sil.pt</t>
+          <t>info@questcapital.eu</t>
         </is>
       </c>
       <c r="E39" s="2" t="inlineStr">
         <is>
-          <t>sil.pt</t>
+          <t>questcapital.eu</t>
         </is>
       </c>
       <c r="F39" s="4" t="inlineStr">
@@ -2807,27 +2787,27 @@
       </c>
       <c r="H39" s="2" t="inlineStr">
         <is>
-          <t>Av. Fontes Pereira de Melo 6, 5º, 1050-121</t>
+          <t>Rua António Maria Cardoso 2, 1200-027 (escritório Porto: Rua Fernandes Tomás 546)</t>
         </is>
       </c>
       <c r="I39" s="2" t="inlineStr">
         <is>
-          <t>Grande Lisboa (Em construção)</t>
+          <t>Antas Atrium (Porto, antigo estádio) (Em construção)</t>
         </is>
       </c>
       <c r="J39" s="2" t="inlineStr">
         <is>
-          <t>Promoção imobiliária desde 1949</t>
+          <t>Com Tikehau Capital. &gt;1B€ sob gestão</t>
         </is>
       </c>
       <c r="K39" s="2" t="inlineStr">
         <is>
-          <t>Pedro Silveira (acionista maioritário/ex-Chairman, destituído judicialmente mai/2025, em recurso)</t>
+          <t>Carlos Vasconcellos (Founding Partner, CEO exato não confirmado)</t>
         </is>
       </c>
       <c r="L39" s="2" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/in/pedro-silveira-88822a20/</t>
+          <t>https://www.linkedin.com/in/vasconcelloscarlos/</t>
         </is>
       </c>
       <c r="M39" s="2" t="inlineStr"/>
@@ -2835,7 +2815,7 @@
     <row r="40" ht="30" customHeight="1">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>SOLYD Property Developers</t>
+          <t>RAR Imobiliária</t>
         </is>
       </c>
       <c r="B40" s="3" t="inlineStr">
@@ -2845,52 +2825,52 @@
       </c>
       <c r="C40" s="4" t="inlineStr">
         <is>
-          <t>+351 211 214 926</t>
+          <t>+351 226 190 530</t>
         </is>
       </c>
       <c r="D40" s="2" t="inlineStr">
         <is>
-          <t>info@elou-solyd.pt</t>
+          <t>geral@rarimobiliaria.pt</t>
         </is>
       </c>
       <c r="E40" s="2" t="inlineStr">
         <is>
-          <t>solyd.pt</t>
+          <t>rarimobiliaria.pt</t>
         </is>
       </c>
       <c r="F40" s="4" t="inlineStr">
         <is>
-          <t>Oeiras</t>
+          <t>Porto</t>
         </is>
       </c>
       <c r="G40" s="4" t="inlineStr">
         <is>
-          <t>Lisboa</t>
+          <t>Porto</t>
         </is>
       </c>
       <c r="H40" s="2" t="inlineStr">
         <is>
-          <t>Torre de Monsanto, Rua Afonso Praça 30, 7º, 1495-061 Algés</t>
+          <t>Rua do Passeio Alegre 600-624, 4169-002</t>
         </is>
       </c>
       <c r="I40" s="2" t="inlineStr">
         <is>
-          <t>Luz Altear (Alta de Lisboa) (Em construção) | ÉLOU (Santo António dos Cavaleiros, Loures) (Em construção/Comercialização)</t>
+          <t>Montebelo Villas (Foz Velha) (Em construção)</t>
         </is>
       </c>
       <c r="J40" s="2" t="inlineStr">
         <is>
-          <t>Estoril Capital Partners + Oaktree. Tel. alternativo 210 966 905</t>
+          <t>Fonte: dinheirovivo.pt, construir.pt</t>
         </is>
       </c>
       <c r="K40" s="2" t="inlineStr">
         <is>
-          <t>Gonçalo Cadete (CEO)</t>
+          <t>Paula Cristina Fernandes (CEO)</t>
         </is>
       </c>
       <c r="L40" s="2" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/in/gon%C3%A7alo-cadete-260692/</t>
+          <t>https://pt.linkedin.com/in/paula-fernandes-349a726</t>
         </is>
       </c>
       <c r="M40" s="2" t="inlineStr"/>
@@ -2898,7 +2878,7 @@
     <row r="41" ht="30" customHeight="1">
       <c r="A41" s="2" t="inlineStr">
         <is>
-          <t>Stone Capital</t>
+          <t>ReVentures – Property Developers</t>
         </is>
       </c>
       <c r="B41" s="3" t="inlineStr">
@@ -2908,17 +2888,17 @@
       </c>
       <c r="C41" s="4" t="inlineStr">
         <is>
-          <t>+351 210 416 350</t>
+          <t>+351 212 402 489</t>
         </is>
       </c>
       <c r="D41" s="2" t="inlineStr">
         <is>
-          <t>info@stonecapital.pt</t>
+          <t>info@reventures.pt</t>
         </is>
       </c>
       <c r="E41" s="2" t="inlineStr">
         <is>
-          <t>stonecapital.pt</t>
+          <t>reventures.pt</t>
         </is>
       </c>
       <c r="F41" s="4" t="inlineStr">
@@ -2933,31 +2913,35 @@
       </c>
       <c r="H41" s="2" t="inlineStr">
         <is>
-          <t>Av. da Liberdade 240, 1250-096</t>
+          <t>Campo Grande 28, 3º A, 1700-093</t>
         </is>
       </c>
       <c r="I41" s="2" t="inlineStr">
         <is>
-          <t>Santa Isabel (Em construção) | Portefólio em desenvolvimento (Em construção)</t>
+          <t>7 residências de estudantes (rede nacional) (Em construção) | Senior Living (Planeamento)</t>
         </is>
       </c>
       <c r="J41" s="2" t="inlineStr">
         <is>
-          <t>Tel. móvel 965 915 993</t>
+          <t>NIF 516390350, capital 800k€. Fonte: construir.pt abr/2026</t>
         </is>
       </c>
       <c r="K41" s="2" t="inlineStr">
         <is>
-          <t>Geoffroy Moreno (Co-Founder)</t>
-        </is>
-      </c>
-      <c r="L41" s="2" t="inlineStr"/>
+          <t>Hugo Gonçalves Pereira (CEO)</t>
+        </is>
+      </c>
+      <c r="L41" s="2" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/hugogpereira/</t>
+        </is>
+      </c>
       <c r="M41" s="2" t="inlineStr"/>
     </row>
     <row r="42" ht="30" customHeight="1">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>Teixeira Duarte Real Estate</t>
+          <t>Rio Capital / Grupo Rio</t>
         </is>
       </c>
       <c r="B42" s="3" t="inlineStr">
@@ -2967,22 +2951,22 @@
       </c>
       <c r="C42" s="4" t="inlineStr">
         <is>
-          <t>+351 217 912 300</t>
+          <t>+351 213 861 065</t>
         </is>
       </c>
       <c r="D42" s="2" t="inlineStr">
         <is>
-          <t>info@tdimobiliaria.pt</t>
+          <t>geral@riocapital.pt</t>
         </is>
       </c>
       <c r="E42" s="2" t="inlineStr">
         <is>
-          <t>tdimobiliaria.pt</t>
+          <t>riocapital.pt</t>
         </is>
       </c>
       <c r="F42" s="4" t="inlineStr">
         <is>
-          <t>Oeiras</t>
+          <t>Lisboa</t>
         </is>
       </c>
       <c r="G42" s="4" t="inlineStr">
@@ -2992,17 +2976,17 @@
       </c>
       <c r="H42" s="2" t="inlineStr">
         <is>
-          <t>Lagoas Park, Edifício 2, 2740-265 Porto Salvo</t>
+          <t>Av. Duarte Pacheco, Amoreiras Torre 2, 14º D</t>
         </is>
       </c>
       <c r="I42" s="2" t="inlineStr">
         <is>
-          <t>Quinta de Cravel (V.N. Gaia) (Comercialização)</t>
+          <t>21 projetos residenciais Grande Porto (Em construção) | Velaris (Porto) (Planeamento) | São Vicente (Maia) (Planeamento) | Metropólis Estúdio Residence (Matosinhos) (Planeamento)</t>
         </is>
       </c>
       <c r="J42" s="2" t="inlineStr">
         <is>
-          <t>Braço imobiliário do grupo Teixeira Duarte</t>
+          <t>Grupo nascido em Monção, liderado por Nuno Afonso. Fonte: idealista/news jun/2026, Público</t>
         </is>
       </c>
       <c r="K42" s="2" t="inlineStr"/>
@@ -3012,7 +2996,7 @@
     <row r="43" ht="30" customHeight="1">
       <c r="A43" s="2" t="inlineStr">
         <is>
-          <t>Thomas &amp; Piron Portugal</t>
+          <t>Rockbuilding – Soluções Imobiliárias</t>
         </is>
       </c>
       <c r="B43" s="3" t="inlineStr">
@@ -3022,52 +3006,48 @@
       </c>
       <c r="C43" s="4" t="inlineStr">
         <is>
-          <t>+351 214 422 464</t>
-        </is>
-      </c>
-      <c r="D43" s="2" t="inlineStr">
-        <is>
-          <t>infopt@thomas-piron.eu</t>
-        </is>
-      </c>
+          <t>+351 217 996 700</t>
+        </is>
+      </c>
+      <c r="D43" s="2" t="inlineStr"/>
       <c r="E43" s="2" t="inlineStr">
         <is>
-          <t>thomas-piron.pt</t>
+          <t>rockbuilding.com</t>
         </is>
       </c>
       <c r="F43" s="4" t="inlineStr">
         <is>
-          <t>Matosinhos</t>
+          <t>Lisboa</t>
         </is>
       </c>
       <c r="G43" s="4" t="inlineStr">
         <is>
-          <t>Porto</t>
+          <t>Lisboa</t>
         </is>
       </c>
       <c r="H43" s="2" t="inlineStr">
         <is>
-          <t>Escritórios em Matosinhos e Sacavém</t>
+          <t>Ed. Amoreiras Plaza, Rua Carlos Alberto da Mota Pinto 9, 7º A, 1070-374</t>
         </is>
       </c>
       <c r="I43" s="2" t="inlineStr">
         <is>
-          <t>Docks Matosinhos (Em construção) | Gaia Hills (V.N. Gaia) (Em construção) | Conde de Lima (Comercialização)</t>
+          <t>Serviços de desenvolvimento para promotores (Em construção)</t>
         </is>
       </c>
       <c r="J43" s="2" t="inlineStr">
         <is>
-          <t>Promotor belga em Portugal desde 2018. Fonte: diarioimobiliario.pt</t>
+          <t>ATENÇÃO: é gestor de projeto/serviços, não promotor puro</t>
         </is>
       </c>
       <c r="K43" s="2" t="inlineStr">
         <is>
-          <t>David Carreira (Diretor Geral/Country Manager)</t>
+          <t>José Pedro Almeida Guerra (Diretor Geral)</t>
         </is>
       </c>
       <c r="L43" s="2" t="inlineStr">
         <is>
-          <t>https://lu.linkedin.com/in/david-carreira-a4082050</t>
+          <t>https://pt.linkedin.com/in/josé-pedro-almeida-guerra-20723679</t>
         </is>
       </c>
       <c r="M43" s="2" t="inlineStr"/>
@@ -3075,7 +3055,7 @@
     <row r="44" ht="30" customHeight="1">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>Vanguard Properties</t>
+          <t>Round Hill Capital</t>
         </is>
       </c>
       <c r="B44" s="3" t="inlineStr">
@@ -3085,17 +3065,13 @@
       </c>
       <c r="C44" s="4" t="inlineStr">
         <is>
-          <t>+351 215 814 094</t>
-        </is>
-      </c>
-      <c r="D44" s="2" t="inlineStr">
-        <is>
-          <t>info@vangproperties.com</t>
-        </is>
-      </c>
+          <t>+351 213 303 727</t>
+        </is>
+      </c>
+      <c r="D44" s="2" t="inlineStr"/>
       <c r="E44" s="2" t="inlineStr">
         <is>
-          <t>vangproperties.com</t>
+          <t>roundhillcapital.com</t>
         </is>
       </c>
       <c r="F44" s="4" t="inlineStr">
@@ -3110,35 +3086,31 @@
       </c>
       <c r="H44" s="2" t="inlineStr">
         <is>
-          <t>Ed. Tivoli Fórum, Av. da Liberdade 180A, 7º, 1250-146</t>
+          <t>Av. D. João II, nº46, 1º B, 1990-095</t>
         </is>
       </c>
       <c r="I44" s="2" t="inlineStr">
         <is>
-          <t>22 projetos (Lisboa, Oeiras, Algarve, Comporta) (Em construção) | Infinity (Lisboa) (Comercialização)</t>
+          <t>Student + residential Lisboa (com TPG) (Planeamento) | Tannery Amial (Porto) (Em construção)</t>
         </is>
       </c>
       <c r="J44" s="2" t="inlineStr">
         <is>
-          <t>Entidade legal Vanguardeagle Asset Management (NIF 514114215). Tel. móvel 915 292 222</t>
+          <t>Sem telefone PT publicado</t>
         </is>
       </c>
       <c r="K44" s="2" t="inlineStr">
         <is>
-          <t>Henrique Rodrigues da Silva (CEO desde fev/2026)</t>
-        </is>
-      </c>
-      <c r="L44" s="2" t="inlineStr">
-        <is>
-          <t>https://www.linkedin.com/in/henrique-rodrigues-da-silva-b396643/</t>
-        </is>
-      </c>
+          <t>Michael Bickford (Founder &amp; CEO global· sem responsável PT confirmado)</t>
+        </is>
+      </c>
+      <c r="L44" s="2" t="inlineStr"/>
       <c r="M44" s="2" t="inlineStr"/>
     </row>
     <row r="45" ht="30" customHeight="1">
       <c r="A45" s="2" t="inlineStr">
         <is>
-          <t>VIC Properties</t>
+          <t>Royal Ventures</t>
         </is>
       </c>
       <c r="B45" s="3" t="inlineStr">
@@ -3148,52 +3120,52 @@
       </c>
       <c r="C45" s="4" t="inlineStr">
         <is>
-          <t>+351 219 347 112</t>
+          <t>+351 916 770 322</t>
         </is>
       </c>
       <c r="D45" s="2" t="inlineStr">
         <is>
-          <t>info@vic-properties.com</t>
+          <t>alex@royal-ventures.com</t>
         </is>
       </c>
       <c r="E45" s="2" t="inlineStr">
         <is>
-          <t>vic-properties.com</t>
+          <t>royal-ventures.com</t>
         </is>
       </c>
       <c r="F45" s="4" t="inlineStr">
         <is>
-          <t>Lisboa</t>
+          <t>Porto</t>
         </is>
       </c>
       <c r="G45" s="4" t="inlineStr">
         <is>
-          <t>Lisboa</t>
+          <t>Porto</t>
         </is>
       </c>
       <c r="H45" s="2" t="inlineStr">
         <is>
-          <t>Av. D. João II, Ed. Mythos 42, 4.03, Parque das Nações, 1990-095</t>
+          <t>Edifício Oceanus, Av. da Boavista 3227, 4100-137</t>
         </is>
       </c>
       <c r="I45" s="2" t="inlineStr">
         <is>
-          <t>Prata Riverside Village (Marvila) (Em construção)</t>
+          <t>Reabilitação centro histórico do Porto (Em construção)</t>
         </is>
       </c>
       <c r="J45" s="2" t="inlineStr">
         <is>
-          <t>Portefólio &gt;3B€. Fundada 2018</t>
+          <t>Sócios israelitas (Udi, Liad) + contacto PT Alexandre. Fonte: royal-ventures.com/contact-us</t>
         </is>
       </c>
       <c r="K45" s="2" t="inlineStr">
         <is>
-          <t>João Cabaça (Co-fundador e CEO)</t>
+          <t>Udi Yadin (fundador/General Partner)</t>
         </is>
       </c>
       <c r="L45" s="2" t="inlineStr">
         <is>
-          <t>https://pt.linkedin.com/in/jo%C3%A3o-caba%C3%A7a-6b293614b</t>
+          <t>https://www.linkedin.com/in/udiyadin/</t>
         </is>
       </c>
       <c r="M45" s="2" t="inlineStr"/>
@@ -3201,7 +3173,7 @@
     <row r="46" ht="30" customHeight="1">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>Vogue Homes</t>
+          <t>Screendomus (Grupo Teixeira)</t>
         </is>
       </c>
       <c r="B46" s="3" t="inlineStr">
@@ -3211,17 +3183,17 @@
       </c>
       <c r="C46" s="4" t="inlineStr">
         <is>
-          <t>+351 213 461 246</t>
+          <t>+351 928 110 064</t>
         </is>
       </c>
       <c r="D46" s="2" t="inlineStr">
         <is>
-          <t>comercial@vogue-homes.com</t>
+          <t>geral@screendomus.com</t>
         </is>
       </c>
       <c r="E46" s="2" t="inlineStr">
         <is>
-          <t>vogue-homes.com</t>
+          <t>screendomus.com</t>
         </is>
       </c>
       <c r="F46" s="4" t="inlineStr">
@@ -3234,589 +3206,761 @@
           <t>Lisboa</t>
         </is>
       </c>
-      <c r="H46" s="2" t="inlineStr">
-        <is>
-          <t>Rua Luz Soriano 15, 1200-246</t>
-        </is>
-      </c>
+      <c r="H46" s="2" t="inlineStr"/>
       <c r="I46" s="2" t="inlineStr">
         <is>
-          <t>Dafundo 24 (Comercialização) | Bom Sucesso (Comercialização) | Westhouse (Cascais) (Comercialização)</t>
+          <t>Altus (Alta de Lisboa) (Em construção)</t>
         </is>
       </c>
       <c r="J46" s="2" t="inlineStr">
         <is>
-          <t>NIF 510933084. Tel. móvel 913 385 846</t>
+          <t>Integra o Grupo Teixeira. Sem telefone confirmado — contacto via screendomus.com</t>
         </is>
       </c>
       <c r="K46" s="2" t="inlineStr">
         <is>
-          <t>Joaquim Lico (CEO)</t>
-        </is>
-      </c>
-      <c r="L46" s="2" t="inlineStr">
-        <is>
-          <t>https://www.linkedin.com/in/joaquim-lico-4383239/</t>
-        </is>
-      </c>
+          <t>Nuno Teixeira (Administrador, perfil LinkedIn não confirmado)</t>
+        </is>
+      </c>
+      <c r="L46" s="2" t="inlineStr"/>
       <c r="M46" s="2" t="inlineStr"/>
     </row>
     <row r="47" ht="30" customHeight="1">
       <c r="A47" s="2" t="inlineStr">
         <is>
+          <t>Sharp Developers</t>
+        </is>
+      </c>
+      <c r="B47" s="3" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+      <c r="C47" s="4" t="inlineStr">
+        <is>
+          <t>+351 933 078 094</t>
+        </is>
+      </c>
+      <c r="D47" s="2" t="inlineStr">
+        <is>
+          <t>info@sharpdevelopers.pt</t>
+        </is>
+      </c>
+      <c r="E47" s="2" t="inlineStr">
+        <is>
+          <t>sharpdevelopers.pt</t>
+        </is>
+      </c>
+      <c r="F47" s="4" t="inlineStr">
+        <is>
+          <t>Porto</t>
+        </is>
+      </c>
+      <c r="G47" s="4" t="inlineStr">
+        <is>
+          <t>Porto</t>
+        </is>
+      </c>
+      <c r="H47" s="2" t="inlineStr">
+        <is>
+          <t>Av. Boavista 1681, Ed. Bristol, Esc. 5.4</t>
+        </is>
+      </c>
+      <c r="I47" s="2" t="inlineStr">
+        <is>
+          <t>Residencial de luxo Porto (Em construção)</t>
+        </is>
+      </c>
+      <c r="J47" s="2" t="inlineStr">
+        <is>
+          <t>CEO Carla Luís</t>
+        </is>
+      </c>
+      <c r="K47" s="2" t="inlineStr">
+        <is>
+          <t>Carla Luís (CEO/cofundadora)</t>
+        </is>
+      </c>
+      <c r="L47" s="2" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/carla-luís-b14a7616/</t>
+        </is>
+      </c>
+      <c r="M47" s="2" t="inlineStr"/>
+    </row>
+    <row r="48" ht="30" customHeight="1">
+      <c r="A48" s="2" t="inlineStr">
+        <is>
+          <t>SILCOGE / Grupo SIL</t>
+        </is>
+      </c>
+      <c r="B48" s="3" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+      <c r="C48" s="4" t="inlineStr">
+        <is>
+          <t>+351 210 124 500</t>
+        </is>
+      </c>
+      <c r="D48" s="2" t="inlineStr">
+        <is>
+          <t>info@sil.pt</t>
+        </is>
+      </c>
+      <c r="E48" s="2" t="inlineStr">
+        <is>
+          <t>sil.pt</t>
+        </is>
+      </c>
+      <c r="F48" s="4" t="inlineStr">
+        <is>
+          <t>Lisboa</t>
+        </is>
+      </c>
+      <c r="G48" s="4" t="inlineStr">
+        <is>
+          <t>Lisboa</t>
+        </is>
+      </c>
+      <c r="H48" s="2" t="inlineStr">
+        <is>
+          <t>Av. Fontes Pereira de Melo 6, 5º, 1050-121</t>
+        </is>
+      </c>
+      <c r="I48" s="2" t="inlineStr">
+        <is>
+          <t>Grande Lisboa (Em construção)</t>
+        </is>
+      </c>
+      <c r="J48" s="2" t="inlineStr">
+        <is>
+          <t>Promoção imobiliária desde 1949</t>
+        </is>
+      </c>
+      <c r="K48" s="2" t="inlineStr">
+        <is>
+          <t>Pedro Silveira (acionista maioritário/ex-Chairman, destituído judicialmente mai/2025, em recurso)</t>
+        </is>
+      </c>
+      <c r="L48" s="2" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/pedro-silveira-88822a20/</t>
+        </is>
+      </c>
+      <c r="M48" s="2" t="inlineStr"/>
+    </row>
+    <row r="49" ht="30" customHeight="1">
+      <c r="A49" s="2" t="inlineStr">
+        <is>
+          <t>SOLYD Property Developers</t>
+        </is>
+      </c>
+      <c r="B49" s="3" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+      <c r="C49" s="4" t="inlineStr">
+        <is>
+          <t>+351 211 214 926</t>
+        </is>
+      </c>
+      <c r="D49" s="2" t="inlineStr">
+        <is>
+          <t>info@elou-solyd.pt</t>
+        </is>
+      </c>
+      <c r="E49" s="2" t="inlineStr">
+        <is>
+          <t>solyd.pt</t>
+        </is>
+      </c>
+      <c r="F49" s="4" t="inlineStr">
+        <is>
+          <t>Oeiras</t>
+        </is>
+      </c>
+      <c r="G49" s="4" t="inlineStr">
+        <is>
+          <t>Lisboa</t>
+        </is>
+      </c>
+      <c r="H49" s="2" t="inlineStr">
+        <is>
+          <t>Torre de Monsanto, Rua Afonso Praça 30, 7º, 1495-061 Algés</t>
+        </is>
+      </c>
+      <c r="I49" s="2" t="inlineStr">
+        <is>
+          <t>Luz Altear (Alta de Lisboa) (Em construção) | ÉLOU (Santo António dos Cavaleiros, Loures) (Em construção/Comercialização)</t>
+        </is>
+      </c>
+      <c r="J49" s="2" t="inlineStr">
+        <is>
+          <t>Estoril Capital Partners + Oaktree. Tel. alternativo 210 966 905</t>
+        </is>
+      </c>
+      <c r="K49" s="2" t="inlineStr">
+        <is>
+          <t>Gonçalo Cadete (CEO)</t>
+        </is>
+      </c>
+      <c r="L49" s="2" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/gon%C3%A7alo-cadete-260692/</t>
+        </is>
+      </c>
+      <c r="M49" s="2" t="inlineStr"/>
+    </row>
+    <row r="50" ht="30" customHeight="1">
+      <c r="A50" s="2" t="inlineStr">
+        <is>
+          <t>Stone Capital</t>
+        </is>
+      </c>
+      <c r="B50" s="3" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+      <c r="C50" s="4" t="inlineStr">
+        <is>
+          <t>+351 210 416 350</t>
+        </is>
+      </c>
+      <c r="D50" s="2" t="inlineStr">
+        <is>
+          <t>info@stonecapital.pt</t>
+        </is>
+      </c>
+      <c r="E50" s="2" t="inlineStr">
+        <is>
+          <t>stonecapital.pt</t>
+        </is>
+      </c>
+      <c r="F50" s="4" t="inlineStr">
+        <is>
+          <t>Lisboa</t>
+        </is>
+      </c>
+      <c r="G50" s="4" t="inlineStr">
+        <is>
+          <t>Lisboa</t>
+        </is>
+      </c>
+      <c r="H50" s="2" t="inlineStr">
+        <is>
+          <t>Av. da Liberdade 240, 1250-096</t>
+        </is>
+      </c>
+      <c r="I50" s="2" t="inlineStr">
+        <is>
+          <t>Santa Isabel (Em construção) | Portefólio em desenvolvimento (Em construção)</t>
+        </is>
+      </c>
+      <c r="J50" s="2" t="inlineStr">
+        <is>
+          <t>Tel. móvel 965 915 993</t>
+        </is>
+      </c>
+      <c r="K50" s="2" t="inlineStr">
+        <is>
+          <t>Geoffroy Moreno (Co-Founder)</t>
+        </is>
+      </c>
+      <c r="L50" s="2" t="inlineStr"/>
+      <c r="M50" s="2" t="inlineStr"/>
+    </row>
+    <row r="51" ht="30" customHeight="1">
+      <c r="A51" s="2" t="inlineStr">
+        <is>
+          <t>Teixeira Duarte Real Estate</t>
+        </is>
+      </c>
+      <c r="B51" s="3" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+      <c r="C51" s="4" t="inlineStr">
+        <is>
+          <t>+351 217 912 300</t>
+        </is>
+      </c>
+      <c r="D51" s="2" t="inlineStr">
+        <is>
+          <t>info@tdimobiliaria.pt</t>
+        </is>
+      </c>
+      <c r="E51" s="2" t="inlineStr">
+        <is>
+          <t>tdimobiliaria.pt</t>
+        </is>
+      </c>
+      <c r="F51" s="4" t="inlineStr">
+        <is>
+          <t>Oeiras</t>
+        </is>
+      </c>
+      <c r="G51" s="4" t="inlineStr">
+        <is>
+          <t>Lisboa</t>
+        </is>
+      </c>
+      <c r="H51" s="2" t="inlineStr">
+        <is>
+          <t>Lagoas Park, Edifício 2, 2740-265 Porto Salvo</t>
+        </is>
+      </c>
+      <c r="I51" s="2" t="inlineStr">
+        <is>
+          <t>Quinta de Cravel (V.N. Gaia) (Comercialização)</t>
+        </is>
+      </c>
+      <c r="J51" s="2" t="inlineStr">
+        <is>
+          <t>Braço imobiliário do grupo Teixeira Duarte</t>
+        </is>
+      </c>
+      <c r="K51" s="2" t="inlineStr"/>
+      <c r="L51" s="2" t="inlineStr"/>
+      <c r="M51" s="2" t="inlineStr"/>
+    </row>
+    <row r="52" ht="30" customHeight="1">
+      <c r="A52" s="2" t="inlineStr">
+        <is>
+          <t>Thomas &amp; Piron Portugal</t>
+        </is>
+      </c>
+      <c r="B52" s="3" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+      <c r="C52" s="4" t="inlineStr">
+        <is>
+          <t>+351 214 422 464</t>
+        </is>
+      </c>
+      <c r="D52" s="2" t="inlineStr">
+        <is>
+          <t>infopt@thomas-piron.eu</t>
+        </is>
+      </c>
+      <c r="E52" s="2" t="inlineStr">
+        <is>
+          <t>thomas-piron.pt</t>
+        </is>
+      </c>
+      <c r="F52" s="4" t="inlineStr">
+        <is>
+          <t>Matosinhos</t>
+        </is>
+      </c>
+      <c r="G52" s="4" t="inlineStr">
+        <is>
+          <t>Porto</t>
+        </is>
+      </c>
+      <c r="H52" s="2" t="inlineStr">
+        <is>
+          <t>Escritórios em Matosinhos e Sacavém</t>
+        </is>
+      </c>
+      <c r="I52" s="2" t="inlineStr">
+        <is>
+          <t>Docks Matosinhos (Em construção) | Gaia Hills (V.N. Gaia) (Em construção) | Conde de Lima (Comercialização)</t>
+        </is>
+      </c>
+      <c r="J52" s="2" t="inlineStr">
+        <is>
+          <t>Promotor belga em Portugal desde 2018. Fonte: diarioimobiliario.pt</t>
+        </is>
+      </c>
+      <c r="K52" s="2" t="inlineStr">
+        <is>
+          <t>David Carreira (Diretor Geral/Country Manager)</t>
+        </is>
+      </c>
+      <c r="L52" s="2" t="inlineStr">
+        <is>
+          <t>https://lu.linkedin.com/in/david-carreira-a4082050</t>
+        </is>
+      </c>
+      <c r="M52" s="2" t="inlineStr"/>
+    </row>
+    <row r="53" ht="30" customHeight="1">
+      <c r="A53" s="2" t="inlineStr">
+        <is>
+          <t>United Investments Portugal (UIP)</t>
+        </is>
+      </c>
+      <c r="B53" s="3" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+      <c r="C53" s="4" t="inlineStr">
+        <is>
+          <t>+351 215 834 534</t>
+        </is>
+      </c>
+      <c r="D53" s="2" t="inlineStr">
+        <is>
+          <t>reception.lisboa@uip.pt</t>
+        </is>
+      </c>
+      <c r="E53" s="2" t="inlineStr">
+        <is>
+          <t>uip.pt</t>
+        </is>
+      </c>
+      <c r="F53" s="4" t="inlineStr">
+        <is>
+          <t>Lisboa</t>
+        </is>
+      </c>
+      <c r="G53" s="4" t="inlineStr">
+        <is>
+          <t>Lisboa</t>
+        </is>
+      </c>
+      <c r="H53" s="2" t="inlineStr">
+        <is>
+          <t>Rua do Mar da China, Ed. Mar do Oriente nº1, Fração 3.2, Parque das Nações, 1990-137</t>
+        </is>
+      </c>
+      <c r="I53" s="2" t="inlineStr">
+        <is>
+          <t>Pine Cliffs (Algarve), Sheraton Cascais, YOTEL Porto, Hyatt Regency Lisboa (Em construção)</t>
+        </is>
+      </c>
+      <c r="J53" s="2" t="inlineStr">
+        <is>
+          <t>Fundada 1985</t>
+        </is>
+      </c>
+      <c r="K53" s="2" t="inlineStr">
+        <is>
+          <t>Carlos Leal (CEO)</t>
+        </is>
+      </c>
+      <c r="L53" s="2" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/carlos-leal-62797227/</t>
+        </is>
+      </c>
+      <c r="M53" s="2" t="inlineStr"/>
+    </row>
+    <row r="54" ht="30" customHeight="1">
+      <c r="A54" s="2" t="inlineStr">
+        <is>
+          <t>Vanguard Properties</t>
+        </is>
+      </c>
+      <c r="B54" s="3" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+      <c r="C54" s="4" t="inlineStr">
+        <is>
+          <t>+351 215 814 094</t>
+        </is>
+      </c>
+      <c r="D54" s="2" t="inlineStr">
+        <is>
+          <t>info@vangproperties.com</t>
+        </is>
+      </c>
+      <c r="E54" s="2" t="inlineStr">
+        <is>
+          <t>vangproperties.com</t>
+        </is>
+      </c>
+      <c r="F54" s="4" t="inlineStr">
+        <is>
+          <t>Lisboa</t>
+        </is>
+      </c>
+      <c r="G54" s="4" t="inlineStr">
+        <is>
+          <t>Lisboa</t>
+        </is>
+      </c>
+      <c r="H54" s="2" t="inlineStr">
+        <is>
+          <t>Ed. Tivoli Fórum, Av. da Liberdade 180A, 7º, 1250-146</t>
+        </is>
+      </c>
+      <c r="I54" s="2" t="inlineStr">
+        <is>
+          <t>22 projetos (Lisboa, Oeiras, Algarve, Comporta) (Em construção) | Infinity (Lisboa) (Comercialização)</t>
+        </is>
+      </c>
+      <c r="J54" s="2" t="inlineStr">
+        <is>
+          <t>Entidade legal Vanguardeagle Asset Management (NIF 514114215). Tel. móvel 915 292 222</t>
+        </is>
+      </c>
+      <c r="K54" s="2" t="inlineStr">
+        <is>
+          <t>Henrique Rodrigues da Silva (CEO desde fev/2026)</t>
+        </is>
+      </c>
+      <c r="L54" s="2" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/henrique-rodrigues-da-silva-b396643/</t>
+        </is>
+      </c>
+      <c r="M54" s="2" t="inlineStr"/>
+    </row>
+    <row r="55" ht="30" customHeight="1">
+      <c r="A55" s="2" t="inlineStr">
+        <is>
+          <t>VIC Properties</t>
+        </is>
+      </c>
+      <c r="B55" s="3" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+      <c r="C55" s="4" t="inlineStr">
+        <is>
+          <t>+351 219 347 112</t>
+        </is>
+      </c>
+      <c r="D55" s="2" t="inlineStr">
+        <is>
+          <t>info@vic-properties.com</t>
+        </is>
+      </c>
+      <c r="E55" s="2" t="inlineStr">
+        <is>
+          <t>vic-properties.com</t>
+        </is>
+      </c>
+      <c r="F55" s="4" t="inlineStr">
+        <is>
+          <t>Lisboa</t>
+        </is>
+      </c>
+      <c r="G55" s="4" t="inlineStr">
+        <is>
+          <t>Lisboa</t>
+        </is>
+      </c>
+      <c r="H55" s="2" t="inlineStr">
+        <is>
+          <t>Av. D. João II, Ed. Mythos 42, 4.03, Parque das Nações, 1990-095</t>
+        </is>
+      </c>
+      <c r="I55" s="2" t="inlineStr">
+        <is>
+          <t>Prata Riverside Village (Marvila) (Em construção)</t>
+        </is>
+      </c>
+      <c r="J55" s="2" t="inlineStr">
+        <is>
+          <t>Portefólio &gt;3B€. Fundada 2018</t>
+        </is>
+      </c>
+      <c r="K55" s="2" t="inlineStr">
+        <is>
+          <t>João Cabaça (Co-fundador e CEO)</t>
+        </is>
+      </c>
+      <c r="L55" s="2" t="inlineStr">
+        <is>
+          <t>https://pt.linkedin.com/in/jo%C3%A3o-caba%C3%A7a-6b293614b</t>
+        </is>
+      </c>
+      <c r="M55" s="2" t="inlineStr"/>
+    </row>
+    <row r="56" ht="30" customHeight="1">
+      <c r="A56" s="2" t="inlineStr">
+        <is>
+          <t>Visabeira Imobiliária (Visabeirahouse)</t>
+        </is>
+      </c>
+      <c r="B56" s="3" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+      <c r="C56" s="4" t="inlineStr">
+        <is>
+          <t>+351 218 429 970</t>
+        </is>
+      </c>
+      <c r="D56" s="2" t="inlineStr"/>
+      <c r="E56" s="2" t="inlineStr">
+        <is>
+          <t>grupovisabeira.com</t>
+        </is>
+      </c>
+      <c r="F56" s="4" t="inlineStr">
+        <is>
+          <t>Lisboa</t>
+        </is>
+      </c>
+      <c r="G56" s="4" t="inlineStr">
+        <is>
+          <t>Lisboa</t>
+        </is>
+      </c>
+      <c r="H56" s="2" t="inlineStr">
+        <is>
+          <t>Av. Almirante Gago Coutinho 78, 1700-031</t>
+        </is>
+      </c>
+      <c r="I56" s="2" t="inlineStr">
+        <is>
+          <t>Areeiro Select (Comercialização)</t>
+        </is>
+      </c>
+      <c r="J56" s="2" t="inlineStr">
+        <is>
+          <t>Fonte: idealista.pt</t>
+        </is>
+      </c>
+      <c r="K56" s="2" t="inlineStr">
+        <is>
+          <t>Paula Santos (Diretora Geral Visabeirahouse)</t>
+        </is>
+      </c>
+      <c r="L56" s="2" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/paula-santos-71083337/</t>
+        </is>
+      </c>
+      <c r="M56" s="2" t="inlineStr"/>
+    </row>
+    <row r="57" ht="30" customHeight="1">
+      <c r="A57" s="2" t="inlineStr">
+        <is>
+          <t>Vogue Homes</t>
+        </is>
+      </c>
+      <c r="B57" s="3" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+      <c r="C57" s="4" t="inlineStr">
+        <is>
+          <t>+351 213 461 246</t>
+        </is>
+      </c>
+      <c r="D57" s="2" t="inlineStr">
+        <is>
+          <t>comercial@vogue-homes.com</t>
+        </is>
+      </c>
+      <c r="E57" s="2" t="inlineStr">
+        <is>
+          <t>vogue-homes.com</t>
+        </is>
+      </c>
+      <c r="F57" s="4" t="inlineStr">
+        <is>
+          <t>Lisboa</t>
+        </is>
+      </c>
+      <c r="G57" s="4" t="inlineStr">
+        <is>
+          <t>Lisboa</t>
+        </is>
+      </c>
+      <c r="H57" s="2" t="inlineStr">
+        <is>
+          <t>Rua Luz Soriano 15, 1200-246</t>
+        </is>
+      </c>
+      <c r="I57" s="2" t="inlineStr">
+        <is>
+          <t>Dafundo 24 (Comercialização) | Bom Sucesso (Comercialização) | Westhouse (Cascais) (Comercialização)</t>
+        </is>
+      </c>
+      <c r="J57" s="2" t="inlineStr">
+        <is>
+          <t>NIF 510933084. Tel. móvel 913 385 846</t>
+        </is>
+      </c>
+      <c r="K57" s="2" t="inlineStr">
+        <is>
+          <t>Joaquim Lico (CEO)</t>
+        </is>
+      </c>
+      <c r="L57" s="2" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/joaquim-lico-4383239/</t>
+        </is>
+      </c>
+      <c r="M57" s="2" t="inlineStr"/>
+    </row>
+    <row r="58" ht="30" customHeight="1">
+      <c r="A58" s="2" t="inlineStr">
+        <is>
           <t>YARD Properties</t>
         </is>
       </c>
-      <c r="B47" s="3" t="inlineStr">
+      <c r="B58" s="3" t="inlineStr">
         <is>
           <t>Sim</t>
         </is>
       </c>
-      <c r="C47" s="4" t="inlineStr">
+      <c r="C58" s="4" t="inlineStr">
         <is>
           <t>+351 918 888 353</t>
         </is>
       </c>
-      <c r="D47" s="2" t="inlineStr">
+      <c r="D58" s="2" t="inlineStr">
         <is>
           <t>sales@355outubro.com</t>
         </is>
       </c>
-      <c r="E47" s="2" t="inlineStr">
+      <c r="E58" s="2" t="inlineStr">
         <is>
           <t>yardproperties.pt</t>
         </is>
       </c>
-      <c r="F47" s="4" t="inlineStr">
-        <is>
-          <t>Lisboa</t>
-        </is>
-      </c>
-      <c r="G47" s="4" t="inlineStr">
-        <is>
-          <t>Lisboa</t>
-        </is>
-      </c>
-      <c r="H47" s="2" t="inlineStr"/>
-      <c r="I47" s="2" t="inlineStr">
+      <c r="F58" s="4" t="inlineStr">
+        <is>
+          <t>Lisboa</t>
+        </is>
+      </c>
+      <c r="G58" s="4" t="inlineStr">
+        <is>
+          <t>Lisboa</t>
+        </is>
+      </c>
+      <c r="H58" s="2" t="inlineStr"/>
+      <c r="I58" s="2" t="inlineStr">
         <is>
           <t>355 Outubro (Av. 5 de Outubro, Lisboa) (Em construção)</t>
         </is>
       </c>
-      <c r="J47" s="2" t="inlineStr">
+      <c r="J58" s="2" t="inlineStr">
         <is>
           <t>Grupo israelita liderado por David Rabbi. Telefone é da linha comercial do projeto 355 Outubro</t>
         </is>
       </c>
-      <c r="K47" s="2" t="inlineStr">
+      <c r="K58" s="2" t="inlineStr">
         <is>
           <t>David Rabbi (fundador)</t>
         </is>
       </c>
-      <c r="L47" s="2" t="inlineStr"/>
-      <c r="M47" s="2" t="inlineStr"/>
-    </row>
-    <row r="48" ht="30" customHeight="1">
-      <c r="A48" s="5" t="inlineStr">
-        <is>
-          <t>AFA (Grupo AFA)</t>
-        </is>
-      </c>
-      <c r="B48" s="6" t="inlineStr">
-        <is>
-          <t>Sim</t>
-        </is>
-      </c>
-      <c r="C48" s="7" t="inlineStr"/>
-      <c r="D48" s="5" t="inlineStr"/>
-      <c r="E48" s="5" t="inlineStr"/>
-      <c r="F48" s="7" t="inlineStr">
-        <is>
-          <t>Lisboa</t>
-        </is>
-      </c>
-      <c r="G48" s="7" t="inlineStr">
-        <is>
-          <t>Lisboa</t>
-        </is>
-      </c>
-      <c r="H48" s="5" t="inlineStr"/>
-      <c r="I48" s="5" t="inlineStr">
-        <is>
-          <t>Savoy Residence D'Ávila (Em construção)</t>
-        </is>
-      </c>
-      <c r="J48" s="5" t="inlineStr">
-        <is>
-          <t>Fonte: diarioimobiliario.pt</t>
-        </is>
-      </c>
-      <c r="K48" s="5" t="inlineStr">
-        <is>
-          <t>Victor de Sousa (Diretor-Geral AFA Real Estate)</t>
-        </is>
-      </c>
-      <c r="L48" s="5" t="inlineStr"/>
-      <c r="M48" s="5" t="inlineStr"/>
-    </row>
-    <row r="49" ht="30" customHeight="1">
-      <c r="A49" s="5" t="inlineStr">
-        <is>
-          <t>Alecrim Real Estate (Lince Capital)</t>
-        </is>
-      </c>
-      <c r="B49" s="6" t="inlineStr">
-        <is>
-          <t>Sim</t>
-        </is>
-      </c>
-      <c r="C49" s="7" t="inlineStr"/>
-      <c r="D49" s="5" t="inlineStr"/>
-      <c r="E49" s="5" t="inlineStr">
-        <is>
-          <t>lince-capital.com</t>
-        </is>
-      </c>
-      <c r="F49" s="7" t="inlineStr">
-        <is>
-          <t>Lisboa</t>
-        </is>
-      </c>
-      <c r="G49" s="7" t="inlineStr">
-        <is>
-          <t>Lisboa</t>
-        </is>
-      </c>
-      <c r="H49" s="5" t="inlineStr">
-        <is>
-          <t>Av. Eng.º Duarte Pacheco, Torre 2, piso 17, 1070-102</t>
-        </is>
-      </c>
-      <c r="I49" s="5" t="inlineStr">
-        <is>
-          <t>Metrass (Campo de Ourique) (Em construção) | 8 projetos em pipeline (Planeamento)</t>
-        </is>
-      </c>
-      <c r="J49" s="5" t="inlineStr">
-        <is>
-          <t>Nova promotora (jan/2026), CEO António Velho da Palma</t>
-        </is>
-      </c>
-      <c r="K49" s="5" t="inlineStr">
-        <is>
-          <t>António Velho da Palma (CEO Alecrim RE)· CEO da holding Lince Capital é Vasco Pereira Coutinho</t>
-        </is>
-      </c>
-      <c r="L49" s="5" t="inlineStr">
-        <is>
-          <t>https://www.linkedin.com/in/ant%C3%B3nio-velho-da-palma-82112282/</t>
-        </is>
-      </c>
-      <c r="M49" s="5" t="inlineStr"/>
-    </row>
-    <row r="50" ht="30" customHeight="1">
-      <c r="A50" s="5" t="inlineStr">
-        <is>
-          <t>Arts Investments, SA</t>
-        </is>
-      </c>
-      <c r="B50" s="6" t="inlineStr">
-        <is>
-          <t>Sim</t>
-        </is>
-      </c>
-      <c r="C50" s="7" t="inlineStr"/>
-      <c r="D50" s="5" t="inlineStr"/>
-      <c r="E50" s="5" t="inlineStr">
-        <is>
-          <t>artsinvestments.com</t>
-        </is>
-      </c>
-      <c r="F50" s="7" t="inlineStr">
-        <is>
-          <t>Lisboa</t>
-        </is>
-      </c>
-      <c r="G50" s="7" t="inlineStr">
-        <is>
-          <t>Lisboa</t>
-        </is>
-      </c>
-      <c r="H50" s="5" t="inlineStr"/>
-      <c r="I50" s="5" t="inlineStr">
-        <is>
-          <t>3 projetos em curso (nomes não encontrados) (Em construção/desenvolvimento)</t>
-        </is>
-      </c>
-      <c r="J50" s="5" t="inlineStr">
-        <is>
-          <t>Fonte: vidaimobiliaria.com</t>
-        </is>
-      </c>
-      <c r="K50" s="5" t="inlineStr"/>
-      <c r="L50" s="5" t="inlineStr"/>
-      <c r="M50" s="5" t="inlineStr"/>
-    </row>
-    <row r="51" ht="30" customHeight="1">
-      <c r="A51" s="5" t="inlineStr">
-        <is>
-          <t>Ceetrus / Nhood Portugal</t>
-        </is>
-      </c>
-      <c r="B51" s="6" t="inlineStr">
-        <is>
-          <t>Sim</t>
-        </is>
-      </c>
-      <c r="C51" s="7" t="inlineStr"/>
-      <c r="D51" s="5" t="inlineStr"/>
-      <c r="E51" s="5" t="inlineStr"/>
-      <c r="F51" s="7" t="inlineStr">
-        <is>
-          <t>Lisboa</t>
-        </is>
-      </c>
-      <c r="G51" s="7" t="inlineStr">
-        <is>
-          <t>nacional</t>
-        </is>
-      </c>
-      <c r="H51" s="5" t="inlineStr"/>
-      <c r="I51" s="5" t="inlineStr">
-        <is>
-          <t>Pipeline nacional 15 cidades (nomes não encontrados) (Planeamento)</t>
-        </is>
-      </c>
-      <c r="J51" s="5" t="inlineStr">
-        <is>
-          <t>Fonte: idealista.pt</t>
-        </is>
-      </c>
-      <c r="K51" s="5" t="inlineStr"/>
-      <c r="L51" s="5" t="inlineStr"/>
-      <c r="M51" s="5" t="inlineStr"/>
-    </row>
-    <row r="52" ht="30" customHeight="1">
-      <c r="A52" s="5" t="inlineStr">
-        <is>
-          <t>Década Paralela (Grupo Latitude, com a TPS)</t>
-        </is>
-      </c>
-      <c r="B52" s="6" t="inlineStr">
-        <is>
-          <t>Sim</t>
-        </is>
-      </c>
-      <c r="C52" s="7" t="inlineStr"/>
-      <c r="D52" s="5" t="inlineStr"/>
-      <c r="E52" s="5" t="inlineStr"/>
-      <c r="F52" s="7" t="inlineStr">
-        <is>
-          <t>Porto</t>
-        </is>
-      </c>
-      <c r="G52" s="7" t="inlineStr">
-        <is>
-          <t>Porto</t>
-        </is>
-      </c>
-      <c r="H52" s="5" t="inlineStr"/>
-      <c r="I52" s="5" t="inlineStr">
-        <is>
-          <t>Fábrica Vilar (Em desenvolvimento)</t>
-        </is>
-      </c>
-      <c r="J52" s="5" t="inlineStr">
-        <is>
-          <t>Fonte: viva-porto.pt</t>
-        </is>
-      </c>
-      <c r="K52" s="5" t="inlineStr">
-        <is>
-          <t>Bruno Soares (CEO, família Soares/Latitude Capital)</t>
-        </is>
-      </c>
-      <c r="L52" s="5" t="inlineStr"/>
-      <c r="M52" s="5" t="inlineStr"/>
-    </row>
-    <row r="53" ht="30" customHeight="1">
-      <c r="A53" s="5" t="inlineStr">
-        <is>
-          <t>Fortera</t>
-        </is>
-      </c>
-      <c r="B53" s="6" t="inlineStr">
-        <is>
-          <t>Sim</t>
-        </is>
-      </c>
-      <c r="C53" s="7" t="inlineStr"/>
-      <c r="D53" s="5" t="inlineStr"/>
-      <c r="E53" s="5" t="inlineStr"/>
-      <c r="F53" s="7" t="inlineStr">
-        <is>
-          <t>Vila Nova de Gaia</t>
-        </is>
-      </c>
-      <c r="G53" s="7" t="inlineStr">
-        <is>
-          <t>Porto</t>
-        </is>
-      </c>
-      <c r="H53" s="5" t="inlineStr">
-        <is>
-          <t>Porto / Gaia</t>
-        </is>
-      </c>
-      <c r="I53" s="5" t="inlineStr">
-        <is>
-          <t>Skyline (V.N. Gaia) (Em construção) | 20 projetos (Porto, Gaia, Espinho, Braga) (Em construção) | Convento do Carmo (Braga) (Em construção)</t>
-        </is>
-      </c>
-      <c r="J53" s="5" t="inlineStr">
-        <is>
-          <t>Israelita (Elad Dror). Sem telefone publicado nas fontes</t>
-        </is>
-      </c>
-      <c r="K53" s="5" t="inlineStr">
-        <is>
-          <t>Pedro Ferreira (CEO desde jun/2023· fundador anterior Elad Dror saiu em 2023)</t>
-        </is>
-      </c>
-      <c r="L53" s="5" t="inlineStr"/>
-      <c r="M53" s="5" t="inlineStr"/>
-    </row>
-    <row r="54" ht="30" customHeight="1">
-      <c r="A54" s="5" t="inlineStr">
-        <is>
-          <t>Fungepi (Grupo Novo Banco)</t>
-        </is>
-      </c>
-      <c r="B54" s="6" t="inlineStr">
-        <is>
-          <t>Sim</t>
-        </is>
-      </c>
-      <c r="C54" s="7" t="inlineStr"/>
-      <c r="D54" s="5" t="inlineStr"/>
-      <c r="E54" s="5" t="inlineStr"/>
-      <c r="F54" s="7" t="inlineStr">
-        <is>
-          <t>Lisboa</t>
-        </is>
-      </c>
-      <c r="G54" s="7" t="inlineStr">
-        <is>
-          <t>Lisboa</t>
-        </is>
-      </c>
-      <c r="H54" s="5" t="inlineStr">
-        <is>
-          <t>Rua de Artilharia 1, Campolide</t>
-        </is>
-      </c>
-      <c r="I54" s="5" t="inlineStr">
-        <is>
-          <t>Urbanização Artilharia Um / Amoreiras (Campolide) (Planeamento (consulta pública fev-mar/2026))</t>
-        </is>
-      </c>
-      <c r="J54" s="5" t="inlineStr">
-        <is>
-          <t>Fundo de Gestão de Património Imobiliário do Grupo Novo Banco. Projeto contestado por moradores (petição + queixa à CE)</t>
-        </is>
-      </c>
-      <c r="K54" s="5" t="inlineStr"/>
-      <c r="L54" s="5" t="inlineStr"/>
-      <c r="M54" s="5" t="inlineStr"/>
-    </row>
-    <row r="55" ht="30" customHeight="1">
-      <c r="A55" s="5" t="inlineStr">
-        <is>
-          <t>Hines Portugal</t>
-        </is>
-      </c>
-      <c r="B55" s="6" t="inlineStr">
-        <is>
-          <t>Sim</t>
-        </is>
-      </c>
-      <c r="C55" s="7" t="inlineStr"/>
-      <c r="D55" s="5" t="inlineStr"/>
-      <c r="E55" s="5" t="inlineStr">
-        <is>
-          <t>hines.com</t>
-        </is>
-      </c>
-      <c r="F55" s="7" t="inlineStr">
-        <is>
-          <t>Lisboa</t>
-        </is>
-      </c>
-      <c r="G55" s="7" t="inlineStr">
-        <is>
-          <t>Lisboa</t>
-        </is>
-      </c>
-      <c r="H55" s="5" t="inlineStr">
-        <is>
-          <t>Lisboa</t>
-        </is>
-      </c>
-      <c r="I55" s="5" t="inlineStr">
-        <is>
-          <t>Residência de estudantes Paranhos (Porto) (Em construção) | Castilho 3 (Lisboa) (Em construção)</t>
-        </is>
-      </c>
-      <c r="J55" s="5" t="inlineStr">
-        <is>
-          <t>Gestora global · sem contacto PT publicado</t>
-        </is>
-      </c>
-      <c r="K55" s="5" t="inlineStr">
-        <is>
-          <t>Vanessa Gelado (Senior Managing Director, Head of Southern Europe)</t>
-        </is>
-      </c>
-      <c r="L55" s="5" t="inlineStr"/>
-      <c r="M55" s="5" t="inlineStr"/>
-    </row>
-    <row r="56" ht="30" customHeight="1">
-      <c r="A56" s="5" t="inlineStr">
-        <is>
-          <t>Imolote</t>
-        </is>
-      </c>
-      <c r="B56" s="6" t="inlineStr">
-        <is>
-          <t>Sim</t>
-        </is>
-      </c>
-      <c r="C56" s="7" t="inlineStr"/>
-      <c r="D56" s="5" t="inlineStr"/>
-      <c r="E56" s="5" t="inlineStr">
-        <is>
-          <t>imolote.pt</t>
-        </is>
-      </c>
-      <c r="F56" s="7" t="inlineStr">
-        <is>
-          <t>Porto</t>
-        </is>
-      </c>
-      <c r="G56" s="7" t="inlineStr">
-        <is>
-          <t>Porto</t>
-        </is>
-      </c>
-      <c r="H56" s="5" t="inlineStr"/>
-      <c r="I56" s="5" t="inlineStr">
-        <is>
-          <t>Monte da Virgem Flats (V.N. Gaia) (Em construção) | 21 projetos entregues (Concluído)</t>
-        </is>
-      </c>
-      <c r="J56" s="5" t="inlineStr">
-        <is>
-          <t>Co-promoção com investidores · CEO Paulo Vaz Ferreira</t>
-        </is>
-      </c>
-      <c r="K56" s="5" t="inlineStr">
-        <is>
-          <t>Paulo Vaz Ferreira (sócio e CEO desde 2019, confiança moderada)</t>
-        </is>
-      </c>
-      <c r="L56" s="5" t="inlineStr"/>
-      <c r="M56" s="5" t="inlineStr"/>
-    </row>
-    <row r="57" ht="30" customHeight="1">
-      <c r="A57" s="5" t="inlineStr">
-        <is>
-          <t>João Magalhães &amp; Alexandre Magalhães (promotores individuais)</t>
-        </is>
-      </c>
-      <c r="B57" s="6" t="inlineStr">
-        <is>
-          <t>Sim</t>
-        </is>
-      </c>
-      <c r="C57" s="7" t="inlineStr"/>
-      <c r="D57" s="5" t="inlineStr"/>
-      <c r="E57" s="5" t="inlineStr"/>
-      <c r="F57" s="7" t="inlineStr">
-        <is>
-          <t>Porto</t>
-        </is>
-      </c>
-      <c r="G57" s="7" t="inlineStr">
-        <is>
-          <t>Porto</t>
-        </is>
-      </c>
-      <c r="H57" s="5" t="inlineStr"/>
-      <c r="I57" s="5" t="inlineStr">
-        <is>
-          <t>Bonjardim 362 (Em construção (conclusão 4T2026))</t>
-        </is>
-      </c>
-      <c r="J57" s="5" t="inlineStr">
-        <is>
-          <t>Fonte: construir.pt</t>
-        </is>
-      </c>
-      <c r="K57" s="5" t="inlineStr">
-        <is>
-          <t>João Magalhães e Alexandre Magalhães (promotores individuais)</t>
-        </is>
-      </c>
-      <c r="L57" s="5" t="inlineStr"/>
-      <c r="M57" s="5" t="inlineStr"/>
-    </row>
-    <row r="58" ht="30" customHeight="1">
-      <c r="A58" s="5" t="inlineStr">
-        <is>
-          <t>KKR Imo, S.A.</t>
-        </is>
-      </c>
-      <c r="B58" s="6" t="inlineStr">
-        <is>
-          <t>Sim</t>
-        </is>
-      </c>
-      <c r="C58" s="7" t="inlineStr"/>
-      <c r="D58" s="5" t="inlineStr"/>
-      <c r="E58" s="5" t="inlineStr"/>
-      <c r="F58" s="7" t="inlineStr">
-        <is>
-          <t>Lisboa</t>
-        </is>
-      </c>
-      <c r="G58" s="7" t="inlineStr">
-        <is>
-          <t>Lisboa</t>
-        </is>
-      </c>
-      <c r="H58" s="5" t="inlineStr"/>
-      <c r="I58" s="5" t="inlineStr">
-        <is>
-          <t>Smart Studios (Janelas Verdes) (Comercialização/Operação)</t>
-        </is>
-      </c>
-      <c r="J58" s="5" t="inlineStr">
-        <is>
-          <t>Fonte: vidaimobiliaria.com</t>
-        </is>
-      </c>
-      <c r="K58" s="5" t="inlineStr">
-        <is>
-          <t>Vera Kendall (administradora, dados de 2018 · confiança baixa)</t>
-        </is>
-      </c>
-      <c r="L58" s="5" t="inlineStr"/>
-      <c r="M58" s="5" t="inlineStr"/>
+      <c r="L58" s="2" t="inlineStr"/>
+      <c r="M58" s="2" t="inlineStr"/>
     </row>
     <row r="59" ht="30" customHeight="1">
       <c r="A59" s="5" t="inlineStr">
         <is>
-          <t>Neptune Developments</t>
+          <t>Alecrim Real Estate (Lince Capital)</t>
         </is>
       </c>
       <c r="B59" s="6" t="inlineStr">
@@ -3828,12 +3972,12 @@
       <c r="D59" s="5" t="inlineStr"/>
       <c r="E59" s="5" t="inlineStr">
         <is>
-          <t>neptune-developments.com</t>
+          <t>lince-capital.com</t>
         </is>
       </c>
       <c r="F59" s="7" t="inlineStr">
         <is>
-          <t>Cascais</t>
+          <t>Lisboa</t>
         </is>
       </c>
       <c r="G59" s="7" t="inlineStr">
@@ -3841,25 +3985,37 @@
           <t>Lisboa</t>
         </is>
       </c>
-      <c r="H59" s="5" t="inlineStr"/>
+      <c r="H59" s="5" t="inlineStr">
+        <is>
+          <t>Av. Eng.º Duarte Pacheco, Torre 2, piso 17, 1070-102</t>
+        </is>
+      </c>
       <c r="I59" s="5" t="inlineStr">
         <is>
-          <t>BellaMary (Cascais) (Comercialização)</t>
+          <t>Metrass (Campo de Ourique) (Em construção) | 8 projetos em pipeline (Planeamento)</t>
         </is>
       </c>
       <c r="J59" s="5" t="inlineStr">
         <is>
-          <t>Sem telefone/CEO confirmados nas fontes</t>
-        </is>
-      </c>
-      <c r="K59" s="5" t="inlineStr"/>
-      <c r="L59" s="5" t="inlineStr"/>
+          <t>Nova promotora (jan/2026), CEO António Velho da Palma</t>
+        </is>
+      </c>
+      <c r="K59" s="5" t="inlineStr">
+        <is>
+          <t>António Velho da Palma (CEO Alecrim RE)· CEO da holding Lince Capital é Vasco Pereira Coutinho</t>
+        </is>
+      </c>
+      <c r="L59" s="5" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/ant%C3%B3nio-velho-da-palma-82112282/</t>
+        </is>
+      </c>
       <c r="M59" s="5" t="inlineStr"/>
     </row>
     <row r="60" ht="30" customHeight="1">
       <c r="A60" s="5" t="inlineStr">
         <is>
-          <t>Onyria Group</t>
+          <t>Década Paralela (Grupo Latitude, com a TPS)</t>
         </is>
       </c>
       <c r="B60" s="6" t="inlineStr">
@@ -3869,35 +4025,31 @@
       </c>
       <c r="C60" s="7" t="inlineStr"/>
       <c r="D60" s="5" t="inlineStr"/>
-      <c r="E60" s="5" t="inlineStr">
-        <is>
-          <t>onyriagroup.com</t>
-        </is>
-      </c>
+      <c r="E60" s="5" t="inlineStr"/>
       <c r="F60" s="7" t="inlineStr">
         <is>
-          <t>Cascais</t>
+          <t>Porto</t>
         </is>
       </c>
       <c r="G60" s="7" t="inlineStr">
         <is>
-          <t>Lisboa</t>
+          <t>Porto</t>
         </is>
       </c>
       <c r="H60" s="5" t="inlineStr"/>
       <c r="I60" s="5" t="inlineStr">
         <is>
-          <t>Onyria Quinta da Marinha Residences (Cascais) (Comercialização)</t>
+          <t>Fábrica Vilar (Em desenvolvimento)</t>
         </is>
       </c>
       <c r="J60" s="5" t="inlineStr">
         <is>
-          <t>Grupo hoteleiro+imobiliário fundado 1986 por José Carlos Pinto Coelho</t>
+          <t>Fonte: viva-porto.pt</t>
         </is>
       </c>
       <c r="K60" s="5" t="inlineStr">
         <is>
-          <t>José Carlos Pinto Coelho (fundador, 1986)</t>
+          <t>Bruno Soares (CEO, família Soares/Latitude Capital)</t>
         </is>
       </c>
       <c r="L60" s="5" t="inlineStr"/>
@@ -3906,7 +4058,7 @@
     <row r="61" ht="30" customHeight="1">
       <c r="A61" s="5" t="inlineStr">
         <is>
-          <t>Overseas</t>
+          <t>Fungepi (Grupo Novo Banco)</t>
         </is>
       </c>
       <c r="B61" s="6" t="inlineStr">
@@ -3929,35 +4081,27 @@
       </c>
       <c r="H61" s="5" t="inlineStr">
         <is>
-          <t>Rua Alexandre Herculano 25, 1º, 1250-008</t>
+          <t>Rua de Artilharia 1, Campolide</t>
         </is>
       </c>
       <c r="I61" s="5" t="inlineStr">
         <is>
-          <t>5 projetos premium (4 Lisboa + Comporta) (Em construção) | JV com Grupo André Guimarães (Lisboa) (Planeamento) | Karl Lagerfeld branded residences (Planeamento) | Telhal 72 Liberdade (Comercialização)</t>
+          <t>Urbanização Artilharia Um / Amoreiras (Campolide) (Planeamento (consulta pública fev-mar/2026))</t>
         </is>
       </c>
       <c r="J61" s="5" t="inlineStr">
         <is>
-          <t>CEO Pedro Vicente (vice-presidente APPII). Sem telefone publicado</t>
-        </is>
-      </c>
-      <c r="K61" s="5" t="inlineStr">
-        <is>
-          <t>Pedro Vicente (CEO)</t>
-        </is>
-      </c>
-      <c r="L61" s="5" t="inlineStr">
-        <is>
-          <t>https://www.linkedin.com/in/pedro-vicente-9aa0b424/</t>
-        </is>
-      </c>
+          <t>Fundo de Gestão de Património Imobiliário do Grupo Novo Banco. Projeto contestado por moradores (petição + queixa à CE)</t>
+        </is>
+      </c>
+      <c r="K61" s="5" t="inlineStr"/>
+      <c r="L61" s="5" t="inlineStr"/>
       <c r="M61" s="5" t="inlineStr"/>
     </row>
     <row r="62" ht="30" customHeight="1">
       <c r="A62" s="5" t="inlineStr">
         <is>
-          <t>Portaviv</t>
+          <t>Hines Portugal</t>
         </is>
       </c>
       <c r="B62" s="6" t="inlineStr">
@@ -3967,31 +4111,39 @@
       </c>
       <c r="C62" s="7" t="inlineStr"/>
       <c r="D62" s="5" t="inlineStr"/>
-      <c r="E62" s="5" t="inlineStr"/>
+      <c r="E62" s="5" t="inlineStr">
+        <is>
+          <t>hines.com</t>
+        </is>
+      </c>
       <c r="F62" s="7" t="inlineStr">
         <is>
-          <t>Porto</t>
+          <t>Lisboa</t>
         </is>
       </c>
       <c r="G62" s="7" t="inlineStr">
         <is>
-          <t>Porto</t>
-        </is>
-      </c>
-      <c r="H62" s="5" t="inlineStr"/>
+          <t>Lisboa</t>
+        </is>
+      </c>
+      <c r="H62" s="5" t="inlineStr">
+        <is>
+          <t>Lisboa</t>
+        </is>
+      </c>
       <c r="I62" s="5" t="inlineStr">
         <is>
-          <t>The Factory Residences Campanhã (Em carteira/comercialização)</t>
+          <t>Residência de estudantes Paranhos (Porto) (Em construção) | Castilho 3 (Lisboa) (Em construção)</t>
         </is>
       </c>
       <c r="J62" s="5" t="inlineStr">
         <is>
-          <t>Fonte: construir.pt</t>
+          <t>Gestora global · sem contacto PT publicado</t>
         </is>
       </c>
       <c r="K62" s="5" t="inlineStr">
         <is>
-          <t>Nuno Cunha (Managing Director)</t>
+          <t>Vanessa Gelado (Senior Managing Director, Head of Southern Europe)</t>
         </is>
       </c>
       <c r="L62" s="5" t="inlineStr"/>
@@ -4000,7 +4152,7 @@
     <row r="63" ht="30" customHeight="1">
       <c r="A63" s="5" t="inlineStr">
         <is>
-          <t>Prime Portugal</t>
+          <t>Imolote</t>
         </is>
       </c>
       <c r="B63" s="6" t="inlineStr">
@@ -4010,35 +4162,35 @@
       </c>
       <c r="C63" s="7" t="inlineStr"/>
       <c r="D63" s="5" t="inlineStr"/>
-      <c r="E63" s="5" t="inlineStr"/>
+      <c r="E63" s="5" t="inlineStr">
+        <is>
+          <t>imolote.pt</t>
+        </is>
+      </c>
       <c r="F63" s="7" t="inlineStr">
         <is>
-          <t>Lisboa</t>
+          <t>Porto</t>
         </is>
       </c>
       <c r="G63" s="7" t="inlineStr">
         <is>
-          <t>Lisboa</t>
-        </is>
-      </c>
-      <c r="H63" s="5" t="inlineStr">
-        <is>
-          <t>Av. Fontes Pereira de Melo 6, 1600-001</t>
-        </is>
-      </c>
+          <t>Porto</t>
+        </is>
+      </c>
+      <c r="H63" s="5" t="inlineStr"/>
       <c r="I63" s="5" t="inlineStr">
         <is>
-          <t>Projetos residenciais Lisboa, Cascais e Melides (Em construção)</t>
+          <t>Monte da Virgem Flats (V.N. Gaia) (Em construção) | 21 projetos entregues (Concluído)</t>
         </is>
       </c>
       <c r="J63" s="5" t="inlineStr">
         <is>
-          <t>Sem telefone/site publicados (APPII)</t>
+          <t>Co-promoção com investidores · CEO Paulo Vaz Ferreira</t>
         </is>
       </c>
       <c r="K63" s="5" t="inlineStr">
         <is>
-          <t>Federico Rosales (cofundador e CEO)</t>
+          <t>Paulo Vaz Ferreira (sócio e CEO desde 2019, confiança moderada)</t>
         </is>
       </c>
       <c r="L63" s="5" t="inlineStr"/>
@@ -4047,7 +4199,7 @@
     <row r="64" ht="30" customHeight="1">
       <c r="A64" s="5" t="inlineStr">
         <is>
-          <t>RAR Imobiliária</t>
+          <t>João Magalhães &amp; Alexandre Magalhães (promotores individuais)</t>
         </is>
       </c>
       <c r="B64" s="6" t="inlineStr">
@@ -4071,17 +4223,17 @@
       <c r="H64" s="5" t="inlineStr"/>
       <c r="I64" s="5" t="inlineStr">
         <is>
-          <t>Montebelo Villas (Foz Velha) (Em construção)</t>
+          <t>Bonjardim 362 (Em construção (conclusão 4T2026))</t>
         </is>
       </c>
       <c r="J64" s="5" t="inlineStr">
         <is>
-          <t>Fonte: dinheirovivo.pt, construir.pt</t>
+          <t>Fonte: construir.pt</t>
         </is>
       </c>
       <c r="K64" s="5" t="inlineStr">
         <is>
-          <t>Paula Fernandes (CEO)</t>
+          <t>João Magalhães e Alexandre Magalhães (promotores individuais)</t>
         </is>
       </c>
       <c r="L64" s="5" t="inlineStr"/>
@@ -4090,7 +4242,7 @@
     <row r="65" ht="30" customHeight="1">
       <c r="A65" s="5" t="inlineStr">
         <is>
-          <t>REDASSET</t>
+          <t>KKR Imo, S.A.</t>
         </is>
       </c>
       <c r="B65" s="6" t="inlineStr">
@@ -4103,7 +4255,7 @@
       <c r="E65" s="5" t="inlineStr"/>
       <c r="F65" s="7" t="inlineStr">
         <is>
-          <t>Amadora</t>
+          <t>Lisboa</t>
         </is>
       </c>
       <c r="G65" s="7" t="inlineStr">
@@ -4114,22 +4266,26 @@
       <c r="H65" s="5" t="inlineStr"/>
       <c r="I65" s="5" t="inlineStr">
         <is>
-          <t>Moinho do Guizo (Mina de Água, Amadora) (Planeamento)</t>
+          <t>Smart Studios (Janelas Verdes) (Comercialização/Operação)</t>
         </is>
       </c>
       <c r="J65" s="5" t="inlineStr">
         <is>
-          <t>Promotor privado em terreno próprio, comercialização sob termos legais definidos</t>
-        </is>
-      </c>
-      <c r="K65" s="5" t="inlineStr"/>
+          <t>Fonte: vidaimobiliaria.com</t>
+        </is>
+      </c>
+      <c r="K65" s="5" t="inlineStr">
+        <is>
+          <t>Vera Kendall (administradora, dados de 2018 · confiança baixa)</t>
+        </is>
+      </c>
       <c r="L65" s="5" t="inlineStr"/>
       <c r="M65" s="5" t="inlineStr"/>
     </row>
     <row r="66" ht="30" customHeight="1">
       <c r="A66" s="5" t="inlineStr">
         <is>
-          <t>RM Promo (JV M2O Group / RJB Home)</t>
+          <t>Neptune Developments</t>
         </is>
       </c>
       <c r="B66" s="6" t="inlineStr">
@@ -4139,26 +4295,30 @@
       </c>
       <c r="C66" s="7" t="inlineStr"/>
       <c r="D66" s="5" t="inlineStr"/>
-      <c r="E66" s="5" t="inlineStr"/>
+      <c r="E66" s="5" t="inlineStr">
+        <is>
+          <t>neptune-developments.com</t>
+        </is>
+      </c>
       <c r="F66" s="7" t="inlineStr">
         <is>
-          <t>Matosinhos</t>
+          <t>Cascais</t>
         </is>
       </c>
       <c r="G66" s="7" t="inlineStr">
         <is>
-          <t>Porto</t>
+          <t>Lisboa</t>
         </is>
       </c>
       <c r="H66" s="5" t="inlineStr"/>
       <c r="I66" s="5" t="inlineStr">
         <is>
-          <t>RM Villas (Início obra 1T2026)</t>
+          <t>BellaMary (Cascais) (Comercialização)</t>
         </is>
       </c>
       <c r="J66" s="5" t="inlineStr">
         <is>
-          <t>Fonte: construir.pt</t>
+          <t>Sem telefone/CEO confirmados nas fontes</t>
         </is>
       </c>
       <c r="K66" s="5" t="inlineStr"/>
@@ -4168,7 +4328,7 @@
     <row r="67" ht="30" customHeight="1">
       <c r="A67" s="5" t="inlineStr">
         <is>
-          <t>Round Hill Capital</t>
+          <t>Onyria Group</t>
         </is>
       </c>
       <c r="B67" s="6" t="inlineStr">
@@ -4180,12 +4340,12 @@
       <c r="D67" s="5" t="inlineStr"/>
       <c r="E67" s="5" t="inlineStr">
         <is>
-          <t>roundhillcapital.com</t>
+          <t>onyriagroup.com</t>
         </is>
       </c>
       <c r="F67" s="7" t="inlineStr">
         <is>
-          <t>Lisboa</t>
+          <t>Cascais</t>
         </is>
       </c>
       <c r="G67" s="7" t="inlineStr">
@@ -4193,24 +4353,20 @@
           <t>Lisboa</t>
         </is>
       </c>
-      <c r="H67" s="5" t="inlineStr">
-        <is>
-          <t>Rua da Escola Politécnica 38, 1250-102</t>
-        </is>
-      </c>
+      <c r="H67" s="5" t="inlineStr"/>
       <c r="I67" s="5" t="inlineStr">
         <is>
-          <t>Student + residential Lisboa (com TPG) (Planeamento) | Tannery Amial (Porto) (Em construção)</t>
+          <t>Onyria Quinta da Marinha Residences (Cascais) (Comercialização)</t>
         </is>
       </c>
       <c r="J67" s="5" t="inlineStr">
         <is>
-          <t>Sem telefone PT publicado</t>
+          <t>Grupo hoteleiro+imobiliário fundado 1986 por José Carlos Pinto Coelho</t>
         </is>
       </c>
       <c r="K67" s="5" t="inlineStr">
         <is>
-          <t>Michael Bickford (Founder &amp; CEO global· sem responsável PT confirmado)</t>
+          <t>José Carlos Pinto Coelho (fundador, 1986)</t>
         </is>
       </c>
       <c r="L67" s="5" t="inlineStr"/>
@@ -4219,7 +4375,7 @@
     <row r="68" ht="30" customHeight="1">
       <c r="A68" s="5" t="inlineStr">
         <is>
-          <t>Screendomus (Grupo Teixeira)</t>
+          <t>Portaviv</t>
         </is>
       </c>
       <c r="B68" s="6" t="inlineStr">
@@ -4228,40 +4384,32 @@
         </is>
       </c>
       <c r="C68" s="7" t="inlineStr"/>
-      <c r="D68" s="5" t="inlineStr">
-        <is>
-          <t>geral@screendomus.com</t>
-        </is>
-      </c>
-      <c r="E68" s="5" t="inlineStr">
-        <is>
-          <t>screendomus.com</t>
-        </is>
-      </c>
+      <c r="D68" s="5" t="inlineStr"/>
+      <c r="E68" s="5" t="inlineStr"/>
       <c r="F68" s="7" t="inlineStr">
         <is>
-          <t>Lisboa</t>
+          <t>Porto</t>
         </is>
       </c>
       <c r="G68" s="7" t="inlineStr">
         <is>
-          <t>Lisboa</t>
+          <t>Porto</t>
         </is>
       </c>
       <c r="H68" s="5" t="inlineStr"/>
       <c r="I68" s="5" t="inlineStr">
         <is>
-          <t>Altus (Alta de Lisboa) (Em construção)</t>
+          <t>The Factory Residences Campanhã (Em carteira/comercialização)</t>
         </is>
       </c>
       <c r="J68" s="5" t="inlineStr">
         <is>
-          <t>Integra o Grupo Teixeira. Sem telefone confirmado — contacto via screendomus.com</t>
+          <t>Fonte: construir.pt</t>
         </is>
       </c>
       <c r="K68" s="5" t="inlineStr">
         <is>
-          <t>Nuno Teixeira (Administrador, perfil LinkedIn não confirmado)</t>
+          <t>Nuno Cunha (Managing Director)</t>
         </is>
       </c>
       <c r="L68" s="5" t="inlineStr"/>
@@ -4270,7 +4418,7 @@
     <row r="69" ht="30" customHeight="1">
       <c r="A69" s="5" t="inlineStr">
         <is>
-          <t>Shalu Investments</t>
+          <t>REDASSET</t>
         </is>
       </c>
       <c r="B69" s="6" t="inlineStr">
@@ -4280,44 +4428,36 @@
       </c>
       <c r="C69" s="7" t="inlineStr"/>
       <c r="D69" s="5" t="inlineStr"/>
-      <c r="E69" s="5" t="inlineStr">
-        <is>
-          <t>shaluinvest.pt</t>
-        </is>
-      </c>
+      <c r="E69" s="5" t="inlineStr"/>
       <c r="F69" s="7" t="inlineStr">
         <is>
-          <t>Porto</t>
+          <t>Amadora</t>
         </is>
       </c>
       <c r="G69" s="7" t="inlineStr">
         <is>
-          <t>Porto</t>
+          <t>Lisboa</t>
         </is>
       </c>
       <c r="H69" s="5" t="inlineStr"/>
       <c r="I69" s="5" t="inlineStr">
         <is>
-          <t>Portefólio residencial Grande Porto (Em desenvolvimento)</t>
+          <t>Moinho do Guizo (Mina de Água, Amadora) (Planeamento)</t>
         </is>
       </c>
       <c r="J69" s="5" t="inlineStr">
         <is>
-          <t>Fundador e Managing Director: Itai Fridman</t>
-        </is>
-      </c>
-      <c r="K69" s="5" t="inlineStr">
-        <is>
-          <t>Itai Fridman (Founder &amp; Managing Director)</t>
-        </is>
-      </c>
+          <t>Promotor privado em terreno próprio, comercialização sob termos legais definidos</t>
+        </is>
+      </c>
+      <c r="K69" s="5" t="inlineStr"/>
       <c r="L69" s="5" t="inlineStr"/>
       <c r="M69" s="5" t="inlineStr"/>
     </row>
     <row r="70" ht="30" customHeight="1">
       <c r="A70" s="5" t="inlineStr">
         <is>
-          <t>Taga Urbanic</t>
+          <t>RM Promo (JV M2O Group / RJB Home)</t>
         </is>
       </c>
       <c r="B70" s="6" t="inlineStr">
@@ -4330,7 +4470,7 @@
       <c r="E70" s="5" t="inlineStr"/>
       <c r="F70" s="7" t="inlineStr">
         <is>
-          <t>Maia</t>
+          <t>Matosinhos</t>
         </is>
       </c>
       <c r="G70" s="7" t="inlineStr">
@@ -4341,12 +4481,12 @@
       <c r="H70" s="5" t="inlineStr"/>
       <c r="I70" s="5" t="inlineStr">
         <is>
-          <t>Verde Vale (Em construção)</t>
+          <t>RM Villas (Início obra 1T2026)</t>
         </is>
       </c>
       <c r="J70" s="5" t="inlineStr">
         <is>
-          <t>Fonte: imobiliario.publico.pt</t>
+          <t>Fonte: construir.pt</t>
         </is>
       </c>
       <c r="K70" s="5" t="inlineStr"/>
@@ -4356,7 +4496,7 @@
     <row r="71" ht="30" customHeight="1">
       <c r="A71" s="5" t="inlineStr">
         <is>
-          <t>United Investments Portugal (UIP)</t>
+          <t>Shalu Investments</t>
         </is>
       </c>
       <c r="B71" s="6" t="inlineStr">
@@ -4368,50 +4508,42 @@
       <c r="D71" s="5" t="inlineStr"/>
       <c r="E71" s="5" t="inlineStr">
         <is>
-          <t>uip.pt</t>
+          <t>shaluinvest.pt</t>
         </is>
       </c>
       <c r="F71" s="7" t="inlineStr">
         <is>
-          <t>Lisboa</t>
+          <t>Porto</t>
         </is>
       </c>
       <c r="G71" s="7" t="inlineStr">
         <is>
-          <t>Lisboa</t>
-        </is>
-      </c>
-      <c r="H71" s="5" t="inlineStr">
-        <is>
-          <t>Lisboa</t>
-        </is>
-      </c>
+          <t>Porto</t>
+        </is>
+      </c>
+      <c r="H71" s="5" t="inlineStr"/>
       <c r="I71" s="5" t="inlineStr">
         <is>
-          <t>Pine Cliffs (Algarve), Sheraton Cascais, YOTEL Porto, Hyatt Regency Lisboa (Em construção)</t>
+          <t>Portefólio residencial Grande Porto (Em desenvolvimento)</t>
         </is>
       </c>
       <c r="J71" s="5" t="inlineStr">
         <is>
-          <t>Fundada 1985 · sem telefone publicado</t>
+          <t>Fundador e Managing Director: Itai Fridman</t>
         </is>
       </c>
       <c r="K71" s="5" t="inlineStr">
         <is>
-          <t>Carlos Leal (CEO)</t>
-        </is>
-      </c>
-      <c r="L71" s="5" t="inlineStr">
-        <is>
-          <t>https://www.linkedin.com/in/carlos-leal-62797227/</t>
-        </is>
-      </c>
+          <t>Itai Fridman (Founder &amp; Managing Director)</t>
+        </is>
+      </c>
+      <c r="L71" s="5" t="inlineStr"/>
       <c r="M71" s="5" t="inlineStr"/>
     </row>
     <row r="72" ht="30" customHeight="1">
       <c r="A72" s="5" t="inlineStr">
         <is>
-          <t>Visabeira Imobiliária (Visabeirahouse)</t>
+          <t>Taga Urbanic</t>
         </is>
       </c>
       <c r="B72" s="6" t="inlineStr">
@@ -4421,42 +4553,30 @@
       </c>
       <c r="C72" s="7" t="inlineStr"/>
       <c r="D72" s="5" t="inlineStr"/>
-      <c r="E72" s="5" t="inlineStr">
-        <is>
-          <t>grupovisabeira.com</t>
-        </is>
-      </c>
+      <c r="E72" s="5" t="inlineStr"/>
       <c r="F72" s="7" t="inlineStr">
         <is>
-          <t>Lisboa</t>
+          <t>Maia</t>
         </is>
       </c>
       <c r="G72" s="7" t="inlineStr">
         <is>
-          <t>Lisboa</t>
+          <t>Porto</t>
         </is>
       </c>
       <c r="H72" s="5" t="inlineStr"/>
       <c r="I72" s="5" t="inlineStr">
         <is>
-          <t>Areeiro Select (Comercialização)</t>
+          <t>Verde Vale (Em construção)</t>
         </is>
       </c>
       <c r="J72" s="5" t="inlineStr">
         <is>
-          <t>Fonte: idealista.pt</t>
-        </is>
-      </c>
-      <c r="K72" s="5" t="inlineStr">
-        <is>
-          <t>Paula Santos (Diretora Geral Visabeirahouse)</t>
-        </is>
-      </c>
-      <c r="L72" s="5" t="inlineStr">
-        <is>
-          <t>https://www.linkedin.com/in/paula-santos-71083337/</t>
-        </is>
-      </c>
+          <t>Fonte: imobiliario.publico.pt</t>
+        </is>
+      </c>
+      <c r="K72" s="5" t="inlineStr"/>
+      <c r="L72" s="5" t="inlineStr"/>
       <c r="M72" s="5" t="inlineStr"/>
     </row>
     <row r="73" ht="30" customHeight="1">
@@ -8807,7 +8927,7 @@
         </is>
       </c>
       <c r="B3" s="9" t="n">
-        <v>71</v>
+        <v>82</v>
       </c>
     </row>
     <row r="4">
@@ -8817,7 +8937,7 @@
         </is>
       </c>
       <c r="B4" s="9" t="n">
-        <v>90</v>
+        <v>79</v>
       </c>
     </row>
     <row r="5">
@@ -8847,7 +8967,7 @@
         </is>
       </c>
       <c r="B7" s="9" t="n">
-        <v>52</v>
+        <v>53</v>
       </c>
     </row>
     <row r="8">

</xml_diff>

<commit_message>
Minor enrichment: Shalu Investments address, Dipe Real Estate CEO LinkedIn
Also confirms (via this search pass) that personal CEO mobile numbers
are not retrievable through open web search for any company tried —
they exist in paywalled data-broker records (RocketReach etc.) that
mask the actual digits, so nothing was added on that front.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01SRBJwGmSsYkTHKJbGCM5ca
</commit_message>
<xml_diff>
--- a/Promotoras_Imobiliarias_Contactos.xlsx
+++ b/Promotoras_Imobiliarias_Contactos.xlsx
@@ -4521,7 +4521,11 @@
           <t>Porto</t>
         </is>
       </c>
-      <c r="H71" s="5" t="inlineStr"/>
+      <c r="H71" s="5" t="inlineStr">
+        <is>
+          <t>Rua Marechal Saldanha 697</t>
+        </is>
+      </c>
       <c r="I71" s="5" t="inlineStr">
         <is>
           <t>Portefólio residencial Grande Porto (Em desenvolvimento)</t>
@@ -5170,7 +5174,11 @@
           <t>Diogo Baptista Antunes (CEO)</t>
         </is>
       </c>
-      <c r="L82" s="2" t="inlineStr"/>
+      <c r="L82" s="2" t="inlineStr">
+        <is>
+          <t>https://pt.linkedin.com/in/diogo-baptista-antunes</t>
+        </is>
+      </c>
       <c r="M82" s="2" t="inlineStr"/>
     </row>
     <row r="83" ht="30" customHeight="1">
@@ -8967,7 +8975,7 @@
         </is>
       </c>
       <c r="B7" s="9" t="n">
-        <v>53</v>
+        <v>54</v>
       </c>
     </row>
     <row r="8">

</xml_diff>

<commit_message>
Add 3 more promoters (164 total): iLanga Capital, Urban Office, Hievila
Also adds the Fercopor CEO's Instagram (Mário Sutil Almeida), supplied
directly by the user and cross-checked against a press interview
confirming he is Fercopor's administrator.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01SRBJwGmSsYkTHKJbGCM5ca
</commit_message>
<xml_diff>
--- a/Promotoras_Imobiliarias_Contactos.xlsx
+++ b/Promotoras_Imobiliarias_Contactos.xlsx
@@ -191,8 +191,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Promotoras" displayName="Promotoras" ref="A1:M162" headerRowCount="1">
-  <autoFilter ref="A1:M162"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Promotoras" displayName="Promotoras" ref="A1:M165" headerRowCount="1">
+  <autoFilter ref="A1:M165"/>
   <tableColumns count="13">
     <tableColumn id="1" name="Nome da Empresa"/>
     <tableColumn id="2" name="Prioritario"/>
@@ -501,7 +501,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M162"/>
+  <dimension ref="A1:M165"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1516,11 +1516,15 @@
       </c>
       <c r="K17" s="2" t="inlineStr">
         <is>
-          <t>Mário Almeida (Administrador)</t>
+          <t>Mário Sutil Almeida (Administrador)</t>
         </is>
       </c>
       <c r="L17" s="2" t="inlineStr"/>
-      <c r="M17" s="2" t="inlineStr"/>
+      <c r="M17" s="2" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/mariosutilalmeida/</t>
+        </is>
+      </c>
     </row>
     <row r="18" ht="30" customHeight="1">
       <c r="A18" s="2" t="inlineStr">
@@ -5597,7 +5601,7 @@
     <row r="90" ht="30" customHeight="1">
       <c r="A90" s="2" t="inlineStr">
         <is>
-          <t>HomeLovers Investment</t>
+          <t>Hievila – Empreendimentos Imobiliários</t>
         </is>
       </c>
       <c r="B90" s="4" t="inlineStr">
@@ -5607,52 +5611,52 @@
       </c>
       <c r="C90" s="4" t="inlineStr">
         <is>
-          <t>+351 913 470 147</t>
-        </is>
-      </c>
-      <c r="D90" s="2" t="inlineStr"/>
+          <t>+351 239 091 692</t>
+        </is>
+      </c>
+      <c r="D90" s="2" t="inlineStr">
+        <is>
+          <t>hievila@hievila.com</t>
+        </is>
+      </c>
       <c r="E90" s="2" t="inlineStr">
         <is>
-          <t>homelovers.pt</t>
+          <t>hievila.com</t>
         </is>
       </c>
       <c r="F90" s="4" t="inlineStr">
         <is>
-          <t>Setúbal</t>
+          <t>Coimbra</t>
         </is>
       </c>
       <c r="G90" s="4" t="inlineStr">
         <is>
-          <t>Setúbal</t>
-        </is>
-      </c>
-      <c r="H90" s="2" t="inlineStr"/>
+          <t>Coimbra</t>
+        </is>
+      </c>
+      <c r="H90" s="2" t="inlineStr">
+        <is>
+          <t>Rua da Casa Branca 13</t>
+        </is>
+      </c>
       <c r="I90" s="2" t="inlineStr">
         <is>
-          <t>Parque da Cidade – Riverside Living Setúbal (Em construção)</t>
+          <t>Portela Flats (Quinta da Portela, Coimbra) (Em construção)</t>
         </is>
       </c>
       <c r="J90" s="2" t="inlineStr">
         <is>
-          <t>Fonte: sapo.pt</t>
-        </is>
-      </c>
-      <c r="K90" s="2" t="inlineStr">
-        <is>
-          <t>Miguel Tilli (fundador e CEO)</t>
-        </is>
-      </c>
-      <c r="L90" s="2" t="inlineStr">
-        <is>
-          <t>https://www.linkedin.com/in/miguel-tilli-a7a41587/</t>
-        </is>
-      </c>
+          <t>Fundada 2008</t>
+        </is>
+      </c>
+      <c r="K90" s="2" t="inlineStr"/>
+      <c r="L90" s="2" t="inlineStr"/>
       <c r="M90" s="2" t="inlineStr"/>
     </row>
     <row r="91" ht="30" customHeight="1">
       <c r="A91" s="2" t="inlineStr">
         <is>
-          <t>JHOMEA Invest</t>
+          <t>HomeLovers Investment</t>
         </is>
       </c>
       <c r="B91" s="4" t="inlineStr">
@@ -5662,56 +5666,52 @@
       </c>
       <c r="C91" s="4" t="inlineStr">
         <is>
-          <t>+351 934 175 642</t>
-        </is>
-      </c>
-      <c r="D91" s="2" t="inlineStr">
-        <is>
-          <t>geral@jhomea.pt</t>
-        </is>
-      </c>
+          <t>+351 913 470 147</t>
+        </is>
+      </c>
+      <c r="D91" s="2" t="inlineStr"/>
       <c r="E91" s="2" t="inlineStr">
         <is>
-          <t>jhomea.pt</t>
+          <t>homelovers.pt</t>
         </is>
       </c>
       <c r="F91" s="4" t="inlineStr">
         <is>
-          <t>Aveiro</t>
+          <t>Setúbal</t>
         </is>
       </c>
       <c r="G91" s="4" t="inlineStr">
         <is>
-          <t>Aveiro</t>
-        </is>
-      </c>
-      <c r="H91" s="2" t="inlineStr">
-        <is>
-          <t>Rua Cristóvão Pinho Queimado 56, 3800-012</t>
-        </is>
-      </c>
+          <t>Setúbal</t>
+        </is>
+      </c>
+      <c r="H91" s="2" t="inlineStr"/>
       <c r="I91" s="2" t="inlineStr">
         <is>
-          <t>Vacivus (Porto) (Em construção)</t>
+          <t>Parque da Cidade – Riverside Living Setúbal (Em construção)</t>
         </is>
       </c>
       <c r="J91" s="2" t="inlineStr">
         <is>
-          <t>AMI 16355. Escritórios Aveiro (+351 914 444 764) e Lisboa (+351 912 325 143)</t>
+          <t>Fonte: sapo.pt</t>
         </is>
       </c>
       <c r="K91" s="2" t="inlineStr">
         <is>
-          <t>José Miguel Afonso (CEO/fundador)</t>
-        </is>
-      </c>
-      <c r="L91" s="2" t="inlineStr"/>
+          <t>Miguel Tilli (fundador e CEO)</t>
+        </is>
+      </c>
+      <c r="L91" s="2" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/miguel-tilli-a7a41587/</t>
+        </is>
+      </c>
       <c r="M91" s="2" t="inlineStr"/>
     </row>
     <row r="92" ht="30" customHeight="1">
       <c r="A92" s="2" t="inlineStr">
         <is>
-          <t>Metathesis</t>
+          <t>iLanga Capital (Ohai Resorts)</t>
         </is>
       </c>
       <c r="B92" s="4" t="inlineStr">
@@ -5721,43 +5721,47 @@
       </c>
       <c r="C92" s="4" t="inlineStr">
         <is>
-          <t>+351 211 650 420</t>
-        </is>
-      </c>
-      <c r="D92" s="2" t="inlineStr"/>
+          <t>+351 262 561 800</t>
+        </is>
+      </c>
+      <c r="D92" s="2" t="inlineStr">
+        <is>
+          <t>info.nazare@ohairesorts.com</t>
+        </is>
+      </c>
       <c r="E92" s="2" t="inlineStr">
         <is>
-          <t>metathesis.pt</t>
+          <t>ohairesorts.com</t>
         </is>
       </c>
       <c r="F92" s="4" t="inlineStr">
         <is>
-          <t>Almada</t>
+          <t>Nazaré</t>
         </is>
       </c>
       <c r="G92" s="4" t="inlineStr">
         <is>
-          <t>Setúbal</t>
+          <t>Leiria</t>
         </is>
       </c>
       <c r="H92" s="2" t="inlineStr">
         <is>
-          <t>R. Marcos de Assunção nº4A, 2805-290</t>
+          <t>Entrada Nacional 242 Km 31.5, 2450-138</t>
         </is>
       </c>
       <c r="I92" s="2" t="inlineStr">
         <is>
-          <t>Reabilitação de imóveis residenciais (Almada) (Em construção)</t>
+          <t>Ohai Peniche (Em construção) | Ohai Nazaré (Concluído/Operação)</t>
         </is>
       </c>
       <c r="J92" s="2" t="inlineStr">
         <is>
-          <t>Gerente: Maria Elisabete da Fonseca Dionísio Dias. Tel. alt. 967 364 611</t>
+          <t>Grupo espanhol de Pelayo Cortina Koplowitz (conde de San Fernando de Peñalver). Tel. alt. 933 089 416</t>
         </is>
       </c>
       <c r="K92" s="2" t="inlineStr">
         <is>
-          <t>Maria Elisabete da Fonseca Dionísio Dias (gerente)</t>
+          <t>Pelayo Cortina Koplowitz (fundador)</t>
         </is>
       </c>
       <c r="L92" s="2" t="inlineStr"/>
@@ -5766,7 +5770,7 @@
     <row r="93" ht="30" customHeight="1">
       <c r="A93" s="2" t="inlineStr">
         <is>
-          <t>Pine Hill</t>
+          <t>JHOMEA Invest</t>
         </is>
       </c>
       <c r="B93" s="4" t="inlineStr">
@@ -5776,56 +5780,56 @@
       </c>
       <c r="C93" s="4" t="inlineStr">
         <is>
-          <t>+351 910 936 732</t>
+          <t>+351 934 175 642</t>
         </is>
       </c>
       <c r="D93" s="2" t="inlineStr">
         <is>
-          <t>info@pinehill.pt</t>
+          <t>geral@jhomea.pt</t>
         </is>
       </c>
       <c r="E93" s="2" t="inlineStr">
         <is>
-          <t>pinehill.pt</t>
+          <t>jhomea.pt</t>
         </is>
       </c>
       <c r="F93" s="4" t="inlineStr">
         <is>
-          <t>Braga</t>
+          <t>Aveiro</t>
         </is>
       </c>
       <c r="G93" s="4" t="inlineStr">
         <is>
-          <t>Braga</t>
-        </is>
-      </c>
-      <c r="H93" s="2" t="inlineStr"/>
+          <t>Aveiro</t>
+        </is>
+      </c>
+      <c r="H93" s="2" t="inlineStr">
+        <is>
+          <t>Rua Cristóvão Pinho Queimado 56, 3800-012</t>
+        </is>
+      </c>
       <c r="I93" s="2" t="inlineStr">
         <is>
-          <t>Braga Premium Flats (Comercialização) | 3 novos projetos em Braga (Planeamento)</t>
+          <t>Vacivus (Porto) (Em construção)</t>
         </is>
       </c>
       <c r="J93" s="2" t="inlineStr">
         <is>
-          <t>Promotora criada em 2025. Fonte: newinbraga.nit.pt, Revista Spot</t>
+          <t>AMI 16355. Escritórios Aveiro (+351 914 444 764) e Lisboa (+351 912 325 143)</t>
         </is>
       </c>
       <c r="K93" s="2" t="inlineStr">
         <is>
-          <t>Nuno Pinheiro (fundador)</t>
-        </is>
-      </c>
-      <c r="L93" s="2" t="inlineStr">
-        <is>
-          <t>https://www.linkedin.com/in/nuno-pinheiro-39968aa4/</t>
-        </is>
-      </c>
+          <t>José Miguel Afonso (CEO/fundador)</t>
+        </is>
+      </c>
+      <c r="L93" s="2" t="inlineStr"/>
       <c r="M93" s="2" t="inlineStr"/>
     </row>
     <row r="94" ht="30" customHeight="1">
       <c r="A94" s="2" t="inlineStr">
         <is>
-          <t>Quinta do Lago Resort</t>
+          <t>Metathesis</t>
         </is>
       </c>
       <c r="B94" s="4" t="inlineStr">
@@ -5835,60 +5839,52 @@
       </c>
       <c r="C94" s="4" t="inlineStr">
         <is>
-          <t>+351 289 390 700</t>
-        </is>
-      </c>
-      <c r="D94" s="2" t="inlineStr">
-        <is>
-          <t>info@quintadolago.com</t>
-        </is>
-      </c>
+          <t>+351 211 650 420</t>
+        </is>
+      </c>
+      <c r="D94" s="2" t="inlineStr"/>
       <c r="E94" s="2" t="inlineStr">
         <is>
-          <t>quintadolago.com</t>
+          <t>metathesis.pt</t>
         </is>
       </c>
       <c r="F94" s="4" t="inlineStr">
         <is>
-          <t>Loulé</t>
+          <t>Almada</t>
         </is>
       </c>
       <c r="G94" s="4" t="inlineStr">
         <is>
-          <t>Faro</t>
+          <t>Setúbal</t>
         </is>
       </c>
       <c r="H94" s="2" t="inlineStr">
         <is>
-          <t>Almancil</t>
+          <t>R. Marcos de Assunção nº4A, 2805-290</t>
         </is>
       </c>
       <c r="I94" s="2" t="inlineStr">
         <is>
-          <t>Quinta do Lago (real estate do resort) (Comercialização)</t>
+          <t>Reabilitação de imóveis residenciais (Almada) (Em construção)</t>
         </is>
       </c>
       <c r="J94" s="2" t="inlineStr">
         <is>
-          <t>Resort residencial/golfe</t>
+          <t>Gerente: Maria Elisabete da Fonseca Dionísio Dias. Tel. alt. 967 364 611</t>
         </is>
       </c>
       <c r="K94" s="2" t="inlineStr">
         <is>
-          <t>Sean Moriarty (CEO)</t>
-        </is>
-      </c>
-      <c r="L94" s="2" t="inlineStr">
-        <is>
-          <t>https://pt.linkedin.com/in/sean-moriarty-6a749133</t>
-        </is>
-      </c>
+          <t>Maria Elisabete da Fonseca Dionísio Dias (gerente)</t>
+        </is>
+      </c>
+      <c r="L94" s="2" t="inlineStr"/>
       <c r="M94" s="2" t="inlineStr"/>
     </row>
     <row r="95" ht="30" customHeight="1">
       <c r="A95" s="2" t="inlineStr">
         <is>
-          <t>Royal Prime</t>
+          <t>Pine Hill</t>
         </is>
       </c>
       <c r="B95" s="4" t="inlineStr">
@@ -5898,52 +5894,56 @@
       </c>
       <c r="C95" s="4" t="inlineStr">
         <is>
-          <t>+351 910 181 312</t>
+          <t>+351 910 936 732</t>
         </is>
       </c>
       <c r="D95" s="2" t="inlineStr">
         <is>
-          <t>rgodinho@royalprime.pt</t>
+          <t>info@pinehill.pt</t>
         </is>
       </c>
       <c r="E95" s="2" t="inlineStr">
         <is>
-          <t>royalprime.pt</t>
+          <t>pinehill.pt</t>
         </is>
       </c>
       <c r="F95" s="4" t="inlineStr">
         <is>
-          <t>Covilhã</t>
+          <t>Braga</t>
         </is>
       </c>
       <c r="G95" s="4" t="inlineStr">
         <is>
-          <t>Castelo Branco</t>
-        </is>
-      </c>
-      <c r="H95" s="2" t="inlineStr">
-        <is>
-          <t>R. Doutor Mário Soares, lote 3, 6200-026</t>
-        </is>
-      </c>
+          <t>Braga</t>
+        </is>
+      </c>
+      <c r="H95" s="2" t="inlineStr"/>
       <c r="I95" s="2" t="inlineStr">
         <is>
-          <t>Tower Residences (Covilhã) (Concluído)</t>
+          <t>Braga Premium Flats (Comercialização) | 3 novos projetos em Braga (Planeamento)</t>
         </is>
       </c>
       <c r="J95" s="2" t="inlineStr">
         <is>
-          <t>Contacto comercial Rita Godinho</t>
-        </is>
-      </c>
-      <c r="K95" s="2" t="inlineStr"/>
-      <c r="L95" s="2" t="inlineStr"/>
+          <t>Promotora criada em 2025. Fonte: newinbraga.nit.pt, Revista Spot</t>
+        </is>
+      </c>
+      <c r="K95" s="2" t="inlineStr">
+        <is>
+          <t>Nuno Pinheiro (fundador)</t>
+        </is>
+      </c>
+      <c r="L95" s="2" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/nuno-pinheiro-39968aa4/</t>
+        </is>
+      </c>
       <c r="M95" s="2" t="inlineStr"/>
     </row>
     <row r="96" ht="30" customHeight="1">
       <c r="A96" s="2" t="inlineStr">
         <is>
-          <t>Salk Properties Portugal</t>
+          <t>Quinta do Lago Resort</t>
         </is>
       </c>
       <c r="B96" s="4" t="inlineStr">
@@ -5953,48 +5953,60 @@
       </c>
       <c r="C96" s="4" t="inlineStr">
         <is>
-          <t>+351 939 443 765</t>
-        </is>
-      </c>
-      <c r="D96" s="2" t="inlineStr"/>
+          <t>+351 289 390 700</t>
+        </is>
+      </c>
+      <c r="D96" s="2" t="inlineStr">
+        <is>
+          <t>info@quintadolago.com</t>
+        </is>
+      </c>
       <c r="E96" s="2" t="inlineStr">
         <is>
-          <t>salkproperties.com</t>
+          <t>quintadolago.com</t>
         </is>
       </c>
       <c r="F96" s="4" t="inlineStr">
         <is>
-          <t>Alcácer do Sal</t>
+          <t>Loulé</t>
         </is>
       </c>
       <c r="G96" s="4" t="inlineStr">
         <is>
-          <t>Setúbal</t>
-        </is>
-      </c>
-      <c r="H96" s="2" t="inlineStr"/>
+          <t>Faro</t>
+        </is>
+      </c>
+      <c r="H96" s="2" t="inlineStr">
+        <is>
+          <t>Almancil</t>
+        </is>
+      </c>
       <c r="I96" s="2" t="inlineStr">
         <is>
-          <t>Alcácer Vintage (Planeamento (consulta pública))</t>
+          <t>Quinta do Lago (real estate do resort) (Comercialização)</t>
         </is>
       </c>
       <c r="J96" s="2" t="inlineStr">
         <is>
-          <t>Fonte: vidaimobiliaria.com</t>
+          <t>Resort residencial/golfe</t>
         </is>
       </c>
       <c r="K96" s="2" t="inlineStr">
         <is>
-          <t>João Luís Ferreira (Chairman &amp; Partner)</t>
-        </is>
-      </c>
-      <c r="L96" s="2" t="inlineStr"/>
+          <t>Sean Moriarty (CEO)</t>
+        </is>
+      </c>
+      <c r="L96" s="2" t="inlineStr">
+        <is>
+          <t>https://pt.linkedin.com/in/sean-moriarty-6a749133</t>
+        </is>
+      </c>
       <c r="M96" s="2" t="inlineStr"/>
     </row>
     <row r="97" ht="30" customHeight="1">
       <c r="A97" s="2" t="inlineStr">
         <is>
-          <t>Scale Property Development</t>
+          <t>Royal Prime</t>
         </is>
       </c>
       <c r="B97" s="4" t="inlineStr">
@@ -6004,52 +6016,52 @@
       </c>
       <c r="C97" s="4" t="inlineStr">
         <is>
-          <t>+351 219 362 960</t>
-        </is>
-      </c>
-      <c r="D97" s="2" t="inlineStr"/>
+          <t>+351 910 181 312</t>
+        </is>
+      </c>
+      <c r="D97" s="2" t="inlineStr">
+        <is>
+          <t>rgodinho@royalprime.pt</t>
+        </is>
+      </c>
       <c r="E97" s="2" t="inlineStr">
         <is>
-          <t>scalepropertydevelopment.com</t>
+          <t>royalprime.pt</t>
         </is>
       </c>
       <c r="F97" s="4" t="inlineStr">
         <is>
-          <t>Setúbal</t>
+          <t>Covilhã</t>
         </is>
       </c>
       <c r="G97" s="4" t="inlineStr">
         <is>
-          <t>Setúbal</t>
-        </is>
-      </c>
-      <c r="H97" s="2" t="inlineStr"/>
+          <t>Castelo Branco</t>
+        </is>
+      </c>
+      <c r="H97" s="2" t="inlineStr">
+        <is>
+          <t>R. Doutor Mário Soares, lote 3, 6200-026</t>
+        </is>
+      </c>
       <c r="I97" s="2" t="inlineStr">
         <is>
-          <t>Parque da Cidade – Riverside Living Setúbal (Em construção)</t>
+          <t>Tower Residences (Covilhã) (Concluído)</t>
         </is>
       </c>
       <c r="J97" s="2" t="inlineStr">
         <is>
-          <t>Fonte: vidaimobiliaria.com</t>
-        </is>
-      </c>
-      <c r="K97" s="2" t="inlineStr">
-        <is>
-          <t>Diogo Sá Viana Rebelo (Co-Founder)</t>
-        </is>
-      </c>
-      <c r="L97" s="2" t="inlineStr">
-        <is>
-          <t>https://www.linkedin.com/in/diogo-s%C3%A1-viana-rebelo-910104143/</t>
-        </is>
-      </c>
+          <t>Contacto comercial Rita Godinho</t>
+        </is>
+      </c>
+      <c r="K97" s="2" t="inlineStr"/>
+      <c r="L97" s="2" t="inlineStr"/>
       <c r="M97" s="2" t="inlineStr"/>
     </row>
     <row r="98" ht="30" customHeight="1">
       <c r="A98" s="2" t="inlineStr">
         <is>
-          <t>TPS – Teixeira, Pinto &amp; Soares</t>
+          <t>Salk Properties Portugal</t>
         </is>
       </c>
       <c r="B98" s="4" t="inlineStr">
@@ -6059,47 +6071,39 @@
       </c>
       <c r="C98" s="4" t="inlineStr">
         <is>
-          <t>+351 255 433 572</t>
-        </is>
-      </c>
-      <c r="D98" s="2" t="inlineStr">
-        <is>
-          <t>geral@tps.com.pt</t>
-        </is>
-      </c>
+          <t>+351 939 443 765</t>
+        </is>
+      </c>
+      <c r="D98" s="2" t="inlineStr"/>
       <c r="E98" s="2" t="inlineStr">
         <is>
-          <t>tps.com.pt</t>
+          <t>salkproperties.com</t>
         </is>
       </c>
       <c r="F98" s="4" t="inlineStr">
         <is>
-          <t>Amarante</t>
+          <t>Alcácer do Sal</t>
         </is>
       </c>
       <c r="G98" s="4" t="inlineStr">
         <is>
-          <t>Porto</t>
-        </is>
-      </c>
-      <c r="H98" s="2" t="inlineStr">
-        <is>
-          <t>Rua do Outeiro 677, Z.I. Telões, 4600-758</t>
-        </is>
-      </c>
+          <t>Setúbal</t>
+        </is>
+      </c>
+      <c r="H98" s="2" t="inlineStr"/>
       <c r="I98" s="2" t="inlineStr">
         <is>
-          <t>JV com Carvoeiro Branco (Lagoa, Portimão, Faro) (Planeamento) | One Lush (Caxias) (Em construção)</t>
+          <t>Alcácer Vintage (Planeamento (consulta pública))</t>
         </is>
       </c>
       <c r="J98" s="2" t="inlineStr">
         <is>
-          <t>Uma das maiores construtoras nacionais · delegações Lisboa e Algarve</t>
+          <t>Fonte: vidaimobiliaria.com</t>
         </is>
       </c>
       <c r="K98" s="2" t="inlineStr">
         <is>
-          <t>Bruno Fernando Macedo Soares (CEO/Presidente do CA)</t>
+          <t>João Luís Ferreira (Chairman &amp; Partner)</t>
         </is>
       </c>
       <c r="L98" s="2" t="inlineStr"/>
@@ -6108,7 +6112,7 @@
     <row r="99" ht="30" customHeight="1">
       <c r="A99" s="2" t="inlineStr">
         <is>
-          <t>Vomera Group</t>
+          <t>Scale Property Development</t>
         </is>
       </c>
       <c r="B99" s="4" t="inlineStr">
@@ -6118,130 +6122,162 @@
       </c>
       <c r="C99" s="4" t="inlineStr">
         <is>
-          <t>351 243 078 442</t>
+          <t>+351 219 362 960</t>
         </is>
       </c>
       <c r="D99" s="2" t="inlineStr"/>
       <c r="E99" s="2" t="inlineStr">
         <is>
-          <t>vomera.pt</t>
+          <t>scalepropertydevelopment.com</t>
         </is>
       </c>
       <c r="F99" s="4" t="inlineStr">
         <is>
-          <t>Santarém</t>
+          <t>Setúbal</t>
         </is>
       </c>
       <c r="G99" s="4" t="inlineStr">
         <is>
-          <t>Santarém</t>
+          <t>Setúbal</t>
         </is>
       </c>
       <c r="H99" s="2" t="inlineStr"/>
       <c r="I99" s="2" t="inlineStr">
         <is>
+          <t>Parque da Cidade – Riverside Living Setúbal (Em construção)</t>
+        </is>
+      </c>
+      <c r="J99" s="2" t="inlineStr">
+        <is>
+          <t>Fonte: vidaimobiliaria.com</t>
+        </is>
+      </c>
+      <c r="K99" s="2" t="inlineStr">
+        <is>
+          <t>Diogo Sá Viana Rebelo (Co-Founder)</t>
+        </is>
+      </c>
+      <c r="L99" s="2" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/diogo-s%C3%A1-viana-rebelo-910104143/</t>
+        </is>
+      </c>
+      <c r="M99" s="2" t="inlineStr"/>
+    </row>
+    <row r="100" ht="30" customHeight="1">
+      <c r="A100" s="2" t="inlineStr">
+        <is>
+          <t>TPS – Teixeira, Pinto &amp; Soares</t>
+        </is>
+      </c>
+      <c r="B100" s="4" t="inlineStr">
+        <is>
+          <t>Nao</t>
+        </is>
+      </c>
+      <c r="C100" s="4" t="inlineStr">
+        <is>
+          <t>+351 255 433 572</t>
+        </is>
+      </c>
+      <c r="D100" s="2" t="inlineStr">
+        <is>
+          <t>geral@tps.com.pt</t>
+        </is>
+      </c>
+      <c r="E100" s="2" t="inlineStr">
+        <is>
+          <t>tps.com.pt</t>
+        </is>
+      </c>
+      <c r="F100" s="4" t="inlineStr">
+        <is>
+          <t>Amarante</t>
+        </is>
+      </c>
+      <c r="G100" s="4" t="inlineStr">
+        <is>
+          <t>Porto</t>
+        </is>
+      </c>
+      <c r="H100" s="2" t="inlineStr">
+        <is>
+          <t>Rua do Outeiro 677, Z.I. Telões, 4600-758</t>
+        </is>
+      </c>
+      <c r="I100" s="2" t="inlineStr">
+        <is>
+          <t>JV com Carvoeiro Branco (Lagoa, Portimão, Faro) (Planeamento) | One Lush (Caxias) (Em construção)</t>
+        </is>
+      </c>
+      <c r="J100" s="2" t="inlineStr">
+        <is>
+          <t>Uma das maiores construtoras nacionais · delegações Lisboa e Algarve</t>
+        </is>
+      </c>
+      <c r="K100" s="2" t="inlineStr">
+        <is>
+          <t>Bruno Fernando Macedo Soares (CEO/Presidente do CA)</t>
+        </is>
+      </c>
+      <c r="L100" s="2" t="inlineStr"/>
+      <c r="M100" s="2" t="inlineStr"/>
+    </row>
+    <row r="101" ht="30" customHeight="1">
+      <c r="A101" s="2" t="inlineStr">
+        <is>
+          <t>Vomera Group</t>
+        </is>
+      </c>
+      <c r="B101" s="4" t="inlineStr">
+        <is>
+          <t>Nao</t>
+        </is>
+      </c>
+      <c r="C101" s="4" t="inlineStr">
+        <is>
+          <t>351 243 078 442</t>
+        </is>
+      </c>
+      <c r="D101" s="2" t="inlineStr"/>
+      <c r="E101" s="2" t="inlineStr">
+        <is>
+          <t>vomera.pt</t>
+        </is>
+      </c>
+      <c r="F101" s="4" t="inlineStr">
+        <is>
+          <t>Santarém</t>
+        </is>
+      </c>
+      <c r="G101" s="4" t="inlineStr">
+        <is>
+          <t>Santarém</t>
+        </is>
+      </c>
+      <c r="H101" s="2" t="inlineStr"/>
+      <c r="I101" s="2" t="inlineStr">
+        <is>
           <t>Empreendimento residencial de luxo (nome não divulgado) (Comercialização/Lançamento)</t>
         </is>
       </c>
-      <c r="J99" s="2" t="inlineStr">
+      <c r="J101" s="2" t="inlineStr">
         <is>
           <t>Fonte: omirante.pt</t>
         </is>
       </c>
-      <c r="K99" s="2" t="inlineStr">
+      <c r="K101" s="2" t="inlineStr">
         <is>
           <t>Sérgio Santos (CEO/fundador, com Delphine Gerardo)</t>
         </is>
       </c>
-      <c r="L99" s="2" t="inlineStr"/>
-      <c r="M99" s="2" t="inlineStr"/>
-    </row>
-    <row r="100" ht="30" customHeight="1">
-      <c r="A100" s="5" t="inlineStr">
-        <is>
-          <t>Algarve Property Shops</t>
-        </is>
-      </c>
-      <c r="B100" s="7" t="inlineStr">
-        <is>
-          <t>Nao</t>
-        </is>
-      </c>
-      <c r="C100" s="7" t="inlineStr"/>
-      <c r="D100" s="5" t="inlineStr"/>
-      <c r="E100" s="5" t="inlineStr"/>
-      <c r="F100" s="7" t="inlineStr">
-        <is>
-          <t>Tavira</t>
-        </is>
-      </c>
-      <c r="G100" s="7" t="inlineStr">
-        <is>
-          <t>Faro</t>
-        </is>
-      </c>
-      <c r="H100" s="5" t="inlineStr"/>
-      <c r="I100" s="5" t="inlineStr">
-        <is>
-          <t>Varandas de Cabanas (Em construção/Comercialização)</t>
-        </is>
-      </c>
-      <c r="J100" s="5" t="inlineStr">
-        <is>
-          <t>Fonte: idealista.pt</t>
-        </is>
-      </c>
-      <c r="K100" s="5" t="inlineStr"/>
-      <c r="L100" s="5" t="inlineStr"/>
-      <c r="M100" s="5" t="inlineStr"/>
-    </row>
-    <row r="101" ht="30" customHeight="1">
-      <c r="A101" s="5" t="inlineStr">
-        <is>
-          <t>Amorim Luxury</t>
-        </is>
-      </c>
-      <c r="B101" s="7" t="inlineStr">
-        <is>
-          <t>Nao</t>
-        </is>
-      </c>
-      <c r="C101" s="7" t="inlineStr"/>
-      <c r="D101" s="5" t="inlineStr"/>
-      <c r="E101" s="5" t="inlineStr"/>
-      <c r="F101" s="7" t="inlineStr">
-        <is>
-          <t>Lisboa/Grândola/Lagoa</t>
-        </is>
-      </c>
-      <c r="G101" s="7" t="inlineStr">
-        <is>
-          <t>Lisboa</t>
-        </is>
-      </c>
-      <c r="H101" s="5" t="inlineStr"/>
-      <c r="I101" s="5" t="inlineStr">
-        <is>
-          <t>JNcQUOI House (Av. Liberdade) (Em construção)</t>
-        </is>
-      </c>
-      <c r="J101" s="5" t="inlineStr">
-        <is>
-          <t>Fonte: idealista.pt, vidaimobiliaria.com</t>
-        </is>
-      </c>
-      <c r="K101" s="5" t="inlineStr">
-        <is>
-          <t>Miguel Guedes de Sousa (Founder &amp; CEO)</t>
-        </is>
-      </c>
-      <c r="L101" s="5" t="inlineStr"/>
-      <c r="M101" s="5" t="inlineStr"/>
+      <c r="L101" s="2" t="inlineStr"/>
+      <c r="M101" s="2" t="inlineStr"/>
     </row>
     <row r="102" ht="30" customHeight="1">
       <c r="A102" s="5" t="inlineStr">
         <is>
-          <t>Aresta Vitalicia</t>
+          <t>Algarve Property Shops</t>
         </is>
       </c>
       <c r="B102" s="7" t="inlineStr">
@@ -6254,23 +6290,23 @@
       <c r="E102" s="5" t="inlineStr"/>
       <c r="F102" s="7" t="inlineStr">
         <is>
-          <t>Setúbal</t>
+          <t>Tavira</t>
         </is>
       </c>
       <c r="G102" s="7" t="inlineStr">
         <is>
-          <t>Setúbal</t>
+          <t>Faro</t>
         </is>
       </c>
       <c r="H102" s="5" t="inlineStr"/>
       <c r="I102" s="5" t="inlineStr">
         <is>
-          <t>WeBuild Castelo (Comercialização)</t>
+          <t>Varandas de Cabanas (Em construção/Comercialização)</t>
         </is>
       </c>
       <c r="J102" s="5" t="inlineStr">
         <is>
-          <t>Fonte: construir.pt</t>
+          <t>Fonte: idealista.pt</t>
         </is>
       </c>
       <c r="K102" s="5" t="inlineStr"/>
@@ -6280,7 +6316,7 @@
     <row r="103" ht="30" customHeight="1">
       <c r="A103" s="5" t="inlineStr">
         <is>
-          <t>Arrow Global Portugal</t>
+          <t>Amorim Luxury</t>
         </is>
       </c>
       <c r="B103" s="7" t="inlineStr">
@@ -6293,28 +6329,28 @@
       <c r="E103" s="5" t="inlineStr"/>
       <c r="F103" s="7" t="inlineStr">
         <is>
-          <t>Loulé (Almancil/Quinta do Lago)</t>
+          <t>Lisboa/Grândola/Lagoa</t>
         </is>
       </c>
       <c r="G103" s="7" t="inlineStr">
         <is>
-          <t>Faro</t>
+          <t>Lisboa</t>
         </is>
       </c>
       <c r="H103" s="5" t="inlineStr"/>
       <c r="I103" s="5" t="inlineStr">
         <is>
-          <t>The Shore Residences (Comercialização)</t>
+          <t>JNcQUOI House (Av. Liberdade) (Em construção)</t>
         </is>
       </c>
       <c r="J103" s="5" t="inlineStr">
         <is>
-          <t>Fonte: idealista.pt, jornaleconomico.sapo.pt</t>
+          <t>Fonte: idealista.pt, vidaimobiliaria.com</t>
         </is>
       </c>
       <c r="K103" s="5" t="inlineStr">
         <is>
-          <t>João Bugalho (CEO)</t>
+          <t>Miguel Guedes de Sousa (Founder &amp; CEO)</t>
         </is>
       </c>
       <c r="L103" s="5" t="inlineStr"/>
@@ -6323,7 +6359,7 @@
     <row r="104" ht="30" customHeight="1">
       <c r="A104" s="5" t="inlineStr">
         <is>
-          <t>Baltor – Engenharia e Construção</t>
+          <t>Aresta Vitalicia</t>
         </is>
       </c>
       <c r="B104" s="7" t="inlineStr">
@@ -6333,14 +6369,10 @@
       </c>
       <c r="C104" s="7" t="inlineStr"/>
       <c r="D104" s="5" t="inlineStr"/>
-      <c r="E104" s="5" t="inlineStr">
-        <is>
-          <t>baltor.pt</t>
-        </is>
-      </c>
+      <c r="E104" s="5" t="inlineStr"/>
       <c r="F104" s="7" t="inlineStr">
         <is>
-          <t>Setúbal (sede Viana do Castelo)</t>
+          <t>Setúbal</t>
         </is>
       </c>
       <c r="G104" s="7" t="inlineStr">
@@ -6351,26 +6383,22 @@
       <c r="H104" s="5" t="inlineStr"/>
       <c r="I104" s="5" t="inlineStr">
         <is>
-          <t>Parque da Cidade – Riverside III (Em construção)</t>
+          <t>WeBuild Castelo (Comercialização)</t>
         </is>
       </c>
       <c r="J104" s="5" t="inlineStr">
         <is>
-          <t>Fonte: ominho.pt</t>
-        </is>
-      </c>
-      <c r="K104" s="5" t="inlineStr">
-        <is>
-          <t>Paulo Balinha e Bruno Torres (fundadores, 2008)</t>
-        </is>
-      </c>
+          <t>Fonte: construir.pt</t>
+        </is>
+      </c>
+      <c r="K104" s="5" t="inlineStr"/>
       <c r="L104" s="5" t="inlineStr"/>
       <c r="M104" s="5" t="inlineStr"/>
     </row>
     <row r="105" ht="30" customHeight="1">
       <c r="A105" s="5" t="inlineStr">
         <is>
-          <t>Bond Group</t>
+          <t>Arrow Global Portugal</t>
         </is>
       </c>
       <c r="B105" s="7" t="inlineStr">
@@ -6383,33 +6411,37 @@
       <c r="E105" s="5" t="inlineStr"/>
       <c r="F105" s="7" t="inlineStr">
         <is>
-          <t>Amares</t>
+          <t>Loulé (Almancil/Quinta do Lago)</t>
         </is>
       </c>
       <c r="G105" s="7" t="inlineStr">
         <is>
-          <t>Braga</t>
+          <t>Faro</t>
         </is>
       </c>
       <c r="H105" s="5" t="inlineStr"/>
       <c r="I105" s="5" t="inlineStr">
         <is>
-          <t>José Azevedo Prime Living (Ferreiros, Amares) (Em construção)</t>
+          <t>The Shore Residences (Comercialização)</t>
         </is>
       </c>
       <c r="J105" s="5" t="inlineStr">
         <is>
-          <t>Grupo imobiliário do Minho. Sem contacto direto confirmado nas fontes</t>
-        </is>
-      </c>
-      <c r="K105" s="5" t="inlineStr"/>
+          <t>Fonte: idealista.pt, jornaleconomico.sapo.pt</t>
+        </is>
+      </c>
+      <c r="K105" s="5" t="inlineStr">
+        <is>
+          <t>João Bugalho (CEO)</t>
+        </is>
+      </c>
       <c r="L105" s="5" t="inlineStr"/>
       <c r="M105" s="5" t="inlineStr"/>
     </row>
     <row r="106" ht="30" customHeight="1">
       <c r="A106" s="5" t="inlineStr">
         <is>
-          <t>Branco Real Estate</t>
+          <t>Baltor – Engenharia e Construção</t>
         </is>
       </c>
       <c r="B106" s="7" t="inlineStr">
@@ -6419,36 +6451,44 @@
       </c>
       <c r="C106" s="7" t="inlineStr"/>
       <c r="D106" s="5" t="inlineStr"/>
-      <c r="E106" s="5" t="inlineStr"/>
+      <c r="E106" s="5" t="inlineStr">
+        <is>
+          <t>baltor.pt</t>
+        </is>
+      </c>
       <c r="F106" s="7" t="inlineStr">
         <is>
-          <t>Lagos</t>
+          <t>Setúbal (sede Viana do Castelo)</t>
         </is>
       </c>
       <c r="G106" s="7" t="inlineStr">
         <is>
-          <t>Faro</t>
+          <t>Setúbal</t>
         </is>
       </c>
       <c r="H106" s="5" t="inlineStr"/>
       <c r="I106" s="5" t="inlineStr">
         <is>
-          <t>Domus (Em construção)</t>
+          <t>Parque da Cidade – Riverside III (Em construção)</t>
         </is>
       </c>
       <c r="J106" s="5" t="inlineStr">
         <is>
-          <t>Fonte: idealista.pt/empreendimento/35004962</t>
-        </is>
-      </c>
-      <c r="K106" s="5" t="inlineStr"/>
+          <t>Fonte: ominho.pt</t>
+        </is>
+      </c>
+      <c r="K106" s="5" t="inlineStr">
+        <is>
+          <t>Paulo Balinha e Bruno Torres (fundadores, 2008)</t>
+        </is>
+      </c>
       <c r="L106" s="5" t="inlineStr"/>
       <c r="M106" s="5" t="inlineStr"/>
     </row>
     <row r="107" ht="30" customHeight="1">
       <c r="A107" s="5" t="inlineStr">
         <is>
-          <t>Casas do Sotavento</t>
+          <t>Bond Group</t>
         </is>
       </c>
       <c r="B107" s="7" t="inlineStr">
@@ -6458,30 +6498,26 @@
       </c>
       <c r="C107" s="7" t="inlineStr"/>
       <c r="D107" s="5" t="inlineStr"/>
-      <c r="E107" s="5" t="inlineStr">
-        <is>
-          <t>casasdosotavento.pt</t>
-        </is>
-      </c>
+      <c r="E107" s="5" t="inlineStr"/>
       <c r="F107" s="7" t="inlineStr">
         <is>
-          <t>Tavira</t>
+          <t>Amares</t>
         </is>
       </c>
       <c r="G107" s="7" t="inlineStr">
         <is>
-          <t>Faro</t>
+          <t>Braga</t>
         </is>
       </c>
       <c r="H107" s="5" t="inlineStr"/>
       <c r="I107" s="5" t="inlineStr">
         <is>
-          <t>Boavista Ocean Tavira (Comercialização)</t>
+          <t>José Azevedo Prime Living (Ferreiros, Amares) (Em construção)</t>
         </is>
       </c>
       <c r="J107" s="5" t="inlineStr">
         <is>
-          <t>Fonte: boavistaoceantavira.com</t>
+          <t>Grupo imobiliário do Minho. Sem contacto direto confirmado nas fontes</t>
         </is>
       </c>
       <c r="K107" s="5" t="inlineStr"/>
@@ -6491,7 +6527,7 @@
     <row r="108" ht="30" customHeight="1">
       <c r="A108" s="5" t="inlineStr">
         <is>
-          <t>Confidential Sphere – Investimento Imobiliário</t>
+          <t>Branco Real Estate</t>
         </is>
       </c>
       <c r="B108" s="7" t="inlineStr">
@@ -6504,7 +6540,7 @@
       <c r="E108" s="5" t="inlineStr"/>
       <c r="F108" s="7" t="inlineStr">
         <is>
-          <t>Silves</t>
+          <t>Lagos</t>
         </is>
       </c>
       <c r="G108" s="7" t="inlineStr">
@@ -6515,12 +6551,12 @@
       <c r="H108" s="5" t="inlineStr"/>
       <c r="I108" s="5" t="inlineStr">
         <is>
-          <t>Quinta do Pateiro / Silves Hills (Planeamento)</t>
+          <t>Domus (Em construção)</t>
         </is>
       </c>
       <c r="J108" s="5" t="inlineStr">
         <is>
-          <t>Fonte: terraruiva.pt, barlavento.pt</t>
+          <t>Fonte: idealista.pt/empreendimento/35004962</t>
         </is>
       </c>
       <c r="K108" s="5" t="inlineStr"/>
@@ -6530,7 +6566,7 @@
     <row r="109" ht="30" customHeight="1">
       <c r="A109" s="5" t="inlineStr">
         <is>
-          <t>CS Ribeiro</t>
+          <t>Casas do Sotavento</t>
         </is>
       </c>
       <c r="B109" s="7" t="inlineStr">
@@ -6540,26 +6576,30 @@
       </c>
       <c r="C109" s="7" t="inlineStr"/>
       <c r="D109" s="5" t="inlineStr"/>
-      <c r="E109" s="5" t="inlineStr"/>
+      <c r="E109" s="5" t="inlineStr">
+        <is>
+          <t>casasdosotavento.pt</t>
+        </is>
+      </c>
       <c r="F109" s="7" t="inlineStr">
         <is>
-          <t>Guarda (atua Viseu/Coimbra)</t>
+          <t>Tavira</t>
         </is>
       </c>
       <c r="G109" s="7" t="inlineStr">
         <is>
-          <t>Guarda</t>
+          <t>Faro</t>
         </is>
       </c>
       <c r="H109" s="5" t="inlineStr"/>
       <c r="I109" s="5" t="inlineStr">
         <is>
-          <t>The Town Signature (Solum, Coimbra) (Em construção)</t>
+          <t>Boavista Ocean Tavira (Comercialização)</t>
         </is>
       </c>
       <c r="J109" s="5" t="inlineStr">
         <is>
-          <t>Fonte: diariocoimbra.pt</t>
+          <t>Fonte: boavistaoceantavira.com</t>
         </is>
       </c>
       <c r="K109" s="5" t="inlineStr"/>
@@ -6569,7 +6609,7 @@
     <row r="110" ht="30" customHeight="1">
       <c r="A110" s="5" t="inlineStr">
         <is>
-          <t>Discovery Land Company</t>
+          <t>Confidential Sphere – Investimento Imobiliário</t>
         </is>
       </c>
       <c r="B110" s="7" t="inlineStr">
@@ -6579,30 +6619,26 @@
       </c>
       <c r="C110" s="7" t="inlineStr"/>
       <c r="D110" s="5" t="inlineStr"/>
-      <c r="E110" s="5" t="inlineStr">
-        <is>
-          <t>discoverylandco.com</t>
-        </is>
-      </c>
+      <c r="E110" s="5" t="inlineStr"/>
       <c r="F110" s="7" t="inlineStr">
         <is>
-          <t>Grândola (Melides)</t>
+          <t>Silves</t>
         </is>
       </c>
       <c r="G110" s="7" t="inlineStr">
         <is>
-          <t>Setúbal</t>
+          <t>Faro</t>
         </is>
       </c>
       <c r="H110" s="5" t="inlineStr"/>
       <c r="I110" s="5" t="inlineStr">
         <is>
-          <t>CostaTerra Golf &amp; Ocean Club (Em construção/Comercialização)</t>
+          <t>Quinta do Pateiro / Silves Hills (Planeamento)</t>
         </is>
       </c>
       <c r="J110" s="5" t="inlineStr">
         <is>
-          <t>Fonte: brainsre.news</t>
+          <t>Fonte: terraruiva.pt, barlavento.pt</t>
         </is>
       </c>
       <c r="K110" s="5" t="inlineStr"/>
@@ -6612,7 +6648,7 @@
     <row r="111" ht="30" customHeight="1">
       <c r="A111" s="5" t="inlineStr">
         <is>
-          <t>DUJA – Sociedade de Construções, Lda</t>
+          <t>CS Ribeiro</t>
         </is>
       </c>
       <c r="B111" s="7" t="inlineStr">
@@ -6625,23 +6661,23 @@
       <c r="E111" s="5" t="inlineStr"/>
       <c r="F111" s="7" t="inlineStr">
         <is>
-          <t>Tavira</t>
+          <t>Guarda (atua Viseu/Coimbra)</t>
         </is>
       </c>
       <c r="G111" s="7" t="inlineStr">
         <is>
-          <t>Faro</t>
+          <t>Guarda</t>
         </is>
       </c>
       <c r="H111" s="5" t="inlineStr"/>
       <c r="I111" s="5" t="inlineStr">
         <is>
-          <t>Royal Cabanas Beach I e II (Comercialização)</t>
+          <t>The Town Signature (Solum, Coimbra) (Em construção)</t>
         </is>
       </c>
       <c r="J111" s="5" t="inlineStr">
         <is>
-          <t>Fonte: remax.pt, tavitel.pt</t>
+          <t>Fonte: diariocoimbra.pt</t>
         </is>
       </c>
       <c r="K111" s="5" t="inlineStr"/>
@@ -6651,7 +6687,7 @@
     <row r="112" ht="30" customHeight="1">
       <c r="A112" s="5" t="inlineStr">
         <is>
-          <t>Emblezart</t>
+          <t>Discovery Land Company</t>
         </is>
       </c>
       <c r="B112" s="7" t="inlineStr">
@@ -6661,44 +6697,40 @@
       </c>
       <c r="C112" s="7" t="inlineStr"/>
       <c r="D112" s="5" t="inlineStr"/>
-      <c r="E112" s="5" t="inlineStr"/>
+      <c r="E112" s="5" t="inlineStr">
+        <is>
+          <t>discoverylandco.com</t>
+        </is>
+      </c>
       <c r="F112" s="7" t="inlineStr">
         <is>
-          <t>Guimarães</t>
+          <t>Grândola (Melides)</t>
         </is>
       </c>
       <c r="G112" s="7" t="inlineStr">
         <is>
-          <t>Braga</t>
+          <t>Setúbal</t>
         </is>
       </c>
       <c r="H112" s="5" t="inlineStr"/>
       <c r="I112" s="5" t="inlineStr">
         <is>
-          <t>Botânico Avenida (Em construção (fase inicial))</t>
+          <t>CostaTerra Golf &amp; Ocean Club (Em construção/Comercialização)</t>
         </is>
       </c>
       <c r="J112" s="5" t="inlineStr">
         <is>
-          <t>Fonte: idealista.pt</t>
-        </is>
-      </c>
-      <c r="K112" s="5" t="inlineStr">
-        <is>
-          <t>David Faria (CEO e sócio único)</t>
-        </is>
-      </c>
-      <c r="L112" s="5" t="inlineStr">
-        <is>
-          <t>https://www.linkedin.com/in/david-faria-a301a466/</t>
-        </is>
-      </c>
+          <t>Fonte: brainsre.news</t>
+        </is>
+      </c>
+      <c r="K112" s="5" t="inlineStr"/>
+      <c r="L112" s="5" t="inlineStr"/>
       <c r="M112" s="5" t="inlineStr"/>
     </row>
     <row r="113" ht="30" customHeight="1">
       <c r="A113" s="5" t="inlineStr">
         <is>
-          <t>Encobarra</t>
+          <t>DUJA – Sociedade de Construções, Lda</t>
         </is>
       </c>
       <c r="B113" s="7" t="inlineStr">
@@ -6711,37 +6743,33 @@
       <c r="E113" s="5" t="inlineStr"/>
       <c r="F113" s="7" t="inlineStr">
         <is>
-          <t>Aveiro (Aradas)</t>
+          <t>Tavira</t>
         </is>
       </c>
       <c r="G113" s="7" t="inlineStr">
         <is>
-          <t>Aveiro</t>
+          <t>Faro</t>
         </is>
       </c>
       <c r="H113" s="5" t="inlineStr"/>
       <c r="I113" s="5" t="inlineStr">
         <is>
-          <t>Quinta da Pinheira (Em construção)</t>
+          <t>Royal Cabanas Beach I e II (Comercialização)</t>
         </is>
       </c>
       <c r="J113" s="5" t="inlineStr">
         <is>
-          <t>Fonte: noticiasdeaveiro.pt, terranova.pt</t>
-        </is>
-      </c>
-      <c r="K113" s="5" t="inlineStr">
-        <is>
-          <t>Aristides Alferes (administrador)</t>
-        </is>
-      </c>
+          <t>Fonte: remax.pt, tavitel.pt</t>
+        </is>
+      </c>
+      <c r="K113" s="5" t="inlineStr"/>
       <c r="L113" s="5" t="inlineStr"/>
       <c r="M113" s="5" t="inlineStr"/>
     </row>
     <row r="114" ht="30" customHeight="1">
       <c r="A114" s="5" t="inlineStr">
         <is>
-          <t>Estrutural Group</t>
+          <t>Emblezart</t>
         </is>
       </c>
       <c r="B114" s="7" t="inlineStr">
@@ -6754,37 +6782,41 @@
       <c r="E114" s="5" t="inlineStr"/>
       <c r="F114" s="7" t="inlineStr">
         <is>
-          <t>Vila Franca de Xira</t>
+          <t>Guimarães</t>
         </is>
       </c>
       <c r="G114" s="7" t="inlineStr">
         <is>
-          <t>Lisboa</t>
+          <t>Braga</t>
         </is>
       </c>
       <c r="H114" s="5" t="inlineStr"/>
       <c r="I114" s="5" t="inlineStr">
         <is>
-          <t>Vila Viva (Em construção)</t>
+          <t>Botânico Avenida (Em construção (fase inicial))</t>
         </is>
       </c>
       <c r="J114" s="5" t="inlineStr">
         <is>
-          <t>Fonte: vidaimobiliaria.com</t>
+          <t>Fonte: idealista.pt</t>
         </is>
       </c>
       <c r="K114" s="5" t="inlineStr">
         <is>
-          <t>Hugo Mendes Pinto (Managing Partner)</t>
-        </is>
-      </c>
-      <c r="L114" s="5" t="inlineStr"/>
+          <t>David Faria (CEO e sócio único)</t>
+        </is>
+      </c>
+      <c r="L114" s="5" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/david-faria-a301a466/</t>
+        </is>
+      </c>
       <c r="M114" s="5" t="inlineStr"/>
     </row>
     <row r="115" ht="30" customHeight="1">
       <c r="A115" s="5" t="inlineStr">
         <is>
-          <t>Explorer Investments (Explorer Real Estate)</t>
+          <t>Encobarra</t>
         </is>
       </c>
       <c r="B115" s="7" t="inlineStr">
@@ -6794,35 +6826,31 @@
       </c>
       <c r="C115" s="7" t="inlineStr"/>
       <c r="D115" s="5" t="inlineStr"/>
-      <c r="E115" s="5" t="inlineStr">
-        <is>
-          <t>explorerinvestments.com</t>
-        </is>
-      </c>
+      <c r="E115" s="5" t="inlineStr"/>
       <c r="F115" s="7" t="inlineStr">
         <is>
-          <t>Sintra</t>
+          <t>Aveiro (Aradas)</t>
         </is>
       </c>
       <c r="G115" s="7" t="inlineStr">
         <is>
-          <t>Lisboa</t>
+          <t>Aveiro</t>
         </is>
       </c>
       <c r="H115" s="5" t="inlineStr"/>
       <c r="I115" s="5" t="inlineStr">
         <is>
-          <t>CPHP / Penha Longa (Operação/Asset management (desde 2018))</t>
+          <t>Quinta da Pinheira (Em construção)</t>
         </is>
       </c>
       <c r="J115" s="5" t="inlineStr">
         <is>
-          <t>Fonte: jornaldenegocios.pt</t>
+          <t>Fonte: noticiasdeaveiro.pt, terranova.pt</t>
         </is>
       </c>
       <c r="K115" s="5" t="inlineStr">
         <is>
-          <t>Elizabeth Rothfield (CEO, Founding Partner)</t>
+          <t>Aristides Alferes (administrador)</t>
         </is>
       </c>
       <c r="L115" s="5" t="inlineStr"/>
@@ -6831,7 +6859,7 @@
     <row r="116" ht="30" customHeight="1">
       <c r="A116" s="5" t="inlineStr">
         <is>
-          <t>Finangeste, S.A.</t>
+          <t>Estrutural Group</t>
         </is>
       </c>
       <c r="B116" s="7" t="inlineStr">
@@ -6844,28 +6872,28 @@
       <c r="E116" s="5" t="inlineStr"/>
       <c r="F116" s="7" t="inlineStr">
         <is>
-          <t>Faro</t>
+          <t>Vila Franca de Xira</t>
         </is>
       </c>
       <c r="G116" s="7" t="inlineStr">
         <is>
-          <t>Faro</t>
+          <t>Lisboa</t>
         </is>
       </c>
       <c r="H116" s="5" t="inlineStr"/>
       <c r="I116" s="5" t="inlineStr">
         <is>
-          <t>PUVA (Planeamento/Em construção)</t>
+          <t>Vila Viva (Em construção)</t>
         </is>
       </c>
       <c r="J116" s="5" t="inlineStr">
         <is>
-          <t>Fonte: jornaldenegocios.pt, idealista.pt</t>
+          <t>Fonte: vidaimobiliaria.com</t>
         </is>
       </c>
       <c r="K116" s="5" t="inlineStr">
         <is>
-          <t>Paul Henri Schelfhout (Presidente do CA) / Armando Lacerda Queiroz (administrador)</t>
+          <t>Hugo Mendes Pinto (Managing Partner)</t>
         </is>
       </c>
       <c r="L116" s="5" t="inlineStr"/>
@@ -6874,7 +6902,7 @@
     <row r="117" ht="30" customHeight="1">
       <c r="A117" s="5" t="inlineStr">
         <is>
-          <t>FourPromo, Lda (Grupo M2O)</t>
+          <t>Explorer Investments (Explorer Real Estate)</t>
         </is>
       </c>
       <c r="B117" s="7" t="inlineStr">
@@ -6884,36 +6912,44 @@
       </c>
       <c r="C117" s="7" t="inlineStr"/>
       <c r="D117" s="5" t="inlineStr"/>
-      <c r="E117" s="5" t="inlineStr"/>
+      <c r="E117" s="5" t="inlineStr">
+        <is>
+          <t>explorerinvestments.com</t>
+        </is>
+      </c>
       <c r="F117" s="7" t="inlineStr">
         <is>
-          <t>Loulé (Vilamoura)</t>
+          <t>Sintra</t>
         </is>
       </c>
       <c r="G117" s="7" t="inlineStr">
         <is>
-          <t>Faro</t>
+          <t>Lisboa</t>
         </is>
       </c>
       <c r="H117" s="5" t="inlineStr"/>
       <c r="I117" s="5" t="inlineStr">
         <is>
-          <t>Rivus (Em construção/Comercialização)</t>
+          <t>CPHP / Penha Longa (Operação/Asset management (desde 2018))</t>
         </is>
       </c>
       <c r="J117" s="5" t="inlineStr">
         <is>
-          <t>Fonte: construir.pt, idealista.pt</t>
-        </is>
-      </c>
-      <c r="K117" s="5" t="inlineStr"/>
+          <t>Fonte: jornaldenegocios.pt</t>
+        </is>
+      </c>
+      <c r="K117" s="5" t="inlineStr">
+        <is>
+          <t>Elizabeth Rothfield (CEO, Founding Partner)</t>
+        </is>
+      </c>
       <c r="L117" s="5" t="inlineStr"/>
       <c r="M117" s="5" t="inlineStr"/>
     </row>
     <row r="118" ht="30" customHeight="1">
       <c r="A118" s="5" t="inlineStr">
         <is>
-          <t>Foz Gala Investments</t>
+          <t>Finangeste, S.A.</t>
         </is>
       </c>
       <c r="B118" s="7" t="inlineStr">
@@ -6926,33 +6962,37 @@
       <c r="E118" s="5" t="inlineStr"/>
       <c r="F118" s="7" t="inlineStr">
         <is>
-          <t>Figueira da Foz</t>
+          <t>Faro</t>
         </is>
       </c>
       <c r="G118" s="7" t="inlineStr">
         <is>
-          <t>Coimbra</t>
+          <t>Faro</t>
         </is>
       </c>
       <c r="H118" s="5" t="inlineStr"/>
       <c r="I118" s="5" t="inlineStr">
         <is>
-          <t>Urbanização antiga fábrica Alberto Gaspar (Planeamento (estudo prévio))</t>
+          <t>PUVA (Planeamento/Em construção)</t>
         </is>
       </c>
       <c r="J118" s="5" t="inlineStr">
         <is>
-          <t>Fonte: idealista.pt, asbeiras.pt</t>
-        </is>
-      </c>
-      <c r="K118" s="5" t="inlineStr"/>
+          <t>Fonte: jornaldenegocios.pt, idealista.pt</t>
+        </is>
+      </c>
+      <c r="K118" s="5" t="inlineStr">
+        <is>
+          <t>Paul Henri Schelfhout (Presidente do CA) / Armando Lacerda Queiroz (administrador)</t>
+        </is>
+      </c>
       <c r="L118" s="5" t="inlineStr"/>
       <c r="M118" s="5" t="inlineStr"/>
     </row>
     <row r="119" ht="30" customHeight="1">
       <c r="A119" s="5" t="inlineStr">
         <is>
-          <t>Galvana Investimentos Imobiliários e Turísticos, Lda</t>
+          <t>FourPromo, Lda (Grupo M2O)</t>
         </is>
       </c>
       <c r="B119" s="7" t="inlineStr">
@@ -6965,7 +7005,7 @@
       <c r="E119" s="5" t="inlineStr"/>
       <c r="F119" s="7" t="inlineStr">
         <is>
-          <t>Albufeira</t>
+          <t>Loulé (Vilamoura)</t>
         </is>
       </c>
       <c r="G119" s="7" t="inlineStr">
@@ -6976,12 +7016,12 @@
       <c r="H119" s="5" t="inlineStr"/>
       <c r="I119" s="5" t="inlineStr">
         <is>
-          <t>Quinta Dourada (Em construção)</t>
+          <t>Rivus (Em construção/Comercialização)</t>
         </is>
       </c>
       <c r="J119" s="5" t="inlineStr">
         <is>
-          <t>Fonte: oconnormurphy.ie, postal.pt</t>
+          <t>Fonte: construir.pt, idealista.pt</t>
         </is>
       </c>
       <c r="K119" s="5" t="inlineStr"/>
@@ -6991,7 +7031,7 @@
     <row r="120" ht="30" customHeight="1">
       <c r="A120" s="5" t="inlineStr">
         <is>
-          <t>Genuino Investments</t>
+          <t>Foz Gala Investments</t>
         </is>
       </c>
       <c r="B120" s="7" t="inlineStr">
@@ -7001,30 +7041,26 @@
       </c>
       <c r="C120" s="7" t="inlineStr"/>
       <c r="D120" s="5" t="inlineStr"/>
-      <c r="E120" s="5" t="inlineStr">
-        <is>
-          <t>genuinoinvestments.com</t>
-        </is>
-      </c>
+      <c r="E120" s="5" t="inlineStr"/>
       <c r="F120" s="7" t="inlineStr">
         <is>
-          <t>Portimão</t>
+          <t>Figueira da Foz</t>
         </is>
       </c>
       <c r="G120" s="7" t="inlineStr">
         <is>
-          <t>Faro</t>
+          <t>Coimbra</t>
         </is>
       </c>
       <c r="H120" s="5" t="inlineStr"/>
       <c r="I120" s="5" t="inlineStr">
         <is>
-          <t>Genuíno Resort / Praia da Rocha (Comercialização)</t>
+          <t>Urbanização antiga fábrica Alberto Gaspar (Planeamento (estudo prévio))</t>
         </is>
       </c>
       <c r="J120" s="5" t="inlineStr">
         <is>
-          <t>Fonte: genuinoinvestments.com</t>
+          <t>Fonte: idealista.pt, asbeiras.pt</t>
         </is>
       </c>
       <c r="K120" s="5" t="inlineStr"/>
@@ -7034,7 +7070,7 @@
     <row r="121" ht="30" customHeight="1">
       <c r="A121" s="5" t="inlineStr">
         <is>
-          <t>GFH (Grupo Ferreira Holding) / Ferreira Build Power (marca BeLiving)</t>
+          <t>Galvana Investimentos Imobiliários e Turísticos, Lda</t>
         </is>
       </c>
       <c r="B121" s="7" t="inlineStr">
@@ -7044,14 +7080,10 @@
       </c>
       <c r="C121" s="7" t="inlineStr"/>
       <c r="D121" s="5" t="inlineStr"/>
-      <c r="E121" s="5" t="inlineStr">
-        <is>
-          <t>ferreirabuildpower.com</t>
-        </is>
-      </c>
+      <c r="E121" s="5" t="inlineStr"/>
       <c r="F121" s="7" t="inlineStr">
         <is>
-          <t>Faro/Loulé</t>
+          <t>Albufeira</t>
         </is>
       </c>
       <c r="G121" s="7" t="inlineStr">
@@ -7062,26 +7094,22 @@
       <c r="H121" s="5" t="inlineStr"/>
       <c r="I121" s="5" t="inlineStr">
         <is>
-          <t>BeLiving Faro / BeLiving HCC Loulé (Em construção)</t>
+          <t>Quinta Dourada (Em construção)</t>
         </is>
       </c>
       <c r="J121" s="5" t="inlineStr">
         <is>
-          <t>Fonte: eco.sapo.pt, jornaldenegocios.pt</t>
-        </is>
-      </c>
-      <c r="K121" s="5" t="inlineStr">
-        <is>
-          <t>Joaquim Silva (CEO Ferreira Build Power)</t>
-        </is>
-      </c>
+          <t>Fonte: oconnormurphy.ie, postal.pt</t>
+        </is>
+      </c>
+      <c r="K121" s="5" t="inlineStr"/>
       <c r="L121" s="5" t="inlineStr"/>
       <c r="M121" s="5" t="inlineStr"/>
     </row>
     <row r="122" ht="30" customHeight="1">
       <c r="A122" s="5" t="inlineStr">
         <is>
-          <t>Glowing</t>
+          <t>Genuino Investments</t>
         </is>
       </c>
       <c r="B122" s="7" t="inlineStr">
@@ -7093,28 +7121,28 @@
       <c r="D122" s="5" t="inlineStr"/>
       <c r="E122" s="5" t="inlineStr">
         <is>
-          <t>glowing.pt</t>
+          <t>genuinoinvestments.com</t>
         </is>
       </c>
       <c r="F122" s="7" t="inlineStr">
         <is>
-          <t>Alcácer do Sal</t>
+          <t>Portimão</t>
         </is>
       </c>
       <c r="G122" s="7" t="inlineStr">
         <is>
-          <t>Setúbal</t>
+          <t>Faro</t>
         </is>
       </c>
       <c r="H122" s="5" t="inlineStr"/>
       <c r="I122" s="5" t="inlineStr">
         <is>
-          <t>FiniSal (Em construção/Comercialização)</t>
+          <t>Genuíno Resort / Praia da Rocha (Comercialização)</t>
         </is>
       </c>
       <c r="J122" s="5" t="inlineStr">
         <is>
-          <t>Fonte: idealista.pt</t>
+          <t>Fonte: genuinoinvestments.com</t>
         </is>
       </c>
       <c r="K122" s="5" t="inlineStr"/>
@@ -7124,7 +7152,7 @@
     <row r="123" ht="30" customHeight="1">
       <c r="A123" s="5" t="inlineStr">
         <is>
-          <t>Grupo A. Silva &amp; Silva</t>
+          <t>GFH (Grupo Ferreira Holding) / Ferreira Build Power (marca BeLiving)</t>
         </is>
       </c>
       <c r="B123" s="7" t="inlineStr">
@@ -7134,36 +7162,44 @@
       </c>
       <c r="C123" s="7" t="inlineStr"/>
       <c r="D123" s="5" t="inlineStr"/>
-      <c r="E123" s="5" t="inlineStr"/>
+      <c r="E123" s="5" t="inlineStr">
+        <is>
+          <t>ferreirabuildpower.com</t>
+        </is>
+      </c>
       <c r="F123" s="7" t="inlineStr">
         <is>
-          <t>Seixal</t>
+          <t>Faro/Loulé</t>
         </is>
       </c>
       <c r="G123" s="7" t="inlineStr">
         <is>
-          <t>Setúbal</t>
+          <t>Faro</t>
         </is>
       </c>
       <c r="H123" s="5" t="inlineStr"/>
       <c r="I123" s="5" t="inlineStr">
         <is>
-          <t>Seixal Baía (Planeamento)</t>
+          <t>BeLiving Faro / BeLiving HCC Loulé (Em construção)</t>
         </is>
       </c>
       <c r="J123" s="5" t="inlineStr">
         <is>
-          <t>Fonte: novoperfil.pt</t>
-        </is>
-      </c>
-      <c r="K123" s="5" t="inlineStr"/>
+          <t>Fonte: eco.sapo.pt, jornaldenegocios.pt</t>
+        </is>
+      </c>
+      <c r="K123" s="5" t="inlineStr">
+        <is>
+          <t>Joaquim Silva (CEO Ferreira Build Power)</t>
+        </is>
+      </c>
       <c r="L123" s="5" t="inlineStr"/>
       <c r="M123" s="5" t="inlineStr"/>
     </row>
     <row r="124" ht="30" customHeight="1">
       <c r="A124" s="5" t="inlineStr">
         <is>
-          <t>Grupo André Guimarães (Portugal)</t>
+          <t>Glowing</t>
         </is>
       </c>
       <c r="B124" s="7" t="inlineStr">
@@ -7175,34 +7211,38 @@
       <c r="D124" s="5" t="inlineStr"/>
       <c r="E124" s="5" t="inlineStr">
         <is>
-          <t>andreguimaraes.com.br</t>
-        </is>
-      </c>
-      <c r="F124" s="7" t="inlineStr"/>
-      <c r="G124" s="7" t="inlineStr"/>
+          <t>glowing.pt</t>
+        </is>
+      </c>
+      <c r="F124" s="7" t="inlineStr">
+        <is>
+          <t>Alcácer do Sal</t>
+        </is>
+      </c>
+      <c r="G124" s="7" t="inlineStr">
+        <is>
+          <t>Setúbal</t>
+        </is>
+      </c>
       <c r="H124" s="5" t="inlineStr"/>
       <c r="I124" s="5" t="inlineStr">
         <is>
-          <t>JV com Overseas (Lisboa) (Planeamento) | Porto, Algarve, Douro, Cascais, Alentejo, Amarante (Em construção)</t>
+          <t>FiniSal (Em construção/Comercialização)</t>
         </is>
       </c>
       <c r="J124" s="5" t="inlineStr">
         <is>
-          <t>Entidade PT: André Guimarães - Portugal, Lda (NIF 517865459). Sem contacto PT</t>
-        </is>
-      </c>
-      <c r="K124" s="5" t="inlineStr">
-        <is>
-          <t>Fundador falecido· hoje liderado pelos filhos (Brasil), sem responsável PT confirmado</t>
-        </is>
-      </c>
+          <t>Fonte: idealista.pt</t>
+        </is>
+      </c>
+      <c r="K124" s="5" t="inlineStr"/>
       <c r="L124" s="5" t="inlineStr"/>
       <c r="M124" s="5" t="inlineStr"/>
     </row>
     <row r="125" ht="30" customHeight="1">
       <c r="A125" s="5" t="inlineStr">
         <is>
-          <t>Grupo André Jordan</t>
+          <t>Grupo A. Silva &amp; Silva</t>
         </is>
       </c>
       <c r="B125" s="7" t="inlineStr">
@@ -7212,44 +7252,36 @@
       </c>
       <c r="C125" s="7" t="inlineStr"/>
       <c r="D125" s="5" t="inlineStr"/>
-      <c r="E125" s="5" t="inlineStr">
-        <is>
-          <t>andrejordangroup.pt</t>
-        </is>
-      </c>
+      <c r="E125" s="5" t="inlineStr"/>
       <c r="F125" s="7" t="inlineStr">
         <is>
-          <t>Sintra</t>
+          <t>Seixal</t>
         </is>
       </c>
       <c r="G125" s="7" t="inlineStr">
         <is>
-          <t>Lisboa</t>
+          <t>Setúbal</t>
         </is>
       </c>
       <c r="H125" s="5" t="inlineStr"/>
       <c r="I125" s="5" t="inlineStr">
         <is>
-          <t>Lisbon Green Valley (Belas Clube de Campo) (Em construção)</t>
+          <t>Seixal Baía (Planeamento)</t>
         </is>
       </c>
       <c r="J125" s="5" t="inlineStr">
         <is>
-          <t>Fonte: idealista.pt</t>
-        </is>
-      </c>
-      <c r="K125" s="5" t="inlineStr">
-        <is>
-          <t>Gilberto Jordan (CEO desde 2009 · sucede a André Jordan, falecido 2024)</t>
-        </is>
-      </c>
+          <t>Fonte: novoperfil.pt</t>
+        </is>
+      </c>
+      <c r="K125" s="5" t="inlineStr"/>
       <c r="L125" s="5" t="inlineStr"/>
       <c r="M125" s="5" t="inlineStr"/>
     </row>
     <row r="126" ht="30" customHeight="1">
       <c r="A126" s="5" t="inlineStr">
         <is>
-          <t>Grupo AOC (Aníbal de Oliveira Cristina)</t>
+          <t>Grupo André Guimarães (Portugal)</t>
         </is>
       </c>
       <c r="B126" s="7" t="inlineStr">
@@ -7259,31 +7291,27 @@
       </c>
       <c r="C126" s="7" t="inlineStr"/>
       <c r="D126" s="5" t="inlineStr"/>
-      <c r="E126" s="5" t="inlineStr"/>
-      <c r="F126" s="7" t="inlineStr">
-        <is>
-          <t>Setúbal</t>
-        </is>
-      </c>
-      <c r="G126" s="7" t="inlineStr">
-        <is>
-          <t>Setúbal</t>
-        </is>
-      </c>
+      <c r="E126" s="5" t="inlineStr">
+        <is>
+          <t>andreguimaraes.com.br</t>
+        </is>
+      </c>
+      <c r="F126" s="7" t="inlineStr"/>
+      <c r="G126" s="7" t="inlineStr"/>
       <c r="H126" s="5" t="inlineStr"/>
       <c r="I126" s="5" t="inlineStr">
         <is>
-          <t>Parque da Cidade – Riverside IV (Em construção)</t>
+          <t>JV com Overseas (Lisboa) (Planeamento) | Porto, Algarve, Douro, Cascais, Alentejo, Amarante (Em construção)</t>
         </is>
       </c>
       <c r="J126" s="5" t="inlineStr">
         <is>
-          <t>Fonte: linkedin.com/company/grupo-aoc</t>
+          <t>Entidade PT: André Guimarães - Portugal, Lda (NIF 517865459). Sem contacto PT</t>
         </is>
       </c>
       <c r="K126" s="5" t="inlineStr">
         <is>
-          <t>Aníbal Cristina (fundador, 1990)</t>
+          <t>Fundador falecido· hoje liderado pelos filhos (Brasil), sem responsável PT confirmado</t>
         </is>
       </c>
       <c r="L126" s="5" t="inlineStr"/>
@@ -7292,7 +7320,7 @@
     <row r="127" ht="30" customHeight="1">
       <c r="A127" s="5" t="inlineStr">
         <is>
-          <t>Grupo Azinor</t>
+          <t>Grupo André Jordan</t>
         </is>
       </c>
       <c r="B127" s="7" t="inlineStr">
@@ -7302,10 +7330,14 @@
       </c>
       <c r="C127" s="7" t="inlineStr"/>
       <c r="D127" s="5" t="inlineStr"/>
-      <c r="E127" s="5" t="inlineStr"/>
+      <c r="E127" s="5" t="inlineStr">
+        <is>
+          <t>andrejordangroup.pt</t>
+        </is>
+      </c>
       <c r="F127" s="7" t="inlineStr">
         <is>
-          <t>Oeiras</t>
+          <t>Sintra</t>
         </is>
       </c>
       <c r="G127" s="7" t="inlineStr">
@@ -7316,7 +7348,7 @@
       <c r="H127" s="5" t="inlineStr"/>
       <c r="I127" s="5" t="inlineStr">
         <is>
-          <t>Porto Cruz (Planeamento (consulta pública))</t>
+          <t>Lisbon Green Valley (Belas Clube de Campo) (Em construção)</t>
         </is>
       </c>
       <c r="J127" s="5" t="inlineStr">
@@ -7326,20 +7358,16 @@
       </c>
       <c r="K127" s="5" t="inlineStr">
         <is>
-          <t>Carlos Silva Neves (administrador)</t>
-        </is>
-      </c>
-      <c r="L127" s="5" t="inlineStr">
-        <is>
-          <t>https://pt.linkedin.com/in/carlos-silva-neves-3b0711142</t>
-        </is>
-      </c>
+          <t>Gilberto Jordan (CEO desde 2009 · sucede a André Jordan, falecido 2024)</t>
+        </is>
+      </c>
+      <c r="L127" s="5" t="inlineStr"/>
       <c r="M127" s="5" t="inlineStr"/>
     </row>
     <row r="128" ht="30" customHeight="1">
       <c r="A128" s="5" t="inlineStr">
         <is>
-          <t>Grupo Mais Empresas / Construções Mais</t>
+          <t>Grupo AOC (Aníbal de Oliveira Cristina)</t>
         </is>
       </c>
       <c r="B128" s="7" t="inlineStr">
@@ -7349,40 +7377,40 @@
       </c>
       <c r="C128" s="7" t="inlineStr"/>
       <c r="D128" s="5" t="inlineStr"/>
-      <c r="E128" s="5" t="inlineStr">
-        <is>
-          <t>grupomaisempresas.pt</t>
-        </is>
-      </c>
+      <c r="E128" s="5" t="inlineStr"/>
       <c r="F128" s="7" t="inlineStr">
         <is>
-          <t>Leiria</t>
+          <t>Setúbal</t>
         </is>
       </c>
       <c r="G128" s="7" t="inlineStr">
         <is>
-          <t>Leiria</t>
+          <t>Setúbal</t>
         </is>
       </c>
       <c r="H128" s="5" t="inlineStr"/>
       <c r="I128" s="5" t="inlineStr">
         <is>
-          <t>Golden Wolf (Em construção)</t>
+          <t>Parque da Cidade – Riverside IV (Em construção)</t>
         </is>
       </c>
       <c r="J128" s="5" t="inlineStr">
         <is>
-          <t>Fonte: idealista.pt</t>
-        </is>
-      </c>
-      <c r="K128" s="5" t="inlineStr"/>
+          <t>Fonte: linkedin.com/company/grupo-aoc</t>
+        </is>
+      </c>
+      <c r="K128" s="5" t="inlineStr">
+        <is>
+          <t>Aníbal Cristina (fundador, 1990)</t>
+        </is>
+      </c>
       <c r="L128" s="5" t="inlineStr"/>
       <c r="M128" s="5" t="inlineStr"/>
     </row>
     <row r="129" ht="30" customHeight="1">
       <c r="A129" s="5" t="inlineStr">
         <is>
-          <t>Grupo NB Portugal</t>
+          <t>Grupo Azinor</t>
         </is>
       </c>
       <c r="B129" s="7" t="inlineStr">
@@ -7392,44 +7420,44 @@
       </c>
       <c r="C129" s="7" t="inlineStr"/>
       <c r="D129" s="5" t="inlineStr"/>
-      <c r="E129" s="5" t="inlineStr">
-        <is>
-          <t>gruponbportugal.pt</t>
-        </is>
-      </c>
+      <c r="E129" s="5" t="inlineStr"/>
       <c r="F129" s="7" t="inlineStr">
         <is>
-          <t>Aveiro</t>
+          <t>Oeiras</t>
         </is>
       </c>
       <c r="G129" s="7" t="inlineStr">
         <is>
-          <t>Aveiro</t>
+          <t>Lisboa</t>
         </is>
       </c>
       <c r="H129" s="5" t="inlineStr"/>
       <c r="I129" s="5" t="inlineStr">
         <is>
-          <t>NB 2040 / NB Garden (estado não confirmado)</t>
+          <t>Porto Cruz (Planeamento (consulta pública))</t>
         </is>
       </c>
       <c r="J129" s="5" t="inlineStr">
         <is>
-          <t>Fonte: gruponb.pt</t>
+          <t>Fonte: idealista.pt</t>
         </is>
       </c>
       <c r="K129" s="5" t="inlineStr">
         <is>
-          <t>Ioav Blanche (presidente)</t>
-        </is>
-      </c>
-      <c r="L129" s="5" t="inlineStr"/>
+          <t>Carlos Silva Neves (administrador)</t>
+        </is>
+      </c>
+      <c r="L129" s="5" t="inlineStr">
+        <is>
+          <t>https://pt.linkedin.com/in/carlos-silva-neves-3b0711142</t>
+        </is>
+      </c>
       <c r="M129" s="5" t="inlineStr"/>
     </row>
     <row r="130" ht="30" customHeight="1">
       <c r="A130" s="5" t="inlineStr">
         <is>
-          <t>Grupo Pestana (Pestana Residences)</t>
+          <t>Grupo Mais Empresas / Construções Mais</t>
         </is>
       </c>
       <c r="B130" s="7" t="inlineStr">
@@ -7441,42 +7469,38 @@
       <c r="D130" s="5" t="inlineStr"/>
       <c r="E130" s="5" t="inlineStr">
         <is>
-          <t>pestana.com</t>
+          <t>grupomaisempresas.pt</t>
         </is>
       </c>
       <c r="F130" s="7" t="inlineStr">
         <is>
-          <t>Sines/Lagoa</t>
+          <t>Leiria</t>
         </is>
       </c>
       <c r="G130" s="7" t="inlineStr">
         <is>
-          <t>Setúbal</t>
+          <t>Leiria</t>
         </is>
       </c>
       <c r="H130" s="5" t="inlineStr"/>
       <c r="I130" s="5" t="inlineStr">
         <is>
-          <t>Pestana Porto Covo Beach Residences (Licenciamento)</t>
+          <t>Golden Wolf (Em construção)</t>
         </is>
       </c>
       <c r="J130" s="5" t="inlineStr">
         <is>
-          <t>Fonte: publico.pt, construir.pt</t>
-        </is>
-      </c>
-      <c r="K130" s="5" t="inlineStr">
-        <is>
-          <t>Dionísio Pestana (Chairman/dono)</t>
-        </is>
-      </c>
+          <t>Fonte: idealista.pt</t>
+        </is>
+      </c>
+      <c r="K130" s="5" t="inlineStr"/>
       <c r="L130" s="5" t="inlineStr"/>
       <c r="M130" s="5" t="inlineStr"/>
     </row>
     <row r="131" ht="30" customHeight="1">
       <c r="A131" s="5" t="inlineStr">
         <is>
-          <t>Hillside House Coimbra, Lda</t>
+          <t>Grupo NB Portugal</t>
         </is>
       </c>
       <c r="B131" s="7" t="inlineStr">
@@ -7488,12 +7512,12 @@
       <c r="D131" s="5" t="inlineStr"/>
       <c r="E131" s="5" t="inlineStr">
         <is>
-          <t>hillside.pt</t>
+          <t>gruponbportugal.pt</t>
         </is>
       </c>
       <c r="F131" s="7" t="inlineStr">
         <is>
-          <t>Mealhada (projeto em Coimbra)</t>
+          <t>Aveiro</t>
         </is>
       </c>
       <c r="G131" s="7" t="inlineStr">
@@ -7504,22 +7528,26 @@
       <c r="H131" s="5" t="inlineStr"/>
       <c r="I131" s="5" t="inlineStr">
         <is>
-          <t>Hillside – Areeiro (2ª fase) (Em construção)</t>
+          <t>NB 2040 / NB Garden (estado não confirmado)</t>
         </is>
       </c>
       <c r="J131" s="5" t="inlineStr">
         <is>
-          <t>Fonte: remax.pt, hillside.pt</t>
-        </is>
-      </c>
-      <c r="K131" s="5" t="inlineStr"/>
+          <t>Fonte: gruponb.pt</t>
+        </is>
+      </c>
+      <c r="K131" s="5" t="inlineStr">
+        <is>
+          <t>Ioav Blanche (presidente)</t>
+        </is>
+      </c>
       <c r="L131" s="5" t="inlineStr"/>
       <c r="M131" s="5" t="inlineStr"/>
     </row>
     <row r="132" ht="30" customHeight="1">
       <c r="A132" s="5" t="inlineStr">
         <is>
-          <t>Iconic Jeunesse, Unipessoal, Lda</t>
+          <t>Grupo Pestana (Pestana Residences)</t>
         </is>
       </c>
       <c r="B132" s="7" t="inlineStr">
@@ -7531,38 +7559,42 @@
       <c r="D132" s="5" t="inlineStr"/>
       <c r="E132" s="5" t="inlineStr">
         <is>
-          <t>zenithresidences.pt</t>
+          <t>pestana.com</t>
         </is>
       </c>
       <c r="F132" s="7" t="inlineStr">
         <is>
-          <t>Portimão</t>
+          <t>Sines/Lagoa</t>
         </is>
       </c>
       <c r="G132" s="7" t="inlineStr">
         <is>
-          <t>Faro</t>
+          <t>Setúbal</t>
         </is>
       </c>
       <c r="H132" s="5" t="inlineStr"/>
       <c r="I132" s="5" t="inlineStr">
         <is>
-          <t>Zenith Residences (Em construção/Planeamento)</t>
+          <t>Pestana Porto Covo Beach Residences (Licenciamento)</t>
         </is>
       </c>
       <c r="J132" s="5" t="inlineStr">
         <is>
-          <t>Fonte: zenithresidences.pt, jamesedition.com</t>
-        </is>
-      </c>
-      <c r="K132" s="5" t="inlineStr"/>
+          <t>Fonte: publico.pt, construir.pt</t>
+        </is>
+      </c>
+      <c r="K132" s="5" t="inlineStr">
+        <is>
+          <t>Dionísio Pestana (Chairman/dono)</t>
+        </is>
+      </c>
       <c r="L132" s="5" t="inlineStr"/>
       <c r="M132" s="5" t="inlineStr"/>
     </row>
     <row r="133" ht="30" customHeight="1">
       <c r="A133" s="5" t="inlineStr">
         <is>
-          <t>Invesquart – Real Estate Promotor</t>
+          <t>Hillside House Coimbra, Lda</t>
         </is>
       </c>
       <c r="B133" s="7" t="inlineStr">
@@ -7572,26 +7604,30 @@
       </c>
       <c r="C133" s="7" t="inlineStr"/>
       <c r="D133" s="5" t="inlineStr"/>
-      <c r="E133" s="5" t="inlineStr"/>
+      <c r="E133" s="5" t="inlineStr">
+        <is>
+          <t>hillside.pt</t>
+        </is>
+      </c>
       <c r="F133" s="7" t="inlineStr">
         <is>
-          <t>Loulé (Quarteira)</t>
+          <t>Mealhada (projeto em Coimbra)</t>
         </is>
       </c>
       <c r="G133" s="7" t="inlineStr">
         <is>
-          <t>Faro</t>
+          <t>Aveiro</t>
         </is>
       </c>
       <c r="H133" s="5" t="inlineStr"/>
       <c r="I133" s="5" t="inlineStr">
         <is>
-          <t>Terraços de Quarteira (Comercialização)</t>
+          <t>Hillside – Areeiro (2ª fase) (Em construção)</t>
         </is>
       </c>
       <c r="J133" s="5" t="inlineStr">
         <is>
-          <t>Fonte: facebook.com/TerracosQuarteira</t>
+          <t>Fonte: remax.pt, hillside.pt</t>
         </is>
       </c>
       <c r="K133" s="5" t="inlineStr"/>
@@ -7601,7 +7637,7 @@
     <row r="134" ht="30" customHeight="1">
       <c r="A134" s="5" t="inlineStr">
         <is>
-          <t>JPAIVA Investimentos / JPAIVA Engenharia e Construção</t>
+          <t>Iconic Jeunesse, Unipessoal, Lda</t>
         </is>
       </c>
       <c r="B134" s="7" t="inlineStr">
@@ -7613,46 +7649,38 @@
       <c r="D134" s="5" t="inlineStr"/>
       <c r="E134" s="5" t="inlineStr">
         <is>
-          <t>jpaiva.pt</t>
+          <t>zenithresidences.pt</t>
         </is>
       </c>
       <c r="F134" s="7" t="inlineStr">
         <is>
-          <t>Coimbra</t>
+          <t>Portimão</t>
         </is>
       </c>
       <c r="G134" s="7" t="inlineStr">
         <is>
-          <t>Coimbra</t>
+          <t>Faro</t>
         </is>
       </c>
       <c r="H134" s="5" t="inlineStr"/>
       <c r="I134" s="5" t="inlineStr">
         <is>
-          <t>Garden Residence 2 (Antanhol) (Em construção/comercialização)</t>
+          <t>Zenith Residences (Em construção/Planeamento)</t>
         </is>
       </c>
       <c r="J134" s="5" t="inlineStr">
         <is>
-          <t>Fonte: jpaiva.pt</t>
-        </is>
-      </c>
-      <c r="K134" s="5" t="inlineStr">
-        <is>
-          <t>Igor Castro (CEO)</t>
-        </is>
-      </c>
-      <c r="L134" s="5" t="inlineStr">
-        <is>
-          <t>https://www.linkedin.com/in/igor-castro-a0026b22b/</t>
-        </is>
-      </c>
+          <t>Fonte: zenithresidences.pt, jamesedition.com</t>
+        </is>
+      </c>
+      <c r="K134" s="5" t="inlineStr"/>
+      <c r="L134" s="5" t="inlineStr"/>
       <c r="M134" s="5" t="inlineStr"/>
     </row>
     <row r="135" ht="30" customHeight="1">
       <c r="A135" s="5" t="inlineStr">
         <is>
-          <t>Le Parc</t>
+          <t>Invesquart – Real Estate Promotor</t>
         </is>
       </c>
       <c r="B135" s="7" t="inlineStr">
@@ -7662,14 +7690,10 @@
       </c>
       <c r="C135" s="7" t="inlineStr"/>
       <c r="D135" s="5" t="inlineStr"/>
-      <c r="E135" s="5" t="inlineStr">
-        <is>
-          <t>leparc.pt</t>
-        </is>
-      </c>
+      <c r="E135" s="5" t="inlineStr"/>
       <c r="F135" s="7" t="inlineStr">
         <is>
-          <t>Faro</t>
+          <t>Loulé (Quarteira)</t>
         </is>
       </c>
       <c r="G135" s="7" t="inlineStr">
@@ -7680,12 +7704,12 @@
       <c r="H135" s="5" t="inlineStr"/>
       <c r="I135" s="5" t="inlineStr">
         <is>
-          <t>Le Parc Faro (Comercialização) | Le Parc Canidelo (V.N. Gaia) (Comercialização)</t>
+          <t>Terraços de Quarteira (Comercialização)</t>
         </is>
       </c>
       <c r="J135" s="5" t="inlineStr">
         <is>
-          <t>Sem telefone próprio confirmado — número encontrado é da comercializadora JLL</t>
+          <t>Fonte: facebook.com/TerracosQuarteira</t>
         </is>
       </c>
       <c r="K135" s="5" t="inlineStr"/>
@@ -7695,7 +7719,7 @@
     <row r="136" ht="30" customHeight="1">
       <c r="A136" s="5" t="inlineStr">
         <is>
-          <t>Lux Premium</t>
+          <t>JPAIVA Investimentos / JPAIVA Engenharia e Construção</t>
         </is>
       </c>
       <c r="B136" s="7" t="inlineStr">
@@ -7707,7 +7731,7 @@
       <c r="D136" s="5" t="inlineStr"/>
       <c r="E136" s="5" t="inlineStr">
         <is>
-          <t>luxpremium.net</t>
+          <t>jpaiva.pt</t>
         </is>
       </c>
       <c r="F136" s="7" t="inlineStr">
@@ -7723,26 +7747,30 @@
       <c r="H136" s="5" t="inlineStr"/>
       <c r="I136" s="5" t="inlineStr">
         <is>
-          <t>Coimbra Premium (Planeamento)</t>
+          <t>Garden Residence 2 (Antanhol) (Em construção/comercialização)</t>
         </is>
       </c>
       <c r="J136" s="5" t="inlineStr">
         <is>
-          <t>Fonte: luxpremium.net</t>
+          <t>Fonte: jpaiva.pt</t>
         </is>
       </c>
       <c r="K136" s="5" t="inlineStr">
         <is>
-          <t>Claude Berda (fundador)</t>
-        </is>
-      </c>
-      <c r="L136" s="5" t="inlineStr"/>
+          <t>Igor Castro (CEO)</t>
+        </is>
+      </c>
+      <c r="L136" s="5" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/igor-castro-a0026b22b/</t>
+        </is>
+      </c>
       <c r="M136" s="5" t="inlineStr"/>
     </row>
     <row r="137" ht="30" customHeight="1">
       <c r="A137" s="5" t="inlineStr">
         <is>
-          <t>MAJA Construções, S.A.</t>
+          <t>Le Parc</t>
         </is>
       </c>
       <c r="B137" s="7" t="inlineStr">
@@ -7752,10 +7780,14 @@
       </c>
       <c r="C137" s="7" t="inlineStr"/>
       <c r="D137" s="5" t="inlineStr"/>
-      <c r="E137" s="5" t="inlineStr"/>
+      <c r="E137" s="5" t="inlineStr">
+        <is>
+          <t>leparc.pt</t>
+        </is>
+      </c>
       <c r="F137" s="7" t="inlineStr">
         <is>
-          <t>Albufeira</t>
+          <t>Faro</t>
         </is>
       </c>
       <c r="G137" s="7" t="inlineStr">
@@ -7766,26 +7798,22 @@
       <c r="H137" s="5" t="inlineStr"/>
       <c r="I137" s="5" t="inlineStr">
         <is>
-          <t>Quinta Dourada (Em construção)</t>
+          <t>Le Parc Faro (Comercialização) | Le Parc Canidelo (V.N. Gaia) (Comercialização)</t>
         </is>
       </c>
       <c r="J137" s="5" t="inlineStr">
         <is>
-          <t>Fonte: oconnormurphy.ie</t>
-        </is>
-      </c>
-      <c r="K137" s="5" t="inlineStr">
-        <is>
-          <t>Manuel António e Jorge Almeida (fundadores, 1972)</t>
-        </is>
-      </c>
+          <t>Sem telefone próprio confirmado — número encontrado é da comercializadora JLL</t>
+        </is>
+      </c>
+      <c r="K137" s="5" t="inlineStr"/>
       <c r="L137" s="5" t="inlineStr"/>
       <c r="M137" s="5" t="inlineStr"/>
     </row>
     <row r="138" ht="30" customHeight="1">
       <c r="A138" s="5" t="inlineStr">
         <is>
-          <t>Mariano Investe – Empreendimentos Imobiliários</t>
+          <t>Lux Premium</t>
         </is>
       </c>
       <c r="B138" s="7" t="inlineStr">
@@ -7795,36 +7823,44 @@
       </c>
       <c r="C138" s="7" t="inlineStr"/>
       <c r="D138" s="5" t="inlineStr"/>
-      <c r="E138" s="5" t="inlineStr"/>
+      <c r="E138" s="5" t="inlineStr">
+        <is>
+          <t>luxpremium.net</t>
+        </is>
+      </c>
       <c r="F138" s="7" t="inlineStr">
         <is>
-          <t>Santarém</t>
+          <t>Coimbra</t>
         </is>
       </c>
       <c r="G138" s="7" t="inlineStr">
         <is>
-          <t>Santarém</t>
+          <t>Coimbra</t>
         </is>
       </c>
       <c r="H138" s="5" t="inlineStr"/>
       <c r="I138" s="5" t="inlineStr">
         <is>
-          <t>Quinta de São Pedro Valley (Em construção)</t>
+          <t>Coimbra Premium (Planeamento)</t>
         </is>
       </c>
       <c r="J138" s="5" t="inlineStr">
         <is>
-          <t>Fonte: idealista.pt</t>
-        </is>
-      </c>
-      <c r="K138" s="5" t="inlineStr"/>
+          <t>Fonte: luxpremium.net</t>
+        </is>
+      </c>
+      <c r="K138" s="5" t="inlineStr">
+        <is>
+          <t>Claude Berda (fundador)</t>
+        </is>
+      </c>
       <c r="L138" s="5" t="inlineStr"/>
       <c r="M138" s="5" t="inlineStr"/>
     </row>
     <row r="139" ht="30" customHeight="1">
       <c r="A139" s="5" t="inlineStr">
         <is>
-          <t>Maven (Maven Invest)</t>
+          <t>MAJA Construções, S.A.</t>
         </is>
       </c>
       <c r="B139" s="7" t="inlineStr">
@@ -7834,35 +7870,31 @@
       </c>
       <c r="C139" s="7" t="inlineStr"/>
       <c r="D139" s="5" t="inlineStr"/>
-      <c r="E139" s="5" t="inlineStr">
-        <is>
-          <t>maveninvest.pt</t>
-        </is>
-      </c>
+      <c r="E139" s="5" t="inlineStr"/>
       <c r="F139" s="7" t="inlineStr">
         <is>
-          <t>Setúbal</t>
+          <t>Albufeira</t>
         </is>
       </c>
       <c r="G139" s="7" t="inlineStr">
         <is>
-          <t>Setúbal</t>
+          <t>Faro</t>
         </is>
       </c>
       <c r="H139" s="5" t="inlineStr"/>
       <c r="I139" s="5" t="inlineStr">
         <is>
-          <t>WeBuild Castelo (Comercialização)</t>
+          <t>Quinta Dourada (Em construção)</t>
         </is>
       </c>
       <c r="J139" s="5" t="inlineStr">
         <is>
-          <t>Fonte: maveninvest.pt</t>
+          <t>Fonte: oconnormurphy.ie</t>
         </is>
       </c>
       <c r="K139" s="5" t="inlineStr">
         <is>
-          <t>Yehonatan Gourvitch (CEO)</t>
+          <t>Manuel António e Jorge Almeida (fundadores, 1972)</t>
         </is>
       </c>
       <c r="L139" s="5" t="inlineStr"/>
@@ -7871,7 +7903,7 @@
     <row r="140" ht="30" customHeight="1">
       <c r="A140" s="5" t="inlineStr">
         <is>
-          <t>Mello RDC</t>
+          <t>Mariano Investe – Empreendimentos Imobiliários</t>
         </is>
       </c>
       <c r="B140" s="7" t="inlineStr">
@@ -7881,48 +7913,36 @@
       </c>
       <c r="C140" s="7" t="inlineStr"/>
       <c r="D140" s="5" t="inlineStr"/>
-      <c r="E140" s="5" t="inlineStr">
-        <is>
-          <t>mellordc.pt</t>
-        </is>
-      </c>
+      <c r="E140" s="5" t="inlineStr"/>
       <c r="F140" s="7" t="inlineStr">
         <is>
-          <t>Grândola (Melides)</t>
+          <t>Santarém</t>
         </is>
       </c>
       <c r="G140" s="7" t="inlineStr">
         <is>
-          <t>Setúbal</t>
+          <t>Santarém</t>
         </is>
       </c>
       <c r="H140" s="5" t="inlineStr"/>
       <c r="I140" s="5" t="inlineStr">
         <is>
-          <t>Projeto hoteleiro em Melides (não divulgado) (Planeamento)</t>
+          <t>Quinta de São Pedro Valley (Em construção)</t>
         </is>
       </c>
       <c r="J140" s="5" t="inlineStr">
         <is>
-          <t>Fonte: vidaimobiliaria.com</t>
-        </is>
-      </c>
-      <c r="K140" s="5" t="inlineStr">
-        <is>
-          <t>António Ribeiro da Cunha (CEO)</t>
-        </is>
-      </c>
-      <c r="L140" s="5" t="inlineStr">
-        <is>
-          <t>https://pt.linkedin.com/in/ant%C3%B3nio-ribeiro-da-cunha-77b974112</t>
-        </is>
-      </c>
+          <t>Fonte: idealista.pt</t>
+        </is>
+      </c>
+      <c r="K140" s="5" t="inlineStr"/>
+      <c r="L140" s="5" t="inlineStr"/>
       <c r="M140" s="5" t="inlineStr"/>
     </row>
     <row r="141" ht="30" customHeight="1">
       <c r="A141" s="5" t="inlineStr">
         <is>
-          <t>Máscarazul – Mediação Imobiliária, Lda</t>
+          <t>Maven (Maven Invest)</t>
         </is>
       </c>
       <c r="B141" s="7" t="inlineStr">
@@ -7932,36 +7952,44 @@
       </c>
       <c r="C141" s="7" t="inlineStr"/>
       <c r="D141" s="5" t="inlineStr"/>
-      <c r="E141" s="5" t="inlineStr"/>
+      <c r="E141" s="5" t="inlineStr">
+        <is>
+          <t>maveninvest.pt</t>
+        </is>
+      </c>
       <c r="F141" s="7" t="inlineStr">
         <is>
-          <t>Albufeira</t>
+          <t>Setúbal</t>
         </is>
       </c>
       <c r="G141" s="7" t="inlineStr">
         <is>
-          <t>Faro</t>
+          <t>Setúbal</t>
         </is>
       </c>
       <c r="H141" s="5" t="inlineStr"/>
       <c r="I141" s="5" t="inlineStr">
         <is>
-          <t>Quinta Dourada (Em construção)</t>
+          <t>WeBuild Castelo (Comercialização)</t>
         </is>
       </c>
       <c r="J141" s="5" t="inlineStr">
         <is>
-          <t>Fonte: ireland-portugal.com</t>
-        </is>
-      </c>
-      <c r="K141" s="5" t="inlineStr"/>
+          <t>Fonte: maveninvest.pt</t>
+        </is>
+      </c>
+      <c r="K141" s="5" t="inlineStr">
+        <is>
+          <t>Yehonatan Gourvitch (CEO)</t>
+        </is>
+      </c>
       <c r="L141" s="5" t="inlineStr"/>
       <c r="M141" s="5" t="inlineStr"/>
     </row>
     <row r="142" ht="30" customHeight="1">
       <c r="A142" s="5" t="inlineStr">
         <is>
-          <t>Nova Atlantic</t>
+          <t>Mello RDC</t>
         </is>
       </c>
       <c r="B142" s="7" t="inlineStr">
@@ -7971,40 +7999,48 @@
       </c>
       <c r="C142" s="7" t="inlineStr"/>
       <c r="D142" s="5" t="inlineStr"/>
-      <c r="E142" s="5" t="inlineStr"/>
+      <c r="E142" s="5" t="inlineStr">
+        <is>
+          <t>mellordc.pt</t>
+        </is>
+      </c>
       <c r="F142" s="7" t="inlineStr">
         <is>
-          <t>Viana do Castelo</t>
+          <t>Grândola (Melides)</t>
         </is>
       </c>
       <c r="G142" s="7" t="inlineStr">
         <is>
-          <t>Viana do Castelo</t>
+          <t>Setúbal</t>
         </is>
       </c>
       <c r="H142" s="5" t="inlineStr"/>
       <c r="I142" s="5" t="inlineStr">
         <is>
-          <t>GREEN HILLS Viana Residences (Comercialização (arrancou set/2026))</t>
+          <t>Projeto hoteleiro em Melides (não divulgado) (Planeamento)</t>
         </is>
       </c>
       <c r="J142" s="5" t="inlineStr">
         <is>
-          <t>Fonte: jornaleconomico.sapo.pt</t>
+          <t>Fonte: vidaimobiliaria.com</t>
         </is>
       </c>
       <c r="K142" s="5" t="inlineStr">
         <is>
-          <t>Matan Amitai (co-fundador)</t>
-        </is>
-      </c>
-      <c r="L142" s="5" t="inlineStr"/>
+          <t>António Ribeiro da Cunha (CEO)</t>
+        </is>
+      </c>
+      <c r="L142" s="5" t="inlineStr">
+        <is>
+          <t>https://pt.linkedin.com/in/ant%C3%B3nio-ribeiro-da-cunha-77b974112</t>
+        </is>
+      </c>
       <c r="M142" s="5" t="inlineStr"/>
     </row>
     <row r="143" ht="30" customHeight="1">
       <c r="A143" s="5" t="inlineStr">
         <is>
-          <t>OCM Portugal (O'Connor Murphy)</t>
+          <t>Máscarazul – Mediação Imobiliária, Lda</t>
         </is>
       </c>
       <c r="B143" s="7" t="inlineStr">
@@ -8014,14 +8050,10 @@
       </c>
       <c r="C143" s="7" t="inlineStr"/>
       <c r="D143" s="5" t="inlineStr"/>
-      <c r="E143" s="5" t="inlineStr">
-        <is>
-          <t>oconnormurphy.ie</t>
-        </is>
-      </c>
+      <c r="E143" s="5" t="inlineStr"/>
       <c r="F143" s="7" t="inlineStr">
         <is>
-          <t>Olhão</t>
+          <t>Albufeira</t>
         </is>
       </c>
       <c r="G143" s="7" t="inlineStr">
@@ -8032,12 +8064,12 @@
       <c r="H143" s="5" t="inlineStr"/>
       <c r="I143" s="5" t="inlineStr">
         <is>
-          <t>Del Mar Waterfront Living (Comercialização)</t>
+          <t>Quinta Dourada (Em construção)</t>
         </is>
       </c>
       <c r="J143" s="5" t="inlineStr">
         <is>
-          <t>Fonte: jll.pt, delmarliving.pt</t>
+          <t>Fonte: ireland-portugal.com</t>
         </is>
       </c>
       <c r="K143" s="5" t="inlineStr"/>
@@ -8047,7 +8079,7 @@
     <row r="144" ht="30" customHeight="1">
       <c r="A144" s="5" t="inlineStr">
         <is>
-          <t>Ombria Resort (Grupo Pontos)</t>
+          <t>Nova Atlantic</t>
         </is>
       </c>
       <c r="B144" s="7" t="inlineStr">
@@ -8057,52 +8089,40 @@
       </c>
       <c r="C144" s="7" t="inlineStr"/>
       <c r="D144" s="5" t="inlineStr"/>
-      <c r="E144" s="5" t="inlineStr">
-        <is>
-          <t>ombria.com</t>
-        </is>
-      </c>
+      <c r="E144" s="5" t="inlineStr"/>
       <c r="F144" s="7" t="inlineStr">
         <is>
-          <t>Loulé</t>
+          <t>Viana do Castelo</t>
         </is>
       </c>
       <c r="G144" s="7" t="inlineStr">
         <is>
-          <t>Faro</t>
-        </is>
-      </c>
-      <c r="H144" s="5" t="inlineStr">
-        <is>
-          <t>Loulé</t>
-        </is>
-      </c>
+          <t>Viana do Castelo</t>
+        </is>
+      </c>
+      <c r="H144" s="5" t="inlineStr"/>
       <c r="I144" s="5" t="inlineStr">
         <is>
-          <t>Ombria Algarve (Em construção)</t>
+          <t>GREEN HILLS Viana Residences (Comercialização (arrancou set/2026))</t>
         </is>
       </c>
       <c r="J144" s="5" t="inlineStr">
         <is>
-          <t>Grupo finlandês Pontos · construtor Gabriel Couto</t>
+          <t>Fonte: jornaleconomico.sapo.pt</t>
         </is>
       </c>
       <c r="K144" s="5" t="inlineStr">
         <is>
-          <t>Patrick Freeman (CEO Ombria desde 2023)· CEO do Grupo Pontos é Timo Kokkila</t>
-        </is>
-      </c>
-      <c r="L144" s="5" t="inlineStr">
-        <is>
-          <t>https://www.linkedin.com/in/patricksfreeman/</t>
-        </is>
-      </c>
+          <t>Matan Amitai (co-fundador)</t>
+        </is>
+      </c>
+      <c r="L144" s="5" t="inlineStr"/>
       <c r="M144" s="5" t="inlineStr"/>
     </row>
     <row r="145" ht="30" customHeight="1">
       <c r="A145" s="5" t="inlineStr">
         <is>
-          <t>PATRIMOINIMMO PORTUGAL</t>
+          <t>OCM Portugal (O'Connor Murphy)</t>
         </is>
       </c>
       <c r="B145" s="7" t="inlineStr">
@@ -8112,10 +8132,14 @@
       </c>
       <c r="C145" s="7" t="inlineStr"/>
       <c r="D145" s="5" t="inlineStr"/>
-      <c r="E145" s="5" t="inlineStr"/>
+      <c r="E145" s="5" t="inlineStr">
+        <is>
+          <t>oconnormurphy.ie</t>
+        </is>
+      </c>
       <c r="F145" s="7" t="inlineStr">
         <is>
-          <t>Lagoa</t>
+          <t>Olhão</t>
         </is>
       </c>
       <c r="G145" s="7" t="inlineStr">
@@ -8126,12 +8150,12 @@
       <c r="H145" s="5" t="inlineStr"/>
       <c r="I145" s="5" t="inlineStr">
         <is>
-          <t>Ferragudo Hills Residência (Comercialização)</t>
+          <t>Del Mar Waterfront Living (Comercialização)</t>
         </is>
       </c>
       <c r="J145" s="5" t="inlineStr">
         <is>
-          <t>Fonte: ferreirabuildpower.com</t>
+          <t>Fonte: jll.pt, delmarliving.pt</t>
         </is>
       </c>
       <c r="K145" s="5" t="inlineStr"/>
@@ -8141,7 +8165,7 @@
     <row r="146" ht="30" customHeight="1">
       <c r="A146" s="5" t="inlineStr">
         <is>
-          <t>Pelicano – Investimento Imobiliário, S.A.</t>
+          <t>Ombria Resort (Grupo Pontos)</t>
         </is>
       </c>
       <c r="B146" s="7" t="inlineStr">
@@ -8151,40 +8175,52 @@
       </c>
       <c r="C146" s="7" t="inlineStr"/>
       <c r="D146" s="5" t="inlineStr"/>
-      <c r="E146" s="5" t="inlineStr"/>
+      <c r="E146" s="5" t="inlineStr">
+        <is>
+          <t>ombria.com</t>
+        </is>
+      </c>
       <c r="F146" s="7" t="inlineStr">
         <is>
-          <t>Palmela</t>
+          <t>Loulé</t>
         </is>
       </c>
       <c r="G146" s="7" t="inlineStr">
         <is>
-          <t>Setúbal</t>
-        </is>
-      </c>
-      <c r="H146" s="5" t="inlineStr"/>
+          <t>Faro</t>
+        </is>
+      </c>
+      <c r="H146" s="5" t="inlineStr">
+        <is>
+          <t>Loulé</t>
+        </is>
+      </c>
       <c r="I146" s="5" t="inlineStr">
         <is>
-          <t>Palmela Village (Comercialização)</t>
+          <t>Ombria Algarve (Em construção)</t>
         </is>
       </c>
       <c r="J146" s="5" t="inlineStr">
         <is>
-          <t>Fonte: racius.com, cnnportugal.iol.pt</t>
+          <t>Grupo finlandês Pontos · construtor Gabriel Couto</t>
         </is>
       </c>
       <c r="K146" s="5" t="inlineStr">
         <is>
-          <t>Joaquim Da Cunha Mendes Duarte (Presidente) / Sergio Manuel Mendes Gomes (Administrador)</t>
-        </is>
-      </c>
-      <c r="L146" s="5" t="inlineStr"/>
+          <t>Patrick Freeman (CEO Ombria desde 2023)· CEO do Grupo Pontos é Timo Kokkila</t>
+        </is>
+      </c>
+      <c r="L146" s="5" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/patricksfreeman/</t>
+        </is>
+      </c>
       <c r="M146" s="5" t="inlineStr"/>
     </row>
     <row r="147" ht="30" customHeight="1">
       <c r="A147" s="5" t="inlineStr">
         <is>
-          <t>Pensaplano</t>
+          <t>PATRIMOINIMMO PORTUGAL</t>
         </is>
       </c>
       <c r="B147" s="7" t="inlineStr">
@@ -8197,23 +8233,23 @@
       <c r="E147" s="5" t="inlineStr"/>
       <c r="F147" s="7" t="inlineStr">
         <is>
-          <t>Coimbra</t>
+          <t>Lagoa</t>
         </is>
       </c>
       <c r="G147" s="7" t="inlineStr">
         <is>
-          <t>Coimbra</t>
+          <t>Faro</t>
         </is>
       </c>
       <c r="H147" s="5" t="inlineStr"/>
       <c r="I147" s="5" t="inlineStr">
         <is>
-          <t>Eleven (Em construção)</t>
+          <t>Ferragudo Hills Residência (Comercialização)</t>
         </is>
       </c>
       <c r="J147" s="5" t="inlineStr">
         <is>
-          <t>Fonte: idealista.pt, construir.pt</t>
+          <t>Fonte: ferreirabuildpower.com</t>
         </is>
       </c>
       <c r="K147" s="5" t="inlineStr"/>
@@ -8223,7 +8259,7 @@
     <row r="148" ht="30" customHeight="1">
       <c r="A148" s="5" t="inlineStr">
         <is>
-          <t>Portugal Slow Living</t>
+          <t>Pelicano – Investimento Imobiliário, S.A.</t>
         </is>
       </c>
       <c r="B148" s="7" t="inlineStr">
@@ -8236,7 +8272,7 @@
       <c r="E148" s="5" t="inlineStr"/>
       <c r="F148" s="7" t="inlineStr">
         <is>
-          <t>Montijo</t>
+          <t>Palmela</t>
         </is>
       </c>
       <c r="G148" s="7" t="inlineStr">
@@ -8247,22 +8283,26 @@
       <c r="H148" s="5" t="inlineStr"/>
       <c r="I148" s="5" t="inlineStr">
         <is>
-          <t>Monville (Comercialização)</t>
+          <t>Palmela Village (Comercialização)</t>
         </is>
       </c>
       <c r="J148" s="5" t="inlineStr">
         <is>
-          <t>Fonte: idealista.pt</t>
-        </is>
-      </c>
-      <c r="K148" s="5" t="inlineStr"/>
+          <t>Fonte: racius.com, cnnportugal.iol.pt</t>
+        </is>
+      </c>
+      <c r="K148" s="5" t="inlineStr">
+        <is>
+          <t>Joaquim Da Cunha Mendes Duarte (Presidente) / Sergio Manuel Mendes Gomes (Administrador)</t>
+        </is>
+      </c>
       <c r="L148" s="5" t="inlineStr"/>
       <c r="M148" s="5" t="inlineStr"/>
     </row>
     <row r="149" ht="30" customHeight="1">
       <c r="A149" s="5" t="inlineStr">
         <is>
-          <t>Rivage Properties</t>
+          <t>Pensaplano</t>
         </is>
       </c>
       <c r="B149" s="7" t="inlineStr">
@@ -8275,37 +8315,33 @@
       <c r="E149" s="5" t="inlineStr"/>
       <c r="F149" s="7" t="inlineStr">
         <is>
-          <t>Gondomar</t>
+          <t>Coimbra</t>
         </is>
       </c>
       <c r="G149" s="7" t="inlineStr">
         <is>
-          <t>Porto</t>
+          <t>Coimbra</t>
         </is>
       </c>
       <c r="H149" s="5" t="inlineStr"/>
       <c r="I149" s="5" t="inlineStr">
         <is>
-          <t>The View II (Em construção (conclusão 2026))</t>
+          <t>Eleven (Em construção)</t>
         </is>
       </c>
       <c r="J149" s="5" t="inlineStr">
         <is>
-          <t>Fonte: jornaldenegocios.pt</t>
-        </is>
-      </c>
-      <c r="K149" s="5" t="inlineStr">
-        <is>
-          <t>João Ribeiro (CEO e fundador, com Jorge Duarte e Fernando Santos)</t>
-        </is>
-      </c>
+          <t>Fonte: idealista.pt, construir.pt</t>
+        </is>
+      </c>
+      <c r="K149" s="5" t="inlineStr"/>
       <c r="L149" s="5" t="inlineStr"/>
       <c r="M149" s="5" t="inlineStr"/>
     </row>
     <row r="150" ht="30" customHeight="1">
       <c r="A150" s="5" t="inlineStr">
         <is>
-          <t>Rodrigues &amp; Vermelho – Construções, S.A.</t>
+          <t>Portugal Slow Living</t>
         </is>
       </c>
       <c r="B150" s="7" t="inlineStr">
@@ -8315,44 +8351,36 @@
       </c>
       <c r="C150" s="7" t="inlineStr"/>
       <c r="D150" s="5" t="inlineStr"/>
-      <c r="E150" s="5" t="inlineStr">
-        <is>
-          <t>rodriguesevermelho.com</t>
-        </is>
-      </c>
+      <c r="E150" s="5" t="inlineStr"/>
       <c r="F150" s="7" t="inlineStr">
         <is>
-          <t>Lagos</t>
+          <t>Montijo</t>
         </is>
       </c>
       <c r="G150" s="7" t="inlineStr">
         <is>
-          <t>Faro</t>
+          <t>Setúbal</t>
         </is>
       </c>
       <c r="H150" s="5" t="inlineStr"/>
       <c r="I150" s="5" t="inlineStr">
         <is>
-          <t>Domus (Domus 22 e 23) (Em construção)</t>
+          <t>Monville (Comercialização)</t>
         </is>
       </c>
       <c r="J150" s="5" t="inlineStr">
         <is>
-          <t>Fonte: sava.pt, thepreplan.com</t>
-        </is>
-      </c>
-      <c r="K150" s="5" t="inlineStr">
-        <is>
-          <t>Celestino Vermelho Rodrigues (contacto)</t>
-        </is>
-      </c>
+          <t>Fonte: idealista.pt</t>
+        </is>
+      </c>
+      <c r="K150" s="5" t="inlineStr"/>
       <c r="L150" s="5" t="inlineStr"/>
       <c r="M150" s="5" t="inlineStr"/>
     </row>
     <row r="151" ht="30" customHeight="1">
       <c r="A151" s="5" t="inlineStr">
         <is>
-          <t>Soccal &amp; Vaz Invest</t>
+          <t>Rivage Properties</t>
         </is>
       </c>
       <c r="B151" s="7" t="inlineStr">
@@ -8362,48 +8390,40 @@
       </c>
       <c r="C151" s="7" t="inlineStr"/>
       <c r="D151" s="5" t="inlineStr"/>
-      <c r="E151" s="5" t="inlineStr">
-        <is>
-          <t>soccal-vaz.com</t>
-        </is>
-      </c>
+      <c r="E151" s="5" t="inlineStr"/>
       <c r="F151" s="7" t="inlineStr">
         <is>
-          <t>Sines</t>
+          <t>Gondomar</t>
         </is>
       </c>
       <c r="G151" s="7" t="inlineStr">
         <is>
-          <t>Setúbal</t>
+          <t>Porto</t>
         </is>
       </c>
       <c r="H151" s="5" t="inlineStr"/>
       <c r="I151" s="5" t="inlineStr">
         <is>
-          <t>Brisa Mar (Em construção)</t>
+          <t>The View II (Em construção (conclusão 2026))</t>
         </is>
       </c>
       <c r="J151" s="5" t="inlineStr">
         <is>
-          <t>Fonte: eco.sapo.pt</t>
+          <t>Fonte: jornaldenegocios.pt</t>
         </is>
       </c>
       <c r="K151" s="5" t="inlineStr">
         <is>
-          <t>António Vaz (fundador e CEO)</t>
-        </is>
-      </c>
-      <c r="L151" s="5" t="inlineStr">
-        <is>
-          <t>https://www.linkedin.com/in/antonio-vaz-9444998a/</t>
-        </is>
-      </c>
+          <t>João Ribeiro (CEO e fundador, com Jorge Duarte e Fernando Santos)</t>
+        </is>
+      </c>
+      <c r="L151" s="5" t="inlineStr"/>
       <c r="M151" s="5" t="inlineStr"/>
     </row>
     <row r="152" ht="30" customHeight="1">
       <c r="A152" s="5" t="inlineStr">
         <is>
-          <t>Solid Sentinel</t>
+          <t>Rodrigues &amp; Vermelho – Construções, S.A.</t>
         </is>
       </c>
       <c r="B152" s="7" t="inlineStr">
@@ -8415,46 +8435,42 @@
       <c r="D152" s="5" t="inlineStr"/>
       <c r="E152" s="5" t="inlineStr">
         <is>
-          <t>solidsentinel.pt</t>
+          <t>rodriguesevermelho.com</t>
         </is>
       </c>
       <c r="F152" s="7" t="inlineStr">
         <is>
-          <t>Barreiro</t>
+          <t>Lagos</t>
         </is>
       </c>
       <c r="G152" s="7" t="inlineStr">
         <is>
-          <t>Setúbal</t>
+          <t>Faro</t>
         </is>
       </c>
       <c r="H152" s="5" t="inlineStr"/>
       <c r="I152" s="5" t="inlineStr">
         <is>
-          <t>NOOBA (Em construção/comercialização)</t>
+          <t>Domus (Domus 22 e 23) (Em construção)</t>
         </is>
       </c>
       <c r="J152" s="5" t="inlineStr">
         <is>
-          <t>Fonte: reportugal.vidaimobiliaria.com</t>
+          <t>Fonte: sava.pt, thepreplan.com</t>
         </is>
       </c>
       <c r="K152" s="5" t="inlineStr">
         <is>
-          <t>Alain Gross (Co-Founder e CEO)</t>
-        </is>
-      </c>
-      <c r="L152" s="5" t="inlineStr">
-        <is>
-          <t>https://www.linkedin.com/in/alain-gross-3351411/</t>
-        </is>
-      </c>
+          <t>Celestino Vermelho Rodrigues (contacto)</t>
+        </is>
+      </c>
+      <c r="L152" s="5" t="inlineStr"/>
       <c r="M152" s="5" t="inlineStr"/>
     </row>
     <row r="153" ht="30" customHeight="1">
       <c r="A153" s="5" t="inlineStr">
         <is>
-          <t>SOLUM PROGRESS</t>
+          <t>Soccal &amp; Vaz Invest</t>
         </is>
       </c>
       <c r="B153" s="7" t="inlineStr">
@@ -8464,36 +8480,48 @@
       </c>
       <c r="C153" s="7" t="inlineStr"/>
       <c r="D153" s="5" t="inlineStr"/>
-      <c r="E153" s="5" t="inlineStr"/>
+      <c r="E153" s="5" t="inlineStr">
+        <is>
+          <t>soccal-vaz.com</t>
+        </is>
+      </c>
       <c r="F153" s="7" t="inlineStr">
         <is>
-          <t>Coimbra</t>
+          <t>Sines</t>
         </is>
       </c>
       <c r="G153" s="7" t="inlineStr">
         <is>
-          <t>Coimbra</t>
+          <t>Setúbal</t>
         </is>
       </c>
       <c r="H153" s="5" t="inlineStr"/>
       <c r="I153" s="5" t="inlineStr">
         <is>
-          <t>Namora Residence (Solum, Sto. António dos Olivais) (Em construção/comercialização)</t>
+          <t>Brisa Mar (Em construção)</t>
         </is>
       </c>
       <c r="J153" s="5" t="inlineStr">
         <is>
-          <t>Fonte: jpaiva.pt, zome.pt</t>
-        </is>
-      </c>
-      <c r="K153" s="5" t="inlineStr"/>
-      <c r="L153" s="5" t="inlineStr"/>
+          <t>Fonte: eco.sapo.pt</t>
+        </is>
+      </c>
+      <c r="K153" s="5" t="inlineStr">
+        <is>
+          <t>António Vaz (fundador e CEO)</t>
+        </is>
+      </c>
+      <c r="L153" s="5" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/antonio-vaz-9444998a/</t>
+        </is>
+      </c>
       <c r="M153" s="5" t="inlineStr"/>
     </row>
     <row r="154" ht="30" customHeight="1">
       <c r="A154" s="5" t="inlineStr">
         <is>
-          <t>Sonae Sierra</t>
+          <t>Solid Sentinel</t>
         </is>
       </c>
       <c r="B154" s="7" t="inlineStr">
@@ -8505,42 +8533,46 @@
       <c r="D154" s="5" t="inlineStr"/>
       <c r="E154" s="5" t="inlineStr">
         <is>
-          <t>sonaesierra.com</t>
+          <t>solidsentinel.pt</t>
         </is>
       </c>
       <c r="F154" s="7" t="inlineStr">
         <is>
-          <t>Lisboa/Porto</t>
+          <t>Barreiro</t>
         </is>
       </c>
       <c r="G154" s="7" t="inlineStr">
         <is>
-          <t>nacional</t>
+          <t>Setúbal</t>
         </is>
       </c>
       <c r="H154" s="5" t="inlineStr"/>
       <c r="I154" s="5" t="inlineStr">
         <is>
-          <t>Pulse Lisboa (Em construção)</t>
+          <t>NOOBA (Em construção/comercialização)</t>
         </is>
       </c>
       <c r="J154" s="5" t="inlineStr">
         <is>
-          <t>Fonte: rtp.pt, idealista.pt</t>
+          <t>Fonte: reportugal.vidaimobiliaria.com</t>
         </is>
       </c>
       <c r="K154" s="5" t="inlineStr">
         <is>
-          <t>Fernando Guedes de Oliveira (CEO)</t>
-        </is>
-      </c>
-      <c r="L154" s="5" t="inlineStr"/>
+          <t>Alain Gross (Co-Founder e CEO)</t>
+        </is>
+      </c>
+      <c r="L154" s="5" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/alain-gross-3351411/</t>
+        </is>
+      </c>
       <c r="M154" s="5" t="inlineStr"/>
     </row>
     <row r="155" ht="30" customHeight="1">
       <c r="A155" s="5" t="inlineStr">
         <is>
-          <t>Southshore Investments</t>
+          <t>SOLUM PROGRESS</t>
         </is>
       </c>
       <c r="B155" s="7" t="inlineStr">
@@ -8550,30 +8582,26 @@
       </c>
       <c r="C155" s="7" t="inlineStr"/>
       <c r="D155" s="5" t="inlineStr"/>
-      <c r="E155" s="5" t="inlineStr">
-        <is>
-          <t>southshoreinvest.com</t>
-        </is>
-      </c>
+      <c r="E155" s="5" t="inlineStr"/>
       <c r="F155" s="7" t="inlineStr">
         <is>
-          <t>Almada</t>
+          <t>Coimbra</t>
         </is>
       </c>
       <c r="G155" s="7" t="inlineStr">
         <is>
-          <t>Setúbal</t>
+          <t>Coimbra</t>
         </is>
       </c>
       <c r="H155" s="5" t="inlineStr"/>
       <c r="I155" s="5" t="inlineStr">
         <is>
-          <t>Tejo City District (Planeamento)</t>
+          <t>Namora Residence (Solum, Sto. António dos Olivais) (Em construção/comercialização)</t>
         </is>
       </c>
       <c r="J155" s="5" t="inlineStr">
         <is>
-          <t>Fonte: southshoreinvest.com</t>
+          <t>Fonte: jpaiva.pt, zome.pt</t>
         </is>
       </c>
       <c r="K155" s="5" t="inlineStr"/>
@@ -8583,7 +8611,7 @@
     <row r="156" ht="30" customHeight="1">
       <c r="A156" s="5" t="inlineStr">
         <is>
-          <t>Square View</t>
+          <t>Sonae Sierra</t>
         </is>
       </c>
       <c r="B156" s="7" t="inlineStr">
@@ -8595,33 +8623,33 @@
       <c r="D156" s="5" t="inlineStr"/>
       <c r="E156" s="5" t="inlineStr">
         <is>
-          <t>squareview.pt</t>
+          <t>sonaesierra.com</t>
         </is>
       </c>
       <c r="F156" s="7" t="inlineStr">
         <is>
-          <t>Lisboa/Ericeira/Melides</t>
+          <t>Lisboa/Porto</t>
         </is>
       </c>
       <c r="G156" s="7" t="inlineStr">
         <is>
-          <t>Lisboa</t>
+          <t>nacional</t>
         </is>
       </c>
       <c r="H156" s="5" t="inlineStr"/>
       <c r="I156" s="5" t="inlineStr">
         <is>
-          <t>4 projetos residenciais multifamiliares (nomes não encontrados) (Em desenvolvimento)</t>
+          <t>Pulse Lisboa (Em construção)</t>
         </is>
       </c>
       <c r="J156" s="5" t="inlineStr">
         <is>
-          <t>Fonte: squareview.pt</t>
+          <t>Fonte: rtp.pt, idealista.pt</t>
         </is>
       </c>
       <c r="K156" s="5" t="inlineStr">
         <is>
-          <t>Luis Horta e Costa (CEO/Fundador)</t>
+          <t>Fernando Guedes de Oliveira (CEO)</t>
         </is>
       </c>
       <c r="L156" s="5" t="inlineStr"/>
@@ -8630,7 +8658,7 @@
     <row r="157" ht="30" customHeight="1">
       <c r="A157" s="5" t="inlineStr">
         <is>
-          <t>Terrace Benefit, Lda</t>
+          <t>Southshore Investments</t>
         </is>
       </c>
       <c r="B157" s="7" t="inlineStr">
@@ -8640,26 +8668,30 @@
       </c>
       <c r="C157" s="7" t="inlineStr"/>
       <c r="D157" s="5" t="inlineStr"/>
-      <c r="E157" s="5" t="inlineStr"/>
+      <c r="E157" s="5" t="inlineStr">
+        <is>
+          <t>southshoreinvest.com</t>
+        </is>
+      </c>
       <c r="F157" s="7" t="inlineStr">
         <is>
-          <t>Loulé (Quarteira)</t>
+          <t>Almada</t>
         </is>
       </c>
       <c r="G157" s="7" t="inlineStr">
         <is>
-          <t>Faro</t>
+          <t>Setúbal</t>
         </is>
       </c>
       <c r="H157" s="5" t="inlineStr"/>
       <c r="I157" s="5" t="inlineStr">
         <is>
-          <t>Forte Novo (Em construção)</t>
+          <t>Tejo City District (Planeamento)</t>
         </is>
       </c>
       <c r="J157" s="5" t="inlineStr">
         <is>
-          <t>Fonte: racius.com, idealista.pt</t>
+          <t>Fonte: southshoreinvest.com</t>
         </is>
       </c>
       <c r="K157" s="5" t="inlineStr"/>
@@ -8669,7 +8701,7 @@
     <row r="158" ht="30" customHeight="1">
       <c r="A158" s="5" t="inlineStr">
         <is>
-          <t>The Epic Group</t>
+          <t>Square View</t>
         </is>
       </c>
       <c r="B158" s="7" t="inlineStr">
@@ -8681,38 +8713,42 @@
       <c r="D158" s="5" t="inlineStr"/>
       <c r="E158" s="5" t="inlineStr">
         <is>
-          <t>valentavillas.com</t>
+          <t>squareview.pt</t>
         </is>
       </c>
       <c r="F158" s="7" t="inlineStr">
         <is>
-          <t>Ílhavo</t>
+          <t>Lisboa/Ericeira/Melides</t>
         </is>
       </c>
       <c r="G158" s="7" t="inlineStr">
         <is>
-          <t>Aveiro</t>
+          <t>Lisboa</t>
         </is>
       </c>
       <c r="H158" s="5" t="inlineStr"/>
       <c r="I158" s="5" t="inlineStr">
         <is>
-          <t>Valenta Villas (Ermida, Ílhavo) (Comercialização)</t>
+          <t>4 projetos residenciais multifamiliares (nomes não encontrados) (Em desenvolvimento)</t>
         </is>
       </c>
       <c r="J158" s="5" t="inlineStr">
         <is>
-          <t>Sem telefone/CEO confirmados nas fontes</t>
-        </is>
-      </c>
-      <c r="K158" s="5" t="inlineStr"/>
+          <t>Fonte: squareview.pt</t>
+        </is>
+      </c>
+      <c r="K158" s="5" t="inlineStr">
+        <is>
+          <t>Luis Horta e Costa (CEO/Fundador)</t>
+        </is>
+      </c>
       <c r="L158" s="5" t="inlineStr"/>
       <c r="M158" s="5" t="inlineStr"/>
     </row>
     <row r="159" ht="30" customHeight="1">
       <c r="A159" s="5" t="inlineStr">
         <is>
-          <t>Udra – Grupo San José</t>
+          <t>Terrace Benefit, Lda</t>
         </is>
       </c>
       <c r="B159" s="7" t="inlineStr">
@@ -8725,23 +8761,23 @@
       <c r="E159" s="5" t="inlineStr"/>
       <c r="F159" s="7" t="inlineStr">
         <is>
-          <t>Setúbal</t>
+          <t>Loulé (Quarteira)</t>
         </is>
       </c>
       <c r="G159" s="7" t="inlineStr">
         <is>
-          <t>Setúbal</t>
+          <t>Faro</t>
         </is>
       </c>
       <c r="H159" s="5" t="inlineStr"/>
       <c r="I159" s="5" t="inlineStr">
         <is>
-          <t>Parque da Cidade – Riverside II (Em construção)</t>
+          <t>Forte Novo (Em construção)</t>
         </is>
       </c>
       <c r="J159" s="5" t="inlineStr">
         <is>
-          <t>Fonte: idealista.pt</t>
+          <t>Fonte: racius.com, idealista.pt</t>
         </is>
       </c>
       <c r="K159" s="5" t="inlineStr"/>
@@ -8751,7 +8787,7 @@
     <row r="160" ht="30" customHeight="1">
       <c r="A160" s="5" t="inlineStr">
         <is>
-          <t>Urban Green Private (UGP)</t>
+          <t>The Epic Group</t>
         </is>
       </c>
       <c r="B160" s="7" t="inlineStr">
@@ -8763,42 +8799,38 @@
       <c r="D160" s="5" t="inlineStr"/>
       <c r="E160" s="5" t="inlineStr">
         <is>
-          <t>ugp.ie</t>
+          <t>valentavillas.com</t>
         </is>
       </c>
       <c r="F160" s="7" t="inlineStr">
         <is>
-          <t>Faro</t>
+          <t>Ílhavo</t>
         </is>
       </c>
       <c r="G160" s="7" t="inlineStr">
         <is>
-          <t>Faro</t>
+          <t>Aveiro</t>
         </is>
       </c>
       <c r="H160" s="5" t="inlineStr"/>
       <c r="I160" s="5" t="inlineStr">
         <is>
-          <t>The Shipyard (Comercialização)</t>
+          <t>Valenta Villas (Ermida, Ílhavo) (Comercialização)</t>
         </is>
       </c>
       <c r="J160" s="5" t="inlineStr">
         <is>
-          <t>Fonte: theshipyard.pt, barlavento.pt</t>
-        </is>
-      </c>
-      <c r="K160" s="5" t="inlineStr">
-        <is>
-          <t>Thomas Coughlan (fundador)</t>
-        </is>
-      </c>
+          <t>Sem telefone/CEO confirmados nas fontes</t>
+        </is>
+      </c>
+      <c r="K160" s="5" t="inlineStr"/>
       <c r="L160" s="5" t="inlineStr"/>
       <c r="M160" s="5" t="inlineStr"/>
     </row>
     <row r="161" ht="30" customHeight="1">
       <c r="A161" s="5" t="inlineStr">
         <is>
-          <t>Vale do Lobo Resort</t>
+          <t>Udra – Grupo San José</t>
         </is>
       </c>
       <c r="B161" s="7" t="inlineStr">
@@ -8808,34 +8840,26 @@
       </c>
       <c r="C161" s="7" t="inlineStr"/>
       <c r="D161" s="5" t="inlineStr"/>
-      <c r="E161" s="5" t="inlineStr">
-        <is>
-          <t>valedolobo.com</t>
-        </is>
-      </c>
+      <c r="E161" s="5" t="inlineStr"/>
       <c r="F161" s="7" t="inlineStr">
         <is>
-          <t>Loulé</t>
+          <t>Setúbal</t>
         </is>
       </c>
       <c r="G161" s="7" t="inlineStr">
         <is>
-          <t>Faro</t>
-        </is>
-      </c>
-      <c r="H161" s="5" t="inlineStr">
-        <is>
-          <t>Parque do Golfe</t>
-        </is>
-      </c>
+          <t>Setúbal</t>
+        </is>
+      </c>
+      <c r="H161" s="5" t="inlineStr"/>
       <c r="I161" s="5" t="inlineStr">
         <is>
-          <t>Vale Real (lotes/moradias em planta) (Planeamento) | Oceano Clube (Comercialização) | The Residences (Comercialização)</t>
+          <t>Parque da Cidade – Riverside II (Em construção)</t>
         </is>
       </c>
       <c r="J161" s="5" t="inlineStr">
         <is>
-          <t>Adquirido 2022 por fundo assessorado pela Davidson Kempner Capital Management. Promotor/gestor operacional: Kronos Real Estate Group</t>
+          <t>Fonte: idealista.pt</t>
         </is>
       </c>
       <c r="K161" s="5" t="inlineStr"/>
@@ -8845,7 +8869,7 @@
     <row r="162" ht="30" customHeight="1">
       <c r="A162" s="5" t="inlineStr">
         <is>
-          <t>Vila Galé</t>
+          <t>Urban Green Private (UGP)</t>
         </is>
       </c>
       <c r="B162" s="7" t="inlineStr">
@@ -8857,33 +8881,174 @@
       <c r="D162" s="5" t="inlineStr"/>
       <c r="E162" s="5" t="inlineStr">
         <is>
-          <t>vilagale.com</t>
+          <t>ugp.ie</t>
         </is>
       </c>
       <c r="F162" s="7" t="inlineStr">
         <is>
-          <t>Golegã</t>
+          <t>Faro</t>
         </is>
       </c>
       <c r="G162" s="7" t="inlineStr">
         <is>
-          <t>Santarém</t>
+          <t>Faro</t>
         </is>
       </c>
       <c r="H162" s="5" t="inlineStr"/>
       <c r="I162" s="5" t="inlineStr">
         <is>
-          <t>Vila Galé Collection Tejo (Quinta da Cardiga) (Em construção)</t>
+          <t>The Shipyard (Comercialização)</t>
         </is>
       </c>
       <c r="J162" s="5" t="inlineStr">
         <is>
-          <t>Fonte: idealista.pt</t>
-        </is>
-      </c>
-      <c r="K162" s="5" t="inlineStr"/>
+          <t>Fonte: theshipyard.pt, barlavento.pt</t>
+        </is>
+      </c>
+      <c r="K162" s="5" t="inlineStr">
+        <is>
+          <t>Thomas Coughlan (fundador)</t>
+        </is>
+      </c>
       <c r="L162" s="5" t="inlineStr"/>
       <c r="M162" s="5" t="inlineStr"/>
+    </row>
+    <row r="163" ht="30" customHeight="1">
+      <c r="A163" s="5" t="inlineStr">
+        <is>
+          <t>Urban Office</t>
+        </is>
+      </c>
+      <c r="B163" s="7" t="inlineStr">
+        <is>
+          <t>Nao</t>
+        </is>
+      </c>
+      <c r="C163" s="7" t="inlineStr"/>
+      <c r="D163" s="5" t="inlineStr"/>
+      <c r="E163" s="5" t="inlineStr">
+        <is>
+          <t>urbanoffice.pt</t>
+        </is>
+      </c>
+      <c r="F163" s="7" t="inlineStr">
+        <is>
+          <t>Torres Vedras</t>
+        </is>
+      </c>
+      <c r="G163" s="7" t="inlineStr">
+        <is>
+          <t>Lisboa</t>
+        </is>
+      </c>
+      <c r="H163" s="5" t="inlineStr">
+        <is>
+          <t>Rua Paiva de Andrade 6A, 2560-357</t>
+        </is>
+      </c>
+      <c r="I163" s="5" t="inlineStr">
+        <is>
+          <t>Torres Prime (Torres Vedras) (Em construção)</t>
+        </is>
+      </c>
+      <c r="J163" s="5" t="inlineStr">
+        <is>
+          <t>Do Grupo Riberalves (&gt;30 anos de história). Nota: site autodenomina-se promotora, mas core histórico é mediação imobiliária</t>
+        </is>
+      </c>
+      <c r="K163" s="5" t="inlineStr"/>
+      <c r="L163" s="5" t="inlineStr"/>
+      <c r="M163" s="5" t="inlineStr"/>
+    </row>
+    <row r="164" ht="30" customHeight="1">
+      <c r="A164" s="5" t="inlineStr">
+        <is>
+          <t>Vale do Lobo Resort</t>
+        </is>
+      </c>
+      <c r="B164" s="7" t="inlineStr">
+        <is>
+          <t>Nao</t>
+        </is>
+      </c>
+      <c r="C164" s="7" t="inlineStr"/>
+      <c r="D164" s="5" t="inlineStr"/>
+      <c r="E164" s="5" t="inlineStr">
+        <is>
+          <t>valedolobo.com</t>
+        </is>
+      </c>
+      <c r="F164" s="7" t="inlineStr">
+        <is>
+          <t>Loulé</t>
+        </is>
+      </c>
+      <c r="G164" s="7" t="inlineStr">
+        <is>
+          <t>Faro</t>
+        </is>
+      </c>
+      <c r="H164" s="5" t="inlineStr">
+        <is>
+          <t>Parque do Golfe</t>
+        </is>
+      </c>
+      <c r="I164" s="5" t="inlineStr">
+        <is>
+          <t>Vale Real (lotes/moradias em planta) (Planeamento) | Oceano Clube (Comercialização) | The Residences (Comercialização)</t>
+        </is>
+      </c>
+      <c r="J164" s="5" t="inlineStr">
+        <is>
+          <t>Adquirido 2022 por fundo assessorado pela Davidson Kempner Capital Management. Promotor/gestor operacional: Kronos Real Estate Group</t>
+        </is>
+      </c>
+      <c r="K164" s="5" t="inlineStr"/>
+      <c r="L164" s="5" t="inlineStr"/>
+      <c r="M164" s="5" t="inlineStr"/>
+    </row>
+    <row r="165" ht="30" customHeight="1">
+      <c r="A165" s="5" t="inlineStr">
+        <is>
+          <t>Vila Galé</t>
+        </is>
+      </c>
+      <c r="B165" s="7" t="inlineStr">
+        <is>
+          <t>Nao</t>
+        </is>
+      </c>
+      <c r="C165" s="7" t="inlineStr"/>
+      <c r="D165" s="5" t="inlineStr"/>
+      <c r="E165" s="5" t="inlineStr">
+        <is>
+          <t>vilagale.com</t>
+        </is>
+      </c>
+      <c r="F165" s="7" t="inlineStr">
+        <is>
+          <t>Golegã</t>
+        </is>
+      </c>
+      <c r="G165" s="7" t="inlineStr">
+        <is>
+          <t>Santarém</t>
+        </is>
+      </c>
+      <c r="H165" s="5" t="inlineStr"/>
+      <c r="I165" s="5" t="inlineStr">
+        <is>
+          <t>Vila Galé Collection Tejo (Quinta da Cardiga) (Em construção)</t>
+        </is>
+      </c>
+      <c r="J165" s="5" t="inlineStr">
+        <is>
+          <t>Fonte: idealista.pt</t>
+        </is>
+      </c>
+      <c r="K165" s="5" t="inlineStr"/>
+      <c r="L165" s="5" t="inlineStr"/>
+      <c r="M165" s="5" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -8925,7 +9090,7 @@
         </is>
       </c>
       <c r="B2" s="9" t="n">
-        <v>161</v>
+        <v>164</v>
       </c>
     </row>
     <row r="3">
@@ -8935,7 +9100,7 @@
         </is>
       </c>
       <c r="B3" s="9" t="n">
-        <v>82</v>
+        <v>84</v>
       </c>
     </row>
     <row r="4">
@@ -8945,7 +9110,7 @@
         </is>
       </c>
       <c r="B4" s="9" t="n">
-        <v>79</v>
+        <v>80</v>
       </c>
     </row>
     <row r="5">
@@ -8965,7 +9130,7 @@
         </is>
       </c>
       <c r="B6" s="9" t="n">
-        <v>110</v>
+        <v>111</v>
       </c>
     </row>
     <row r="7">

</xml_diff>